<commit_message>
Fix dual-tail state persistence in MinusLock v2
</commit_message>
<xml_diff>
--- a/work/MinusLock_SelfCompressing_BigSmall_v2/MinusLock_SelfCompressing_BigSmall_v2.xlsx
+++ b/work/MinusLock_SelfCompressing_BigSmall_v2/MinusLock_SelfCompressing_BigSmall_v2.xlsx
@@ -17,10 +17,10 @@
     <sheet name="Examples" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Calculator'!$A$1:$AZ$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Trend_UP'!$A$1:$AZ$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Trend_DOWN'!$A$1:$AZ$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tests'!$A$1:$H$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Calculator'!$A$1:$BG$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Trend_UP'!$A$1:$BG$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Trend_DOWN'!$A$1:$BG$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tests'!$A$1:$H$55</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -900,7 +900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ11"/>
+  <dimension ref="A1:BG11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -955,6 +955,13 @@
     <col width="18" customWidth="1" min="50" max="50"/>
     <col width="18" customWidth="1" min="51" max="51"/>
     <col width="18" customWidth="1" min="52" max="52"/>
+    <col width="20" customWidth="1" min="53" max="53"/>
+    <col width="20" customWidth="1" min="54" max="54"/>
+    <col width="20" customWidth="1" min="55" max="55"/>
+    <col width="20" customWidth="1" min="56" max="56"/>
+    <col width="20" customWidth="1" min="57" max="57"/>
+    <col width="20" customWidth="1" min="58" max="58"/>
+    <col width="22" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1218,6 +1225,41 @@
           <t>CostsFarClose</t>
         </is>
       </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>ActiveOldFarLot</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>ActiveNewFarLot</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>DualTailTotalLot</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>ManualOldFarCloseLot</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>ManualNewFarCloseLot</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>ManualClosePL</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>ManualAllowNewLevel</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="n">
@@ -1322,15 +1364,15 @@
         <v>0</v>
       </c>
       <c r="AA2" s="12">
-        <f>IF($B2="BLOCKED",$Z2,IF($B2="BIG_SIDE",$Z2+$AX2-$AS2-$AZ2,IF($B2="SMALL_SIDE",$Z2+$S2+$AI2,$Z2+$S2)))</f>
+        <f>IF($B2="BLOCKED",$Z2+$BF2,IF($B2="BIG_SIDE",$Z2+$AX2-$AS2-$AZ2,IF($B2="SMALL_SIDE",$Z2+$S2+$AI2,$Z2+$S2)))</f>
         <v/>
       </c>
       <c r="AB2" s="12">
-        <f>IF($B2="BLOCKED",IF(ROW()=2,0,$AG1+$AJ1),$D2+$G2+$J2)</f>
+        <f>IF($B2="BLOCKED",$BC2,$D2+$G2+$J2)</f>
         <v/>
       </c>
       <c r="AC2" s="12">
-        <f>IF($B2="BLOCKED",$AB2,IF($B2="BIG_SIDE",$W2,$AG2+$AJ2))</f>
+        <f>IF($B2="BLOCKED",$BC2,IF($B2="BIG_SIDE",$W2,IF($AK2=TRUE,$BC2,$AG2)))</f>
         <v/>
       </c>
       <c r="AD2" s="12">
@@ -1342,11 +1384,11 @@
         <v/>
       </c>
       <c r="AF2" s="12">
-        <f>IF($B2="BLOCKED",IF(ROW()=2,$C2,$AF1),IF($B2="SMALL_SIDE",$E2,$C2))</f>
+        <f>IF($B2="BLOCKED",IF($BB2&gt;0,$AF2,$C2),IF($B2="SMALL_SIDE",$E2,$C2))</f>
         <v/>
       </c>
       <c r="AG2" s="12">
-        <f>IF($B2="BLOCKED",IF(ROW()=2,0,$AG1),IF($B2="SMALL_SIDE",$AM2,$W2))</f>
+        <f>IF($B2="BLOCKED",IF($BB2&gt;0,$BB2,$BA2),IF($B2="SMALL_SIDE",$AM2,$W2))</f>
         <v/>
       </c>
       <c r="AH2" s="13" t="inlineStr">
@@ -1382,15 +1424,15 @@
         <v/>
       </c>
       <c r="AP2" s="12">
-        <f>IF(OR($AQ2="DUAL_TAIL",$AQ2="DANGER",$AQ2="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ2="MANUAL_READY",$BG2="YES"),"YES",IF(OR($AQ2="DUAL_TAIL",$AQ2="DANGER",$AQ2="STOP",$AQ2="STOP_CLEARED",$AQ2="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ2" s="12">
-        <f>IF($B2="BLOCKED","STOP",IF($AK2=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G2/$D2,0)&gt;Settings!$B$16,IFERROR($J2/$G2,0)&gt;Settings!$B$17,$AE2&gt;$AD2,$Y2&lt;0,$AG2&gt;$D2*1.0001,$S2&lt;-100),"DANGER",IF(OR(AND($B2="BIG_SIDE",$U2&lt;=0),$S2&lt;=0,$X2=0,$AE2&gt;$AD2*0.95),"WARNING","OK"))))</f>
+        <f>IF($B2="BLOCKED",IF($BC2=0,"STOP_CLEARED",IF(OR(AND($BA2=0,$BB2&gt;0),AND($BA2&gt;0,$BB2=0)),"MANUAL_READY","STOP")),IF($AK2=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G2/$D2,0)&gt;Settings!$B$16,IFERROR($J2/$G2,0)&gt;Settings!$B$17,$AE2&gt;$AD2,$Y2&lt;0,$AG2&gt;$D2*1.0001,$S2&lt;-100),"DANGER",IF(OR(AND($B2="BIG_SIDE",$U2&lt;=0),$S2&lt;=0,$X2=0,$AE2&gt;$AD2*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR2" s="12">
-        <f>IF($B2="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B2="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ2="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B2="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B2="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ2="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS2" s="20">
@@ -1410,7 +1452,7 @@
         <v/>
       </c>
       <c r="AW2" s="12">
-        <f>IF($B2="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B2="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX2" s="12">
@@ -1424,6 +1466,32 @@
       <c r="AZ2" s="12">
         <f>IF($B2="BIG_SIDE",$V2*$AU2,0)</f>
         <v/>
+      </c>
+      <c r="BA2" s="12">
+        <f>IF($AK2=TRUE,MAX(0,$AJ2-$BD2),0)</f>
+        <v/>
+      </c>
+      <c r="BB2" s="12">
+        <f>IF($AK2=TRUE,MAX(0,$AG2-$BE2),0)</f>
+        <v/>
+      </c>
+      <c r="BC2" s="12">
+        <f>$BA2+$BB2</f>
+        <v/>
+      </c>
+      <c r="BD2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -1431,15 +1499,15 @@
         <v>2</v>
       </c>
       <c r="B3" s="13">
-        <f>IF(OR($AP2="NO",$AQ2="DUAL_TAIL",$AQ2="DANGER",$AQ2="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ2="MANUAL_READY",$BG2="YES"),"BIG_SIDE",IF(OR($AP2="NO",$AQ2="DUAL_TAIL",$AQ2="DANGER",$AQ2="STOP",$AQ2="MANUAL_READY",$AQ2="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C3" s="13">
-        <f>IF($B3="BLOCKED",$AF2,IF($AP2="YES",$AF2,$C2))</f>
+        <f>IF($B3="BLOCKED",$AF2,IF(AND($AQ2="MANUAL_READY",$BG2="YES"),$AF2,IF($AP2="YES",$AF2,$C2)))</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF($B3="BLOCKED",0,IF($AP2="YES",MAX(0,$AG2),$D2))</f>
+        <f>IF($B3="BLOCKED",0,IF(AND($AQ2="MANUAL_READY",$BG2="YES"),MAX($BA2,$BB2),IF($AP2="YES",MAX(0,$AG2),$D2)))</f>
         <v/>
       </c>
       <c r="E3" s="12">
@@ -1528,15 +1596,15 @@
         <v/>
       </c>
       <c r="AA3" s="12">
-        <f>IF($B3="BLOCKED",$Z3,IF($B3="BIG_SIDE",$Z3+$AX3-$AS3-$AZ3,IF($B3="SMALL_SIDE",$Z3+$S3+$AI3,$Z3+$S3)))</f>
+        <f>IF($B3="BLOCKED",$Z3+$BF3,IF($B3="BIG_SIDE",$Z3+$AX3-$AS3-$AZ3,IF($B3="SMALL_SIDE",$Z3+$S3+$AI3,$Z3+$S3)))</f>
         <v/>
       </c>
       <c r="AB3" s="12">
-        <f>IF($B3="BLOCKED",IF(ROW()=2,0,$AG2+$AJ2),$D3+$G3+$J3)</f>
+        <f>IF($B3="BLOCKED",$BC3,$D3+$G3+$J3)</f>
         <v/>
       </c>
       <c r="AC3" s="12">
-        <f>IF($B3="BLOCKED",$AB3,IF($B3="BIG_SIDE",$W3,$AG3+$AJ3))</f>
+        <f>IF($B3="BLOCKED",$BC3,IF($B3="BIG_SIDE",$W3,IF($AK3=TRUE,$BC3,$AG3)))</f>
         <v/>
       </c>
       <c r="AD3" s="12">
@@ -1548,11 +1616,11 @@
         <v/>
       </c>
       <c r="AF3" s="12">
-        <f>IF($B3="BLOCKED",IF(ROW()=2,$C3,$AF2),IF($B3="SMALL_SIDE",$E3,$C3))</f>
+        <f>IF($B3="BLOCKED",IF($BB3&gt;0,$AF2,$C3),IF($B3="SMALL_SIDE",$E3,$C3))</f>
         <v/>
       </c>
       <c r="AG3" s="12">
-        <f>IF($B3="BLOCKED",IF(ROW()=2,0,$AG2),IF($B3="SMALL_SIDE",$AM3,$W3))</f>
+        <f>IF($B3="BLOCKED",IF($BB3&gt;0,$BB3,$BA3),IF($B3="SMALL_SIDE",$AM3,$W3))</f>
         <v/>
       </c>
       <c r="AH3" s="13" t="inlineStr">
@@ -1588,15 +1656,15 @@
         <v/>
       </c>
       <c r="AP3" s="12">
-        <f>IF(OR($AQ3="DUAL_TAIL",$AQ3="DANGER",$AQ3="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ3="MANUAL_READY",$BG3="YES"),"YES",IF(OR($AQ3="DUAL_TAIL",$AQ3="DANGER",$AQ3="STOP",$AQ3="STOP_CLEARED",$AQ3="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ3" s="12">
-        <f>IF($B3="BLOCKED","STOP",IF($AK3=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G3/$D3,0)&gt;Settings!$B$16,IFERROR($J3/$G3,0)&gt;Settings!$B$17,$AE3&gt;$AD3,$Y3&lt;0,$AG3&gt;$D3*1.0001,$S3&lt;-100),"DANGER",IF(OR(AND($B3="BIG_SIDE",$U3&lt;=0),$S3&lt;=0,$X3=0,$AE3&gt;$AD3*0.95),"WARNING","OK"))))</f>
+        <f>IF($B3="BLOCKED",IF($BC3=0,"STOP_CLEARED",IF(OR(AND($BA3=0,$BB3&gt;0),AND($BA3&gt;0,$BB3=0)),"MANUAL_READY","STOP")),IF($AK3=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G3/$D3,0)&gt;Settings!$B$16,IFERROR($J3/$G3,0)&gt;Settings!$B$17,$AE3&gt;$AD3,$Y3&lt;0,$AG3&gt;$D3*1.0001,$S3&lt;-100),"DANGER",IF(OR(AND($B3="BIG_SIDE",$U3&lt;=0),$S3&lt;=0,$X3=0,$AE3&gt;$AD3*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR3" s="12">
-        <f>IF($B3="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B3="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ3="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B3="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B3="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ3="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS3" s="20">
@@ -1616,7 +1684,7 @@
         <v/>
       </c>
       <c r="AW3" s="12">
-        <f>IF($B3="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B3="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX3" s="12">
@@ -1630,6 +1698,32 @@
       <c r="AZ3" s="12">
         <f>IF($B3="BIG_SIDE",$V3*$AU3,0)</f>
         <v/>
+      </c>
+      <c r="BA3" s="12">
+        <f>IF($AK3=TRUE,MAX(0,$AJ3-$BD3),IF($B3="BLOCKED",MAX(0,$BA2-$BD3),0))</f>
+        <v/>
+      </c>
+      <c r="BB3" s="12">
+        <f>IF($AK3=TRUE,MAX(0,$AG3-$BE3),IF($B3="BLOCKED",MAX(0,$BB2-$BE3),0))</f>
+        <v/>
+      </c>
+      <c r="BC3" s="12">
+        <f>$BA3+$BB3</f>
+        <v/>
+      </c>
+      <c r="BD3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF3" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG3" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -1637,15 +1731,15 @@
         <v>3</v>
       </c>
       <c r="B4" s="13">
-        <f>IF(OR($AP3="NO",$AQ3="DUAL_TAIL",$AQ3="DANGER",$AQ3="STOP"),"BLOCKED","SMALL_SIDE")</f>
+        <f>IF(AND($AQ3="MANUAL_READY",$BG3="YES"),"SMALL_SIDE",IF(OR($AP3="NO",$AQ3="DUAL_TAIL",$AQ3="DANGER",$AQ3="STOP",$AQ3="MANUAL_READY",$AQ3="STOP_CLEARED"),"BLOCKED","SMALL_SIDE"))</f>
         <v/>
       </c>
       <c r="C4" s="13">
-        <f>IF($B4="BLOCKED",$AF3,IF($AP3="YES",$AF3,$C3))</f>
+        <f>IF($B4="BLOCKED",$AF3,IF(AND($AQ3="MANUAL_READY",$BG3="YES"),$AF3,IF($AP3="YES",$AF3,$C3)))</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>IF($B4="BLOCKED",0,IF($AP3="YES",MAX(0,$AG3),$D3))</f>
+        <f>IF($B4="BLOCKED",0,IF(AND($AQ3="MANUAL_READY",$BG3="YES"),MAX($BA3,$BB3),IF($AP3="YES",MAX(0,$AG3),$D3)))</f>
         <v/>
       </c>
       <c r="E4" s="12">
@@ -1734,15 +1828,15 @@
         <v/>
       </c>
       <c r="AA4" s="12">
-        <f>IF($B4="BLOCKED",$Z4,IF($B4="BIG_SIDE",$Z4+$AX4-$AS4-$AZ4,IF($B4="SMALL_SIDE",$Z4+$S4+$AI4,$Z4+$S4)))</f>
+        <f>IF($B4="BLOCKED",$Z4+$BF4,IF($B4="BIG_SIDE",$Z4+$AX4-$AS4-$AZ4,IF($B4="SMALL_SIDE",$Z4+$S4+$AI4,$Z4+$S4)))</f>
         <v/>
       </c>
       <c r="AB4" s="12">
-        <f>IF($B4="BLOCKED",IF(ROW()=2,0,$AG3+$AJ3),$D4+$G4+$J4)</f>
+        <f>IF($B4="BLOCKED",$BC4,$D4+$G4+$J4)</f>
         <v/>
       </c>
       <c r="AC4" s="12">
-        <f>IF($B4="BLOCKED",$AB4,IF($B4="BIG_SIDE",$W4,$AG4+$AJ4))</f>
+        <f>IF($B4="BLOCKED",$BC4,IF($B4="BIG_SIDE",$W4,IF($AK4=TRUE,$BC4,$AG4)))</f>
         <v/>
       </c>
       <c r="AD4" s="12">
@@ -1754,11 +1848,11 @@
         <v/>
       </c>
       <c r="AF4" s="12">
-        <f>IF($B4="BLOCKED",IF(ROW()=2,$C4,$AF3),IF($B4="SMALL_SIDE",$E4,$C4))</f>
+        <f>IF($B4="BLOCKED",IF($BB4&gt;0,$AF3,$C4),IF($B4="SMALL_SIDE",$E4,$C4))</f>
         <v/>
       </c>
       <c r="AG4" s="12">
-        <f>IF($B4="BLOCKED",IF(ROW()=2,0,$AG3),IF($B4="SMALL_SIDE",$AM4,$W4))</f>
+        <f>IF($B4="BLOCKED",IF($BB4&gt;0,$BB4,$BA4),IF($B4="SMALL_SIDE",$AM4,$W4))</f>
         <v/>
       </c>
       <c r="AH4" s="13" t="inlineStr">
@@ -1794,15 +1888,15 @@
         <v/>
       </c>
       <c r="AP4" s="12">
-        <f>IF(OR($AQ4="DUAL_TAIL",$AQ4="DANGER",$AQ4="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ4="MANUAL_READY",$BG4="YES"),"YES",IF(OR($AQ4="DUAL_TAIL",$AQ4="DANGER",$AQ4="STOP",$AQ4="STOP_CLEARED",$AQ4="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ4" s="12">
-        <f>IF($B4="BLOCKED","STOP",IF($AK4=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G4/$D4,0)&gt;Settings!$B$16,IFERROR($J4/$G4,0)&gt;Settings!$B$17,$AE4&gt;$AD4,$Y4&lt;0,$AG4&gt;$D4*1.0001,$S4&lt;-100),"DANGER",IF(OR(AND($B4="BIG_SIDE",$U4&lt;=0),$S4&lt;=0,$X4=0,$AE4&gt;$AD4*0.95),"WARNING","OK"))))</f>
+        <f>IF($B4="BLOCKED",IF($BC4=0,"STOP_CLEARED",IF(OR(AND($BA4=0,$BB4&gt;0),AND($BA4&gt;0,$BB4=0)),"MANUAL_READY","STOP")),IF($AK4=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G4/$D4,0)&gt;Settings!$B$16,IFERROR($J4/$G4,0)&gt;Settings!$B$17,$AE4&gt;$AD4,$Y4&lt;0,$AG4&gt;$D4*1.0001,$S4&lt;-100),"DANGER",IF(OR(AND($B4="BIG_SIDE",$U4&lt;=0),$S4&lt;=0,$X4=0,$AE4&gt;$AD4*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR4" s="12">
-        <f>IF($B4="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B4="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ4="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B4="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B4="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ4="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS4" s="20">
@@ -1822,7 +1916,7 @@
         <v/>
       </c>
       <c r="AW4" s="12">
-        <f>IF($B4="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B4="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX4" s="12">
@@ -1836,6 +1930,32 @@
       <c r="AZ4" s="12">
         <f>IF($B4="BIG_SIDE",$V4*$AU4,0)</f>
         <v/>
+      </c>
+      <c r="BA4" s="12">
+        <f>IF($AK4=TRUE,MAX(0,$AJ4-$BD4),IF($B4="BLOCKED",MAX(0,$BA3-$BD4),0))</f>
+        <v/>
+      </c>
+      <c r="BB4" s="12">
+        <f>IF($AK4=TRUE,MAX(0,$AG4-$BE4),IF($B4="BLOCKED",MAX(0,$BB3-$BE4),0))</f>
+        <v/>
+      </c>
+      <c r="BC4" s="12">
+        <f>$BA4+$BB4</f>
+        <v/>
+      </c>
+      <c r="BD4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG4" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1843,15 +1963,15 @@
         <v>4</v>
       </c>
       <c r="B5" s="13">
-        <f>IF(OR($AP4="NO",$AQ4="DUAL_TAIL",$AQ4="DANGER",$AQ4="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ4="MANUAL_READY",$BG4="YES"),"BIG_SIDE",IF(OR($AP4="NO",$AQ4="DUAL_TAIL",$AQ4="DANGER",$AQ4="STOP",$AQ4="MANUAL_READY",$AQ4="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C5" s="13">
-        <f>IF($B5="BLOCKED",$AF4,IF($AP4="YES",$AF4,$C4))</f>
+        <f>IF($B5="BLOCKED",$AF4,IF(AND($AQ4="MANUAL_READY",$BG4="YES"),$AF4,IF($AP4="YES",$AF4,$C4)))</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>IF($B5="BLOCKED",0,IF($AP4="YES",MAX(0,$AG4),$D4))</f>
+        <f>IF($B5="BLOCKED",0,IF(AND($AQ4="MANUAL_READY",$BG4="YES"),MAX($BA4,$BB4),IF($AP4="YES",MAX(0,$AG4),$D4)))</f>
         <v/>
       </c>
       <c r="E5" s="12">
@@ -1940,15 +2060,15 @@
         <v/>
       </c>
       <c r="AA5" s="12">
-        <f>IF($B5="BLOCKED",$Z5,IF($B5="BIG_SIDE",$Z5+$AX5-$AS5-$AZ5,IF($B5="SMALL_SIDE",$Z5+$S5+$AI5,$Z5+$S5)))</f>
+        <f>IF($B5="BLOCKED",$Z5+$BF5,IF($B5="BIG_SIDE",$Z5+$AX5-$AS5-$AZ5,IF($B5="SMALL_SIDE",$Z5+$S5+$AI5,$Z5+$S5)))</f>
         <v/>
       </c>
       <c r="AB5" s="12">
-        <f>IF($B5="BLOCKED",IF(ROW()=2,0,$AG4+$AJ4),$D5+$G5+$J5)</f>
+        <f>IF($B5="BLOCKED",$BC5,$D5+$G5+$J5)</f>
         <v/>
       </c>
       <c r="AC5" s="12">
-        <f>IF($B5="BLOCKED",$AB5,IF($B5="BIG_SIDE",$W5,$AG5+$AJ5))</f>
+        <f>IF($B5="BLOCKED",$BC5,IF($B5="BIG_SIDE",$W5,IF($AK5=TRUE,$BC5,$AG5)))</f>
         <v/>
       </c>
       <c r="AD5" s="12">
@@ -1960,11 +2080,11 @@
         <v/>
       </c>
       <c r="AF5" s="12">
-        <f>IF($B5="BLOCKED",IF(ROW()=2,$C5,$AF4),IF($B5="SMALL_SIDE",$E5,$C5))</f>
+        <f>IF($B5="BLOCKED",IF($BB5&gt;0,$AF4,$C5),IF($B5="SMALL_SIDE",$E5,$C5))</f>
         <v/>
       </c>
       <c r="AG5" s="12">
-        <f>IF($B5="BLOCKED",IF(ROW()=2,0,$AG4),IF($B5="SMALL_SIDE",$AM5,$W5))</f>
+        <f>IF($B5="BLOCKED",IF($BB5&gt;0,$BB5,$BA5),IF($B5="SMALL_SIDE",$AM5,$W5))</f>
         <v/>
       </c>
       <c r="AH5" s="13" t="inlineStr">
@@ -2000,15 +2120,15 @@
         <v/>
       </c>
       <c r="AP5" s="12">
-        <f>IF(OR($AQ5="DUAL_TAIL",$AQ5="DANGER",$AQ5="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ5="MANUAL_READY",$BG5="YES"),"YES",IF(OR($AQ5="DUAL_TAIL",$AQ5="DANGER",$AQ5="STOP",$AQ5="STOP_CLEARED",$AQ5="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ5" s="12">
-        <f>IF($B5="BLOCKED","STOP",IF($AK5=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G5/$D5,0)&gt;Settings!$B$16,IFERROR($J5/$G5,0)&gt;Settings!$B$17,$AE5&gt;$AD5,$Y5&lt;0,$AG5&gt;$D5*1.0001,$S5&lt;-100),"DANGER",IF(OR(AND($B5="BIG_SIDE",$U5&lt;=0),$S5&lt;=0,$X5=0,$AE5&gt;$AD5*0.95),"WARNING","OK"))))</f>
+        <f>IF($B5="BLOCKED",IF($BC5=0,"STOP_CLEARED",IF(OR(AND($BA5=0,$BB5&gt;0),AND($BA5&gt;0,$BB5=0)),"MANUAL_READY","STOP")),IF($AK5=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G5/$D5,0)&gt;Settings!$B$16,IFERROR($J5/$G5,0)&gt;Settings!$B$17,$AE5&gt;$AD5,$Y5&lt;0,$AG5&gt;$D5*1.0001,$S5&lt;-100),"DANGER",IF(OR(AND($B5="BIG_SIDE",$U5&lt;=0),$S5&lt;=0,$X5=0,$AE5&gt;$AD5*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR5" s="12">
-        <f>IF($B5="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B5="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ5="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B5="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B5="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ5="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS5" s="20">
@@ -2028,7 +2148,7 @@
         <v/>
       </c>
       <c r="AW5" s="12">
-        <f>IF($B5="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B5="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX5" s="12">
@@ -2042,6 +2162,32 @@
       <c r="AZ5" s="12">
         <f>IF($B5="BIG_SIDE",$V5*$AU5,0)</f>
         <v/>
+      </c>
+      <c r="BA5" s="12">
+        <f>IF($AK5=TRUE,MAX(0,$AJ5-$BD5),IF($B5="BLOCKED",MAX(0,$BA4-$BD5),0))</f>
+        <v/>
+      </c>
+      <c r="BB5" s="12">
+        <f>IF($AK5=TRUE,MAX(0,$AG5-$BE5),IF($B5="BLOCKED",MAX(0,$BB4-$BE5),0))</f>
+        <v/>
+      </c>
+      <c r="BC5" s="12">
+        <f>$BA5+$BB5</f>
+        <v/>
+      </c>
+      <c r="BD5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF5" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG5" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -2049,15 +2195,15 @@
         <v>5</v>
       </c>
       <c r="B6" s="13">
-        <f>IF(OR($AP5="NO",$AQ5="DUAL_TAIL",$AQ5="DANGER",$AQ5="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ5="MANUAL_READY",$BG5="YES"),"BIG_SIDE",IF(OR($AP5="NO",$AQ5="DUAL_TAIL",$AQ5="DANGER",$AQ5="STOP",$AQ5="MANUAL_READY",$AQ5="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C6" s="13">
-        <f>IF($B6="BLOCKED",$AF5,IF($AP5="YES",$AF5,$C5))</f>
+        <f>IF($B6="BLOCKED",$AF5,IF(AND($AQ5="MANUAL_READY",$BG5="YES"),$AF5,IF($AP5="YES",$AF5,$C5)))</f>
         <v/>
       </c>
       <c r="D6" s="13">
-        <f>IF($B6="BLOCKED",0,IF($AP5="YES",MAX(0,$AG5),$D5))</f>
+        <f>IF($B6="BLOCKED",0,IF(AND($AQ5="MANUAL_READY",$BG5="YES"),MAX($BA5,$BB5),IF($AP5="YES",MAX(0,$AG5),$D5)))</f>
         <v/>
       </c>
       <c r="E6" s="12">
@@ -2146,15 +2292,15 @@
         <v/>
       </c>
       <c r="AA6" s="12">
-        <f>IF($B6="BLOCKED",$Z6,IF($B6="BIG_SIDE",$Z6+$AX6-$AS6-$AZ6,IF($B6="SMALL_SIDE",$Z6+$S6+$AI6,$Z6+$S6)))</f>
+        <f>IF($B6="BLOCKED",$Z6+$BF6,IF($B6="BIG_SIDE",$Z6+$AX6-$AS6-$AZ6,IF($B6="SMALL_SIDE",$Z6+$S6+$AI6,$Z6+$S6)))</f>
         <v/>
       </c>
       <c r="AB6" s="12">
-        <f>IF($B6="BLOCKED",IF(ROW()=2,0,$AG5+$AJ5),$D6+$G6+$J6)</f>
+        <f>IF($B6="BLOCKED",$BC6,$D6+$G6+$J6)</f>
         <v/>
       </c>
       <c r="AC6" s="12">
-        <f>IF($B6="BLOCKED",$AB6,IF($B6="BIG_SIDE",$W6,$AG6+$AJ6))</f>
+        <f>IF($B6="BLOCKED",$BC6,IF($B6="BIG_SIDE",$W6,IF($AK6=TRUE,$BC6,$AG6)))</f>
         <v/>
       </c>
       <c r="AD6" s="12">
@@ -2166,11 +2312,11 @@
         <v/>
       </c>
       <c r="AF6" s="12">
-        <f>IF($B6="BLOCKED",IF(ROW()=2,$C6,$AF5),IF($B6="SMALL_SIDE",$E6,$C6))</f>
+        <f>IF($B6="BLOCKED",IF($BB6&gt;0,$AF5,$C6),IF($B6="SMALL_SIDE",$E6,$C6))</f>
         <v/>
       </c>
       <c r="AG6" s="12">
-        <f>IF($B6="BLOCKED",IF(ROW()=2,0,$AG5),IF($B6="SMALL_SIDE",$AM6,$W6))</f>
+        <f>IF($B6="BLOCKED",IF($BB6&gt;0,$BB6,$BA6),IF($B6="SMALL_SIDE",$AM6,$W6))</f>
         <v/>
       </c>
       <c r="AH6" s="13" t="inlineStr">
@@ -2206,15 +2352,15 @@
         <v/>
       </c>
       <c r="AP6" s="12">
-        <f>IF(OR($AQ6="DUAL_TAIL",$AQ6="DANGER",$AQ6="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ6="MANUAL_READY",$BG6="YES"),"YES",IF(OR($AQ6="DUAL_TAIL",$AQ6="DANGER",$AQ6="STOP",$AQ6="STOP_CLEARED",$AQ6="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ6" s="12">
-        <f>IF($B6="BLOCKED","STOP",IF($AK6=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G6/$D6,0)&gt;Settings!$B$16,IFERROR($J6/$G6,0)&gt;Settings!$B$17,$AE6&gt;$AD6,$Y6&lt;0,$AG6&gt;$D6*1.0001,$S6&lt;-100),"DANGER",IF(OR(AND($B6="BIG_SIDE",$U6&lt;=0),$S6&lt;=0,$X6=0,$AE6&gt;$AD6*0.95),"WARNING","OK"))))</f>
+        <f>IF($B6="BLOCKED",IF($BC6=0,"STOP_CLEARED",IF(OR(AND($BA6=0,$BB6&gt;0),AND($BA6&gt;0,$BB6=0)),"MANUAL_READY","STOP")),IF($AK6=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G6/$D6,0)&gt;Settings!$B$16,IFERROR($J6/$G6,0)&gt;Settings!$B$17,$AE6&gt;$AD6,$Y6&lt;0,$AG6&gt;$D6*1.0001,$S6&lt;-100),"DANGER",IF(OR(AND($B6="BIG_SIDE",$U6&lt;=0),$S6&lt;=0,$X6=0,$AE6&gt;$AD6*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR6" s="12">
-        <f>IF($B6="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B6="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ6="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B6="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B6="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ6="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS6" s="20">
@@ -2234,7 +2380,7 @@
         <v/>
       </c>
       <c r="AW6" s="12">
-        <f>IF($B6="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B6="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX6" s="12">
@@ -2248,6 +2394,32 @@
       <c r="AZ6" s="12">
         <f>IF($B6="BIG_SIDE",$V6*$AU6,0)</f>
         <v/>
+      </c>
+      <c r="BA6" s="12">
+        <f>IF($AK6=TRUE,MAX(0,$AJ6-$BD6),IF($B6="BLOCKED",MAX(0,$BA5-$BD6),0))</f>
+        <v/>
+      </c>
+      <c r="BB6" s="12">
+        <f>IF($AK6=TRUE,MAX(0,$AG6-$BE6),IF($B6="BLOCKED",MAX(0,$BB5-$BE6),0))</f>
+        <v/>
+      </c>
+      <c r="BC6" s="12">
+        <f>$BA6+$BB6</f>
+        <v/>
+      </c>
+      <c r="BD6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF6" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG6" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -2255,15 +2427,15 @@
         <v>6</v>
       </c>
       <c r="B7" s="13">
-        <f>IF(OR($AP6="NO",$AQ6="DUAL_TAIL",$AQ6="DANGER",$AQ6="STOP"),"BLOCKED","SMALL_SIDE")</f>
+        <f>IF(AND($AQ6="MANUAL_READY",$BG6="YES"),"SMALL_SIDE",IF(OR($AP6="NO",$AQ6="DUAL_TAIL",$AQ6="DANGER",$AQ6="STOP",$AQ6="MANUAL_READY",$AQ6="STOP_CLEARED"),"BLOCKED","SMALL_SIDE"))</f>
         <v/>
       </c>
       <c r="C7" s="13">
-        <f>IF($B7="BLOCKED",$AF6,IF($AP6="YES",$AF6,$C6))</f>
+        <f>IF($B7="BLOCKED",$AF6,IF(AND($AQ6="MANUAL_READY",$BG6="YES"),$AF6,IF($AP6="YES",$AF6,$C6)))</f>
         <v/>
       </c>
       <c r="D7" s="13">
-        <f>IF($B7="BLOCKED",0,IF($AP6="YES",MAX(0,$AG6),$D6))</f>
+        <f>IF($B7="BLOCKED",0,IF(AND($AQ6="MANUAL_READY",$BG6="YES"),MAX($BA6,$BB6),IF($AP6="YES",MAX(0,$AG6),$D6)))</f>
         <v/>
       </c>
       <c r="E7" s="12">
@@ -2352,15 +2524,15 @@
         <v/>
       </c>
       <c r="AA7" s="12">
-        <f>IF($B7="BLOCKED",$Z7,IF($B7="BIG_SIDE",$Z7+$AX7-$AS7-$AZ7,IF($B7="SMALL_SIDE",$Z7+$S7+$AI7,$Z7+$S7)))</f>
+        <f>IF($B7="BLOCKED",$Z7+$BF7,IF($B7="BIG_SIDE",$Z7+$AX7-$AS7-$AZ7,IF($B7="SMALL_SIDE",$Z7+$S7+$AI7,$Z7+$S7)))</f>
         <v/>
       </c>
       <c r="AB7" s="12">
-        <f>IF($B7="BLOCKED",IF(ROW()=2,0,$AG6+$AJ6),$D7+$G7+$J7)</f>
+        <f>IF($B7="BLOCKED",$BC7,$D7+$G7+$J7)</f>
         <v/>
       </c>
       <c r="AC7" s="12">
-        <f>IF($B7="BLOCKED",$AB7,IF($B7="BIG_SIDE",$W7,$AG7+$AJ7))</f>
+        <f>IF($B7="BLOCKED",$BC7,IF($B7="BIG_SIDE",$W7,IF($AK7=TRUE,$BC7,$AG7)))</f>
         <v/>
       </c>
       <c r="AD7" s="12">
@@ -2372,11 +2544,11 @@
         <v/>
       </c>
       <c r="AF7" s="12">
-        <f>IF($B7="BLOCKED",IF(ROW()=2,$C7,$AF6),IF($B7="SMALL_SIDE",$E7,$C7))</f>
+        <f>IF($B7="BLOCKED",IF($BB7&gt;0,$AF6,$C7),IF($B7="SMALL_SIDE",$E7,$C7))</f>
         <v/>
       </c>
       <c r="AG7" s="12">
-        <f>IF($B7="BLOCKED",IF(ROW()=2,0,$AG6),IF($B7="SMALL_SIDE",$AM7,$W7))</f>
+        <f>IF($B7="BLOCKED",IF($BB7&gt;0,$BB7,$BA7),IF($B7="SMALL_SIDE",$AM7,$W7))</f>
         <v/>
       </c>
       <c r="AH7" s="13" t="inlineStr">
@@ -2412,15 +2584,15 @@
         <v/>
       </c>
       <c r="AP7" s="12">
-        <f>IF(OR($AQ7="DUAL_TAIL",$AQ7="DANGER",$AQ7="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ7="MANUAL_READY",$BG7="YES"),"YES",IF(OR($AQ7="DUAL_TAIL",$AQ7="DANGER",$AQ7="STOP",$AQ7="STOP_CLEARED",$AQ7="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ7" s="12">
-        <f>IF($B7="BLOCKED","STOP",IF($AK7=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G7/$D7,0)&gt;Settings!$B$16,IFERROR($J7/$G7,0)&gt;Settings!$B$17,$AE7&gt;$AD7,$Y7&lt;0,$AG7&gt;$D7*1.0001,$S7&lt;-100),"DANGER",IF(OR(AND($B7="BIG_SIDE",$U7&lt;=0),$S7&lt;=0,$X7=0,$AE7&gt;$AD7*0.95),"WARNING","OK"))))</f>
+        <f>IF($B7="BLOCKED",IF($BC7=0,"STOP_CLEARED",IF(OR(AND($BA7=0,$BB7&gt;0),AND($BA7&gt;0,$BB7=0)),"MANUAL_READY","STOP")),IF($AK7=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G7/$D7,0)&gt;Settings!$B$16,IFERROR($J7/$G7,0)&gt;Settings!$B$17,$AE7&gt;$AD7,$Y7&lt;0,$AG7&gt;$D7*1.0001,$S7&lt;-100),"DANGER",IF(OR(AND($B7="BIG_SIDE",$U7&lt;=0),$S7&lt;=0,$X7=0,$AE7&gt;$AD7*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR7" s="12">
-        <f>IF($B7="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B7="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ7="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B7="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B7="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ7="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS7" s="20">
@@ -2440,7 +2612,7 @@
         <v/>
       </c>
       <c r="AW7" s="12">
-        <f>IF($B7="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B7="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX7" s="12">
@@ -2454,6 +2626,32 @@
       <c r="AZ7" s="12">
         <f>IF($B7="BIG_SIDE",$V7*$AU7,0)</f>
         <v/>
+      </c>
+      <c r="BA7" s="12">
+        <f>IF($AK7=TRUE,MAX(0,$AJ7-$BD7),IF($B7="BLOCKED",MAX(0,$BA6-$BD7),0))</f>
+        <v/>
+      </c>
+      <c r="BB7" s="12">
+        <f>IF($AK7=TRUE,MAX(0,$AG7-$BE7),IF($B7="BLOCKED",MAX(0,$BB6-$BE7),0))</f>
+        <v/>
+      </c>
+      <c r="BC7" s="12">
+        <f>$BA7+$BB7</f>
+        <v/>
+      </c>
+      <c r="BD7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF7" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG7" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -2461,15 +2659,15 @@
         <v>7</v>
       </c>
       <c r="B8" s="13">
-        <f>IF(OR($AP7="NO",$AQ7="DUAL_TAIL",$AQ7="DANGER",$AQ7="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ7="MANUAL_READY",$BG7="YES"),"BIG_SIDE",IF(OR($AP7="NO",$AQ7="DUAL_TAIL",$AQ7="DANGER",$AQ7="STOP",$AQ7="MANUAL_READY",$AQ7="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C8" s="13">
-        <f>IF($B8="BLOCKED",$AF7,IF($AP7="YES",$AF7,$C7))</f>
+        <f>IF($B8="BLOCKED",$AF7,IF(AND($AQ7="MANUAL_READY",$BG7="YES"),$AF7,IF($AP7="YES",$AF7,$C7)))</f>
         <v/>
       </c>
       <c r="D8" s="13">
-        <f>IF($B8="BLOCKED",0,IF($AP7="YES",MAX(0,$AG7),$D7))</f>
+        <f>IF($B8="BLOCKED",0,IF(AND($AQ7="MANUAL_READY",$BG7="YES"),MAX($BA7,$BB7),IF($AP7="YES",MAX(0,$AG7),$D7)))</f>
         <v/>
       </c>
       <c r="E8" s="12">
@@ -2558,15 +2756,15 @@
         <v/>
       </c>
       <c r="AA8" s="12">
-        <f>IF($B8="BLOCKED",$Z8,IF($B8="BIG_SIDE",$Z8+$AX8-$AS8-$AZ8,IF($B8="SMALL_SIDE",$Z8+$S8+$AI8,$Z8+$S8)))</f>
+        <f>IF($B8="BLOCKED",$Z8+$BF8,IF($B8="BIG_SIDE",$Z8+$AX8-$AS8-$AZ8,IF($B8="SMALL_SIDE",$Z8+$S8+$AI8,$Z8+$S8)))</f>
         <v/>
       </c>
       <c r="AB8" s="12">
-        <f>IF($B8="BLOCKED",IF(ROW()=2,0,$AG7+$AJ7),$D8+$G8+$J8)</f>
+        <f>IF($B8="BLOCKED",$BC8,$D8+$G8+$J8)</f>
         <v/>
       </c>
       <c r="AC8" s="12">
-        <f>IF($B8="BLOCKED",$AB8,IF($B8="BIG_SIDE",$W8,$AG8+$AJ8))</f>
+        <f>IF($B8="BLOCKED",$BC8,IF($B8="BIG_SIDE",$W8,IF($AK8=TRUE,$BC8,$AG8)))</f>
         <v/>
       </c>
       <c r="AD8" s="12">
@@ -2578,11 +2776,11 @@
         <v/>
       </c>
       <c r="AF8" s="12">
-        <f>IF($B8="BLOCKED",IF(ROW()=2,$C8,$AF7),IF($B8="SMALL_SIDE",$E8,$C8))</f>
+        <f>IF($B8="BLOCKED",IF($BB8&gt;0,$AF7,$C8),IF($B8="SMALL_SIDE",$E8,$C8))</f>
         <v/>
       </c>
       <c r="AG8" s="12">
-        <f>IF($B8="BLOCKED",IF(ROW()=2,0,$AG7),IF($B8="SMALL_SIDE",$AM8,$W8))</f>
+        <f>IF($B8="BLOCKED",IF($BB8&gt;0,$BB8,$BA8),IF($B8="SMALL_SIDE",$AM8,$W8))</f>
         <v/>
       </c>
       <c r="AH8" s="13" t="inlineStr">
@@ -2618,15 +2816,15 @@
         <v/>
       </c>
       <c r="AP8" s="12">
-        <f>IF(OR($AQ8="DUAL_TAIL",$AQ8="DANGER",$AQ8="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ8="MANUAL_READY",$BG8="YES"),"YES",IF(OR($AQ8="DUAL_TAIL",$AQ8="DANGER",$AQ8="STOP",$AQ8="STOP_CLEARED",$AQ8="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ8" s="12">
-        <f>IF($B8="BLOCKED","STOP",IF($AK8=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G8/$D8,0)&gt;Settings!$B$16,IFERROR($J8/$G8,0)&gt;Settings!$B$17,$AE8&gt;$AD8,$Y8&lt;0,$AG8&gt;$D8*1.0001,$S8&lt;-100),"DANGER",IF(OR(AND($B8="BIG_SIDE",$U8&lt;=0),$S8&lt;=0,$X8=0,$AE8&gt;$AD8*0.95),"WARNING","OK"))))</f>
+        <f>IF($B8="BLOCKED",IF($BC8=0,"STOP_CLEARED",IF(OR(AND($BA8=0,$BB8&gt;0),AND($BA8&gt;0,$BB8=0)),"MANUAL_READY","STOP")),IF($AK8=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G8/$D8,0)&gt;Settings!$B$16,IFERROR($J8/$G8,0)&gt;Settings!$B$17,$AE8&gt;$AD8,$Y8&lt;0,$AG8&gt;$D8*1.0001,$S8&lt;-100),"DANGER",IF(OR(AND($B8="BIG_SIDE",$U8&lt;=0),$S8&lt;=0,$X8=0,$AE8&gt;$AD8*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR8" s="12">
-        <f>IF($B8="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B8="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ8="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B8="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B8="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ8="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS8" s="20">
@@ -2646,7 +2844,7 @@
         <v/>
       </c>
       <c r="AW8" s="12">
-        <f>IF($B8="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B8="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX8" s="12">
@@ -2660,6 +2858,32 @@
       <c r="AZ8" s="12">
         <f>IF($B8="BIG_SIDE",$V8*$AU8,0)</f>
         <v/>
+      </c>
+      <c r="BA8" s="12">
+        <f>IF($AK8=TRUE,MAX(0,$AJ8-$BD8),IF($B8="BLOCKED",MAX(0,$BA7-$BD8),0))</f>
+        <v/>
+      </c>
+      <c r="BB8" s="12">
+        <f>IF($AK8=TRUE,MAX(0,$AG8-$BE8),IF($B8="BLOCKED",MAX(0,$BB7-$BE8),0))</f>
+        <v/>
+      </c>
+      <c r="BC8" s="12">
+        <f>$BA8+$BB8</f>
+        <v/>
+      </c>
+      <c r="BD8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF8" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG8" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -2667,15 +2891,15 @@
         <v>8</v>
       </c>
       <c r="B9" s="13">
-        <f>IF(OR($AP8="NO",$AQ8="DUAL_TAIL",$AQ8="DANGER",$AQ8="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ8="MANUAL_READY",$BG8="YES"),"BIG_SIDE",IF(OR($AP8="NO",$AQ8="DUAL_TAIL",$AQ8="DANGER",$AQ8="STOP",$AQ8="MANUAL_READY",$AQ8="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C9" s="13">
-        <f>IF($B9="BLOCKED",$AF8,IF($AP8="YES",$AF8,$C8))</f>
+        <f>IF($B9="BLOCKED",$AF8,IF(AND($AQ8="MANUAL_READY",$BG8="YES"),$AF8,IF($AP8="YES",$AF8,$C8)))</f>
         <v/>
       </c>
       <c r="D9" s="13">
-        <f>IF($B9="BLOCKED",0,IF($AP8="YES",MAX(0,$AG8),$D8))</f>
+        <f>IF($B9="BLOCKED",0,IF(AND($AQ8="MANUAL_READY",$BG8="YES"),MAX($BA8,$BB8),IF($AP8="YES",MAX(0,$AG8),$D8)))</f>
         <v/>
       </c>
       <c r="E9" s="12">
@@ -2764,15 +2988,15 @@
         <v/>
       </c>
       <c r="AA9" s="12">
-        <f>IF($B9="BLOCKED",$Z9,IF($B9="BIG_SIDE",$Z9+$AX9-$AS9-$AZ9,IF($B9="SMALL_SIDE",$Z9+$S9+$AI9,$Z9+$S9)))</f>
+        <f>IF($B9="BLOCKED",$Z9+$BF9,IF($B9="BIG_SIDE",$Z9+$AX9-$AS9-$AZ9,IF($B9="SMALL_SIDE",$Z9+$S9+$AI9,$Z9+$S9)))</f>
         <v/>
       </c>
       <c r="AB9" s="12">
-        <f>IF($B9="BLOCKED",IF(ROW()=2,0,$AG8+$AJ8),$D9+$G9+$J9)</f>
+        <f>IF($B9="BLOCKED",$BC9,$D9+$G9+$J9)</f>
         <v/>
       </c>
       <c r="AC9" s="12">
-        <f>IF($B9="BLOCKED",$AB9,IF($B9="BIG_SIDE",$W9,$AG9+$AJ9))</f>
+        <f>IF($B9="BLOCKED",$BC9,IF($B9="BIG_SIDE",$W9,IF($AK9=TRUE,$BC9,$AG9)))</f>
         <v/>
       </c>
       <c r="AD9" s="12">
@@ -2784,11 +3008,11 @@
         <v/>
       </c>
       <c r="AF9" s="12">
-        <f>IF($B9="BLOCKED",IF(ROW()=2,$C9,$AF8),IF($B9="SMALL_SIDE",$E9,$C9))</f>
+        <f>IF($B9="BLOCKED",IF($BB9&gt;0,$AF8,$C9),IF($B9="SMALL_SIDE",$E9,$C9))</f>
         <v/>
       </c>
       <c r="AG9" s="12">
-        <f>IF($B9="BLOCKED",IF(ROW()=2,0,$AG8),IF($B9="SMALL_SIDE",$AM9,$W9))</f>
+        <f>IF($B9="BLOCKED",IF($BB9&gt;0,$BB9,$BA9),IF($B9="SMALL_SIDE",$AM9,$W9))</f>
         <v/>
       </c>
       <c r="AH9" s="13" t="inlineStr">
@@ -2824,15 +3048,15 @@
         <v/>
       </c>
       <c r="AP9" s="12">
-        <f>IF(OR($AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ9="MANUAL_READY",$BG9="YES"),"YES",IF(OR($AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP",$AQ9="STOP_CLEARED",$AQ9="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ9" s="12">
-        <f>IF($B9="BLOCKED","STOP",IF($AK9=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G9/$D9,0)&gt;Settings!$B$16,IFERROR($J9/$G9,0)&gt;Settings!$B$17,$AE9&gt;$AD9,$Y9&lt;0,$AG9&gt;$D9*1.0001,$S9&lt;-100),"DANGER",IF(OR(AND($B9="BIG_SIDE",$U9&lt;=0),$S9&lt;=0,$X9=0,$AE9&gt;$AD9*0.95),"WARNING","OK"))))</f>
+        <f>IF($B9="BLOCKED",IF($BC9=0,"STOP_CLEARED",IF(OR(AND($BA9=0,$BB9&gt;0),AND($BA9&gt;0,$BB9=0)),"MANUAL_READY","STOP")),IF($AK9=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G9/$D9,0)&gt;Settings!$B$16,IFERROR($J9/$G9,0)&gt;Settings!$B$17,$AE9&gt;$AD9,$Y9&lt;0,$AG9&gt;$D9*1.0001,$S9&lt;-100),"DANGER",IF(OR(AND($B9="BIG_SIDE",$U9&lt;=0),$S9&lt;=0,$X9=0,$AE9&gt;$AD9*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR9" s="12">
-        <f>IF($B9="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B9="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ9="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B9="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B9="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ9="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS9" s="20">
@@ -2852,7 +3076,7 @@
         <v/>
       </c>
       <c r="AW9" s="12">
-        <f>IF($B9="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B9="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX9" s="12">
@@ -2866,6 +3090,32 @@
       <c r="AZ9" s="12">
         <f>IF($B9="BIG_SIDE",$V9*$AU9,0)</f>
         <v/>
+      </c>
+      <c r="BA9" s="12">
+        <f>IF($AK9=TRUE,MAX(0,$AJ9-$BD9),IF($B9="BLOCKED",MAX(0,$BA8-$BD9),0))</f>
+        <v/>
+      </c>
+      <c r="BB9" s="12">
+        <f>IF($AK9=TRUE,MAX(0,$AG9-$BE9),IF($B9="BLOCKED",MAX(0,$BB8-$BE9),0))</f>
+        <v/>
+      </c>
+      <c r="BC9" s="12">
+        <f>$BA9+$BB9</f>
+        <v/>
+      </c>
+      <c r="BD9" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE9" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF9" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG9" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -2873,15 +3123,15 @@
         <v>9</v>
       </c>
       <c r="B10" s="13">
-        <f>IF(OR($AP9="NO",$AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ9="MANUAL_READY",$BG9="YES"),"BIG_SIDE",IF(OR($AP9="NO",$AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP",$AQ9="MANUAL_READY",$AQ9="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C10" s="13">
-        <f>IF($B10="BLOCKED",$AF9,IF($AP9="YES",$AF9,$C9))</f>
+        <f>IF($B10="BLOCKED",$AF9,IF(AND($AQ9="MANUAL_READY",$BG9="YES"),$AF9,IF($AP9="YES",$AF9,$C9)))</f>
         <v/>
       </c>
       <c r="D10" s="13">
-        <f>IF($B10="BLOCKED",0,IF($AP9="YES",MAX(0,$AG9),$D9))</f>
+        <f>IF($B10="BLOCKED",0,IF(AND($AQ9="MANUAL_READY",$BG9="YES"),MAX($BA9,$BB9),IF($AP9="YES",MAX(0,$AG9),$D9)))</f>
         <v/>
       </c>
       <c r="E10" s="12">
@@ -2970,15 +3220,15 @@
         <v/>
       </c>
       <c r="AA10" s="12">
-        <f>IF($B10="BLOCKED",$Z10,IF($B10="BIG_SIDE",$Z10+$AX10-$AS10-$AZ10,IF($B10="SMALL_SIDE",$Z10+$S10+$AI10,$Z10+$S10)))</f>
+        <f>IF($B10="BLOCKED",$Z10+$BF10,IF($B10="BIG_SIDE",$Z10+$AX10-$AS10-$AZ10,IF($B10="SMALL_SIDE",$Z10+$S10+$AI10,$Z10+$S10)))</f>
         <v/>
       </c>
       <c r="AB10" s="12">
-        <f>IF($B10="BLOCKED",IF(ROW()=2,0,$AG9+$AJ9),$D10+$G10+$J10)</f>
+        <f>IF($B10="BLOCKED",$BC10,$D10+$G10+$J10)</f>
         <v/>
       </c>
       <c r="AC10" s="12">
-        <f>IF($B10="BLOCKED",$AB10,IF($B10="BIG_SIDE",$W10,$AG10+$AJ10))</f>
+        <f>IF($B10="BLOCKED",$BC10,IF($B10="BIG_SIDE",$W10,IF($AK10=TRUE,$BC10,$AG10)))</f>
         <v/>
       </c>
       <c r="AD10" s="12">
@@ -2990,11 +3240,11 @@
         <v/>
       </c>
       <c r="AF10" s="12">
-        <f>IF($B10="BLOCKED",IF(ROW()=2,$C10,$AF9),IF($B10="SMALL_SIDE",$E10,$C10))</f>
+        <f>IF($B10="BLOCKED",IF($BB10&gt;0,$AF9,$C10),IF($B10="SMALL_SIDE",$E10,$C10))</f>
         <v/>
       </c>
       <c r="AG10" s="12">
-        <f>IF($B10="BLOCKED",IF(ROW()=2,0,$AG9),IF($B10="SMALL_SIDE",$AM10,$W10))</f>
+        <f>IF($B10="BLOCKED",IF($BB10&gt;0,$BB10,$BA10),IF($B10="SMALL_SIDE",$AM10,$W10))</f>
         <v/>
       </c>
       <c r="AH10" s="13" t="inlineStr">
@@ -3030,15 +3280,15 @@
         <v/>
       </c>
       <c r="AP10" s="12">
-        <f>IF(OR($AQ10="DUAL_TAIL",$AQ10="DANGER",$AQ10="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ10="MANUAL_READY",$BG10="YES"),"YES",IF(OR($AQ10="DUAL_TAIL",$AQ10="DANGER",$AQ10="STOP",$AQ10="STOP_CLEARED",$AQ10="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ10" s="12">
-        <f>IF($B10="BLOCKED","STOP",IF($AK10=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G10/$D10,0)&gt;Settings!$B$16,IFERROR($J10/$G10,0)&gt;Settings!$B$17,$AE10&gt;$AD10,$Y10&lt;0,$AG10&gt;$D10*1.0001,$S10&lt;-100),"DANGER",IF(OR(AND($B10="BIG_SIDE",$U10&lt;=0),$S10&lt;=0,$X10=0,$AE10&gt;$AD10*0.95),"WARNING","OK"))))</f>
+        <f>IF($B10="BLOCKED",IF($BC10=0,"STOP_CLEARED",IF(OR(AND($BA10=0,$BB10&gt;0),AND($BA10&gt;0,$BB10=0)),"MANUAL_READY","STOP")),IF($AK10=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G10/$D10,0)&gt;Settings!$B$16,IFERROR($J10/$G10,0)&gt;Settings!$B$17,$AE10&gt;$AD10,$Y10&lt;0,$AG10&gt;$D10*1.0001,$S10&lt;-100),"DANGER",IF(OR(AND($B10="BIG_SIDE",$U10&lt;=0),$S10&lt;=0,$X10=0,$AE10&gt;$AD10*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR10" s="12">
-        <f>IF($B10="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B10="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ10="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B10="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B10="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ10="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS10" s="20">
@@ -3058,7 +3308,7 @@
         <v/>
       </c>
       <c r="AW10" s="12">
-        <f>IF($B10="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B10="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX10" s="12">
@@ -3072,6 +3322,32 @@
       <c r="AZ10" s="12">
         <f>IF($B10="BIG_SIDE",$V10*$AU10,0)</f>
         <v/>
+      </c>
+      <c r="BA10" s="12">
+        <f>IF($AK10=TRUE,MAX(0,$AJ10-$BD10),IF($B10="BLOCKED",MAX(0,$BA9-$BD10),0))</f>
+        <v/>
+      </c>
+      <c r="BB10" s="12">
+        <f>IF($AK10=TRUE,MAX(0,$AG10-$BE10),IF($B10="BLOCKED",MAX(0,$BB9-$BE10),0))</f>
+        <v/>
+      </c>
+      <c r="BC10" s="12">
+        <f>$BA10+$BB10</f>
+        <v/>
+      </c>
+      <c r="BD10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF10" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG10" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -3079,15 +3355,15 @@
         <v>10</v>
       </c>
       <c r="B11" s="13">
-        <f>IF(OR($AP10="NO",$AQ10="DUAL_TAIL",$AQ10="DANGER",$AQ10="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ10="MANUAL_READY",$BG10="YES"),"BIG_SIDE",IF(OR($AP10="NO",$AQ10="DUAL_TAIL",$AQ10="DANGER",$AQ10="STOP",$AQ10="MANUAL_READY",$AQ10="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C11" s="13">
-        <f>IF($B11="BLOCKED",$AF10,IF($AP10="YES",$AF10,$C10))</f>
+        <f>IF($B11="BLOCKED",$AF10,IF(AND($AQ10="MANUAL_READY",$BG10="YES"),$AF10,IF($AP10="YES",$AF10,$C10)))</f>
         <v/>
       </c>
       <c r="D11" s="13">
-        <f>IF($B11="BLOCKED",0,IF($AP10="YES",MAX(0,$AG10),$D10))</f>
+        <f>IF($B11="BLOCKED",0,IF(AND($AQ10="MANUAL_READY",$BG10="YES"),MAX($BA10,$BB10),IF($AP10="YES",MAX(0,$AG10),$D10)))</f>
         <v/>
       </c>
       <c r="E11" s="12">
@@ -3176,15 +3452,15 @@
         <v/>
       </c>
       <c r="AA11" s="12">
-        <f>IF($B11="BLOCKED",$Z11,IF($B11="BIG_SIDE",$Z11+$AX11-$AS11-$AZ11,IF($B11="SMALL_SIDE",$Z11+$S11+$AI11,$Z11+$S11)))</f>
+        <f>IF($B11="BLOCKED",$Z11+$BF11,IF($B11="BIG_SIDE",$Z11+$AX11-$AS11-$AZ11,IF($B11="SMALL_SIDE",$Z11+$S11+$AI11,$Z11+$S11)))</f>
         <v/>
       </c>
       <c r="AB11" s="12">
-        <f>IF($B11="BLOCKED",IF(ROW()=2,0,$AG10+$AJ10),$D11+$G11+$J11)</f>
+        <f>IF($B11="BLOCKED",$BC11,$D11+$G11+$J11)</f>
         <v/>
       </c>
       <c r="AC11" s="12">
-        <f>IF($B11="BLOCKED",$AB11,IF($B11="BIG_SIDE",$W11,$AG11+$AJ11))</f>
+        <f>IF($B11="BLOCKED",$BC11,IF($B11="BIG_SIDE",$W11,IF($AK11=TRUE,$BC11,$AG11)))</f>
         <v/>
       </c>
       <c r="AD11" s="12">
@@ -3196,11 +3472,11 @@
         <v/>
       </c>
       <c r="AF11" s="12">
-        <f>IF($B11="BLOCKED",IF(ROW()=2,$C11,$AF10),IF($B11="SMALL_SIDE",$E11,$C11))</f>
+        <f>IF($B11="BLOCKED",IF($BB11&gt;0,$AF10,$C11),IF($B11="SMALL_SIDE",$E11,$C11))</f>
         <v/>
       </c>
       <c r="AG11" s="12">
-        <f>IF($B11="BLOCKED",IF(ROW()=2,0,$AG10),IF($B11="SMALL_SIDE",$AM11,$W11))</f>
+        <f>IF($B11="BLOCKED",IF($BB11&gt;0,$BB11,$BA11),IF($B11="SMALL_SIDE",$AM11,$W11))</f>
         <v/>
       </c>
       <c r="AH11" s="13" t="inlineStr">
@@ -3236,15 +3512,15 @@
         <v/>
       </c>
       <c r="AP11" s="12">
-        <f>IF(OR($AQ11="DUAL_TAIL",$AQ11="DANGER",$AQ11="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ11="MANUAL_READY",$BG11="YES"),"YES",IF(OR($AQ11="DUAL_TAIL",$AQ11="DANGER",$AQ11="STOP",$AQ11="STOP_CLEARED",$AQ11="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ11" s="12">
-        <f>IF($B11="BLOCKED","STOP",IF($AK11=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G11/$D11,0)&gt;Settings!$B$16,IFERROR($J11/$G11,0)&gt;Settings!$B$17,$AE11&gt;$AD11,$Y11&lt;0,$AG11&gt;$D11*1.0001,$S11&lt;-100),"DANGER",IF(OR(AND($B11="BIG_SIDE",$U11&lt;=0),$S11&lt;=0,$X11=0,$AE11&gt;$AD11*0.95),"WARNING","OK"))))</f>
+        <f>IF($B11="BLOCKED",IF($BC11=0,"STOP_CLEARED",IF(OR(AND($BA11=0,$BB11&gt;0),AND($BA11&gt;0,$BB11=0)),"MANUAL_READY","STOP")),IF($AK11=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G11/$D11,0)&gt;Settings!$B$16,IFERROR($J11/$G11,0)&gt;Settings!$B$17,$AE11&gt;$AD11,$Y11&lt;0,$AG11&gt;$D11*1.0001,$S11&lt;-100),"DANGER",IF(OR(AND($B11="BIG_SIDE",$U11&lt;=0),$S11&lt;=0,$X11=0,$AE11&gt;$AD11*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR11" s="12">
-        <f>IF($B11="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B11="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ11="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B11="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B11="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ11="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS11" s="20">
@@ -3264,7 +3540,7 @@
         <v/>
       </c>
       <c r="AW11" s="12">
-        <f>IF($B11="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B11="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX11" s="12">
@@ -3279,9 +3555,35 @@
         <f>IF($B11="BIG_SIDE",$V11*$AU11,0)</f>
         <v/>
       </c>
+      <c r="BA11" s="12">
+        <f>IF($AK11=TRUE,MAX(0,$AJ11-$BD11),IF($B11="BLOCKED",MAX(0,$BA10-$BD11),0))</f>
+        <v/>
+      </c>
+      <c r="BB11" s="12">
+        <f>IF($AK11=TRUE,MAX(0,$AG11-$BE11),IF($B11="BLOCKED",MAX(0,$BB10-$BE11),0))</f>
+        <v/>
+      </c>
+      <c r="BC11" s="12">
+        <f>$BA11+$BB11</f>
+        <v/>
+      </c>
+      <c r="BD11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF11" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG11" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AZ11"/>
+  <autoFilter ref="A1:BG11"/>
   <conditionalFormatting sqref="AQ2:AQ11">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AQ2="WARNING"</formula>
@@ -3317,7 +3619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ11"/>
+  <dimension ref="A1:BG11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3372,6 +3674,13 @@
     <col width="18" customWidth="1" min="50" max="50"/>
     <col width="18" customWidth="1" min="51" max="51"/>
     <col width="18" customWidth="1" min="52" max="52"/>
+    <col width="20" customWidth="1" min="53" max="53"/>
+    <col width="20" customWidth="1" min="54" max="54"/>
+    <col width="20" customWidth="1" min="55" max="55"/>
+    <col width="20" customWidth="1" min="56" max="56"/>
+    <col width="20" customWidth="1" min="57" max="57"/>
+    <col width="20" customWidth="1" min="58" max="58"/>
+    <col width="22" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3635,6 +3944,41 @@
           <t>CostsFarClose</t>
         </is>
       </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>ActiveOldFarLot</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>ActiveNewFarLot</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>DualTailTotalLot</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>ManualOldFarCloseLot</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>ManualNewFarCloseLot</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>ManualClosePL</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>ManualAllowNewLevel</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="n">
@@ -3739,15 +4083,15 @@
         <v>0</v>
       </c>
       <c r="AA2" s="12">
-        <f>IF($B2="BLOCKED",$Z2,IF($B2="BIG_SIDE",$Z2+$AX2-$AS2-$AZ2,IF($B2="SMALL_SIDE",$Z2+$S2+$AI2,$Z2+$S2)))</f>
+        <f>IF($B2="BLOCKED",$Z2+$BF2,IF($B2="BIG_SIDE",$Z2+$AX2-$AS2-$AZ2,IF($B2="SMALL_SIDE",$Z2+$S2+$AI2,$Z2+$S2)))</f>
         <v/>
       </c>
       <c r="AB2" s="12">
-        <f>IF($B2="BLOCKED",IF(ROW()=2,0,$AG1+$AJ1),$D2+$G2+$J2)</f>
+        <f>IF($B2="BLOCKED",$BC2,$D2+$G2+$J2)</f>
         <v/>
       </c>
       <c r="AC2" s="12">
-        <f>IF($B2="BLOCKED",$AB2,IF($B2="BIG_SIDE",$W2,$AG2+$AJ2))</f>
+        <f>IF($B2="BLOCKED",$BC2,IF($B2="BIG_SIDE",$W2,IF($AK2=TRUE,$BC2,$AG2)))</f>
         <v/>
       </c>
       <c r="AD2" s="12">
@@ -3759,11 +4103,11 @@
         <v/>
       </c>
       <c r="AF2" s="12">
-        <f>IF($B2="BLOCKED",IF(ROW()=2,$C2,$AF1),IF($B2="SMALL_SIDE",$E2,$C2))</f>
+        <f>IF($B2="BLOCKED",IF($BB2&gt;0,$AF2,$C2),IF($B2="SMALL_SIDE",$E2,$C2))</f>
         <v/>
       </c>
       <c r="AG2" s="12">
-        <f>IF($B2="BLOCKED",IF(ROW()=2,0,$AG1),IF($B2="SMALL_SIDE",$AM2,$W2))</f>
+        <f>IF($B2="BLOCKED",IF($BB2&gt;0,$BB2,$BA2),IF($B2="SMALL_SIDE",$AM2,$W2))</f>
         <v/>
       </c>
       <c r="AH2" s="13" t="inlineStr">
@@ -3799,15 +4143,15 @@
         <v/>
       </c>
       <c r="AP2" s="12">
-        <f>IF(OR($AQ2="DUAL_TAIL",$AQ2="DANGER",$AQ2="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ2="MANUAL_READY",$BG2="YES"),"YES",IF(OR($AQ2="DUAL_TAIL",$AQ2="DANGER",$AQ2="STOP",$AQ2="STOP_CLEARED",$AQ2="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ2" s="12">
-        <f>IF($B2="BLOCKED","STOP",IF($AK2=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G2/$D2,0)&gt;Settings!$B$16,IFERROR($J2/$G2,0)&gt;Settings!$B$17,$AE2&gt;$AD2,$Y2&lt;0,$AG2&gt;$D2*1.0001,$S2&lt;-100),"DANGER",IF(OR(AND($B2="BIG_SIDE",$U2&lt;=0),$S2&lt;=0,$X2=0,$AE2&gt;$AD2*0.95),"WARNING","OK"))))</f>
+        <f>IF($B2="BLOCKED",IF($BC2=0,"STOP_CLEARED",IF(OR(AND($BA2=0,$BB2&gt;0),AND($BA2&gt;0,$BB2=0)),"MANUAL_READY","STOP")),IF($AK2=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G2/$D2,0)&gt;Settings!$B$16,IFERROR($J2/$G2,0)&gt;Settings!$B$17,$AE2&gt;$AD2,$Y2&lt;0,$AG2&gt;$D2*1.0001,$S2&lt;-100),"DANGER",IF(OR(AND($B2="BIG_SIDE",$U2&lt;=0),$S2&lt;=0,$X2=0,$AE2&gt;$AD2*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR2" s="12">
-        <f>IF($B2="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B2="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ2="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B2="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B2="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ2="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS2" s="20">
@@ -3827,7 +4171,7 @@
         <v/>
       </c>
       <c r="AW2" s="12">
-        <f>IF($B2="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B2="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX2" s="12">
@@ -3841,6 +4185,32 @@
       <c r="AZ2" s="12">
         <f>IF($B2="BIG_SIDE",$V2*$AU2,0)</f>
         <v/>
+      </c>
+      <c r="BA2" s="12">
+        <f>IF($AK2=TRUE,MAX(0,$AJ2-$BD2),0)</f>
+        <v/>
+      </c>
+      <c r="BB2" s="12">
+        <f>IF($AK2=TRUE,MAX(0,$AG2-$BE2),0)</f>
+        <v/>
+      </c>
+      <c r="BC2" s="12">
+        <f>$BA2+$BB2</f>
+        <v/>
+      </c>
+      <c r="BD2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -3848,15 +4218,15 @@
         <v>2</v>
       </c>
       <c r="B3" s="13">
-        <f>IF(OR($AP2="NO",$AQ2="DUAL_TAIL",$AQ2="DANGER",$AQ2="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ2="MANUAL_READY",$BG2="YES"),"BIG_SIDE",IF(OR($AP2="NO",$AQ2="DUAL_TAIL",$AQ2="DANGER",$AQ2="STOP",$AQ2="MANUAL_READY",$AQ2="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C3" s="13">
-        <f>IF($B3="BLOCKED",$AF2,IF($AP2="YES",$AF2,$C2))</f>
+        <f>IF($B3="BLOCKED",$AF2,IF(AND($AQ2="MANUAL_READY",$BG2="YES"),$AF2,IF($AP2="YES",$AF2,$C2)))</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF($B3="BLOCKED",0,IF($AP2="YES",MAX(0,$AG2),$D2))</f>
+        <f>IF($B3="BLOCKED",0,IF(AND($AQ2="MANUAL_READY",$BG2="YES"),MAX($BA2,$BB2),IF($AP2="YES",MAX(0,$AG2),$D2)))</f>
         <v/>
       </c>
       <c r="E3" s="12">
@@ -3945,15 +4315,15 @@
         <v/>
       </c>
       <c r="AA3" s="12">
-        <f>IF($B3="BLOCKED",$Z3,IF($B3="BIG_SIDE",$Z3+$AX3-$AS3-$AZ3,IF($B3="SMALL_SIDE",$Z3+$S3+$AI3,$Z3+$S3)))</f>
+        <f>IF($B3="BLOCKED",$Z3+$BF3,IF($B3="BIG_SIDE",$Z3+$AX3-$AS3-$AZ3,IF($B3="SMALL_SIDE",$Z3+$S3+$AI3,$Z3+$S3)))</f>
         <v/>
       </c>
       <c r="AB3" s="12">
-        <f>IF($B3="BLOCKED",IF(ROW()=2,0,$AG2+$AJ2),$D3+$G3+$J3)</f>
+        <f>IF($B3="BLOCKED",$BC3,$D3+$G3+$J3)</f>
         <v/>
       </c>
       <c r="AC3" s="12">
-        <f>IF($B3="BLOCKED",$AB3,IF($B3="BIG_SIDE",$W3,$AG3+$AJ3))</f>
+        <f>IF($B3="BLOCKED",$BC3,IF($B3="BIG_SIDE",$W3,IF($AK3=TRUE,$BC3,$AG3)))</f>
         <v/>
       </c>
       <c r="AD3" s="12">
@@ -3965,11 +4335,11 @@
         <v/>
       </c>
       <c r="AF3" s="12">
-        <f>IF($B3="BLOCKED",IF(ROW()=2,$C3,$AF2),IF($B3="SMALL_SIDE",$E3,$C3))</f>
+        <f>IF($B3="BLOCKED",IF($BB3&gt;0,$AF2,$C3),IF($B3="SMALL_SIDE",$E3,$C3))</f>
         <v/>
       </c>
       <c r="AG3" s="12">
-        <f>IF($B3="BLOCKED",IF(ROW()=2,0,$AG2),IF($B3="SMALL_SIDE",$AM3,$W3))</f>
+        <f>IF($B3="BLOCKED",IF($BB3&gt;0,$BB3,$BA3),IF($B3="SMALL_SIDE",$AM3,$W3))</f>
         <v/>
       </c>
       <c r="AH3" s="13" t="inlineStr">
@@ -4005,15 +4375,15 @@
         <v/>
       </c>
       <c r="AP3" s="12">
-        <f>IF(OR($AQ3="DUAL_TAIL",$AQ3="DANGER",$AQ3="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ3="MANUAL_READY",$BG3="YES"),"YES",IF(OR($AQ3="DUAL_TAIL",$AQ3="DANGER",$AQ3="STOP",$AQ3="STOP_CLEARED",$AQ3="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ3" s="12">
-        <f>IF($B3="BLOCKED","STOP",IF($AK3=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G3/$D3,0)&gt;Settings!$B$16,IFERROR($J3/$G3,0)&gt;Settings!$B$17,$AE3&gt;$AD3,$Y3&lt;0,$AG3&gt;$D3*1.0001,$S3&lt;-100),"DANGER",IF(OR(AND($B3="BIG_SIDE",$U3&lt;=0),$S3&lt;=0,$X3=0,$AE3&gt;$AD3*0.95),"WARNING","OK"))))</f>
+        <f>IF($B3="BLOCKED",IF($BC3=0,"STOP_CLEARED",IF(OR(AND($BA3=0,$BB3&gt;0),AND($BA3&gt;0,$BB3=0)),"MANUAL_READY","STOP")),IF($AK3=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G3/$D3,0)&gt;Settings!$B$16,IFERROR($J3/$G3,0)&gt;Settings!$B$17,$AE3&gt;$AD3,$Y3&lt;0,$AG3&gt;$D3*1.0001,$S3&lt;-100),"DANGER",IF(OR(AND($B3="BIG_SIDE",$U3&lt;=0),$S3&lt;=0,$X3=0,$AE3&gt;$AD3*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR3" s="12">
-        <f>IF($B3="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B3="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ3="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B3="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B3="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ3="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS3" s="20">
@@ -4033,7 +4403,7 @@
         <v/>
       </c>
       <c r="AW3" s="12">
-        <f>IF($B3="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B3="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX3" s="12">
@@ -4047,6 +4417,32 @@
       <c r="AZ3" s="12">
         <f>IF($B3="BIG_SIDE",$V3*$AU3,0)</f>
         <v/>
+      </c>
+      <c r="BA3" s="12">
+        <f>IF($AK3=TRUE,MAX(0,$AJ3-$BD3),IF($B3="BLOCKED",MAX(0,$BA2-$BD3),0))</f>
+        <v/>
+      </c>
+      <c r="BB3" s="12">
+        <f>IF($AK3=TRUE,MAX(0,$AG3-$BE3),IF($B3="BLOCKED",MAX(0,$BB2-$BE3),0))</f>
+        <v/>
+      </c>
+      <c r="BC3" s="12">
+        <f>$BA3+$BB3</f>
+        <v/>
+      </c>
+      <c r="BD3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF3" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG3" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -4054,15 +4450,15 @@
         <v>3</v>
       </c>
       <c r="B4" s="13">
-        <f>IF(OR($AP3="NO",$AQ3="DUAL_TAIL",$AQ3="DANGER",$AQ3="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ3="MANUAL_READY",$BG3="YES"),"BIG_SIDE",IF(OR($AP3="NO",$AQ3="DUAL_TAIL",$AQ3="DANGER",$AQ3="STOP",$AQ3="MANUAL_READY",$AQ3="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C4" s="13">
-        <f>IF($B4="BLOCKED",$AF3,IF($AP3="YES",$AF3,$C3))</f>
+        <f>IF($B4="BLOCKED",$AF3,IF(AND($AQ3="MANUAL_READY",$BG3="YES"),$AF3,IF($AP3="YES",$AF3,$C3)))</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>IF($B4="BLOCKED",0,IF($AP3="YES",MAX(0,$AG3),$D3))</f>
+        <f>IF($B4="BLOCKED",0,IF(AND($AQ3="MANUAL_READY",$BG3="YES"),MAX($BA3,$BB3),IF($AP3="YES",MAX(0,$AG3),$D3)))</f>
         <v/>
       </c>
       <c r="E4" s="12">
@@ -4151,15 +4547,15 @@
         <v/>
       </c>
       <c r="AA4" s="12">
-        <f>IF($B4="BLOCKED",$Z4,IF($B4="BIG_SIDE",$Z4+$AX4-$AS4-$AZ4,IF($B4="SMALL_SIDE",$Z4+$S4+$AI4,$Z4+$S4)))</f>
+        <f>IF($B4="BLOCKED",$Z4+$BF4,IF($B4="BIG_SIDE",$Z4+$AX4-$AS4-$AZ4,IF($B4="SMALL_SIDE",$Z4+$S4+$AI4,$Z4+$S4)))</f>
         <v/>
       </c>
       <c r="AB4" s="12">
-        <f>IF($B4="BLOCKED",IF(ROW()=2,0,$AG3+$AJ3),$D4+$G4+$J4)</f>
+        <f>IF($B4="BLOCKED",$BC4,$D4+$G4+$J4)</f>
         <v/>
       </c>
       <c r="AC4" s="12">
-        <f>IF($B4="BLOCKED",$AB4,IF($B4="BIG_SIDE",$W4,$AG4+$AJ4))</f>
+        <f>IF($B4="BLOCKED",$BC4,IF($B4="BIG_SIDE",$W4,IF($AK4=TRUE,$BC4,$AG4)))</f>
         <v/>
       </c>
       <c r="AD4" s="12">
@@ -4171,11 +4567,11 @@
         <v/>
       </c>
       <c r="AF4" s="12">
-        <f>IF($B4="BLOCKED",IF(ROW()=2,$C4,$AF3),IF($B4="SMALL_SIDE",$E4,$C4))</f>
+        <f>IF($B4="BLOCKED",IF($BB4&gt;0,$AF3,$C4),IF($B4="SMALL_SIDE",$E4,$C4))</f>
         <v/>
       </c>
       <c r="AG4" s="12">
-        <f>IF($B4="BLOCKED",IF(ROW()=2,0,$AG3),IF($B4="SMALL_SIDE",$AM4,$W4))</f>
+        <f>IF($B4="BLOCKED",IF($BB4&gt;0,$BB4,$BA4),IF($B4="SMALL_SIDE",$AM4,$W4))</f>
         <v/>
       </c>
       <c r="AH4" s="13" t="inlineStr">
@@ -4211,15 +4607,15 @@
         <v/>
       </c>
       <c r="AP4" s="12">
-        <f>IF(OR($AQ4="DUAL_TAIL",$AQ4="DANGER",$AQ4="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ4="MANUAL_READY",$BG4="YES"),"YES",IF(OR($AQ4="DUAL_TAIL",$AQ4="DANGER",$AQ4="STOP",$AQ4="STOP_CLEARED",$AQ4="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ4" s="12">
-        <f>IF($B4="BLOCKED","STOP",IF($AK4=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G4/$D4,0)&gt;Settings!$B$16,IFERROR($J4/$G4,0)&gt;Settings!$B$17,$AE4&gt;$AD4,$Y4&lt;0,$AG4&gt;$D4*1.0001,$S4&lt;-100),"DANGER",IF(OR(AND($B4="BIG_SIDE",$U4&lt;=0),$S4&lt;=0,$X4=0,$AE4&gt;$AD4*0.95),"WARNING","OK"))))</f>
+        <f>IF($B4="BLOCKED",IF($BC4=0,"STOP_CLEARED",IF(OR(AND($BA4=0,$BB4&gt;0),AND($BA4&gt;0,$BB4=0)),"MANUAL_READY","STOP")),IF($AK4=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G4/$D4,0)&gt;Settings!$B$16,IFERROR($J4/$G4,0)&gt;Settings!$B$17,$AE4&gt;$AD4,$Y4&lt;0,$AG4&gt;$D4*1.0001,$S4&lt;-100),"DANGER",IF(OR(AND($B4="BIG_SIDE",$U4&lt;=0),$S4&lt;=0,$X4=0,$AE4&gt;$AD4*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR4" s="12">
-        <f>IF($B4="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B4="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ4="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B4="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B4="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ4="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS4" s="20">
@@ -4239,7 +4635,7 @@
         <v/>
       </c>
       <c r="AW4" s="12">
-        <f>IF($B4="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B4="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX4" s="12">
@@ -4253,6 +4649,32 @@
       <c r="AZ4" s="12">
         <f>IF($B4="BIG_SIDE",$V4*$AU4,0)</f>
         <v/>
+      </c>
+      <c r="BA4" s="12">
+        <f>IF($AK4=TRUE,MAX(0,$AJ4-$BD4),IF($B4="BLOCKED",MAX(0,$BA3-$BD4),0))</f>
+        <v/>
+      </c>
+      <c r="BB4" s="12">
+        <f>IF($AK4=TRUE,MAX(0,$AG4-$BE4),IF($B4="BLOCKED",MAX(0,$BB3-$BE4),0))</f>
+        <v/>
+      </c>
+      <c r="BC4" s="12">
+        <f>$BA4+$BB4</f>
+        <v/>
+      </c>
+      <c r="BD4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG4" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -4260,15 +4682,15 @@
         <v>4</v>
       </c>
       <c r="B5" s="13">
-        <f>IF(OR($AP4="NO",$AQ4="DUAL_TAIL",$AQ4="DANGER",$AQ4="STOP"),"BLOCKED","SMALL_SIDE")</f>
+        <f>IF(AND($AQ4="MANUAL_READY",$BG4="YES"),"SMALL_SIDE",IF(OR($AP4="NO",$AQ4="DUAL_TAIL",$AQ4="DANGER",$AQ4="STOP",$AQ4="MANUAL_READY",$AQ4="STOP_CLEARED"),"BLOCKED","SMALL_SIDE"))</f>
         <v/>
       </c>
       <c r="C5" s="13">
-        <f>IF($B5="BLOCKED",$AF4,IF($AP4="YES",$AF4,$C4))</f>
+        <f>IF($B5="BLOCKED",$AF4,IF(AND($AQ4="MANUAL_READY",$BG4="YES"),$AF4,IF($AP4="YES",$AF4,$C4)))</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>IF($B5="BLOCKED",0,IF($AP4="YES",MAX(0,$AG4),$D4))</f>
+        <f>IF($B5="BLOCKED",0,IF(AND($AQ4="MANUAL_READY",$BG4="YES"),MAX($BA4,$BB4),IF($AP4="YES",MAX(0,$AG4),$D4)))</f>
         <v/>
       </c>
       <c r="E5" s="12">
@@ -4357,15 +4779,15 @@
         <v/>
       </c>
       <c r="AA5" s="12">
-        <f>IF($B5="BLOCKED",$Z5,IF($B5="BIG_SIDE",$Z5+$AX5-$AS5-$AZ5,IF($B5="SMALL_SIDE",$Z5+$S5+$AI5,$Z5+$S5)))</f>
+        <f>IF($B5="BLOCKED",$Z5+$BF5,IF($B5="BIG_SIDE",$Z5+$AX5-$AS5-$AZ5,IF($B5="SMALL_SIDE",$Z5+$S5+$AI5,$Z5+$S5)))</f>
         <v/>
       </c>
       <c r="AB5" s="12">
-        <f>IF($B5="BLOCKED",IF(ROW()=2,0,$AG4+$AJ4),$D5+$G5+$J5)</f>
+        <f>IF($B5="BLOCKED",$BC5,$D5+$G5+$J5)</f>
         <v/>
       </c>
       <c r="AC5" s="12">
-        <f>IF($B5="BLOCKED",$AB5,IF($B5="BIG_SIDE",$W5,$AG5+$AJ5))</f>
+        <f>IF($B5="BLOCKED",$BC5,IF($B5="BIG_SIDE",$W5,IF($AK5=TRUE,$BC5,$AG5)))</f>
         <v/>
       </c>
       <c r="AD5" s="12">
@@ -4377,11 +4799,11 @@
         <v/>
       </c>
       <c r="AF5" s="12">
-        <f>IF($B5="BLOCKED",IF(ROW()=2,$C5,$AF4),IF($B5="SMALL_SIDE",$E5,$C5))</f>
+        <f>IF($B5="BLOCKED",IF($BB5&gt;0,$AF4,$C5),IF($B5="SMALL_SIDE",$E5,$C5))</f>
         <v/>
       </c>
       <c r="AG5" s="12">
-        <f>IF($B5="BLOCKED",IF(ROW()=2,0,$AG4),IF($B5="SMALL_SIDE",$AM5,$W5))</f>
+        <f>IF($B5="BLOCKED",IF($BB5&gt;0,$BB5,$BA5),IF($B5="SMALL_SIDE",$AM5,$W5))</f>
         <v/>
       </c>
       <c r="AH5" s="13" t="inlineStr">
@@ -4417,15 +4839,15 @@
         <v/>
       </c>
       <c r="AP5" s="12">
-        <f>IF(OR($AQ5="DUAL_TAIL",$AQ5="DANGER",$AQ5="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ5="MANUAL_READY",$BG5="YES"),"YES",IF(OR($AQ5="DUAL_TAIL",$AQ5="DANGER",$AQ5="STOP",$AQ5="STOP_CLEARED",$AQ5="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ5" s="12">
-        <f>IF($B5="BLOCKED","STOP",IF($AK5=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G5/$D5,0)&gt;Settings!$B$16,IFERROR($J5/$G5,0)&gt;Settings!$B$17,$AE5&gt;$AD5,$Y5&lt;0,$AG5&gt;$D5*1.0001,$S5&lt;-100),"DANGER",IF(OR(AND($B5="BIG_SIDE",$U5&lt;=0),$S5&lt;=0,$X5=0,$AE5&gt;$AD5*0.95),"WARNING","OK"))))</f>
+        <f>IF($B5="BLOCKED",IF($BC5=0,"STOP_CLEARED",IF(OR(AND($BA5=0,$BB5&gt;0),AND($BA5&gt;0,$BB5=0)),"MANUAL_READY","STOP")),IF($AK5=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G5/$D5,0)&gt;Settings!$B$16,IFERROR($J5/$G5,0)&gt;Settings!$B$17,$AE5&gt;$AD5,$Y5&lt;0,$AG5&gt;$D5*1.0001,$S5&lt;-100),"DANGER",IF(OR(AND($B5="BIG_SIDE",$U5&lt;=0),$S5&lt;=0,$X5=0,$AE5&gt;$AD5*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR5" s="12">
-        <f>IF($B5="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B5="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ5="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B5="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B5="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ5="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS5" s="20">
@@ -4445,7 +4867,7 @@
         <v/>
       </c>
       <c r="AW5" s="12">
-        <f>IF($B5="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B5="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX5" s="12">
@@ -4459,6 +4881,32 @@
       <c r="AZ5" s="12">
         <f>IF($B5="BIG_SIDE",$V5*$AU5,0)</f>
         <v/>
+      </c>
+      <c r="BA5" s="12">
+        <f>IF($AK5=TRUE,MAX(0,$AJ5-$BD5),IF($B5="BLOCKED",MAX(0,$BA4-$BD5),0))</f>
+        <v/>
+      </c>
+      <c r="BB5" s="12">
+        <f>IF($AK5=TRUE,MAX(0,$AG5-$BE5),IF($B5="BLOCKED",MAX(0,$BB4-$BE5),0))</f>
+        <v/>
+      </c>
+      <c r="BC5" s="12">
+        <f>$BA5+$BB5</f>
+        <v/>
+      </c>
+      <c r="BD5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF5" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG5" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -4466,15 +4914,15 @@
         <v>5</v>
       </c>
       <c r="B6" s="13">
-        <f>IF(OR($AP5="NO",$AQ5="DUAL_TAIL",$AQ5="DANGER",$AQ5="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ5="MANUAL_READY",$BG5="YES"),"BIG_SIDE",IF(OR($AP5="NO",$AQ5="DUAL_TAIL",$AQ5="DANGER",$AQ5="STOP",$AQ5="MANUAL_READY",$AQ5="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C6" s="13">
-        <f>IF($B6="BLOCKED",$AF5,IF($AP5="YES",$AF5,$C5))</f>
+        <f>IF($B6="BLOCKED",$AF5,IF(AND($AQ5="MANUAL_READY",$BG5="YES"),$AF5,IF($AP5="YES",$AF5,$C5)))</f>
         <v/>
       </c>
       <c r="D6" s="13">
-        <f>IF($B6="BLOCKED",0,IF($AP5="YES",MAX(0,$AG5),$D5))</f>
+        <f>IF($B6="BLOCKED",0,IF(AND($AQ5="MANUAL_READY",$BG5="YES"),MAX($BA5,$BB5),IF($AP5="YES",MAX(0,$AG5),$D5)))</f>
         <v/>
       </c>
       <c r="E6" s="12">
@@ -4563,15 +5011,15 @@
         <v/>
       </c>
       <c r="AA6" s="12">
-        <f>IF($B6="BLOCKED",$Z6,IF($B6="BIG_SIDE",$Z6+$AX6-$AS6-$AZ6,IF($B6="SMALL_SIDE",$Z6+$S6+$AI6,$Z6+$S6)))</f>
+        <f>IF($B6="BLOCKED",$Z6+$BF6,IF($B6="BIG_SIDE",$Z6+$AX6-$AS6-$AZ6,IF($B6="SMALL_SIDE",$Z6+$S6+$AI6,$Z6+$S6)))</f>
         <v/>
       </c>
       <c r="AB6" s="12">
-        <f>IF($B6="BLOCKED",IF(ROW()=2,0,$AG5+$AJ5),$D6+$G6+$J6)</f>
+        <f>IF($B6="BLOCKED",$BC6,$D6+$G6+$J6)</f>
         <v/>
       </c>
       <c r="AC6" s="12">
-        <f>IF($B6="BLOCKED",$AB6,IF($B6="BIG_SIDE",$W6,$AG6+$AJ6))</f>
+        <f>IF($B6="BLOCKED",$BC6,IF($B6="BIG_SIDE",$W6,IF($AK6=TRUE,$BC6,$AG6)))</f>
         <v/>
       </c>
       <c r="AD6" s="12">
@@ -4583,11 +5031,11 @@
         <v/>
       </c>
       <c r="AF6" s="12">
-        <f>IF($B6="BLOCKED",IF(ROW()=2,$C6,$AF5),IF($B6="SMALL_SIDE",$E6,$C6))</f>
+        <f>IF($B6="BLOCKED",IF($BB6&gt;0,$AF5,$C6),IF($B6="SMALL_SIDE",$E6,$C6))</f>
         <v/>
       </c>
       <c r="AG6" s="12">
-        <f>IF($B6="BLOCKED",IF(ROW()=2,0,$AG5),IF($B6="SMALL_SIDE",$AM6,$W6))</f>
+        <f>IF($B6="BLOCKED",IF($BB6&gt;0,$BB6,$BA6),IF($B6="SMALL_SIDE",$AM6,$W6))</f>
         <v/>
       </c>
       <c r="AH6" s="13" t="inlineStr">
@@ -4623,15 +5071,15 @@
         <v/>
       </c>
       <c r="AP6" s="12">
-        <f>IF(OR($AQ6="DUAL_TAIL",$AQ6="DANGER",$AQ6="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ6="MANUAL_READY",$BG6="YES"),"YES",IF(OR($AQ6="DUAL_TAIL",$AQ6="DANGER",$AQ6="STOP",$AQ6="STOP_CLEARED",$AQ6="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ6" s="12">
-        <f>IF($B6="BLOCKED","STOP",IF($AK6=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G6/$D6,0)&gt;Settings!$B$16,IFERROR($J6/$G6,0)&gt;Settings!$B$17,$AE6&gt;$AD6,$Y6&lt;0,$AG6&gt;$D6*1.0001,$S6&lt;-100),"DANGER",IF(OR(AND($B6="BIG_SIDE",$U6&lt;=0),$S6&lt;=0,$X6=0,$AE6&gt;$AD6*0.95),"WARNING","OK"))))</f>
+        <f>IF($B6="BLOCKED",IF($BC6=0,"STOP_CLEARED",IF(OR(AND($BA6=0,$BB6&gt;0),AND($BA6&gt;0,$BB6=0)),"MANUAL_READY","STOP")),IF($AK6=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G6/$D6,0)&gt;Settings!$B$16,IFERROR($J6/$G6,0)&gt;Settings!$B$17,$AE6&gt;$AD6,$Y6&lt;0,$AG6&gt;$D6*1.0001,$S6&lt;-100),"DANGER",IF(OR(AND($B6="BIG_SIDE",$U6&lt;=0),$S6&lt;=0,$X6=0,$AE6&gt;$AD6*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR6" s="12">
-        <f>IF($B6="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B6="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ6="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B6="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B6="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ6="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS6" s="20">
@@ -4651,7 +5099,7 @@
         <v/>
       </c>
       <c r="AW6" s="12">
-        <f>IF($B6="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B6="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX6" s="12">
@@ -4665,6 +5113,32 @@
       <c r="AZ6" s="12">
         <f>IF($B6="BIG_SIDE",$V6*$AU6,0)</f>
         <v/>
+      </c>
+      <c r="BA6" s="12">
+        <f>IF($AK6=TRUE,MAX(0,$AJ6-$BD6),IF($B6="BLOCKED",MAX(0,$BA5-$BD6),0))</f>
+        <v/>
+      </c>
+      <c r="BB6" s="12">
+        <f>IF($AK6=TRUE,MAX(0,$AG6-$BE6),IF($B6="BLOCKED",MAX(0,$BB5-$BE6),0))</f>
+        <v/>
+      </c>
+      <c r="BC6" s="12">
+        <f>$BA6+$BB6</f>
+        <v/>
+      </c>
+      <c r="BD6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF6" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG6" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -4672,15 +5146,15 @@
         <v>6</v>
       </c>
       <c r="B7" s="13">
-        <f>IF(OR($AP6="NO",$AQ6="DUAL_TAIL",$AQ6="DANGER",$AQ6="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ6="MANUAL_READY",$BG6="YES"),"BIG_SIDE",IF(OR($AP6="NO",$AQ6="DUAL_TAIL",$AQ6="DANGER",$AQ6="STOP",$AQ6="MANUAL_READY",$AQ6="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C7" s="13">
-        <f>IF($B7="BLOCKED",$AF6,IF($AP6="YES",$AF6,$C6))</f>
+        <f>IF($B7="BLOCKED",$AF6,IF(AND($AQ6="MANUAL_READY",$BG6="YES"),$AF6,IF($AP6="YES",$AF6,$C6)))</f>
         <v/>
       </c>
       <c r="D7" s="13">
-        <f>IF($B7="BLOCKED",0,IF($AP6="YES",MAX(0,$AG6),$D6))</f>
+        <f>IF($B7="BLOCKED",0,IF(AND($AQ6="MANUAL_READY",$BG6="YES"),MAX($BA6,$BB6),IF($AP6="YES",MAX(0,$AG6),$D6)))</f>
         <v/>
       </c>
       <c r="E7" s="12">
@@ -4769,15 +5243,15 @@
         <v/>
       </c>
       <c r="AA7" s="12">
-        <f>IF($B7="BLOCKED",$Z7,IF($B7="BIG_SIDE",$Z7+$AX7-$AS7-$AZ7,IF($B7="SMALL_SIDE",$Z7+$S7+$AI7,$Z7+$S7)))</f>
+        <f>IF($B7="BLOCKED",$Z7+$BF7,IF($B7="BIG_SIDE",$Z7+$AX7-$AS7-$AZ7,IF($B7="SMALL_SIDE",$Z7+$S7+$AI7,$Z7+$S7)))</f>
         <v/>
       </c>
       <c r="AB7" s="12">
-        <f>IF($B7="BLOCKED",IF(ROW()=2,0,$AG6+$AJ6),$D7+$G7+$J7)</f>
+        <f>IF($B7="BLOCKED",$BC7,$D7+$G7+$J7)</f>
         <v/>
       </c>
       <c r="AC7" s="12">
-        <f>IF($B7="BLOCKED",$AB7,IF($B7="BIG_SIDE",$W7,$AG7+$AJ7))</f>
+        <f>IF($B7="BLOCKED",$BC7,IF($B7="BIG_SIDE",$W7,IF($AK7=TRUE,$BC7,$AG7)))</f>
         <v/>
       </c>
       <c r="AD7" s="12">
@@ -4789,11 +5263,11 @@
         <v/>
       </c>
       <c r="AF7" s="12">
-        <f>IF($B7="BLOCKED",IF(ROW()=2,$C7,$AF6),IF($B7="SMALL_SIDE",$E7,$C7))</f>
+        <f>IF($B7="BLOCKED",IF($BB7&gt;0,$AF6,$C7),IF($B7="SMALL_SIDE",$E7,$C7))</f>
         <v/>
       </c>
       <c r="AG7" s="12">
-        <f>IF($B7="BLOCKED",IF(ROW()=2,0,$AG6),IF($B7="SMALL_SIDE",$AM7,$W7))</f>
+        <f>IF($B7="BLOCKED",IF($BB7&gt;0,$BB7,$BA7),IF($B7="SMALL_SIDE",$AM7,$W7))</f>
         <v/>
       </c>
       <c r="AH7" s="13" t="inlineStr">
@@ -4829,15 +5303,15 @@
         <v/>
       </c>
       <c r="AP7" s="12">
-        <f>IF(OR($AQ7="DUAL_TAIL",$AQ7="DANGER",$AQ7="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ7="MANUAL_READY",$BG7="YES"),"YES",IF(OR($AQ7="DUAL_TAIL",$AQ7="DANGER",$AQ7="STOP",$AQ7="STOP_CLEARED",$AQ7="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ7" s="12">
-        <f>IF($B7="BLOCKED","STOP",IF($AK7=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G7/$D7,0)&gt;Settings!$B$16,IFERROR($J7/$G7,0)&gt;Settings!$B$17,$AE7&gt;$AD7,$Y7&lt;0,$AG7&gt;$D7*1.0001,$S7&lt;-100),"DANGER",IF(OR(AND($B7="BIG_SIDE",$U7&lt;=0),$S7&lt;=0,$X7=0,$AE7&gt;$AD7*0.95),"WARNING","OK"))))</f>
+        <f>IF($B7="BLOCKED",IF($BC7=0,"STOP_CLEARED",IF(OR(AND($BA7=0,$BB7&gt;0),AND($BA7&gt;0,$BB7=0)),"MANUAL_READY","STOP")),IF($AK7=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G7/$D7,0)&gt;Settings!$B$16,IFERROR($J7/$G7,0)&gt;Settings!$B$17,$AE7&gt;$AD7,$Y7&lt;0,$AG7&gt;$D7*1.0001,$S7&lt;-100),"DANGER",IF(OR(AND($B7="BIG_SIDE",$U7&lt;=0),$S7&lt;=0,$X7=0,$AE7&gt;$AD7*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR7" s="12">
-        <f>IF($B7="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B7="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ7="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B7="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B7="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ7="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS7" s="20">
@@ -4857,7 +5331,7 @@
         <v/>
       </c>
       <c r="AW7" s="12">
-        <f>IF($B7="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B7="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX7" s="12">
@@ -4871,6 +5345,32 @@
       <c r="AZ7" s="12">
         <f>IF($B7="BIG_SIDE",$V7*$AU7,0)</f>
         <v/>
+      </c>
+      <c r="BA7" s="12">
+        <f>IF($AK7=TRUE,MAX(0,$AJ7-$BD7),IF($B7="BLOCKED",MAX(0,$BA6-$BD7),0))</f>
+        <v/>
+      </c>
+      <c r="BB7" s="12">
+        <f>IF($AK7=TRUE,MAX(0,$AG7-$BE7),IF($B7="BLOCKED",MAX(0,$BB6-$BE7),0))</f>
+        <v/>
+      </c>
+      <c r="BC7" s="12">
+        <f>$BA7+$BB7</f>
+        <v/>
+      </c>
+      <c r="BD7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF7" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG7" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -4878,15 +5378,15 @@
         <v>7</v>
       </c>
       <c r="B8" s="13">
-        <f>IF(OR($AP7="NO",$AQ7="DUAL_TAIL",$AQ7="DANGER",$AQ7="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ7="MANUAL_READY",$BG7="YES"),"BIG_SIDE",IF(OR($AP7="NO",$AQ7="DUAL_TAIL",$AQ7="DANGER",$AQ7="STOP",$AQ7="MANUAL_READY",$AQ7="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C8" s="13">
-        <f>IF($B8="BLOCKED",$AF7,IF($AP7="YES",$AF7,$C7))</f>
+        <f>IF($B8="BLOCKED",$AF7,IF(AND($AQ7="MANUAL_READY",$BG7="YES"),$AF7,IF($AP7="YES",$AF7,$C7)))</f>
         <v/>
       </c>
       <c r="D8" s="13">
-        <f>IF($B8="BLOCKED",0,IF($AP7="YES",MAX(0,$AG7),$D7))</f>
+        <f>IF($B8="BLOCKED",0,IF(AND($AQ7="MANUAL_READY",$BG7="YES"),MAX($BA7,$BB7),IF($AP7="YES",MAX(0,$AG7),$D7)))</f>
         <v/>
       </c>
       <c r="E8" s="12">
@@ -4975,15 +5475,15 @@
         <v/>
       </c>
       <c r="AA8" s="12">
-        <f>IF($B8="BLOCKED",$Z8,IF($B8="BIG_SIDE",$Z8+$AX8-$AS8-$AZ8,IF($B8="SMALL_SIDE",$Z8+$S8+$AI8,$Z8+$S8)))</f>
+        <f>IF($B8="BLOCKED",$Z8+$BF8,IF($B8="BIG_SIDE",$Z8+$AX8-$AS8-$AZ8,IF($B8="SMALL_SIDE",$Z8+$S8+$AI8,$Z8+$S8)))</f>
         <v/>
       </c>
       <c r="AB8" s="12">
-        <f>IF($B8="BLOCKED",IF(ROW()=2,0,$AG7+$AJ7),$D8+$G8+$J8)</f>
+        <f>IF($B8="BLOCKED",$BC8,$D8+$G8+$J8)</f>
         <v/>
       </c>
       <c r="AC8" s="12">
-        <f>IF($B8="BLOCKED",$AB8,IF($B8="BIG_SIDE",$W8,$AG8+$AJ8))</f>
+        <f>IF($B8="BLOCKED",$BC8,IF($B8="BIG_SIDE",$W8,IF($AK8=TRUE,$BC8,$AG8)))</f>
         <v/>
       </c>
       <c r="AD8" s="12">
@@ -4995,11 +5495,11 @@
         <v/>
       </c>
       <c r="AF8" s="12">
-        <f>IF($B8="BLOCKED",IF(ROW()=2,$C8,$AF7),IF($B8="SMALL_SIDE",$E8,$C8))</f>
+        <f>IF($B8="BLOCKED",IF($BB8&gt;0,$AF7,$C8),IF($B8="SMALL_SIDE",$E8,$C8))</f>
         <v/>
       </c>
       <c r="AG8" s="12">
-        <f>IF($B8="BLOCKED",IF(ROW()=2,0,$AG7),IF($B8="SMALL_SIDE",$AM8,$W8))</f>
+        <f>IF($B8="BLOCKED",IF($BB8&gt;0,$BB8,$BA8),IF($B8="SMALL_SIDE",$AM8,$W8))</f>
         <v/>
       </c>
       <c r="AH8" s="13" t="inlineStr">
@@ -5035,15 +5535,15 @@
         <v/>
       </c>
       <c r="AP8" s="12">
-        <f>IF(OR($AQ8="DUAL_TAIL",$AQ8="DANGER",$AQ8="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ8="MANUAL_READY",$BG8="YES"),"YES",IF(OR($AQ8="DUAL_TAIL",$AQ8="DANGER",$AQ8="STOP",$AQ8="STOP_CLEARED",$AQ8="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ8" s="12">
-        <f>IF($B8="BLOCKED","STOP",IF($AK8=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G8/$D8,0)&gt;Settings!$B$16,IFERROR($J8/$G8,0)&gt;Settings!$B$17,$AE8&gt;$AD8,$Y8&lt;0,$AG8&gt;$D8*1.0001,$S8&lt;-100),"DANGER",IF(OR(AND($B8="BIG_SIDE",$U8&lt;=0),$S8&lt;=0,$X8=0,$AE8&gt;$AD8*0.95),"WARNING","OK"))))</f>
+        <f>IF($B8="BLOCKED",IF($BC8=0,"STOP_CLEARED",IF(OR(AND($BA8=0,$BB8&gt;0),AND($BA8&gt;0,$BB8=0)),"MANUAL_READY","STOP")),IF($AK8=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G8/$D8,0)&gt;Settings!$B$16,IFERROR($J8/$G8,0)&gt;Settings!$B$17,$AE8&gt;$AD8,$Y8&lt;0,$AG8&gt;$D8*1.0001,$S8&lt;-100),"DANGER",IF(OR(AND($B8="BIG_SIDE",$U8&lt;=0),$S8&lt;=0,$X8=0,$AE8&gt;$AD8*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR8" s="12">
-        <f>IF($B8="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B8="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ8="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B8="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B8="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ8="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS8" s="20">
@@ -5063,7 +5563,7 @@
         <v/>
       </c>
       <c r="AW8" s="12">
-        <f>IF($B8="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B8="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX8" s="12">
@@ -5077,6 +5577,32 @@
       <c r="AZ8" s="12">
         <f>IF($B8="BIG_SIDE",$V8*$AU8,0)</f>
         <v/>
+      </c>
+      <c r="BA8" s="12">
+        <f>IF($AK8=TRUE,MAX(0,$AJ8-$BD8),IF($B8="BLOCKED",MAX(0,$BA7-$BD8),0))</f>
+        <v/>
+      </c>
+      <c r="BB8" s="12">
+        <f>IF($AK8=TRUE,MAX(0,$AG8-$BE8),IF($B8="BLOCKED",MAX(0,$BB7-$BE8),0))</f>
+        <v/>
+      </c>
+      <c r="BC8" s="12">
+        <f>$BA8+$BB8</f>
+        <v/>
+      </c>
+      <c r="BD8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF8" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG8" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -5084,15 +5610,15 @@
         <v>8</v>
       </c>
       <c r="B9" s="13">
-        <f>IF(OR($AP8="NO",$AQ8="DUAL_TAIL",$AQ8="DANGER",$AQ8="STOP"),"BLOCKED","SMALL_SIDE")</f>
+        <f>IF(AND($AQ8="MANUAL_READY",$BG8="YES"),"SMALL_SIDE",IF(OR($AP8="NO",$AQ8="DUAL_TAIL",$AQ8="DANGER",$AQ8="STOP",$AQ8="MANUAL_READY",$AQ8="STOP_CLEARED"),"BLOCKED","SMALL_SIDE"))</f>
         <v/>
       </c>
       <c r="C9" s="13">
-        <f>IF($B9="BLOCKED",$AF8,IF($AP8="YES",$AF8,$C8))</f>
+        <f>IF($B9="BLOCKED",$AF8,IF(AND($AQ8="MANUAL_READY",$BG8="YES"),$AF8,IF($AP8="YES",$AF8,$C8)))</f>
         <v/>
       </c>
       <c r="D9" s="13">
-        <f>IF($B9="BLOCKED",0,IF($AP8="YES",MAX(0,$AG8),$D8))</f>
+        <f>IF($B9="BLOCKED",0,IF(AND($AQ8="MANUAL_READY",$BG8="YES"),MAX($BA8,$BB8),IF($AP8="YES",MAX(0,$AG8),$D8)))</f>
         <v/>
       </c>
       <c r="E9" s="12">
@@ -5181,15 +5707,15 @@
         <v/>
       </c>
       <c r="AA9" s="12">
-        <f>IF($B9="BLOCKED",$Z9,IF($B9="BIG_SIDE",$Z9+$AX9-$AS9-$AZ9,IF($B9="SMALL_SIDE",$Z9+$S9+$AI9,$Z9+$S9)))</f>
+        <f>IF($B9="BLOCKED",$Z9+$BF9,IF($B9="BIG_SIDE",$Z9+$AX9-$AS9-$AZ9,IF($B9="SMALL_SIDE",$Z9+$S9+$AI9,$Z9+$S9)))</f>
         <v/>
       </c>
       <c r="AB9" s="12">
-        <f>IF($B9="BLOCKED",IF(ROW()=2,0,$AG8+$AJ8),$D9+$G9+$J9)</f>
+        <f>IF($B9="BLOCKED",$BC9,$D9+$G9+$J9)</f>
         <v/>
       </c>
       <c r="AC9" s="12">
-        <f>IF($B9="BLOCKED",$AB9,IF($B9="BIG_SIDE",$W9,$AG9+$AJ9))</f>
+        <f>IF($B9="BLOCKED",$BC9,IF($B9="BIG_SIDE",$W9,IF($AK9=TRUE,$BC9,$AG9)))</f>
         <v/>
       </c>
       <c r="AD9" s="12">
@@ -5201,11 +5727,11 @@
         <v/>
       </c>
       <c r="AF9" s="12">
-        <f>IF($B9="BLOCKED",IF(ROW()=2,$C9,$AF8),IF($B9="SMALL_SIDE",$E9,$C9))</f>
+        <f>IF($B9="BLOCKED",IF($BB9&gt;0,$AF8,$C9),IF($B9="SMALL_SIDE",$E9,$C9))</f>
         <v/>
       </c>
       <c r="AG9" s="12">
-        <f>IF($B9="BLOCKED",IF(ROW()=2,0,$AG8),IF($B9="SMALL_SIDE",$AM9,$W9))</f>
+        <f>IF($B9="BLOCKED",IF($BB9&gt;0,$BB9,$BA9),IF($B9="SMALL_SIDE",$AM9,$W9))</f>
         <v/>
       </c>
       <c r="AH9" s="13" t="inlineStr">
@@ -5241,15 +5767,15 @@
         <v/>
       </c>
       <c r="AP9" s="12">
-        <f>IF(OR($AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ9="MANUAL_READY",$BG9="YES"),"YES",IF(OR($AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP",$AQ9="STOP_CLEARED",$AQ9="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ9" s="12">
-        <f>IF($B9="BLOCKED","STOP",IF($AK9=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G9/$D9,0)&gt;Settings!$B$16,IFERROR($J9/$G9,0)&gt;Settings!$B$17,$AE9&gt;$AD9,$Y9&lt;0,$AG9&gt;$D9*1.0001,$S9&lt;-100),"DANGER",IF(OR(AND($B9="BIG_SIDE",$U9&lt;=0),$S9&lt;=0,$X9=0,$AE9&gt;$AD9*0.95),"WARNING","OK"))))</f>
+        <f>IF($B9="BLOCKED",IF($BC9=0,"STOP_CLEARED",IF(OR(AND($BA9=0,$BB9&gt;0),AND($BA9&gt;0,$BB9=0)),"MANUAL_READY","STOP")),IF($AK9=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G9/$D9,0)&gt;Settings!$B$16,IFERROR($J9/$G9,0)&gt;Settings!$B$17,$AE9&gt;$AD9,$Y9&lt;0,$AG9&gt;$D9*1.0001,$S9&lt;-100),"DANGER",IF(OR(AND($B9="BIG_SIDE",$U9&lt;=0),$S9&lt;=0,$X9=0,$AE9&gt;$AD9*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR9" s="12">
-        <f>IF($B9="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B9="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ9="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B9="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B9="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ9="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS9" s="20">
@@ -5269,7 +5795,7 @@
         <v/>
       </c>
       <c r="AW9" s="12">
-        <f>IF($B9="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B9="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX9" s="12">
@@ -5283,6 +5809,32 @@
       <c r="AZ9" s="12">
         <f>IF($B9="BIG_SIDE",$V9*$AU9,0)</f>
         <v/>
+      </c>
+      <c r="BA9" s="12">
+        <f>IF($AK9=TRUE,MAX(0,$AJ9-$BD9),IF($B9="BLOCKED",MAX(0,$BA8-$BD9),0))</f>
+        <v/>
+      </c>
+      <c r="BB9" s="12">
+        <f>IF($AK9=TRUE,MAX(0,$AG9-$BE9),IF($B9="BLOCKED",MAX(0,$BB8-$BE9),0))</f>
+        <v/>
+      </c>
+      <c r="BC9" s="12">
+        <f>$BA9+$BB9</f>
+        <v/>
+      </c>
+      <c r="BD9" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE9" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF9" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG9" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -5290,15 +5842,15 @@
         <v>9</v>
       </c>
       <c r="B10" s="13">
-        <f>IF(OR($AP9="NO",$AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ9="MANUAL_READY",$BG9="YES"),"BIG_SIDE",IF(OR($AP9="NO",$AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP",$AQ9="MANUAL_READY",$AQ9="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C10" s="13">
-        <f>IF($B10="BLOCKED",$AF9,IF($AP9="YES",$AF9,$C9))</f>
+        <f>IF($B10="BLOCKED",$AF9,IF(AND($AQ9="MANUAL_READY",$BG9="YES"),$AF9,IF($AP9="YES",$AF9,$C9)))</f>
         <v/>
       </c>
       <c r="D10" s="13">
-        <f>IF($B10="BLOCKED",0,IF($AP9="YES",MAX(0,$AG9),$D9))</f>
+        <f>IF($B10="BLOCKED",0,IF(AND($AQ9="MANUAL_READY",$BG9="YES"),MAX($BA9,$BB9),IF($AP9="YES",MAX(0,$AG9),$D9)))</f>
         <v/>
       </c>
       <c r="E10" s="12">
@@ -5387,15 +5939,15 @@
         <v/>
       </c>
       <c r="AA10" s="12">
-        <f>IF($B10="BLOCKED",$Z10,IF($B10="BIG_SIDE",$Z10+$AX10-$AS10-$AZ10,IF($B10="SMALL_SIDE",$Z10+$S10+$AI10,$Z10+$S10)))</f>
+        <f>IF($B10="BLOCKED",$Z10+$BF10,IF($B10="BIG_SIDE",$Z10+$AX10-$AS10-$AZ10,IF($B10="SMALL_SIDE",$Z10+$S10+$AI10,$Z10+$S10)))</f>
         <v/>
       </c>
       <c r="AB10" s="12">
-        <f>IF($B10="BLOCKED",IF(ROW()=2,0,$AG9+$AJ9),$D10+$G10+$J10)</f>
+        <f>IF($B10="BLOCKED",$BC10,$D10+$G10+$J10)</f>
         <v/>
       </c>
       <c r="AC10" s="12">
-        <f>IF($B10="BLOCKED",$AB10,IF($B10="BIG_SIDE",$W10,$AG10+$AJ10))</f>
+        <f>IF($B10="BLOCKED",$BC10,IF($B10="BIG_SIDE",$W10,IF($AK10=TRUE,$BC10,$AG10)))</f>
         <v/>
       </c>
       <c r="AD10" s="12">
@@ -5407,11 +5959,11 @@
         <v/>
       </c>
       <c r="AF10" s="12">
-        <f>IF($B10="BLOCKED",IF(ROW()=2,$C10,$AF9),IF($B10="SMALL_SIDE",$E10,$C10))</f>
+        <f>IF($B10="BLOCKED",IF($BB10&gt;0,$AF9,$C10),IF($B10="SMALL_SIDE",$E10,$C10))</f>
         <v/>
       </c>
       <c r="AG10" s="12">
-        <f>IF($B10="BLOCKED",IF(ROW()=2,0,$AG9),IF($B10="SMALL_SIDE",$AM10,$W10))</f>
+        <f>IF($B10="BLOCKED",IF($BB10&gt;0,$BB10,$BA10),IF($B10="SMALL_SIDE",$AM10,$W10))</f>
         <v/>
       </c>
       <c r="AH10" s="13" t="inlineStr">
@@ -5447,15 +5999,15 @@
         <v/>
       </c>
       <c r="AP10" s="12">
-        <f>IF(OR($AQ10="DUAL_TAIL",$AQ10="DANGER",$AQ10="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ10="MANUAL_READY",$BG10="YES"),"YES",IF(OR($AQ10="DUAL_TAIL",$AQ10="DANGER",$AQ10="STOP",$AQ10="STOP_CLEARED",$AQ10="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ10" s="12">
-        <f>IF($B10="BLOCKED","STOP",IF($AK10=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G10/$D10,0)&gt;Settings!$B$16,IFERROR($J10/$G10,0)&gt;Settings!$B$17,$AE10&gt;$AD10,$Y10&lt;0,$AG10&gt;$D10*1.0001,$S10&lt;-100),"DANGER",IF(OR(AND($B10="BIG_SIDE",$U10&lt;=0),$S10&lt;=0,$X10=0,$AE10&gt;$AD10*0.95),"WARNING","OK"))))</f>
+        <f>IF($B10="BLOCKED",IF($BC10=0,"STOP_CLEARED",IF(OR(AND($BA10=0,$BB10&gt;0),AND($BA10&gt;0,$BB10=0)),"MANUAL_READY","STOP")),IF($AK10=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G10/$D10,0)&gt;Settings!$B$16,IFERROR($J10/$G10,0)&gt;Settings!$B$17,$AE10&gt;$AD10,$Y10&lt;0,$AG10&gt;$D10*1.0001,$S10&lt;-100),"DANGER",IF(OR(AND($B10="BIG_SIDE",$U10&lt;=0),$S10&lt;=0,$X10=0,$AE10&gt;$AD10*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR10" s="12">
-        <f>IF($B10="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B10="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ10="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B10="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B10="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ10="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS10" s="20">
@@ -5475,7 +6027,7 @@
         <v/>
       </c>
       <c r="AW10" s="12">
-        <f>IF($B10="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B10="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX10" s="12">
@@ -5489,6 +6041,32 @@
       <c r="AZ10" s="12">
         <f>IF($B10="BIG_SIDE",$V10*$AU10,0)</f>
         <v/>
+      </c>
+      <c r="BA10" s="12">
+        <f>IF($AK10=TRUE,MAX(0,$AJ10-$BD10),IF($B10="BLOCKED",MAX(0,$BA9-$BD10),0))</f>
+        <v/>
+      </c>
+      <c r="BB10" s="12">
+        <f>IF($AK10=TRUE,MAX(0,$AG10-$BE10),IF($B10="BLOCKED",MAX(0,$BB9-$BE10),0))</f>
+        <v/>
+      </c>
+      <c r="BC10" s="12">
+        <f>$BA10+$BB10</f>
+        <v/>
+      </c>
+      <c r="BD10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF10" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG10" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -5496,15 +6074,15 @@
         <v>10</v>
       </c>
       <c r="B11" s="13">
-        <f>IF(OR($AP10="NO",$AQ10="DUAL_TAIL",$AQ10="DANGER",$AQ10="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ10="MANUAL_READY",$BG10="YES"),"BIG_SIDE",IF(OR($AP10="NO",$AQ10="DUAL_TAIL",$AQ10="DANGER",$AQ10="STOP",$AQ10="MANUAL_READY",$AQ10="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C11" s="13">
-        <f>IF($B11="BLOCKED",$AF10,IF($AP10="YES",$AF10,$C10))</f>
+        <f>IF($B11="BLOCKED",$AF10,IF(AND($AQ10="MANUAL_READY",$BG10="YES"),$AF10,IF($AP10="YES",$AF10,$C10)))</f>
         <v/>
       </c>
       <c r="D11" s="13">
-        <f>IF($B11="BLOCKED",0,IF($AP10="YES",MAX(0,$AG10),$D10))</f>
+        <f>IF($B11="BLOCKED",0,IF(AND($AQ10="MANUAL_READY",$BG10="YES"),MAX($BA10,$BB10),IF($AP10="YES",MAX(0,$AG10),$D10)))</f>
         <v/>
       </c>
       <c r="E11" s="12">
@@ -5593,15 +6171,15 @@
         <v/>
       </c>
       <c r="AA11" s="12">
-        <f>IF($B11="BLOCKED",$Z11,IF($B11="BIG_SIDE",$Z11+$AX11-$AS11-$AZ11,IF($B11="SMALL_SIDE",$Z11+$S11+$AI11,$Z11+$S11)))</f>
+        <f>IF($B11="BLOCKED",$Z11+$BF11,IF($B11="BIG_SIDE",$Z11+$AX11-$AS11-$AZ11,IF($B11="SMALL_SIDE",$Z11+$S11+$AI11,$Z11+$S11)))</f>
         <v/>
       </c>
       <c r="AB11" s="12">
-        <f>IF($B11="BLOCKED",IF(ROW()=2,0,$AG10+$AJ10),$D11+$G11+$J11)</f>
+        <f>IF($B11="BLOCKED",$BC11,$D11+$G11+$J11)</f>
         <v/>
       </c>
       <c r="AC11" s="12">
-        <f>IF($B11="BLOCKED",$AB11,IF($B11="BIG_SIDE",$W11,$AG11+$AJ11))</f>
+        <f>IF($B11="BLOCKED",$BC11,IF($B11="BIG_SIDE",$W11,IF($AK11=TRUE,$BC11,$AG11)))</f>
         <v/>
       </c>
       <c r="AD11" s="12">
@@ -5613,11 +6191,11 @@
         <v/>
       </c>
       <c r="AF11" s="12">
-        <f>IF($B11="BLOCKED",IF(ROW()=2,$C11,$AF10),IF($B11="SMALL_SIDE",$E11,$C11))</f>
+        <f>IF($B11="BLOCKED",IF($BB11&gt;0,$AF10,$C11),IF($B11="SMALL_SIDE",$E11,$C11))</f>
         <v/>
       </c>
       <c r="AG11" s="12">
-        <f>IF($B11="BLOCKED",IF(ROW()=2,0,$AG10),IF($B11="SMALL_SIDE",$AM11,$W11))</f>
+        <f>IF($B11="BLOCKED",IF($BB11&gt;0,$BB11,$BA11),IF($B11="SMALL_SIDE",$AM11,$W11))</f>
         <v/>
       </c>
       <c r="AH11" s="13" t="inlineStr">
@@ -5653,15 +6231,15 @@
         <v/>
       </c>
       <c r="AP11" s="12">
-        <f>IF(OR($AQ11="DUAL_TAIL",$AQ11="DANGER",$AQ11="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ11="MANUAL_READY",$BG11="YES"),"YES",IF(OR($AQ11="DUAL_TAIL",$AQ11="DANGER",$AQ11="STOP",$AQ11="STOP_CLEARED",$AQ11="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ11" s="12">
-        <f>IF($B11="BLOCKED","STOP",IF($AK11=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G11/$D11,0)&gt;Settings!$B$16,IFERROR($J11/$G11,0)&gt;Settings!$B$17,$AE11&gt;$AD11,$Y11&lt;0,$AG11&gt;$D11*1.0001,$S11&lt;-100),"DANGER",IF(OR(AND($B11="BIG_SIDE",$U11&lt;=0),$S11&lt;=0,$X11=0,$AE11&gt;$AD11*0.95),"WARNING","OK"))))</f>
+        <f>IF($B11="BLOCKED",IF($BC11=0,"STOP_CLEARED",IF(OR(AND($BA11=0,$BB11&gt;0),AND($BA11&gt;0,$BB11=0)),"MANUAL_READY","STOP")),IF($AK11=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G11/$D11,0)&gt;Settings!$B$16,IFERROR($J11/$G11,0)&gt;Settings!$B$17,$AE11&gt;$AD11,$Y11&lt;0,$AG11&gt;$D11*1.0001,$S11&lt;-100),"DANGER",IF(OR(AND($B11="BIG_SIDE",$U11&lt;=0),$S11&lt;=0,$X11=0,$AE11&gt;$AD11*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR11" s="12">
-        <f>IF($B11="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B11="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ11="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B11="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B11="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ11="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS11" s="20">
@@ -5681,7 +6259,7 @@
         <v/>
       </c>
       <c r="AW11" s="12">
-        <f>IF($B11="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B11="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX11" s="12">
@@ -5696,9 +6274,35 @@
         <f>IF($B11="BIG_SIDE",$V11*$AU11,0)</f>
         <v/>
       </c>
+      <c r="BA11" s="12">
+        <f>IF($AK11=TRUE,MAX(0,$AJ11-$BD11),IF($B11="BLOCKED",MAX(0,$BA10-$BD11),0))</f>
+        <v/>
+      </c>
+      <c r="BB11" s="12">
+        <f>IF($AK11=TRUE,MAX(0,$AG11-$BE11),IF($B11="BLOCKED",MAX(0,$BB10-$BE11),0))</f>
+        <v/>
+      </c>
+      <c r="BC11" s="12">
+        <f>$BA11+$BB11</f>
+        <v/>
+      </c>
+      <c r="BD11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF11" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG11" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AZ11"/>
+  <autoFilter ref="A1:BG11"/>
   <conditionalFormatting sqref="AQ2:AQ11">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AQ2="WARNING"</formula>
@@ -5734,7 +6338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ11"/>
+  <dimension ref="A1:BG11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5789,6 +6393,13 @@
     <col width="18" customWidth="1" min="50" max="50"/>
     <col width="18" customWidth="1" min="51" max="51"/>
     <col width="18" customWidth="1" min="52" max="52"/>
+    <col width="20" customWidth="1" min="53" max="53"/>
+    <col width="20" customWidth="1" min="54" max="54"/>
+    <col width="20" customWidth="1" min="55" max="55"/>
+    <col width="20" customWidth="1" min="56" max="56"/>
+    <col width="20" customWidth="1" min="57" max="57"/>
+    <col width="20" customWidth="1" min="58" max="58"/>
+    <col width="22" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6052,6 +6663,41 @@
           <t>CostsFarClose</t>
         </is>
       </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>ActiveOldFarLot</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>ActiveNewFarLot</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>DualTailTotalLot</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>ManualOldFarCloseLot</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>ManualNewFarCloseLot</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>ManualClosePL</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>ManualAllowNewLevel</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="n">
@@ -6156,15 +6802,15 @@
         <v>0</v>
       </c>
       <c r="AA2" s="12">
-        <f>IF($B2="BLOCKED",$Z2,IF($B2="BIG_SIDE",$Z2+$AX2-$AS2-$AZ2,IF($B2="SMALL_SIDE",$Z2+$S2+$AI2,$Z2+$S2)))</f>
+        <f>IF($B2="BLOCKED",$Z2+$BF2,IF($B2="BIG_SIDE",$Z2+$AX2-$AS2-$AZ2,IF($B2="SMALL_SIDE",$Z2+$S2+$AI2,$Z2+$S2)))</f>
         <v/>
       </c>
       <c r="AB2" s="12">
-        <f>IF($B2="BLOCKED",IF(ROW()=2,0,$AG1+$AJ1),$D2+$G2+$J2)</f>
+        <f>IF($B2="BLOCKED",$BC2,$D2+$G2+$J2)</f>
         <v/>
       </c>
       <c r="AC2" s="12">
-        <f>IF($B2="BLOCKED",$AB2,IF($B2="BIG_SIDE",$W2,$AG2+$AJ2))</f>
+        <f>IF($B2="BLOCKED",$BC2,IF($B2="BIG_SIDE",$W2,IF($AK2=TRUE,$BC2,$AG2)))</f>
         <v/>
       </c>
       <c r="AD2" s="12">
@@ -6176,11 +6822,11 @@
         <v/>
       </c>
       <c r="AF2" s="12">
-        <f>IF($B2="BLOCKED",IF(ROW()=2,$C2,$AF1),IF($B2="SMALL_SIDE",$E2,$C2))</f>
+        <f>IF($B2="BLOCKED",IF($BB2&gt;0,$AF2,$C2),IF($B2="SMALL_SIDE",$E2,$C2))</f>
         <v/>
       </c>
       <c r="AG2" s="12">
-        <f>IF($B2="BLOCKED",IF(ROW()=2,0,$AG1),IF($B2="SMALL_SIDE",$AM2,$W2))</f>
+        <f>IF($B2="BLOCKED",IF($BB2&gt;0,$BB2,$BA2),IF($B2="SMALL_SIDE",$AM2,$W2))</f>
         <v/>
       </c>
       <c r="AH2" s="13" t="inlineStr">
@@ -6216,15 +6862,15 @@
         <v/>
       </c>
       <c r="AP2" s="12">
-        <f>IF(OR($AQ2="DUAL_TAIL",$AQ2="DANGER",$AQ2="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ2="MANUAL_READY",$BG2="YES"),"YES",IF(OR($AQ2="DUAL_TAIL",$AQ2="DANGER",$AQ2="STOP",$AQ2="STOP_CLEARED",$AQ2="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ2" s="12">
-        <f>IF($B2="BLOCKED","STOP",IF($AK2=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G2/$D2,0)&gt;Settings!$B$16,IFERROR($J2/$G2,0)&gt;Settings!$B$17,$AE2&gt;$AD2,$Y2&lt;0,$AG2&gt;$D2*1.0001,$S2&lt;-100),"DANGER",IF(OR(AND($B2="BIG_SIDE",$U2&lt;=0),$S2&lt;=0,$X2=0,$AE2&gt;$AD2*0.95),"WARNING","OK"))))</f>
+        <f>IF($B2="BLOCKED",IF($BC2=0,"STOP_CLEARED",IF(OR(AND($BA2=0,$BB2&gt;0),AND($BA2&gt;0,$BB2=0)),"MANUAL_READY","STOP")),IF($AK2=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G2/$D2,0)&gt;Settings!$B$16,IFERROR($J2/$G2,0)&gt;Settings!$B$17,$AE2&gt;$AD2,$Y2&lt;0,$AG2&gt;$D2*1.0001,$S2&lt;-100),"DANGER",IF(OR(AND($B2="BIG_SIDE",$U2&lt;=0),$S2&lt;=0,$X2=0,$AE2&gt;$AD2*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR2" s="12">
-        <f>IF($B2="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B2="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ2="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B2="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B2="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ2="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS2" s="20">
@@ -6244,7 +6890,7 @@
         <v/>
       </c>
       <c r="AW2" s="12">
-        <f>IF($B2="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B2="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX2" s="12">
@@ -6258,6 +6904,32 @@
       <c r="AZ2" s="12">
         <f>IF($B2="BIG_SIDE",$V2*$AU2,0)</f>
         <v/>
+      </c>
+      <c r="BA2" s="12">
+        <f>IF($AK2=TRUE,MAX(0,$AJ2-$BD2),0)</f>
+        <v/>
+      </c>
+      <c r="BB2" s="12">
+        <f>IF($AK2=TRUE,MAX(0,$AG2-$BE2),0)</f>
+        <v/>
+      </c>
+      <c r="BC2" s="12">
+        <f>$BA2+$BB2</f>
+        <v/>
+      </c>
+      <c r="BD2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -6265,15 +6937,15 @@
         <v>2</v>
       </c>
       <c r="B3" s="13">
-        <f>IF(OR($AP2="NO",$AQ2="DUAL_TAIL",$AQ2="DANGER",$AQ2="STOP"),"BLOCKED","SMALL_SIDE")</f>
+        <f>IF(AND($AQ2="MANUAL_READY",$BG2="YES"),"SMALL_SIDE",IF(OR($AP2="NO",$AQ2="DUAL_TAIL",$AQ2="DANGER",$AQ2="STOP",$AQ2="MANUAL_READY",$AQ2="STOP_CLEARED"),"BLOCKED","SMALL_SIDE"))</f>
         <v/>
       </c>
       <c r="C3" s="13">
-        <f>IF($B3="BLOCKED",$AF2,IF($AP2="YES",$AF2,$C2))</f>
+        <f>IF($B3="BLOCKED",$AF2,IF(AND($AQ2="MANUAL_READY",$BG2="YES"),$AF2,IF($AP2="YES",$AF2,$C2)))</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF($B3="BLOCKED",0,IF($AP2="YES",MAX(0,$AG2),$D2))</f>
+        <f>IF($B3="BLOCKED",0,IF(AND($AQ2="MANUAL_READY",$BG2="YES"),MAX($BA2,$BB2),IF($AP2="YES",MAX(0,$AG2),$D2)))</f>
         <v/>
       </c>
       <c r="E3" s="12">
@@ -6362,15 +7034,15 @@
         <v/>
       </c>
       <c r="AA3" s="12">
-        <f>IF($B3="BLOCKED",$Z3,IF($B3="BIG_SIDE",$Z3+$AX3-$AS3-$AZ3,IF($B3="SMALL_SIDE",$Z3+$S3+$AI3,$Z3+$S3)))</f>
+        <f>IF($B3="BLOCKED",$Z3+$BF3,IF($B3="BIG_SIDE",$Z3+$AX3-$AS3-$AZ3,IF($B3="SMALL_SIDE",$Z3+$S3+$AI3,$Z3+$S3)))</f>
         <v/>
       </c>
       <c r="AB3" s="12">
-        <f>IF($B3="BLOCKED",IF(ROW()=2,0,$AG2+$AJ2),$D3+$G3+$J3)</f>
+        <f>IF($B3="BLOCKED",$BC3,$D3+$G3+$J3)</f>
         <v/>
       </c>
       <c r="AC3" s="12">
-        <f>IF($B3="BLOCKED",$AB3,IF($B3="BIG_SIDE",$W3,$AG3+$AJ3))</f>
+        <f>IF($B3="BLOCKED",$BC3,IF($B3="BIG_SIDE",$W3,IF($AK3=TRUE,$BC3,$AG3)))</f>
         <v/>
       </c>
       <c r="AD3" s="12">
@@ -6382,11 +7054,11 @@
         <v/>
       </c>
       <c r="AF3" s="12">
-        <f>IF($B3="BLOCKED",IF(ROW()=2,$C3,$AF2),IF($B3="SMALL_SIDE",$E3,$C3))</f>
+        <f>IF($B3="BLOCKED",IF($BB3&gt;0,$AF2,$C3),IF($B3="SMALL_SIDE",$E3,$C3))</f>
         <v/>
       </c>
       <c r="AG3" s="12">
-        <f>IF($B3="BLOCKED",IF(ROW()=2,0,$AG2),IF($B3="SMALL_SIDE",$AM3,$W3))</f>
+        <f>IF($B3="BLOCKED",IF($BB3&gt;0,$BB3,$BA3),IF($B3="SMALL_SIDE",$AM3,$W3))</f>
         <v/>
       </c>
       <c r="AH3" s="13" t="inlineStr">
@@ -6422,15 +7094,15 @@
         <v/>
       </c>
       <c r="AP3" s="12">
-        <f>IF(OR($AQ3="DUAL_TAIL",$AQ3="DANGER",$AQ3="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ3="MANUAL_READY",$BG3="YES"),"YES",IF(OR($AQ3="DUAL_TAIL",$AQ3="DANGER",$AQ3="STOP",$AQ3="STOP_CLEARED",$AQ3="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ3" s="12">
-        <f>IF($B3="BLOCKED","STOP",IF($AK3=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G3/$D3,0)&gt;Settings!$B$16,IFERROR($J3/$G3,0)&gt;Settings!$B$17,$AE3&gt;$AD3,$Y3&lt;0,$AG3&gt;$D3*1.0001,$S3&lt;-100),"DANGER",IF(OR(AND($B3="BIG_SIDE",$U3&lt;=0),$S3&lt;=0,$X3=0,$AE3&gt;$AD3*0.95),"WARNING","OK"))))</f>
+        <f>IF($B3="BLOCKED",IF($BC3=0,"STOP_CLEARED",IF(OR(AND($BA3=0,$BB3&gt;0),AND($BA3&gt;0,$BB3=0)),"MANUAL_READY","STOP")),IF($AK3=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G3/$D3,0)&gt;Settings!$B$16,IFERROR($J3/$G3,0)&gt;Settings!$B$17,$AE3&gt;$AD3,$Y3&lt;0,$AG3&gt;$D3*1.0001,$S3&lt;-100),"DANGER",IF(OR(AND($B3="BIG_SIDE",$U3&lt;=0),$S3&lt;=0,$X3=0,$AE3&gt;$AD3*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR3" s="12">
-        <f>IF($B3="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B3="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ3="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B3="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B3="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ3="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS3" s="20">
@@ -6450,7 +7122,7 @@
         <v/>
       </c>
       <c r="AW3" s="12">
-        <f>IF($B3="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B3="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX3" s="12">
@@ -6464,6 +7136,32 @@
       <c r="AZ3" s="12">
         <f>IF($B3="BIG_SIDE",$V3*$AU3,0)</f>
         <v/>
+      </c>
+      <c r="BA3" s="12">
+        <f>IF($AK3=TRUE,MAX(0,$AJ3-$BD3),IF($B3="BLOCKED",MAX(0,$BA2-$BD3),0))</f>
+        <v/>
+      </c>
+      <c r="BB3" s="12">
+        <f>IF($AK3=TRUE,MAX(0,$AG3-$BE3),IF($B3="BLOCKED",MAX(0,$BB2-$BE3),0))</f>
+        <v/>
+      </c>
+      <c r="BC3" s="12">
+        <f>$BA3+$BB3</f>
+        <v/>
+      </c>
+      <c r="BD3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF3" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG3" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -6471,15 +7169,15 @@
         <v>3</v>
       </c>
       <c r="B4" s="13">
-        <f>IF(OR($AP3="NO",$AQ3="DUAL_TAIL",$AQ3="DANGER",$AQ3="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ3="MANUAL_READY",$BG3="YES"),"BIG_SIDE",IF(OR($AP3="NO",$AQ3="DUAL_TAIL",$AQ3="DANGER",$AQ3="STOP",$AQ3="MANUAL_READY",$AQ3="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C4" s="13">
-        <f>IF($B4="BLOCKED",$AF3,IF($AP3="YES",$AF3,$C3))</f>
+        <f>IF($B4="BLOCKED",$AF3,IF(AND($AQ3="MANUAL_READY",$BG3="YES"),$AF3,IF($AP3="YES",$AF3,$C3)))</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>IF($B4="BLOCKED",0,IF($AP3="YES",MAX(0,$AG3),$D3))</f>
+        <f>IF($B4="BLOCKED",0,IF(AND($AQ3="MANUAL_READY",$BG3="YES"),MAX($BA3,$BB3),IF($AP3="YES",MAX(0,$AG3),$D3)))</f>
         <v/>
       </c>
       <c r="E4" s="12">
@@ -6568,15 +7266,15 @@
         <v/>
       </c>
       <c r="AA4" s="12">
-        <f>IF($B4="BLOCKED",$Z4,IF($B4="BIG_SIDE",$Z4+$AX4-$AS4-$AZ4,IF($B4="SMALL_SIDE",$Z4+$S4+$AI4,$Z4+$S4)))</f>
+        <f>IF($B4="BLOCKED",$Z4+$BF4,IF($B4="BIG_SIDE",$Z4+$AX4-$AS4-$AZ4,IF($B4="SMALL_SIDE",$Z4+$S4+$AI4,$Z4+$S4)))</f>
         <v/>
       </c>
       <c r="AB4" s="12">
-        <f>IF($B4="BLOCKED",IF(ROW()=2,0,$AG3+$AJ3),$D4+$G4+$J4)</f>
+        <f>IF($B4="BLOCKED",$BC4,$D4+$G4+$J4)</f>
         <v/>
       </c>
       <c r="AC4" s="12">
-        <f>IF($B4="BLOCKED",$AB4,IF($B4="BIG_SIDE",$W4,$AG4+$AJ4))</f>
+        <f>IF($B4="BLOCKED",$BC4,IF($B4="BIG_SIDE",$W4,IF($AK4=TRUE,$BC4,$AG4)))</f>
         <v/>
       </c>
       <c r="AD4" s="12">
@@ -6588,11 +7286,11 @@
         <v/>
       </c>
       <c r="AF4" s="12">
-        <f>IF($B4="BLOCKED",IF(ROW()=2,$C4,$AF3),IF($B4="SMALL_SIDE",$E4,$C4))</f>
+        <f>IF($B4="BLOCKED",IF($BB4&gt;0,$AF3,$C4),IF($B4="SMALL_SIDE",$E4,$C4))</f>
         <v/>
       </c>
       <c r="AG4" s="12">
-        <f>IF($B4="BLOCKED",IF(ROW()=2,0,$AG3),IF($B4="SMALL_SIDE",$AM4,$W4))</f>
+        <f>IF($B4="BLOCKED",IF($BB4&gt;0,$BB4,$BA4),IF($B4="SMALL_SIDE",$AM4,$W4))</f>
         <v/>
       </c>
       <c r="AH4" s="13" t="inlineStr">
@@ -6628,15 +7326,15 @@
         <v/>
       </c>
       <c r="AP4" s="12">
-        <f>IF(OR($AQ4="DUAL_TAIL",$AQ4="DANGER",$AQ4="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ4="MANUAL_READY",$BG4="YES"),"YES",IF(OR($AQ4="DUAL_TAIL",$AQ4="DANGER",$AQ4="STOP",$AQ4="STOP_CLEARED",$AQ4="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ4" s="12">
-        <f>IF($B4="BLOCKED","STOP",IF($AK4=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G4/$D4,0)&gt;Settings!$B$16,IFERROR($J4/$G4,0)&gt;Settings!$B$17,$AE4&gt;$AD4,$Y4&lt;0,$AG4&gt;$D4*1.0001,$S4&lt;-100),"DANGER",IF(OR(AND($B4="BIG_SIDE",$U4&lt;=0),$S4&lt;=0,$X4=0,$AE4&gt;$AD4*0.95),"WARNING","OK"))))</f>
+        <f>IF($B4="BLOCKED",IF($BC4=0,"STOP_CLEARED",IF(OR(AND($BA4=0,$BB4&gt;0),AND($BA4&gt;0,$BB4=0)),"MANUAL_READY","STOP")),IF($AK4=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G4/$D4,0)&gt;Settings!$B$16,IFERROR($J4/$G4,0)&gt;Settings!$B$17,$AE4&gt;$AD4,$Y4&lt;0,$AG4&gt;$D4*1.0001,$S4&lt;-100),"DANGER",IF(OR(AND($B4="BIG_SIDE",$U4&lt;=0),$S4&lt;=0,$X4=0,$AE4&gt;$AD4*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR4" s="12">
-        <f>IF($B4="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B4="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ4="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B4="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B4="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ4="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS4" s="20">
@@ -6656,7 +7354,7 @@
         <v/>
       </c>
       <c r="AW4" s="12">
-        <f>IF($B4="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B4="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX4" s="12">
@@ -6670,6 +7368,32 @@
       <c r="AZ4" s="12">
         <f>IF($B4="BIG_SIDE",$V4*$AU4,0)</f>
         <v/>
+      </c>
+      <c r="BA4" s="12">
+        <f>IF($AK4=TRUE,MAX(0,$AJ4-$BD4),IF($B4="BLOCKED",MAX(0,$BA3-$BD4),0))</f>
+        <v/>
+      </c>
+      <c r="BB4" s="12">
+        <f>IF($AK4=TRUE,MAX(0,$AG4-$BE4),IF($B4="BLOCKED",MAX(0,$BB3-$BE4),0))</f>
+        <v/>
+      </c>
+      <c r="BC4" s="12">
+        <f>$BA4+$BB4</f>
+        <v/>
+      </c>
+      <c r="BD4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG4" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -6677,15 +7401,15 @@
         <v>4</v>
       </c>
       <c r="B5" s="13">
-        <f>IF(OR($AP4="NO",$AQ4="DUAL_TAIL",$AQ4="DANGER",$AQ4="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ4="MANUAL_READY",$BG4="YES"),"BIG_SIDE",IF(OR($AP4="NO",$AQ4="DUAL_TAIL",$AQ4="DANGER",$AQ4="STOP",$AQ4="MANUAL_READY",$AQ4="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C5" s="13">
-        <f>IF($B5="BLOCKED",$AF4,IF($AP4="YES",$AF4,$C4))</f>
+        <f>IF($B5="BLOCKED",$AF4,IF(AND($AQ4="MANUAL_READY",$BG4="YES"),$AF4,IF($AP4="YES",$AF4,$C4)))</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>IF($B5="BLOCKED",0,IF($AP4="YES",MAX(0,$AG4),$D4))</f>
+        <f>IF($B5="BLOCKED",0,IF(AND($AQ4="MANUAL_READY",$BG4="YES"),MAX($BA4,$BB4),IF($AP4="YES",MAX(0,$AG4),$D4)))</f>
         <v/>
       </c>
       <c r="E5" s="12">
@@ -6774,15 +7498,15 @@
         <v/>
       </c>
       <c r="AA5" s="12">
-        <f>IF($B5="BLOCKED",$Z5,IF($B5="BIG_SIDE",$Z5+$AX5-$AS5-$AZ5,IF($B5="SMALL_SIDE",$Z5+$S5+$AI5,$Z5+$S5)))</f>
+        <f>IF($B5="BLOCKED",$Z5+$BF5,IF($B5="BIG_SIDE",$Z5+$AX5-$AS5-$AZ5,IF($B5="SMALL_SIDE",$Z5+$S5+$AI5,$Z5+$S5)))</f>
         <v/>
       </c>
       <c r="AB5" s="12">
-        <f>IF($B5="BLOCKED",IF(ROW()=2,0,$AG4+$AJ4),$D5+$G5+$J5)</f>
+        <f>IF($B5="BLOCKED",$BC5,$D5+$G5+$J5)</f>
         <v/>
       </c>
       <c r="AC5" s="12">
-        <f>IF($B5="BLOCKED",$AB5,IF($B5="BIG_SIDE",$W5,$AG5+$AJ5))</f>
+        <f>IF($B5="BLOCKED",$BC5,IF($B5="BIG_SIDE",$W5,IF($AK5=TRUE,$BC5,$AG5)))</f>
         <v/>
       </c>
       <c r="AD5" s="12">
@@ -6794,11 +7518,11 @@
         <v/>
       </c>
       <c r="AF5" s="12">
-        <f>IF($B5="BLOCKED",IF(ROW()=2,$C5,$AF4),IF($B5="SMALL_SIDE",$E5,$C5))</f>
+        <f>IF($B5="BLOCKED",IF($BB5&gt;0,$AF4,$C5),IF($B5="SMALL_SIDE",$E5,$C5))</f>
         <v/>
       </c>
       <c r="AG5" s="12">
-        <f>IF($B5="BLOCKED",IF(ROW()=2,0,$AG4),IF($B5="SMALL_SIDE",$AM5,$W5))</f>
+        <f>IF($B5="BLOCKED",IF($BB5&gt;0,$BB5,$BA5),IF($B5="SMALL_SIDE",$AM5,$W5))</f>
         <v/>
       </c>
       <c r="AH5" s="13" t="inlineStr">
@@ -6834,15 +7558,15 @@
         <v/>
       </c>
       <c r="AP5" s="12">
-        <f>IF(OR($AQ5="DUAL_TAIL",$AQ5="DANGER",$AQ5="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ5="MANUAL_READY",$BG5="YES"),"YES",IF(OR($AQ5="DUAL_TAIL",$AQ5="DANGER",$AQ5="STOP",$AQ5="STOP_CLEARED",$AQ5="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ5" s="12">
-        <f>IF($B5="BLOCKED","STOP",IF($AK5=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G5/$D5,0)&gt;Settings!$B$16,IFERROR($J5/$G5,0)&gt;Settings!$B$17,$AE5&gt;$AD5,$Y5&lt;0,$AG5&gt;$D5*1.0001,$S5&lt;-100),"DANGER",IF(OR(AND($B5="BIG_SIDE",$U5&lt;=0),$S5&lt;=0,$X5=0,$AE5&gt;$AD5*0.95),"WARNING","OK"))))</f>
+        <f>IF($B5="BLOCKED",IF($BC5=0,"STOP_CLEARED",IF(OR(AND($BA5=0,$BB5&gt;0),AND($BA5&gt;0,$BB5=0)),"MANUAL_READY","STOP")),IF($AK5=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G5/$D5,0)&gt;Settings!$B$16,IFERROR($J5/$G5,0)&gt;Settings!$B$17,$AE5&gt;$AD5,$Y5&lt;0,$AG5&gt;$D5*1.0001,$S5&lt;-100),"DANGER",IF(OR(AND($B5="BIG_SIDE",$U5&lt;=0),$S5&lt;=0,$X5=0,$AE5&gt;$AD5*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR5" s="12">
-        <f>IF($B5="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B5="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ5="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B5="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B5="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ5="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS5" s="20">
@@ -6862,7 +7586,7 @@
         <v/>
       </c>
       <c r="AW5" s="12">
-        <f>IF($B5="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B5="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX5" s="12">
@@ -6876,6 +7600,32 @@
       <c r="AZ5" s="12">
         <f>IF($B5="BIG_SIDE",$V5*$AU5,0)</f>
         <v/>
+      </c>
+      <c r="BA5" s="12">
+        <f>IF($AK5=TRUE,MAX(0,$AJ5-$BD5),IF($B5="BLOCKED",MAX(0,$BA4-$BD5),0))</f>
+        <v/>
+      </c>
+      <c r="BB5" s="12">
+        <f>IF($AK5=TRUE,MAX(0,$AG5-$BE5),IF($B5="BLOCKED",MAX(0,$BB4-$BE5),0))</f>
+        <v/>
+      </c>
+      <c r="BC5" s="12">
+        <f>$BA5+$BB5</f>
+        <v/>
+      </c>
+      <c r="BD5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF5" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG5" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -6883,15 +7633,15 @@
         <v>5</v>
       </c>
       <c r="B6" s="13">
-        <f>IF(OR($AP5="NO",$AQ5="DUAL_TAIL",$AQ5="DANGER",$AQ5="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ5="MANUAL_READY",$BG5="YES"),"BIG_SIDE",IF(OR($AP5="NO",$AQ5="DUAL_TAIL",$AQ5="DANGER",$AQ5="STOP",$AQ5="MANUAL_READY",$AQ5="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C6" s="13">
-        <f>IF($B6="BLOCKED",$AF5,IF($AP5="YES",$AF5,$C5))</f>
+        <f>IF($B6="BLOCKED",$AF5,IF(AND($AQ5="MANUAL_READY",$BG5="YES"),$AF5,IF($AP5="YES",$AF5,$C5)))</f>
         <v/>
       </c>
       <c r="D6" s="13">
-        <f>IF($B6="BLOCKED",0,IF($AP5="YES",MAX(0,$AG5),$D5))</f>
+        <f>IF($B6="BLOCKED",0,IF(AND($AQ5="MANUAL_READY",$BG5="YES"),MAX($BA5,$BB5),IF($AP5="YES",MAX(0,$AG5),$D5)))</f>
         <v/>
       </c>
       <c r="E6" s="12">
@@ -6980,15 +7730,15 @@
         <v/>
       </c>
       <c r="AA6" s="12">
-        <f>IF($B6="BLOCKED",$Z6,IF($B6="BIG_SIDE",$Z6+$AX6-$AS6-$AZ6,IF($B6="SMALL_SIDE",$Z6+$S6+$AI6,$Z6+$S6)))</f>
+        <f>IF($B6="BLOCKED",$Z6+$BF6,IF($B6="BIG_SIDE",$Z6+$AX6-$AS6-$AZ6,IF($B6="SMALL_SIDE",$Z6+$S6+$AI6,$Z6+$S6)))</f>
         <v/>
       </c>
       <c r="AB6" s="12">
-        <f>IF($B6="BLOCKED",IF(ROW()=2,0,$AG5+$AJ5),$D6+$G6+$J6)</f>
+        <f>IF($B6="BLOCKED",$BC6,$D6+$G6+$J6)</f>
         <v/>
       </c>
       <c r="AC6" s="12">
-        <f>IF($B6="BLOCKED",$AB6,IF($B6="BIG_SIDE",$W6,$AG6+$AJ6))</f>
+        <f>IF($B6="BLOCKED",$BC6,IF($B6="BIG_SIDE",$W6,IF($AK6=TRUE,$BC6,$AG6)))</f>
         <v/>
       </c>
       <c r="AD6" s="12">
@@ -7000,11 +7750,11 @@
         <v/>
       </c>
       <c r="AF6" s="12">
-        <f>IF($B6="BLOCKED",IF(ROW()=2,$C6,$AF5),IF($B6="SMALL_SIDE",$E6,$C6))</f>
+        <f>IF($B6="BLOCKED",IF($BB6&gt;0,$AF5,$C6),IF($B6="SMALL_SIDE",$E6,$C6))</f>
         <v/>
       </c>
       <c r="AG6" s="12">
-        <f>IF($B6="BLOCKED",IF(ROW()=2,0,$AG5),IF($B6="SMALL_SIDE",$AM6,$W6))</f>
+        <f>IF($B6="BLOCKED",IF($BB6&gt;0,$BB6,$BA6),IF($B6="SMALL_SIDE",$AM6,$W6))</f>
         <v/>
       </c>
       <c r="AH6" s="13" t="inlineStr">
@@ -7040,15 +7790,15 @@
         <v/>
       </c>
       <c r="AP6" s="12">
-        <f>IF(OR($AQ6="DUAL_TAIL",$AQ6="DANGER",$AQ6="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ6="MANUAL_READY",$BG6="YES"),"YES",IF(OR($AQ6="DUAL_TAIL",$AQ6="DANGER",$AQ6="STOP",$AQ6="STOP_CLEARED",$AQ6="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ6" s="12">
-        <f>IF($B6="BLOCKED","STOP",IF($AK6=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G6/$D6,0)&gt;Settings!$B$16,IFERROR($J6/$G6,0)&gt;Settings!$B$17,$AE6&gt;$AD6,$Y6&lt;0,$AG6&gt;$D6*1.0001,$S6&lt;-100),"DANGER",IF(OR(AND($B6="BIG_SIDE",$U6&lt;=0),$S6&lt;=0,$X6=0,$AE6&gt;$AD6*0.95),"WARNING","OK"))))</f>
+        <f>IF($B6="BLOCKED",IF($BC6=0,"STOP_CLEARED",IF(OR(AND($BA6=0,$BB6&gt;0),AND($BA6&gt;0,$BB6=0)),"MANUAL_READY","STOP")),IF($AK6=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G6/$D6,0)&gt;Settings!$B$16,IFERROR($J6/$G6,0)&gt;Settings!$B$17,$AE6&gt;$AD6,$Y6&lt;0,$AG6&gt;$D6*1.0001,$S6&lt;-100),"DANGER",IF(OR(AND($B6="BIG_SIDE",$U6&lt;=0),$S6&lt;=0,$X6=0,$AE6&gt;$AD6*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR6" s="12">
-        <f>IF($B6="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B6="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ6="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B6="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B6="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ6="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS6" s="20">
@@ -7068,7 +7818,7 @@
         <v/>
       </c>
       <c r="AW6" s="12">
-        <f>IF($B6="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B6="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX6" s="12">
@@ -7082,6 +7832,32 @@
       <c r="AZ6" s="12">
         <f>IF($B6="BIG_SIDE",$V6*$AU6,0)</f>
         <v/>
+      </c>
+      <c r="BA6" s="12">
+        <f>IF($AK6=TRUE,MAX(0,$AJ6-$BD6),IF($B6="BLOCKED",MAX(0,$BA5-$BD6),0))</f>
+        <v/>
+      </c>
+      <c r="BB6" s="12">
+        <f>IF($AK6=TRUE,MAX(0,$AG6-$BE6),IF($B6="BLOCKED",MAX(0,$BB5-$BE6),0))</f>
+        <v/>
+      </c>
+      <c r="BC6" s="12">
+        <f>$BA6+$BB6</f>
+        <v/>
+      </c>
+      <c r="BD6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF6" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG6" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -7089,15 +7865,15 @@
         <v>6</v>
       </c>
       <c r="B7" s="13">
-        <f>IF(OR($AP6="NO",$AQ6="DUAL_TAIL",$AQ6="DANGER",$AQ6="STOP"),"BLOCKED","SMALL_SIDE")</f>
+        <f>IF(AND($AQ6="MANUAL_READY",$BG6="YES"),"SMALL_SIDE",IF(OR($AP6="NO",$AQ6="DUAL_TAIL",$AQ6="DANGER",$AQ6="STOP",$AQ6="MANUAL_READY",$AQ6="STOP_CLEARED"),"BLOCKED","SMALL_SIDE"))</f>
         <v/>
       </c>
       <c r="C7" s="13">
-        <f>IF($B7="BLOCKED",$AF6,IF($AP6="YES",$AF6,$C6))</f>
+        <f>IF($B7="BLOCKED",$AF6,IF(AND($AQ6="MANUAL_READY",$BG6="YES"),$AF6,IF($AP6="YES",$AF6,$C6)))</f>
         <v/>
       </c>
       <c r="D7" s="13">
-        <f>IF($B7="BLOCKED",0,IF($AP6="YES",MAX(0,$AG6),$D6))</f>
+        <f>IF($B7="BLOCKED",0,IF(AND($AQ6="MANUAL_READY",$BG6="YES"),MAX($BA6,$BB6),IF($AP6="YES",MAX(0,$AG6),$D6)))</f>
         <v/>
       </c>
       <c r="E7" s="12">
@@ -7186,15 +7962,15 @@
         <v/>
       </c>
       <c r="AA7" s="12">
-        <f>IF($B7="BLOCKED",$Z7,IF($B7="BIG_SIDE",$Z7+$AX7-$AS7-$AZ7,IF($B7="SMALL_SIDE",$Z7+$S7+$AI7,$Z7+$S7)))</f>
+        <f>IF($B7="BLOCKED",$Z7+$BF7,IF($B7="BIG_SIDE",$Z7+$AX7-$AS7-$AZ7,IF($B7="SMALL_SIDE",$Z7+$S7+$AI7,$Z7+$S7)))</f>
         <v/>
       </c>
       <c r="AB7" s="12">
-        <f>IF($B7="BLOCKED",IF(ROW()=2,0,$AG6+$AJ6),$D7+$G7+$J7)</f>
+        <f>IF($B7="BLOCKED",$BC7,$D7+$G7+$J7)</f>
         <v/>
       </c>
       <c r="AC7" s="12">
-        <f>IF($B7="BLOCKED",$AB7,IF($B7="BIG_SIDE",$W7,$AG7+$AJ7))</f>
+        <f>IF($B7="BLOCKED",$BC7,IF($B7="BIG_SIDE",$W7,IF($AK7=TRUE,$BC7,$AG7)))</f>
         <v/>
       </c>
       <c r="AD7" s="12">
@@ -7206,11 +7982,11 @@
         <v/>
       </c>
       <c r="AF7" s="12">
-        <f>IF($B7="BLOCKED",IF(ROW()=2,$C7,$AF6),IF($B7="SMALL_SIDE",$E7,$C7))</f>
+        <f>IF($B7="BLOCKED",IF($BB7&gt;0,$AF6,$C7),IF($B7="SMALL_SIDE",$E7,$C7))</f>
         <v/>
       </c>
       <c r="AG7" s="12">
-        <f>IF($B7="BLOCKED",IF(ROW()=2,0,$AG6),IF($B7="SMALL_SIDE",$AM7,$W7))</f>
+        <f>IF($B7="BLOCKED",IF($BB7&gt;0,$BB7,$BA7),IF($B7="SMALL_SIDE",$AM7,$W7))</f>
         <v/>
       </c>
       <c r="AH7" s="13" t="inlineStr">
@@ -7246,15 +8022,15 @@
         <v/>
       </c>
       <c r="AP7" s="12">
-        <f>IF(OR($AQ7="DUAL_TAIL",$AQ7="DANGER",$AQ7="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ7="MANUAL_READY",$BG7="YES"),"YES",IF(OR($AQ7="DUAL_TAIL",$AQ7="DANGER",$AQ7="STOP",$AQ7="STOP_CLEARED",$AQ7="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ7" s="12">
-        <f>IF($B7="BLOCKED","STOP",IF($AK7=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G7/$D7,0)&gt;Settings!$B$16,IFERROR($J7/$G7,0)&gt;Settings!$B$17,$AE7&gt;$AD7,$Y7&lt;0,$AG7&gt;$D7*1.0001,$S7&lt;-100),"DANGER",IF(OR(AND($B7="BIG_SIDE",$U7&lt;=0),$S7&lt;=0,$X7=0,$AE7&gt;$AD7*0.95),"WARNING","OK"))))</f>
+        <f>IF($B7="BLOCKED",IF($BC7=0,"STOP_CLEARED",IF(OR(AND($BA7=0,$BB7&gt;0),AND($BA7&gt;0,$BB7=0)),"MANUAL_READY","STOP")),IF($AK7=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G7/$D7,0)&gt;Settings!$B$16,IFERROR($J7/$G7,0)&gt;Settings!$B$17,$AE7&gt;$AD7,$Y7&lt;0,$AG7&gt;$D7*1.0001,$S7&lt;-100),"DANGER",IF(OR(AND($B7="BIG_SIDE",$U7&lt;=0),$S7&lt;=0,$X7=0,$AE7&gt;$AD7*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR7" s="12">
-        <f>IF($B7="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B7="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ7="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B7="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B7="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ7="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS7" s="20">
@@ -7274,7 +8050,7 @@
         <v/>
       </c>
       <c r="AW7" s="12">
-        <f>IF($B7="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B7="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX7" s="12">
@@ -7288,6 +8064,32 @@
       <c r="AZ7" s="12">
         <f>IF($B7="BIG_SIDE",$V7*$AU7,0)</f>
         <v/>
+      </c>
+      <c r="BA7" s="12">
+        <f>IF($AK7=TRUE,MAX(0,$AJ7-$BD7),IF($B7="BLOCKED",MAX(0,$BA6-$BD7),0))</f>
+        <v/>
+      </c>
+      <c r="BB7" s="12">
+        <f>IF($AK7=TRUE,MAX(0,$AG7-$BE7),IF($B7="BLOCKED",MAX(0,$BB6-$BE7),0))</f>
+        <v/>
+      </c>
+      <c r="BC7" s="12">
+        <f>$BA7+$BB7</f>
+        <v/>
+      </c>
+      <c r="BD7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF7" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG7" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -7295,15 +8097,15 @@
         <v>7</v>
       </c>
       <c r="B8" s="13">
-        <f>IF(OR($AP7="NO",$AQ7="DUAL_TAIL",$AQ7="DANGER",$AQ7="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ7="MANUAL_READY",$BG7="YES"),"BIG_SIDE",IF(OR($AP7="NO",$AQ7="DUAL_TAIL",$AQ7="DANGER",$AQ7="STOP",$AQ7="MANUAL_READY",$AQ7="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C8" s="13">
-        <f>IF($B8="BLOCKED",$AF7,IF($AP7="YES",$AF7,$C7))</f>
+        <f>IF($B8="BLOCKED",$AF7,IF(AND($AQ7="MANUAL_READY",$BG7="YES"),$AF7,IF($AP7="YES",$AF7,$C7)))</f>
         <v/>
       </c>
       <c r="D8" s="13">
-        <f>IF($B8="BLOCKED",0,IF($AP7="YES",MAX(0,$AG7),$D7))</f>
+        <f>IF($B8="BLOCKED",0,IF(AND($AQ7="MANUAL_READY",$BG7="YES"),MAX($BA7,$BB7),IF($AP7="YES",MAX(0,$AG7),$D7)))</f>
         <v/>
       </c>
       <c r="E8" s="12">
@@ -7392,15 +8194,15 @@
         <v/>
       </c>
       <c r="AA8" s="12">
-        <f>IF($B8="BLOCKED",$Z8,IF($B8="BIG_SIDE",$Z8+$AX8-$AS8-$AZ8,IF($B8="SMALL_SIDE",$Z8+$S8+$AI8,$Z8+$S8)))</f>
+        <f>IF($B8="BLOCKED",$Z8+$BF8,IF($B8="BIG_SIDE",$Z8+$AX8-$AS8-$AZ8,IF($B8="SMALL_SIDE",$Z8+$S8+$AI8,$Z8+$S8)))</f>
         <v/>
       </c>
       <c r="AB8" s="12">
-        <f>IF($B8="BLOCKED",IF(ROW()=2,0,$AG7+$AJ7),$D8+$G8+$J8)</f>
+        <f>IF($B8="BLOCKED",$BC8,$D8+$G8+$J8)</f>
         <v/>
       </c>
       <c r="AC8" s="12">
-        <f>IF($B8="BLOCKED",$AB8,IF($B8="BIG_SIDE",$W8,$AG8+$AJ8))</f>
+        <f>IF($B8="BLOCKED",$BC8,IF($B8="BIG_SIDE",$W8,IF($AK8=TRUE,$BC8,$AG8)))</f>
         <v/>
       </c>
       <c r="AD8" s="12">
@@ -7412,11 +8214,11 @@
         <v/>
       </c>
       <c r="AF8" s="12">
-        <f>IF($B8="BLOCKED",IF(ROW()=2,$C8,$AF7),IF($B8="SMALL_SIDE",$E8,$C8))</f>
+        <f>IF($B8="BLOCKED",IF($BB8&gt;0,$AF7,$C8),IF($B8="SMALL_SIDE",$E8,$C8))</f>
         <v/>
       </c>
       <c r="AG8" s="12">
-        <f>IF($B8="BLOCKED",IF(ROW()=2,0,$AG7),IF($B8="SMALL_SIDE",$AM8,$W8))</f>
+        <f>IF($B8="BLOCKED",IF($BB8&gt;0,$BB8,$BA8),IF($B8="SMALL_SIDE",$AM8,$W8))</f>
         <v/>
       </c>
       <c r="AH8" s="13" t="inlineStr">
@@ -7452,15 +8254,15 @@
         <v/>
       </c>
       <c r="AP8" s="12">
-        <f>IF(OR($AQ8="DUAL_TAIL",$AQ8="DANGER",$AQ8="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ8="MANUAL_READY",$BG8="YES"),"YES",IF(OR($AQ8="DUAL_TAIL",$AQ8="DANGER",$AQ8="STOP",$AQ8="STOP_CLEARED",$AQ8="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ8" s="12">
-        <f>IF($B8="BLOCKED","STOP",IF($AK8=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G8/$D8,0)&gt;Settings!$B$16,IFERROR($J8/$G8,0)&gt;Settings!$B$17,$AE8&gt;$AD8,$Y8&lt;0,$AG8&gt;$D8*1.0001,$S8&lt;-100),"DANGER",IF(OR(AND($B8="BIG_SIDE",$U8&lt;=0),$S8&lt;=0,$X8=0,$AE8&gt;$AD8*0.95),"WARNING","OK"))))</f>
+        <f>IF($B8="BLOCKED",IF($BC8=0,"STOP_CLEARED",IF(OR(AND($BA8=0,$BB8&gt;0),AND($BA8&gt;0,$BB8=0)),"MANUAL_READY","STOP")),IF($AK8=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G8/$D8,0)&gt;Settings!$B$16,IFERROR($J8/$G8,0)&gt;Settings!$B$17,$AE8&gt;$AD8,$Y8&lt;0,$AG8&gt;$D8*1.0001,$S8&lt;-100),"DANGER",IF(OR(AND($B8="BIG_SIDE",$U8&lt;=0),$S8&lt;=0,$X8=0,$AE8&gt;$AD8*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR8" s="12">
-        <f>IF($B8="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B8="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ8="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B8="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B8="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ8="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS8" s="20">
@@ -7480,7 +8282,7 @@
         <v/>
       </c>
       <c r="AW8" s="12">
-        <f>IF($B8="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B8="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX8" s="12">
@@ -7494,6 +8296,32 @@
       <c r="AZ8" s="12">
         <f>IF($B8="BIG_SIDE",$V8*$AU8,0)</f>
         <v/>
+      </c>
+      <c r="BA8" s="12">
+        <f>IF($AK8=TRUE,MAX(0,$AJ8-$BD8),IF($B8="BLOCKED",MAX(0,$BA7-$BD8),0))</f>
+        <v/>
+      </c>
+      <c r="BB8" s="12">
+        <f>IF($AK8=TRUE,MAX(0,$AG8-$BE8),IF($B8="BLOCKED",MAX(0,$BB7-$BE8),0))</f>
+        <v/>
+      </c>
+      <c r="BC8" s="12">
+        <f>$BA8+$BB8</f>
+        <v/>
+      </c>
+      <c r="BD8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF8" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG8" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -7501,15 +8329,15 @@
         <v>8</v>
       </c>
       <c r="B9" s="13">
-        <f>IF(OR($AP8="NO",$AQ8="DUAL_TAIL",$AQ8="DANGER",$AQ8="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ8="MANUAL_READY",$BG8="YES"),"BIG_SIDE",IF(OR($AP8="NO",$AQ8="DUAL_TAIL",$AQ8="DANGER",$AQ8="STOP",$AQ8="MANUAL_READY",$AQ8="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C9" s="13">
-        <f>IF($B9="BLOCKED",$AF8,IF($AP8="YES",$AF8,$C8))</f>
+        <f>IF($B9="BLOCKED",$AF8,IF(AND($AQ8="MANUAL_READY",$BG8="YES"),$AF8,IF($AP8="YES",$AF8,$C8)))</f>
         <v/>
       </c>
       <c r="D9" s="13">
-        <f>IF($B9="BLOCKED",0,IF($AP8="YES",MAX(0,$AG8),$D8))</f>
+        <f>IF($B9="BLOCKED",0,IF(AND($AQ8="MANUAL_READY",$BG8="YES"),MAX($BA8,$BB8),IF($AP8="YES",MAX(0,$AG8),$D8)))</f>
         <v/>
       </c>
       <c r="E9" s="12">
@@ -7598,15 +8426,15 @@
         <v/>
       </c>
       <c r="AA9" s="12">
-        <f>IF($B9="BLOCKED",$Z9,IF($B9="BIG_SIDE",$Z9+$AX9-$AS9-$AZ9,IF($B9="SMALL_SIDE",$Z9+$S9+$AI9,$Z9+$S9)))</f>
+        <f>IF($B9="BLOCKED",$Z9+$BF9,IF($B9="BIG_SIDE",$Z9+$AX9-$AS9-$AZ9,IF($B9="SMALL_SIDE",$Z9+$S9+$AI9,$Z9+$S9)))</f>
         <v/>
       </c>
       <c r="AB9" s="12">
-        <f>IF($B9="BLOCKED",IF(ROW()=2,0,$AG8+$AJ8),$D9+$G9+$J9)</f>
+        <f>IF($B9="BLOCKED",$BC9,$D9+$G9+$J9)</f>
         <v/>
       </c>
       <c r="AC9" s="12">
-        <f>IF($B9="BLOCKED",$AB9,IF($B9="BIG_SIDE",$W9,$AG9+$AJ9))</f>
+        <f>IF($B9="BLOCKED",$BC9,IF($B9="BIG_SIDE",$W9,IF($AK9=TRUE,$BC9,$AG9)))</f>
         <v/>
       </c>
       <c r="AD9" s="12">
@@ -7618,11 +8446,11 @@
         <v/>
       </c>
       <c r="AF9" s="12">
-        <f>IF($B9="BLOCKED",IF(ROW()=2,$C9,$AF8),IF($B9="SMALL_SIDE",$E9,$C9))</f>
+        <f>IF($B9="BLOCKED",IF($BB9&gt;0,$AF8,$C9),IF($B9="SMALL_SIDE",$E9,$C9))</f>
         <v/>
       </c>
       <c r="AG9" s="12">
-        <f>IF($B9="BLOCKED",IF(ROW()=2,0,$AG8),IF($B9="SMALL_SIDE",$AM9,$W9))</f>
+        <f>IF($B9="BLOCKED",IF($BB9&gt;0,$BB9,$BA9),IF($B9="SMALL_SIDE",$AM9,$W9))</f>
         <v/>
       </c>
       <c r="AH9" s="13" t="inlineStr">
@@ -7658,15 +8486,15 @@
         <v/>
       </c>
       <c r="AP9" s="12">
-        <f>IF(OR($AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ9="MANUAL_READY",$BG9="YES"),"YES",IF(OR($AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP",$AQ9="STOP_CLEARED",$AQ9="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ9" s="12">
-        <f>IF($B9="BLOCKED","STOP",IF($AK9=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G9/$D9,0)&gt;Settings!$B$16,IFERROR($J9/$G9,0)&gt;Settings!$B$17,$AE9&gt;$AD9,$Y9&lt;0,$AG9&gt;$D9*1.0001,$S9&lt;-100),"DANGER",IF(OR(AND($B9="BIG_SIDE",$U9&lt;=0),$S9&lt;=0,$X9=0,$AE9&gt;$AD9*0.95),"WARNING","OK"))))</f>
+        <f>IF($B9="BLOCKED",IF($BC9=0,"STOP_CLEARED",IF(OR(AND($BA9=0,$BB9&gt;0),AND($BA9&gt;0,$BB9=0)),"MANUAL_READY","STOP")),IF($AK9=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G9/$D9,0)&gt;Settings!$B$16,IFERROR($J9/$G9,0)&gt;Settings!$B$17,$AE9&gt;$AD9,$Y9&lt;0,$AG9&gt;$D9*1.0001,$S9&lt;-100),"DANGER",IF(OR(AND($B9="BIG_SIDE",$U9&lt;=0),$S9&lt;=0,$X9=0,$AE9&gt;$AD9*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR9" s="12">
-        <f>IF($B9="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B9="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ9="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B9="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B9="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ9="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS9" s="20">
@@ -7686,7 +8514,7 @@
         <v/>
       </c>
       <c r="AW9" s="12">
-        <f>IF($B9="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B9="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX9" s="12">
@@ -7700,6 +8528,32 @@
       <c r="AZ9" s="12">
         <f>IF($B9="BIG_SIDE",$V9*$AU9,0)</f>
         <v/>
+      </c>
+      <c r="BA9" s="12">
+        <f>IF($AK9=TRUE,MAX(0,$AJ9-$BD9),IF($B9="BLOCKED",MAX(0,$BA8-$BD9),0))</f>
+        <v/>
+      </c>
+      <c r="BB9" s="12">
+        <f>IF($AK9=TRUE,MAX(0,$AG9-$BE9),IF($B9="BLOCKED",MAX(0,$BB8-$BE9),0))</f>
+        <v/>
+      </c>
+      <c r="BC9" s="12">
+        <f>$BA9+$BB9</f>
+        <v/>
+      </c>
+      <c r="BD9" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE9" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF9" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG9" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -7707,15 +8561,15 @@
         <v>9</v>
       </c>
       <c r="B10" s="13">
-        <f>IF(OR($AP9="NO",$AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ9="MANUAL_READY",$BG9="YES"),"BIG_SIDE",IF(OR($AP9="NO",$AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP",$AQ9="MANUAL_READY",$AQ9="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C10" s="13">
-        <f>IF($B10="BLOCKED",$AF9,IF($AP9="YES",$AF9,$C9))</f>
+        <f>IF($B10="BLOCKED",$AF9,IF(AND($AQ9="MANUAL_READY",$BG9="YES"),$AF9,IF($AP9="YES",$AF9,$C9)))</f>
         <v/>
       </c>
       <c r="D10" s="13">
-        <f>IF($B10="BLOCKED",0,IF($AP9="YES",MAX(0,$AG9),$D9))</f>
+        <f>IF($B10="BLOCKED",0,IF(AND($AQ9="MANUAL_READY",$BG9="YES"),MAX($BA9,$BB9),IF($AP9="YES",MAX(0,$AG9),$D9)))</f>
         <v/>
       </c>
       <c r="E10" s="12">
@@ -7804,15 +8658,15 @@
         <v/>
       </c>
       <c r="AA10" s="12">
-        <f>IF($B10="BLOCKED",$Z10,IF($B10="BIG_SIDE",$Z10+$AX10-$AS10-$AZ10,IF($B10="SMALL_SIDE",$Z10+$S10+$AI10,$Z10+$S10)))</f>
+        <f>IF($B10="BLOCKED",$Z10+$BF10,IF($B10="BIG_SIDE",$Z10+$AX10-$AS10-$AZ10,IF($B10="SMALL_SIDE",$Z10+$S10+$AI10,$Z10+$S10)))</f>
         <v/>
       </c>
       <c r="AB10" s="12">
-        <f>IF($B10="BLOCKED",IF(ROW()=2,0,$AG9+$AJ9),$D10+$G10+$J10)</f>
+        <f>IF($B10="BLOCKED",$BC10,$D10+$G10+$J10)</f>
         <v/>
       </c>
       <c r="AC10" s="12">
-        <f>IF($B10="BLOCKED",$AB10,IF($B10="BIG_SIDE",$W10,$AG10+$AJ10))</f>
+        <f>IF($B10="BLOCKED",$BC10,IF($B10="BIG_SIDE",$W10,IF($AK10=TRUE,$BC10,$AG10)))</f>
         <v/>
       </c>
       <c r="AD10" s="12">
@@ -7824,11 +8678,11 @@
         <v/>
       </c>
       <c r="AF10" s="12">
-        <f>IF($B10="BLOCKED",IF(ROW()=2,$C10,$AF9),IF($B10="SMALL_SIDE",$E10,$C10))</f>
+        <f>IF($B10="BLOCKED",IF($BB10&gt;0,$AF9,$C10),IF($B10="SMALL_SIDE",$E10,$C10))</f>
         <v/>
       </c>
       <c r="AG10" s="12">
-        <f>IF($B10="BLOCKED",IF(ROW()=2,0,$AG9),IF($B10="SMALL_SIDE",$AM10,$W10))</f>
+        <f>IF($B10="BLOCKED",IF($BB10&gt;0,$BB10,$BA10),IF($B10="SMALL_SIDE",$AM10,$W10))</f>
         <v/>
       </c>
       <c r="AH10" s="13" t="inlineStr">
@@ -7864,15 +8718,15 @@
         <v/>
       </c>
       <c r="AP10" s="12">
-        <f>IF(OR($AQ10="DUAL_TAIL",$AQ10="DANGER",$AQ10="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ10="MANUAL_READY",$BG10="YES"),"YES",IF(OR($AQ10="DUAL_TAIL",$AQ10="DANGER",$AQ10="STOP",$AQ10="STOP_CLEARED",$AQ10="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ10" s="12">
-        <f>IF($B10="BLOCKED","STOP",IF($AK10=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G10/$D10,0)&gt;Settings!$B$16,IFERROR($J10/$G10,0)&gt;Settings!$B$17,$AE10&gt;$AD10,$Y10&lt;0,$AG10&gt;$D10*1.0001,$S10&lt;-100),"DANGER",IF(OR(AND($B10="BIG_SIDE",$U10&lt;=0),$S10&lt;=0,$X10=0,$AE10&gt;$AD10*0.95),"WARNING","OK"))))</f>
+        <f>IF($B10="BLOCKED",IF($BC10=0,"STOP_CLEARED",IF(OR(AND($BA10=0,$BB10&gt;0),AND($BA10&gt;0,$BB10=0)),"MANUAL_READY","STOP")),IF($AK10=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G10/$D10,0)&gt;Settings!$B$16,IFERROR($J10/$G10,0)&gt;Settings!$B$17,$AE10&gt;$AD10,$Y10&lt;0,$AG10&gt;$D10*1.0001,$S10&lt;-100),"DANGER",IF(OR(AND($B10="BIG_SIDE",$U10&lt;=0),$S10&lt;=0,$X10=0,$AE10&gt;$AD10*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR10" s="12">
-        <f>IF($B10="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B10="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ10="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B10="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B10="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ10="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS10" s="20">
@@ -7892,7 +8746,7 @@
         <v/>
       </c>
       <c r="AW10" s="12">
-        <f>IF($B10="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B10="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX10" s="12">
@@ -7906,6 +8760,32 @@
       <c r="AZ10" s="12">
         <f>IF($B10="BIG_SIDE",$V10*$AU10,0)</f>
         <v/>
+      </c>
+      <c r="BA10" s="12">
+        <f>IF($AK10=TRUE,MAX(0,$AJ10-$BD10),IF($B10="BLOCKED",MAX(0,$BA9-$BD10),0))</f>
+        <v/>
+      </c>
+      <c r="BB10" s="12">
+        <f>IF($AK10=TRUE,MAX(0,$AG10-$BE10),IF($B10="BLOCKED",MAX(0,$BB9-$BE10),0))</f>
+        <v/>
+      </c>
+      <c r="BC10" s="12">
+        <f>$BA10+$BB10</f>
+        <v/>
+      </c>
+      <c r="BD10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF10" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG10" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -7913,15 +8793,15 @@
         <v>10</v>
       </c>
       <c r="B11" s="13">
-        <f>IF(OR($AP10="NO",$AQ10="DUAL_TAIL",$AQ10="DANGER",$AQ10="STOP"),"BLOCKED","BIG_SIDE")</f>
+        <f>IF(AND($AQ10="MANUAL_READY",$BG10="YES"),"BIG_SIDE",IF(OR($AP10="NO",$AQ10="DUAL_TAIL",$AQ10="DANGER",$AQ10="STOP",$AQ10="MANUAL_READY",$AQ10="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
         <v/>
       </c>
       <c r="C11" s="13">
-        <f>IF($B11="BLOCKED",$AF10,IF($AP10="YES",$AF10,$C10))</f>
+        <f>IF($B11="BLOCKED",$AF10,IF(AND($AQ10="MANUAL_READY",$BG10="YES"),$AF10,IF($AP10="YES",$AF10,$C10)))</f>
         <v/>
       </c>
       <c r="D11" s="13">
-        <f>IF($B11="BLOCKED",0,IF($AP10="YES",MAX(0,$AG10),$D10))</f>
+        <f>IF($B11="BLOCKED",0,IF(AND($AQ10="MANUAL_READY",$BG10="YES"),MAX($BA10,$BB10),IF($AP10="YES",MAX(0,$AG10),$D10)))</f>
         <v/>
       </c>
       <c r="E11" s="12">
@@ -8010,15 +8890,15 @@
         <v/>
       </c>
       <c r="AA11" s="12">
-        <f>IF($B11="BLOCKED",$Z11,IF($B11="BIG_SIDE",$Z11+$AX11-$AS11-$AZ11,IF($B11="SMALL_SIDE",$Z11+$S11+$AI11,$Z11+$S11)))</f>
+        <f>IF($B11="BLOCKED",$Z11+$BF11,IF($B11="BIG_SIDE",$Z11+$AX11-$AS11-$AZ11,IF($B11="SMALL_SIDE",$Z11+$S11+$AI11,$Z11+$S11)))</f>
         <v/>
       </c>
       <c r="AB11" s="12">
-        <f>IF($B11="BLOCKED",IF(ROW()=2,0,$AG10+$AJ10),$D11+$G11+$J11)</f>
+        <f>IF($B11="BLOCKED",$BC11,$D11+$G11+$J11)</f>
         <v/>
       </c>
       <c r="AC11" s="12">
-        <f>IF($B11="BLOCKED",$AB11,IF($B11="BIG_SIDE",$W11,$AG11+$AJ11))</f>
+        <f>IF($B11="BLOCKED",$BC11,IF($B11="BIG_SIDE",$W11,IF($AK11=TRUE,$BC11,$AG11)))</f>
         <v/>
       </c>
       <c r="AD11" s="12">
@@ -8030,11 +8910,11 @@
         <v/>
       </c>
       <c r="AF11" s="12">
-        <f>IF($B11="BLOCKED",IF(ROW()=2,$C11,$AF10),IF($B11="SMALL_SIDE",$E11,$C11))</f>
+        <f>IF($B11="BLOCKED",IF($BB11&gt;0,$AF10,$C11),IF($B11="SMALL_SIDE",$E11,$C11))</f>
         <v/>
       </c>
       <c r="AG11" s="12">
-        <f>IF($B11="BLOCKED",IF(ROW()=2,0,$AG10),IF($B11="SMALL_SIDE",$AM11,$W11))</f>
+        <f>IF($B11="BLOCKED",IF($BB11&gt;0,$BB11,$BA11),IF($B11="SMALL_SIDE",$AM11,$W11))</f>
         <v/>
       </c>
       <c r="AH11" s="13" t="inlineStr">
@@ -8070,15 +8950,15 @@
         <v/>
       </c>
       <c r="AP11" s="12">
-        <f>IF(OR($AQ11="DUAL_TAIL",$AQ11="DANGER",$AQ11="STOP"),"NO","YES")</f>
+        <f>IF(AND($AQ11="MANUAL_READY",$BG11="YES"),"YES",IF(OR($AQ11="DUAL_TAIL",$AQ11="DANGER",$AQ11="STOP",$AQ11="STOP_CLEARED",$AQ11="MANUAL_READY"),"NO","YES"))</f>
         <v/>
       </c>
       <c r="AQ11" s="12">
-        <f>IF($B11="BLOCKED","STOP",IF($AK11=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G11/$D11,0)&gt;Settings!$B$16,IFERROR($J11/$G11,0)&gt;Settings!$B$17,$AE11&gt;$AD11,$Y11&lt;0,$AG11&gt;$D11*1.0001,$S11&lt;-100),"DANGER",IF(OR(AND($B11="BIG_SIDE",$U11&lt;=0),$S11&lt;=0,$X11=0,$AE11&gt;$AD11*0.95),"WARNING","OK"))))</f>
+        <f>IF($B11="BLOCKED",IF($BC11=0,"STOP_CLEARED",IF(OR(AND($BA11=0,$BB11&gt;0),AND($BA11&gt;0,$BB11=0)),"MANUAL_READY","STOP")),IF($AK11=TRUE,"DUAL_TAIL",IF(OR(IFERROR($G11/$D11,0)&gt;Settings!$B$16,IFERROR($J11/$G11,0)&gt;Settings!$B$17,$AE11&gt;$AD11,$Y11&lt;0,$AG11&gt;$D11*1.0001,$S11&lt;-100),"DANGER",IF(OR(AND($B11="BIG_SIDE",$U11&lt;=0),$S11&lt;=0,$X11=0,$AE11&gt;$AD11*0.95),"WARNING","OK"))))</f>
         <v/>
       </c>
       <c r="AR11" s="12">
-        <f>IF($B11="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень",IF($B11="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ11="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
+        <f>IF($B11="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B11="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ11="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
         <v/>
       </c>
       <c r="AS11" s="20">
@@ -8098,7 +8978,7 @@
         <v/>
       </c>
       <c r="AW11" s="12">
-        <f>IF($B11="BLOCKED","Заблокировано: предыдущий уровень не разрешил новый полноценный уровень","")</f>
+        <f>IF($B11="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия","")</f>
         <v/>
       </c>
       <c r="AX11" s="12">
@@ -8113,9 +8993,35 @@
         <f>IF($B11="BIG_SIDE",$V11*$AU11,0)</f>
         <v/>
       </c>
+      <c r="BA11" s="12">
+        <f>IF($AK11=TRUE,MAX(0,$AJ11-$BD11),IF($B11="BLOCKED",MAX(0,$BA10-$BD11),0))</f>
+        <v/>
+      </c>
+      <c r="BB11" s="12">
+        <f>IF($AK11=TRUE,MAX(0,$AG11-$BE11),IF($B11="BLOCKED",MAX(0,$BB10-$BE11),0))</f>
+        <v/>
+      </c>
+      <c r="BC11" s="12">
+        <f>$BA11+$BB11</f>
+        <v/>
+      </c>
+      <c r="BD11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF11" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG11" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AZ11"/>
+  <autoFilter ref="A1:BG11"/>
   <conditionalFormatting sqref="AQ2:AQ11">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AQ2="WARNING"</formula>
@@ -8151,7 +9057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8397,6 +9303,134 @@
       </c>
       <c r="C15" s="3">
         <f>LOOKUP(2,1/(Calculator!AQ2:AQ11&lt;&gt;""),Calculator!AQ2:AQ11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Max DualTail Exposure</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>MAX DualTailTotalLot</t>
+        </is>
+      </c>
+      <c r="C16" s="3">
+        <f>MAX(Calculator!BC2:BC11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Final ActiveOldFarLot</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>last ActiveOldFarLot</t>
+        </is>
+      </c>
+      <c r="C17" s="3">
+        <f>LOOKUP(2,1/(Calculator!BA2:BA11&lt;&gt;""),Calculator!BA2:BA11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Final ActiveNewFarLot</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>last ActiveNewFarLot</t>
+        </is>
+      </c>
+      <c r="C18" s="3">
+        <f>LOOKUP(2,1/(Calculator!BB2:BB11&lt;&gt;""),Calculator!BB2:BB11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Final DualTailTotalLot</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>last DualTailTotalLot</t>
+        </is>
+      </c>
+      <c r="C19" s="3">
+        <f>LOOKUP(2,1/(Calculator!BC2:BC11&lt;&gt;""),Calculator!BC2:BC11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Manual Close PL</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>SUM ManualClosePL</t>
+        </is>
+      </c>
+      <c r="C20" s="3">
+        <f>SUM(Calculator!BF2:BF11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Blocked Levels Count</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>COUNTIF Scenario BLOCKED</t>
+        </is>
+      </c>
+      <c r="C21" s="3">
+        <f>COUNTIF(Calculator!B2:B11,"BLOCKED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Stop Cleared Count</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>COUNTIF Status STOP_CLEARED</t>
+        </is>
+      </c>
+      <c r="C22" s="3">
+        <f>COUNTIF(Calculator!AQ2:AQ11,"STOP_CLEARED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Manual Ready Count</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>COUNTIF Status MANUAL_READY</t>
+        </is>
+      </c>
+      <c r="C23" s="3">
+        <f>COUNTIF(Calculator!AQ2:AQ11,"MANUAL_READY")</f>
         <v/>
       </c>
     </row>
@@ -8411,7 +9445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10103,8 +11137,638 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>T40</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>DUAL_TAIL ActiveOldFarLot equals OldFarRemainLot</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>DUAL_TAIL row</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>ActiveOldFarLot = OldFarRemainLot unless manual close</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>BA = AJ - ManualOldFarCloseLot</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>BA formula</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Старый хвост фиксируется в активном состоянии.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>T41</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>DUAL_TAIL ActiveNewFarLot equals NewFarStartLot</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>DUAL_TAIL row</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>ActiveNewFarLot = NewFarStartLot unless manual close</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>BB = AG - ManualNewFarCloseLot</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>BB formula</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Новый хвост фиксируется отдельно.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>T42</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>DualTailTotalLot sums active tails</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Any DUAL/BLOCKED row</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>DualTailTotalLot = ActiveOldFarLot + ActiveNewFarLot</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>BC=BA+BB</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>BC formula</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Суммарная экспозиция двух хвостов не теряется.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>T43</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Next BLOCKED keeps both tails</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Row after DUAL_TAIL</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>ActiveOld/New copy previous active tails minus manual close</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>BA/BB previous carry</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>BA/BB blocked formulas</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Следующий заблокированный уровень сохраняет оба хвоста.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>T44</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Second BLOCKED keeps both tails</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Second blocked row</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Old tail still present without manual close</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>BA persists</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>BA formula</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Старый хвост не исчезает во второй BLOCKED строке.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>T45</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>OpenLotsAfter BLOCKED equals DualTailTotalLot</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>BLOCKED row</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>OpenLotsAfter = DualTailTotalLot</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>AC=BC</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>AC formula</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Открытые лоты после блокировки считаются по двум хвостам.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>T46</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>MarginAfter BLOCKED from both tails</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>BLOCKED row</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>MarginAfter = DualTailTotalLot × MarginPerLot</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>AE=AC*MarginPerLot</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>AE formula</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Маржа не падает искусственно.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>T47</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>BigLot zero in BLOCKED</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>BLOCKED row</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>BigLot = 0</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>G=0 when B=BLOCKED</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>G formula</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Новый Big не открывается.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>T48</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>SmallLot zero in BLOCKED</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>BLOCKED row</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>SmallLot = 0</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>J=0 when B=BLOCKED</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>J formula</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Новый Small не открывается.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>T49</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Status remains STOP while two tails active</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>BLOCKED with BA&gt;0 and BB&gt;0</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Status = STOP</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>AQ STOP</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>AQ formula</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Без ручного закрытия статус не OK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>T50</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Old tail cannot disappear without manual close</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>ManualOldFarCloseLot=0</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>ActiveOldFarLot persists</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>BA current=BA previous</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>BA formula</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Старый хвост не обнуляется автоматически.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>T51</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>New tail cannot disappear without manual close</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>ManualNewFarCloseLot=0</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>ActiveNewFarLot persists</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>BB current=BB previous</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>BB formula</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Новый хвост не обнуляется автоматически.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>T52</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>ManualOldFarCloseLot reduces old tail</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Manual close input</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>ActiveOldFarLot = PreviousActiveOldFarLot - ManualOldFarCloseLot</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>BA=MAX(0,BAprev-BD)</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>BA formula</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Ручное закрытие уменьшает старый хвост.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>T53</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Full old-tail manual close creates MANUAL_READY</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>BA=0 and BB&gt;0</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Status = MANUAL_READY</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>AQ MANUAL_READY branch</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>AQ formula</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Один оставшийся хвост требует ручного разрешения.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>T54</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>New level requires ManualAllowNewLevel YES</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>MANUAL_READY previous</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Next row BLOCKED unless ManualAllowNewLevel=YES</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>B checks BG="YES"</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>B formula</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Автоматический перезапуск запрещён без ручного разрешения.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H40"/>
+  <autoFilter ref="A1:H55"/>
   <conditionalFormatting sqref="D2:D18">
     <cfRule type="expression" priority="1" dxfId="2">
       <formula>$D2="FAIL"</formula>

</xml_diff>

<commit_message>
Fix circular references and global risk sync
</commit_message>
<xml_diff>
--- a/work/MinusLock_SelfCompressing_BigSmall_v2/MinusLock_SelfCompressing_BigSmall_v2.xlsx
+++ b/work/MinusLock_SelfCompressing_BigSmall_v2/MinusLock_SelfCompressing_BigSmall_v2.xlsx
@@ -1378,7 +1378,7 @@
         <v/>
       </c>
       <c r="X2" s="19">
-        <f>IF($B2="BIG_SIDE",IF($AX2&gt;0,$AX2-$AS2,0),IF($S2&gt;0,$S2*0.5,0))</f>
+        <f>IF($B2="BIG_SIDE",IF($AX$2&gt;0,$AX$2-$AS$2,0),IF($S$2&gt;0,$S$2*0.5,0))</f>
         <v/>
       </c>
       <c r="Y2" s="19">
@@ -1409,11 +1409,11 @@
         <v/>
       </c>
       <c r="AF2" s="12">
-        <f>IF($B2="BLOCKED",IF($BB2&gt;0,$AF2,$C2),IF($B2="SMALL_SIDE",$E2,$C2))</f>
+        <f>IF($B2="BLOCKED",$C2,IF($B2="SMALL_SIDE",$E2,$C2))</f>
         <v/>
       </c>
       <c r="AG2" s="12">
-        <f>IF($B2="BLOCKED",IF($BB2&gt;0,$BB2,$BA2),IF($B2="SMALL_SIDE",$AM2,$W2))</f>
+        <f>IF($B2="BLOCKED",0,IF($B2="SMALL_SIDE",$AM2,$W2))</f>
         <v/>
       </c>
       <c r="AH2" s="13" t="inlineStr">
@@ -1481,7 +1481,7 @@
         <v/>
       </c>
       <c r="AX2" s="12">
-        <f>IF($B2="BIG_SIDE",$N2-$P2-$AY2,IF($B2="SMALL_SIDE",$O2-$Q2-$R2,0))</f>
+        <f>IF($B2="BIG_SIDE",$N2-$P2-$AY2,0)</f>
         <v/>
       </c>
       <c r="AY2" s="12">
@@ -1609,7 +1609,7 @@
         <v/>
       </c>
       <c r="X3" s="19">
-        <f>IF($B3="BIG_SIDE",IF($AX3&gt;0,$AX3-$AS3,0),IF($S3&gt;0,$S3*0.5,0))</f>
+        <f>IF($B3="BIG_SIDE",IF($AX$3&gt;0,$AX$3-$AS$3,0),IF($S$3&gt;0,$S$3*0.5,0))</f>
         <v/>
       </c>
       <c r="Y3" s="19">
@@ -1645,7 +1645,7 @@
         <v/>
       </c>
       <c r="AG3" s="12">
-        <f>IF($B3="BLOCKED",IF($BB3&gt;0,$BB3,$BA3),IF($B3="SMALL_SIDE",$AM3,$W3))</f>
+        <f>IF($B3="BLOCKED",IF($BB2&gt;0,$BB2,$BA2),IF($B3="SMALL_SIDE",$AM3,$W3))</f>
         <v/>
       </c>
       <c r="AH3" s="13" t="inlineStr">
@@ -1713,7 +1713,7 @@
         <v/>
       </c>
       <c r="AX3" s="12">
-        <f>IF($B3="BIG_SIDE",$N3-$P3-$AY3,IF($B3="SMALL_SIDE",$O3-$Q3-$R3,0))</f>
+        <f>IF($B3="BIG_SIDE",$N3-$P3-$AY3,0)</f>
         <v/>
       </c>
       <c r="AY3" s="12">
@@ -1841,7 +1841,7 @@
         <v/>
       </c>
       <c r="X4" s="19">
-        <f>IF($B4="BIG_SIDE",IF($AX4&gt;0,$AX4-$AS4,0),IF($S4&gt;0,$S4*0.5,0))</f>
+        <f>IF($B4="BIG_SIDE",IF($AX$4&gt;0,$AX$4-$AS$4,0),IF($S$4&gt;0,$S$4*0.5,0))</f>
         <v/>
       </c>
       <c r="Y4" s="19">
@@ -1877,7 +1877,7 @@
         <v/>
       </c>
       <c r="AG4" s="12">
-        <f>IF($B4="BLOCKED",IF($BB4&gt;0,$BB4,$BA4),IF($B4="SMALL_SIDE",$AM4,$W4))</f>
+        <f>IF($B4="BLOCKED",IF($BB3&gt;0,$BB3,$BA3),IF($B4="SMALL_SIDE",$AM4,$W4))</f>
         <v/>
       </c>
       <c r="AH4" s="13" t="inlineStr">
@@ -1945,7 +1945,7 @@
         <v/>
       </c>
       <c r="AX4" s="12">
-        <f>IF($B4="BIG_SIDE",$N4-$P4-$AY4,IF($B4="SMALL_SIDE",$O4-$Q4-$R4,0))</f>
+        <f>IF($B4="BIG_SIDE",$N4-$P4-$AY4,0)</f>
         <v/>
       </c>
       <c r="AY4" s="12">
@@ -2073,7 +2073,7 @@
         <v/>
       </c>
       <c r="X5" s="19">
-        <f>IF($B5="BIG_SIDE",IF($AX5&gt;0,$AX5-$AS5,0),IF($S5&gt;0,$S5*0.5,0))</f>
+        <f>IF($B5="BIG_SIDE",IF($AX$5&gt;0,$AX$5-$AS$5,0),IF($S$5&gt;0,$S$5*0.5,0))</f>
         <v/>
       </c>
       <c r="Y5" s="19">
@@ -2109,7 +2109,7 @@
         <v/>
       </c>
       <c r="AG5" s="12">
-        <f>IF($B5="BLOCKED",IF($BB5&gt;0,$BB5,$BA5),IF($B5="SMALL_SIDE",$AM5,$W5))</f>
+        <f>IF($B5="BLOCKED",IF($BB4&gt;0,$BB4,$BA4),IF($B5="SMALL_SIDE",$AM5,$W5))</f>
         <v/>
       </c>
       <c r="AH5" s="13" t="inlineStr">
@@ -2177,7 +2177,7 @@
         <v/>
       </c>
       <c r="AX5" s="12">
-        <f>IF($B5="BIG_SIDE",$N5-$P5-$AY5,IF($B5="SMALL_SIDE",$O5-$Q5-$R5,0))</f>
+        <f>IF($B5="BIG_SIDE",$N5-$P5-$AY5,0)</f>
         <v/>
       </c>
       <c r="AY5" s="12">
@@ -2305,7 +2305,7 @@
         <v/>
       </c>
       <c r="X6" s="19">
-        <f>IF($B6="BIG_SIDE",IF($AX6&gt;0,$AX6-$AS6,0),IF($S6&gt;0,$S6*0.5,0))</f>
+        <f>IF($B6="BIG_SIDE",IF($AX$6&gt;0,$AX$6-$AS$6,0),IF($S$6&gt;0,$S$6*0.5,0))</f>
         <v/>
       </c>
       <c r="Y6" s="19">
@@ -2341,7 +2341,7 @@
         <v/>
       </c>
       <c r="AG6" s="12">
-        <f>IF($B6="BLOCKED",IF($BB6&gt;0,$BB6,$BA6),IF($B6="SMALL_SIDE",$AM6,$W6))</f>
+        <f>IF($B6="BLOCKED",IF($BB5&gt;0,$BB5,$BA5),IF($B6="SMALL_SIDE",$AM6,$W6))</f>
         <v/>
       </c>
       <c r="AH6" s="13" t="inlineStr">
@@ -2409,7 +2409,7 @@
         <v/>
       </c>
       <c r="AX6" s="12">
-        <f>IF($B6="BIG_SIDE",$N6-$P6-$AY6,IF($B6="SMALL_SIDE",$O6-$Q6-$R6,0))</f>
+        <f>IF($B6="BIG_SIDE",$N6-$P6-$AY6,0)</f>
         <v/>
       </c>
       <c r="AY6" s="12">
@@ -2537,7 +2537,7 @@
         <v/>
       </c>
       <c r="X7" s="19">
-        <f>IF($B7="BIG_SIDE",IF($AX7&gt;0,$AX7-$AS7,0),IF($S7&gt;0,$S7*0.5,0))</f>
+        <f>IF($B7="BIG_SIDE",IF($AX$7&gt;0,$AX$7-$AS$7,0),IF($S$7&gt;0,$S$7*0.5,0))</f>
         <v/>
       </c>
       <c r="Y7" s="19">
@@ -2573,7 +2573,7 @@
         <v/>
       </c>
       <c r="AG7" s="12">
-        <f>IF($B7="BLOCKED",IF($BB7&gt;0,$BB7,$BA7),IF($B7="SMALL_SIDE",$AM7,$W7))</f>
+        <f>IF($B7="BLOCKED",IF($BB6&gt;0,$BB6,$BA6),IF($B7="SMALL_SIDE",$AM7,$W7))</f>
         <v/>
       </c>
       <c r="AH7" s="13" t="inlineStr">
@@ -2641,7 +2641,7 @@
         <v/>
       </c>
       <c r="AX7" s="12">
-        <f>IF($B7="BIG_SIDE",$N7-$P7-$AY7,IF($B7="SMALL_SIDE",$O7-$Q7-$R7,0))</f>
+        <f>IF($B7="BIG_SIDE",$N7-$P7-$AY7,0)</f>
         <v/>
       </c>
       <c r="AY7" s="12">
@@ -2769,7 +2769,7 @@
         <v/>
       </c>
       <c r="X8" s="19">
-        <f>IF($B8="BIG_SIDE",IF($AX8&gt;0,$AX8-$AS8,0),IF($S8&gt;0,$S8*0.5,0))</f>
+        <f>IF($B8="BIG_SIDE",IF($AX$8&gt;0,$AX$8-$AS$8,0),IF($S$8&gt;0,$S$8*0.5,0))</f>
         <v/>
       </c>
       <c r="Y8" s="19">
@@ -2805,7 +2805,7 @@
         <v/>
       </c>
       <c r="AG8" s="12">
-        <f>IF($B8="BLOCKED",IF($BB8&gt;0,$BB8,$BA8),IF($B8="SMALL_SIDE",$AM8,$W8))</f>
+        <f>IF($B8="BLOCKED",IF($BB7&gt;0,$BB7,$BA7),IF($B8="SMALL_SIDE",$AM8,$W8))</f>
         <v/>
       </c>
       <c r="AH8" s="13" t="inlineStr">
@@ -2873,7 +2873,7 @@
         <v/>
       </c>
       <c r="AX8" s="12">
-        <f>IF($B8="BIG_SIDE",$N8-$P8-$AY8,IF($B8="SMALL_SIDE",$O8-$Q8-$R8,0))</f>
+        <f>IF($B8="BIG_SIDE",$N8-$P8-$AY8,0)</f>
         <v/>
       </c>
       <c r="AY8" s="12">
@@ -3001,7 +3001,7 @@
         <v/>
       </c>
       <c r="X9" s="19">
-        <f>IF($B9="BIG_SIDE",IF($AX9&gt;0,$AX9-$AS9,0),IF($S9&gt;0,$S9*0.5,0))</f>
+        <f>IF($B9="BIG_SIDE",IF($AX$9&gt;0,$AX$9-$AS$9,0),IF($S$9&gt;0,$S$9*0.5,0))</f>
         <v/>
       </c>
       <c r="Y9" s="19">
@@ -3037,7 +3037,7 @@
         <v/>
       </c>
       <c r="AG9" s="12">
-        <f>IF($B9="BLOCKED",IF($BB9&gt;0,$BB9,$BA9),IF($B9="SMALL_SIDE",$AM9,$W9))</f>
+        <f>IF($B9="BLOCKED",IF($BB8&gt;0,$BB8,$BA8),IF($B9="SMALL_SIDE",$AM9,$W9))</f>
         <v/>
       </c>
       <c r="AH9" s="13" t="inlineStr">
@@ -3105,7 +3105,7 @@
         <v/>
       </c>
       <c r="AX9" s="12">
-        <f>IF($B9="BIG_SIDE",$N9-$P9-$AY9,IF($B9="SMALL_SIDE",$O9-$Q9-$R9,0))</f>
+        <f>IF($B9="BIG_SIDE",$N9-$P9-$AY9,0)</f>
         <v/>
       </c>
       <c r="AY9" s="12">
@@ -3233,7 +3233,7 @@
         <v/>
       </c>
       <c r="X10" s="19">
-        <f>IF($B10="BIG_SIDE",IF($AX10&gt;0,$AX10-$AS10,0),IF($S10&gt;0,$S10*0.5,0))</f>
+        <f>IF($B10="BIG_SIDE",IF($AX$10&gt;0,$AX$10-$AS$10,0),IF($S$10&gt;0,$S$10*0.5,0))</f>
         <v/>
       </c>
       <c r="Y10" s="19">
@@ -3269,7 +3269,7 @@
         <v/>
       </c>
       <c r="AG10" s="12">
-        <f>IF($B10="BLOCKED",IF($BB10&gt;0,$BB10,$BA10),IF($B10="SMALL_SIDE",$AM10,$W10))</f>
+        <f>IF($B10="BLOCKED",IF($BB9&gt;0,$BB9,$BA9),IF($B10="SMALL_SIDE",$AM10,$W10))</f>
         <v/>
       </c>
       <c r="AH10" s="13" t="inlineStr">
@@ -3337,7 +3337,7 @@
         <v/>
       </c>
       <c r="AX10" s="12">
-        <f>IF($B10="BIG_SIDE",$N10-$P10-$AY10,IF($B10="SMALL_SIDE",$O10-$Q10-$R10,0))</f>
+        <f>IF($B10="BIG_SIDE",$N10-$P10-$AY10,0)</f>
         <v/>
       </c>
       <c r="AY10" s="12">
@@ -3465,7 +3465,7 @@
         <v/>
       </c>
       <c r="X11" s="19">
-        <f>IF($B11="BIG_SIDE",IF($AX11&gt;0,$AX11-$AS11,0),IF($S11&gt;0,$S11*0.5,0))</f>
+        <f>IF($B11="BIG_SIDE",IF($AX$11&gt;0,$AX$11-$AS$11,0),IF($S$11&gt;0,$S$11*0.5,0))</f>
         <v/>
       </c>
       <c r="Y11" s="19">
@@ -3501,7 +3501,7 @@
         <v/>
       </c>
       <c r="AG11" s="12">
-        <f>IF($B11="BLOCKED",IF($BB11&gt;0,$BB11,$BA11),IF($B11="SMALL_SIDE",$AM11,$W11))</f>
+        <f>IF($B11="BLOCKED",IF($BB10&gt;0,$BB10,$BA10),IF($B11="SMALL_SIDE",$AM11,$W11))</f>
         <v/>
       </c>
       <c r="AH11" s="13" t="inlineStr">
@@ -3569,7 +3569,7 @@
         <v/>
       </c>
       <c r="AX11" s="12">
-        <f>IF($B11="BIG_SIDE",$N11-$P11-$AY11,IF($B11="SMALL_SIDE",$O11-$Q11-$R11,0))</f>
+        <f>IF($B11="BIG_SIDE",$N11-$P11-$AY11,0)</f>
         <v/>
       </c>
       <c r="AY11" s="12">
@@ -4097,7 +4097,7 @@
         <v/>
       </c>
       <c r="X2" s="19">
-        <f>IF($B2="BIG_SIDE",IF($AX2&gt;0,$AX2-$AS2,0),IF($S2&gt;0,$S2*0.5,0))</f>
+        <f>IF($B2="BIG_SIDE",IF($AX$2&gt;0,$AX$2-$AS$2,0),IF($S$2&gt;0,$S$2*0.5,0))</f>
         <v/>
       </c>
       <c r="Y2" s="19">
@@ -4128,11 +4128,11 @@
         <v/>
       </c>
       <c r="AF2" s="12">
-        <f>IF($B2="BLOCKED",IF($BB2&gt;0,$AF2,$C2),IF($B2="SMALL_SIDE",$E2,$C2))</f>
+        <f>IF($B2="BLOCKED",$C2,IF($B2="SMALL_SIDE",$E2,$C2))</f>
         <v/>
       </c>
       <c r="AG2" s="12">
-        <f>IF($B2="BLOCKED",IF($BB2&gt;0,$BB2,$BA2),IF($B2="SMALL_SIDE",$AM2,$W2))</f>
+        <f>IF($B2="BLOCKED",0,IF($B2="SMALL_SIDE",$AM2,$W2))</f>
         <v/>
       </c>
       <c r="AH2" s="13" t="inlineStr">
@@ -4200,7 +4200,7 @@
         <v/>
       </c>
       <c r="AX2" s="12">
-        <f>IF($B2="BIG_SIDE",$N2-$P2-$AY2,IF($B2="SMALL_SIDE",$O2-$Q2-$R2,0))</f>
+        <f>IF($B2="BIG_SIDE",$N2-$P2-$AY2,0)</f>
         <v/>
       </c>
       <c r="AY2" s="12">
@@ -4328,7 +4328,7 @@
         <v/>
       </c>
       <c r="X3" s="19">
-        <f>IF($B3="BIG_SIDE",IF($AX3&gt;0,$AX3-$AS3,0),IF($S3&gt;0,$S3*0.5,0))</f>
+        <f>IF($B3="BIG_SIDE",IF($AX$3&gt;0,$AX$3-$AS$3,0),IF($S$3&gt;0,$S$3*0.5,0))</f>
         <v/>
       </c>
       <c r="Y3" s="19">
@@ -4364,7 +4364,7 @@
         <v/>
       </c>
       <c r="AG3" s="12">
-        <f>IF($B3="BLOCKED",IF($BB3&gt;0,$BB3,$BA3),IF($B3="SMALL_SIDE",$AM3,$W3))</f>
+        <f>IF($B3="BLOCKED",IF($BB2&gt;0,$BB2,$BA2),IF($B3="SMALL_SIDE",$AM3,$W3))</f>
         <v/>
       </c>
       <c r="AH3" s="13" t="inlineStr">
@@ -4432,7 +4432,7 @@
         <v/>
       </c>
       <c r="AX3" s="12">
-        <f>IF($B3="BIG_SIDE",$N3-$P3-$AY3,IF($B3="SMALL_SIDE",$O3-$Q3-$R3,0))</f>
+        <f>IF($B3="BIG_SIDE",$N3-$P3-$AY3,0)</f>
         <v/>
       </c>
       <c r="AY3" s="12">
@@ -4560,7 +4560,7 @@
         <v/>
       </c>
       <c r="X4" s="19">
-        <f>IF($B4="BIG_SIDE",IF($AX4&gt;0,$AX4-$AS4,0),IF($S4&gt;0,$S4*0.5,0))</f>
+        <f>IF($B4="BIG_SIDE",IF($AX$4&gt;0,$AX$4-$AS$4,0),IF($S$4&gt;0,$S$4*0.5,0))</f>
         <v/>
       </c>
       <c r="Y4" s="19">
@@ -4596,7 +4596,7 @@
         <v/>
       </c>
       <c r="AG4" s="12">
-        <f>IF($B4="BLOCKED",IF($BB4&gt;0,$BB4,$BA4),IF($B4="SMALL_SIDE",$AM4,$W4))</f>
+        <f>IF($B4="BLOCKED",IF($BB3&gt;0,$BB3,$BA3),IF($B4="SMALL_SIDE",$AM4,$W4))</f>
         <v/>
       </c>
       <c r="AH4" s="13" t="inlineStr">
@@ -4664,7 +4664,7 @@
         <v/>
       </c>
       <c r="AX4" s="12">
-        <f>IF($B4="BIG_SIDE",$N4-$P4-$AY4,IF($B4="SMALL_SIDE",$O4-$Q4-$R4,0))</f>
+        <f>IF($B4="BIG_SIDE",$N4-$P4-$AY4,0)</f>
         <v/>
       </c>
       <c r="AY4" s="12">
@@ -4792,7 +4792,7 @@
         <v/>
       </c>
       <c r="X5" s="19">
-        <f>IF($B5="BIG_SIDE",IF($AX5&gt;0,$AX5-$AS5,0),IF($S5&gt;0,$S5*0.5,0))</f>
+        <f>IF($B5="BIG_SIDE",IF($AX$5&gt;0,$AX$5-$AS$5,0),IF($S$5&gt;0,$S$5*0.5,0))</f>
         <v/>
       </c>
       <c r="Y5" s="19">
@@ -4828,7 +4828,7 @@
         <v/>
       </c>
       <c r="AG5" s="12">
-        <f>IF($B5="BLOCKED",IF($BB5&gt;0,$BB5,$BA5),IF($B5="SMALL_SIDE",$AM5,$W5))</f>
+        <f>IF($B5="BLOCKED",IF($BB4&gt;0,$BB4,$BA4),IF($B5="SMALL_SIDE",$AM5,$W5))</f>
         <v>0.468</v>
       </c>
       <c r="AH5" s="13" t="inlineStr">
@@ -4896,7 +4896,7 @@
         <v/>
       </c>
       <c r="AX5" s="12">
-        <f>IF($B5="BIG_SIDE",$N5-$P5-$AY5,IF($B5="SMALL_SIDE",$O5-$Q5-$R5,0))</f>
+        <f>IF($B5="BIG_SIDE",$N5-$P5-$AY5,0)</f>
         <v/>
       </c>
       <c r="AY5" s="12">
@@ -5024,7 +5024,7 @@
         <v/>
       </c>
       <c r="X6" s="19">
-        <f>IF($B6="BIG_SIDE",IF($AX6&gt;0,$AX6-$AS6,0),IF($S6&gt;0,$S6*0.5,0))</f>
+        <f>IF($B6="BIG_SIDE",IF($AX$6&gt;0,$AX$6-$AS$6,0),IF($S$6&gt;0,$S$6*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y6" s="19">
@@ -5060,7 +5060,7 @@
         <v/>
       </c>
       <c r="AG6" s="12">
-        <f>IF($B6="BLOCKED",IF($BB6&gt;0,$BB6,$BA6),IF($B6="SMALL_SIDE",$AM6,$W6))</f>
+        <f>IF($B6="BLOCKED",IF($BB5&gt;0,$BB5,$BA5),IF($B6="SMALL_SIDE",$AM6,$W6))</f>
         <v/>
       </c>
       <c r="AH6" s="13" t="inlineStr">
@@ -5105,7 +5105,7 @@
       </c>
       <c r="AR6" s="12" t="str">
         <f>IF($B6="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B6="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ6="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS6" s="20">
         <f>IF($B6="BIG_SIDE",$V6*$U6,0)</f>
@@ -5128,7 +5128,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX6" s="12">
-        <f>IF($B6="BIG_SIDE",$N6-$P6-$AY6,IF($B6="SMALL_SIDE",$O6-$Q6-$R6,0))</f>
+        <f>IF($B6="BIG_SIDE",$N6-$P6-$AY6,0)</f>
         <v/>
       </c>
       <c r="AY6" s="12">
@@ -5256,7 +5256,7 @@
         <v/>
       </c>
       <c r="X7" s="19">
-        <f>IF($B7="BIG_SIDE",IF($AX7&gt;0,$AX7-$AS7,0),IF($S7&gt;0,$S7*0.5,0))</f>
+        <f>IF($B7="BIG_SIDE",IF($AX$7&gt;0,$AX$7-$AS$7,0),IF($S$7&gt;0,$S$7*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y7" s="19">
@@ -5292,7 +5292,7 @@
         <v/>
       </c>
       <c r="AG7" s="12">
-        <f>IF($B7="BLOCKED",IF($BB7&gt;0,$BB7,$BA7),IF($B7="SMALL_SIDE",$AM7,$W7))</f>
+        <f>IF($B7="BLOCKED",IF($BB6&gt;0,$BB6,$BA6),IF($B7="SMALL_SIDE",$AM7,$W7))</f>
         <v/>
       </c>
       <c r="AH7" s="13" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="AR7" s="12" t="str">
         <f>IF($B7="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B7="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ7="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS7" s="20">
         <f>IF($B7="BIG_SIDE",$V7*$U7,0)</f>
@@ -5360,7 +5360,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX7" s="12">
-        <f>IF($B7="BIG_SIDE",$N7-$P7-$AY7,IF($B7="SMALL_SIDE",$O7-$Q7-$R7,0))</f>
+        <f>IF($B7="BIG_SIDE",$N7-$P7-$AY7,0)</f>
         <v/>
       </c>
       <c r="AY7" s="12">
@@ -5488,7 +5488,7 @@
         <v/>
       </c>
       <c r="X8" s="19">
-        <f>IF($B8="BIG_SIDE",IF($AX8&gt;0,$AX8-$AS8,0),IF($S8&gt;0,$S8*0.5,0))</f>
+        <f>IF($B8="BIG_SIDE",IF($AX$8&gt;0,$AX$8-$AS$8,0),IF($S$8&gt;0,$S$8*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y8" s="19">
@@ -5524,7 +5524,7 @@
         <v/>
       </c>
       <c r="AG8" s="12">
-        <f>IF($B8="BLOCKED",IF($BB8&gt;0,$BB8,$BA8),IF($B8="SMALL_SIDE",$AM8,$W8))</f>
+        <f>IF($B8="BLOCKED",IF($BB7&gt;0,$BB7,$BA7),IF($B8="SMALL_SIDE",$AM8,$W8))</f>
         <v/>
       </c>
       <c r="AH8" s="13" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="AR8" s="12" t="str">
         <f>IF($B8="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B8="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ8="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS8" s="20">
         <f>IF($B8="BIG_SIDE",$V8*$U8,0)</f>
@@ -5592,7 +5592,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX8" s="12">
-        <f>IF($B8="BIG_SIDE",$N8-$P8-$AY8,IF($B8="SMALL_SIDE",$O8-$Q8-$R8,0))</f>
+        <f>IF($B8="BIG_SIDE",$N8-$P8-$AY8,0)</f>
         <v/>
       </c>
       <c r="AY8" s="12">
@@ -5720,7 +5720,7 @@
         <v/>
       </c>
       <c r="X9" s="19">
-        <f>IF($B9="BIG_SIDE",IF($AX9&gt;0,$AX9-$AS9,0),IF($S9&gt;0,$S9*0.5,0))</f>
+        <f>IF($B9="BIG_SIDE",IF($AX$9&gt;0,$AX$9-$AS$9,0),IF($S$9&gt;0,$S$9*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y9" s="19">
@@ -5756,7 +5756,7 @@
         <v/>
       </c>
       <c r="AG9" s="12">
-        <f>IF($B9="BLOCKED",IF($BB9&gt;0,$BB9,$BA9),IF($B9="SMALL_SIDE",$AM9,$W9))</f>
+        <f>IF($B9="BLOCKED",IF($BB8&gt;0,$BB8,$BA8),IF($B9="SMALL_SIDE",$AM9,$W9))</f>
         <v/>
       </c>
       <c r="AH9" s="13" t="inlineStr">
@@ -5801,7 +5801,7 @@
       </c>
       <c r="AR9" s="12" t="str">
         <f>IF($B9="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B9="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ9="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS9" s="20">
         <f>IF($B9="BIG_SIDE",$V9*$U9,0)</f>
@@ -5824,7 +5824,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX9" s="12">
-        <f>IF($B9="BIG_SIDE",$N9-$P9-$AY9,IF($B9="SMALL_SIDE",$O9-$Q9-$R9,0))</f>
+        <f>IF($B9="BIG_SIDE",$N9-$P9-$AY9,0)</f>
         <v/>
       </c>
       <c r="AY9" s="12">
@@ -5952,7 +5952,7 @@
         <v/>
       </c>
       <c r="X10" s="19">
-        <f>IF($B10="BIG_SIDE",IF($AX10&gt;0,$AX10-$AS10,0),IF($S10&gt;0,$S10*0.5,0))</f>
+        <f>IF($B10="BIG_SIDE",IF($AX$10&gt;0,$AX$10-$AS$10,0),IF($S$10&gt;0,$S$10*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y10" s="19">
@@ -5988,7 +5988,7 @@
         <v/>
       </c>
       <c r="AG10" s="12">
-        <f>IF($B10="BLOCKED",IF($BB10&gt;0,$BB10,$BA10),IF($B10="SMALL_SIDE",$AM10,$W10))</f>
+        <f>IF($B10="BLOCKED",IF($BB9&gt;0,$BB9,$BA9),IF($B10="SMALL_SIDE",$AM10,$W10))</f>
         <v/>
       </c>
       <c r="AH10" s="13" t="inlineStr">
@@ -6033,7 +6033,7 @@
       </c>
       <c r="AR10" s="12" t="str">
         <f>IF($B10="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B10="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ10="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS10" s="20">
         <f>IF($B10="BIG_SIDE",$V10*$U10,0)</f>
@@ -6056,7 +6056,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX10" s="12">
-        <f>IF($B10="BIG_SIDE",$N10-$P10-$AY10,IF($B10="SMALL_SIDE",$O10-$Q10-$R10,0))</f>
+        <f>IF($B10="BIG_SIDE",$N10-$P10-$AY10,0)</f>
         <v/>
       </c>
       <c r="AY10" s="12">
@@ -6184,7 +6184,7 @@
         <v/>
       </c>
       <c r="X11" s="19">
-        <f>IF($B11="BIG_SIDE",IF($AX11&gt;0,$AX11-$AS11,0),IF($S11&gt;0,$S11*0.5,0))</f>
+        <f>IF($B11="BIG_SIDE",IF($AX$11&gt;0,$AX$11-$AS$11,0),IF($S$11&gt;0,$S$11*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y11" s="19">
@@ -6220,7 +6220,7 @@
         <v/>
       </c>
       <c r="AG11" s="12">
-        <f>IF($B11="BLOCKED",IF($BB11&gt;0,$BB11,$BA11),IF($B11="SMALL_SIDE",$AM11,$W11))</f>
+        <f>IF($B11="BLOCKED",IF($BB10&gt;0,$BB10,$BA10),IF($B11="SMALL_SIDE",$AM11,$W11))</f>
         <v/>
       </c>
       <c r="AH11" s="13" t="inlineStr">
@@ -6265,7 +6265,7 @@
       </c>
       <c r="AR11" s="12" t="str">
         <f>IF($B11="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B11="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ11="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS11" s="20">
         <f>IF($B11="BIG_SIDE",$V11*$U11,0)</f>
@@ -6288,7 +6288,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX11" s="12">
-        <f>IF($B11="BIG_SIDE",$N11-$P11-$AY11,IF($B11="SMALL_SIDE",$O11-$Q11-$R11,0))</f>
+        <f>IF($B11="BIG_SIDE",$N11-$P11-$AY11,0)</f>
         <v/>
       </c>
       <c r="AY11" s="12">
@@ -6816,7 +6816,7 @@
         <v/>
       </c>
       <c r="X2" s="19">
-        <f>IF($B2="BIG_SIDE",IF($AX2&gt;0,$AX2-$AS2,0),IF($S2&gt;0,$S2*0.5,0))</f>
+        <f>IF($B2="BIG_SIDE",IF($AX$2&gt;0,$AX$2-$AS$2,0),IF($S$2&gt;0,$S$2*0.5,0))</f>
         <v/>
       </c>
       <c r="Y2" s="19">
@@ -6847,11 +6847,11 @@
         <v/>
       </c>
       <c r="AF2" s="12">
-        <f>IF($B2="BLOCKED",IF($BB2&gt;0,$AF2,$C2),IF($B2="SMALL_SIDE",$E2,$C2))</f>
+        <f>IF($B2="BLOCKED",$C2,IF($B2="SMALL_SIDE",$E2,$C2))</f>
         <v/>
       </c>
       <c r="AG2" s="12">
-        <f>IF($B2="BLOCKED",IF($BB2&gt;0,$BB2,$BA2),IF($B2="SMALL_SIDE",$AM2,$W2))</f>
+        <f>IF($B2="BLOCKED",0,IF($B2="SMALL_SIDE",$AM2,$W2))</f>
         <v/>
       </c>
       <c r="AH2" s="13" t="inlineStr">
@@ -6919,7 +6919,7 @@
         <v/>
       </c>
       <c r="AX2" s="12">
-        <f>IF($B2="BIG_SIDE",$N2-$P2-$AY2,IF($B2="SMALL_SIDE",$O2-$Q2-$R2,0))</f>
+        <f>IF($B2="BIG_SIDE",$N2-$P2-$AY2,0)</f>
         <v/>
       </c>
       <c r="AY2" s="12">
@@ -7047,7 +7047,7 @@
         <v/>
       </c>
       <c r="X3" s="19">
-        <f>IF($B3="BIG_SIDE",IF($AX3&gt;0,$AX3-$AS3,0),IF($S3&gt;0,$S3*0.5,0))</f>
+        <f>IF($B3="BIG_SIDE",IF($AX$3&gt;0,$AX$3-$AS$3,0),IF($S$3&gt;0,$S$3*0.5,0))</f>
         <v/>
       </c>
       <c r="Y3" s="19">
@@ -7068,7 +7068,7 @@
       </c>
       <c r="AC3" s="12">
         <f>IF($B3="BLOCKED",$BC3,IF($B3="BIG_SIDE",$W3,IF($AK3=TRUE,$BC3,$AG3)))</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AD3" s="12">
         <f>$AB3*Settings!$B$10</f>
@@ -7076,15 +7076,15 @@
       </c>
       <c r="AE3" s="12">
         <f>$AC3*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AF3" s="12">
         <f>IF($B3="BLOCKED",IF($BB3&gt;0,$AF2,$C3),IF($B3="SMALL_SIDE",$E3,$C3))</f>
         <v/>
       </c>
       <c r="AG3" s="12">
-        <f>IF($B3="BLOCKED",IF($BB3&gt;0,$BB3,$BA3),IF($B3="SMALL_SIDE",$AM3,$W3))</f>
-        <v>0.897</v>
+        <f>IF($B3="BLOCKED",IF($BB2&gt;0,$BB2,$BA2),IF($B3="SMALL_SIDE",$AM3,$W3))</f>
+        <v>0.7254</v>
       </c>
       <c r="AH3" s="13" t="inlineStr">
         <is>
@@ -7096,7 +7096,7 @@
       </c>
       <c r="AJ3" s="12">
         <f>IF($B3="SMALL_SIDE",MAX(0,$D3-$AV3),0)</f>
-        <v>0.8</v>
+        <v>0.8052</v>
       </c>
       <c r="AK3" s="12">
         <f>IF(AND($AJ3&gt;0,$AG3&gt;0),TRUE,FALSE)</f>
@@ -7151,7 +7151,7 @@
         <v/>
       </c>
       <c r="AX3" s="12">
-        <f>IF($B3="BIG_SIDE",$N3-$P3-$AY3,IF($B3="SMALL_SIDE",$O3-$Q3-$R3,0))</f>
+        <f>IF($B3="BIG_SIDE",$N3-$P3-$AY3,0)</f>
         <v/>
       </c>
       <c r="AY3" s="12">
@@ -7164,15 +7164,15 @@
       </c>
       <c r="BA3" s="12">
         <f>IF($AK3=TRUE,MAX(0,$AJ3-$BD3),IF($B3="BLOCKED",MAX(0,$BA2-$BD3),0))</f>
-        <v>0.8</v>
+        <v>0.8052</v>
       </c>
       <c r="BB3" s="12">
         <f>IF($AK3=TRUE,MAX(0,$AG3-$BE3),IF($B3="BLOCKED",MAX(0,$BB2-$BE3),0))</f>
-        <v>0.897</v>
+        <v>0.7254</v>
       </c>
       <c r="BC3" s="12">
         <f>$BA3+$BB3</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="BD3" s="13">
         <v>0</v>
@@ -7279,7 +7279,7 @@
         <v/>
       </c>
       <c r="X4" s="19">
-        <f>IF($B4="BIG_SIDE",IF($AX4&gt;0,$AX4-$AS4,0),IF($S4&gt;0,$S4*0.5,0))</f>
+        <f>IF($B4="BIG_SIDE",IF($AX$4&gt;0,$AX$4-$AS$4,0),IF($S$4&gt;0,$S$4*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y4" s="19">
@@ -7296,26 +7296,26 @@
       </c>
       <c r="AB4" s="12">
         <f>IF($B4="BLOCKED",$BC4,$D4+$G4+$J4)</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AC4" s="12">
         <f>IF($B4="BLOCKED",$BC4,IF($B4="BIG_SIDE",$W4,IF($AK4=TRUE,$BC4,$AG4)))</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AD4" s="12">
         <f>$AB4*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AE4" s="12">
         <f>$AC4*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AF4" s="12">
         <f>IF($B4="BLOCKED",IF($BB4&gt;0,$AF3,$C4),IF($B4="SMALL_SIDE",$E4,$C4))</f>
         <v/>
       </c>
       <c r="AG4" s="12">
-        <f>IF($B4="BLOCKED",IF($BB4&gt;0,$BB4,$BA4),IF($B4="SMALL_SIDE",$AM4,$W4))</f>
+        <f>IF($B4="BLOCKED",IF($BB3&gt;0,$BB3,$BA3),IF($B4="SMALL_SIDE",$AM4,$W4))</f>
         <v/>
       </c>
       <c r="AH4" s="13" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="AR4" s="12" t="str">
         <f>IF($B4="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B4="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ4="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS4" s="20">
         <f>IF($B4="BIG_SIDE",$V4*$U4,0)</f>
@@ -7383,7 +7383,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX4" s="12">
-        <f>IF($B4="BIG_SIDE",$N4-$P4-$AY4,IF($B4="SMALL_SIDE",$O4-$Q4-$R4,0))</f>
+        <f>IF($B4="BIG_SIDE",$N4-$P4-$AY4,0)</f>
         <v/>
       </c>
       <c r="AY4" s="12">
@@ -7396,15 +7396,15 @@
       </c>
       <c r="BA4" s="12">
         <f>IF($AK4=TRUE,MAX(0,$AJ4-$BD4),IF($B4="BLOCKED",MAX(0,$BA3-$BD4),0))</f>
-        <v>0.8</v>
+        <v>0.8052</v>
       </c>
       <c r="BB4" s="12">
         <f>IF($AK4=TRUE,MAX(0,$AG4-$BE4),IF($B4="BLOCKED",MAX(0,$BB3-$BE4),0))</f>
-        <v>0.897</v>
+        <v>0.7254</v>
       </c>
       <c r="BC4" s="12">
         <f>$BA4+$BB4</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="BD4" s="13">
         <v>0</v>
@@ -7511,7 +7511,7 @@
         <v/>
       </c>
       <c r="X5" s="19">
-        <f>IF($B5="BIG_SIDE",IF($AX5&gt;0,$AX5-$AS5,0),IF($S5&gt;0,$S5*0.5,0))</f>
+        <f>IF($B5="BIG_SIDE",IF($AX$5&gt;0,$AX$5-$AS$5,0),IF($S$5&gt;0,$S$5*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y5" s="19">
@@ -7528,26 +7528,26 @@
       </c>
       <c r="AB5" s="12">
         <f>IF($B5="BLOCKED",$BC5,$D5+$G5+$J5)</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AC5" s="12">
         <f>IF($B5="BLOCKED",$BC5,IF($B5="BIG_SIDE",$W5,IF($AK5=TRUE,$BC5,$AG5)))</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AD5" s="12">
         <f>$AB5*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AE5" s="12">
         <f>$AC5*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AF5" s="12">
         <f>IF($B5="BLOCKED",IF($BB5&gt;0,$AF4,$C5),IF($B5="SMALL_SIDE",$E5,$C5))</f>
         <v/>
       </c>
       <c r="AG5" s="12">
-        <f>IF($B5="BLOCKED",IF($BB5&gt;0,$BB5,$BA5),IF($B5="SMALL_SIDE",$AM5,$W5))</f>
+        <f>IF($B5="BLOCKED",IF($BB4&gt;0,$BB4,$BA4),IF($B5="SMALL_SIDE",$AM5,$W5))</f>
         <v/>
       </c>
       <c r="AH5" s="13" t="inlineStr">
@@ -7592,7 +7592,7 @@
       </c>
       <c r="AR5" s="12" t="str">
         <f>IF($B5="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B5="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ5="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS5" s="20">
         <f>IF($B5="BIG_SIDE",$V5*$U5,0)</f>
@@ -7615,7 +7615,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX5" s="12">
-        <f>IF($B5="BIG_SIDE",$N5-$P5-$AY5,IF($B5="SMALL_SIDE",$O5-$Q5-$R5,0))</f>
+        <f>IF($B5="BIG_SIDE",$N5-$P5-$AY5,0)</f>
         <v/>
       </c>
       <c r="AY5" s="12">
@@ -7628,15 +7628,15 @@
       </c>
       <c r="BA5" s="12">
         <f>IF($AK5=TRUE,MAX(0,$AJ5-$BD5),IF($B5="BLOCKED",MAX(0,$BA4-$BD5),0))</f>
-        <v>0.8</v>
+        <v>0.8052</v>
       </c>
       <c r="BB5" s="12">
         <f>IF($AK5=TRUE,MAX(0,$AG5-$BE5),IF($B5="BLOCKED",MAX(0,$BB4-$BE5),0))</f>
-        <v>0.897</v>
+        <v>0.7254</v>
       </c>
       <c r="BC5" s="12">
         <f>$BA5+$BB5</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="BD5" s="13">
         <v>0</v>
@@ -7743,7 +7743,7 @@
         <v/>
       </c>
       <c r="X6" s="19">
-        <f>IF($B6="BIG_SIDE",IF($AX6&gt;0,$AX6-$AS6,0),IF($S6&gt;0,$S6*0.5,0))</f>
+        <f>IF($B6="BIG_SIDE",IF($AX$6&gt;0,$AX$6-$AS$6,0),IF($S$6&gt;0,$S$6*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y6" s="19">
@@ -7760,26 +7760,26 @@
       </c>
       <c r="AB6" s="12">
         <f>IF($B6="BLOCKED",$BC6,$D6+$G6+$J6)</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AC6" s="12">
         <f>IF($B6="BLOCKED",$BC6,IF($B6="BIG_SIDE",$W6,IF($AK6=TRUE,$BC6,$AG6)))</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AD6" s="12">
         <f>$AB6*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AE6" s="12">
         <f>$AC6*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AF6" s="12">
         <f>IF($B6="BLOCKED",IF($BB6&gt;0,$AF5,$C6),IF($B6="SMALL_SIDE",$E6,$C6))</f>
         <v/>
       </c>
       <c r="AG6" s="12">
-        <f>IF($B6="BLOCKED",IF($BB6&gt;0,$BB6,$BA6),IF($B6="SMALL_SIDE",$AM6,$W6))</f>
+        <f>IF($B6="BLOCKED",IF($BB5&gt;0,$BB5,$BA5),IF($B6="SMALL_SIDE",$AM6,$W6))</f>
         <v/>
       </c>
       <c r="AH6" s="13" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="AR6" s="12" t="str">
         <f>IF($B6="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B6="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ6="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS6" s="20">
         <f>IF($B6="BIG_SIDE",$V6*$U6,0)</f>
@@ -7847,7 +7847,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX6" s="12">
-        <f>IF($B6="BIG_SIDE",$N6-$P6-$AY6,IF($B6="SMALL_SIDE",$O6-$Q6-$R6,0))</f>
+        <f>IF($B6="BIG_SIDE",$N6-$P6-$AY6,0)</f>
         <v/>
       </c>
       <c r="AY6" s="12">
@@ -7860,15 +7860,15 @@
       </c>
       <c r="BA6" s="12">
         <f>IF($AK6=TRUE,MAX(0,$AJ6-$BD6),IF($B6="BLOCKED",MAX(0,$BA5-$BD6),0))</f>
-        <v>0.8</v>
+        <v>0.8052</v>
       </c>
       <c r="BB6" s="12">
         <f>IF($AK6=TRUE,MAX(0,$AG6-$BE6),IF($B6="BLOCKED",MAX(0,$BB5-$BE6),0))</f>
-        <v>0.897</v>
+        <v>0.7254</v>
       </c>
       <c r="BC6" s="12">
         <f>$BA6+$BB6</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="BD6" s="13">
         <v>0</v>
@@ -7975,7 +7975,7 @@
         <v/>
       </c>
       <c r="X7" s="19">
-        <f>IF($B7="BIG_SIDE",IF($AX7&gt;0,$AX7-$AS7,0),IF($S7&gt;0,$S7*0.5,0))</f>
+        <f>IF($B7="BIG_SIDE",IF($AX$7&gt;0,$AX$7-$AS$7,0),IF($S$7&gt;0,$S$7*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y7" s="19">
@@ -7992,26 +7992,26 @@
       </c>
       <c r="AB7" s="12">
         <f>IF($B7="BLOCKED",$BC7,$D7+$G7+$J7)</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AC7" s="12">
         <f>IF($B7="BLOCKED",$BC7,IF($B7="BIG_SIDE",$W7,IF($AK7=TRUE,$BC7,$AG7)))</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AD7" s="12">
         <f>$AB7*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AE7" s="12">
         <f>$AC7*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AF7" s="12">
         <f>IF($B7="BLOCKED",IF($BB7&gt;0,$AF6,$C7),IF($B7="SMALL_SIDE",$E7,$C7))</f>
         <v/>
       </c>
       <c r="AG7" s="12">
-        <f>IF($B7="BLOCKED",IF($BB7&gt;0,$BB7,$BA7),IF($B7="SMALL_SIDE",$AM7,$W7))</f>
+        <f>IF($B7="BLOCKED",IF($BB6&gt;0,$BB6,$BA6),IF($B7="SMALL_SIDE",$AM7,$W7))</f>
         <v/>
       </c>
       <c r="AH7" s="13" t="inlineStr">
@@ -8056,7 +8056,7 @@
       </c>
       <c r="AR7" s="12" t="str">
         <f>IF($B7="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B7="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ7="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS7" s="20">
         <f>IF($B7="BIG_SIDE",$V7*$U7,0)</f>
@@ -8079,7 +8079,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX7" s="12">
-        <f>IF($B7="BIG_SIDE",$N7-$P7-$AY7,IF($B7="SMALL_SIDE",$O7-$Q7-$R7,0))</f>
+        <f>IF($B7="BIG_SIDE",$N7-$P7-$AY7,0)</f>
         <v/>
       </c>
       <c r="AY7" s="12">
@@ -8092,15 +8092,15 @@
       </c>
       <c r="BA7" s="12">
         <f>IF($AK7=TRUE,MAX(0,$AJ7-$BD7),IF($B7="BLOCKED",MAX(0,$BA6-$BD7),0))</f>
-        <v>0.8</v>
+        <v>0.8052</v>
       </c>
       <c r="BB7" s="12">
         <f>IF($AK7=TRUE,MAX(0,$AG7-$BE7),IF($B7="BLOCKED",MAX(0,$BB6-$BE7),0))</f>
-        <v>0.897</v>
+        <v>0.7254</v>
       </c>
       <c r="BC7" s="12">
         <f>$BA7+$BB7</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="BD7" s="13">
         <v>0</v>
@@ -8207,7 +8207,7 @@
         <v/>
       </c>
       <c r="X8" s="19">
-        <f>IF($B8="BIG_SIDE",IF($AX8&gt;0,$AX8-$AS8,0),IF($S8&gt;0,$S8*0.5,0))</f>
+        <f>IF($B8="BIG_SIDE",IF($AX$8&gt;0,$AX$8-$AS$8,0),IF($S$8&gt;0,$S$8*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y8" s="19">
@@ -8224,26 +8224,26 @@
       </c>
       <c r="AB8" s="12">
         <f>IF($B8="BLOCKED",$BC8,$D8+$G8+$J8)</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AC8" s="12">
         <f>IF($B8="BLOCKED",$BC8,IF($B8="BIG_SIDE",$W8,IF($AK8=TRUE,$BC8,$AG8)))</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AD8" s="12">
         <f>$AB8*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AE8" s="12">
         <f>$AC8*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AF8" s="12">
         <f>IF($B8="BLOCKED",IF($BB8&gt;0,$AF7,$C8),IF($B8="SMALL_SIDE",$E8,$C8))</f>
         <v/>
       </c>
       <c r="AG8" s="12">
-        <f>IF($B8="BLOCKED",IF($BB8&gt;0,$BB8,$BA8),IF($B8="SMALL_SIDE",$AM8,$W8))</f>
+        <f>IF($B8="BLOCKED",IF($BB7&gt;0,$BB7,$BA7),IF($B8="SMALL_SIDE",$AM8,$W8))</f>
         <v/>
       </c>
       <c r="AH8" s="13" t="inlineStr">
@@ -8288,7 +8288,7 @@
       </c>
       <c r="AR8" s="12" t="str">
         <f>IF($B8="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B8="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ8="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS8" s="20">
         <f>IF($B8="BIG_SIDE",$V8*$U8,0)</f>
@@ -8311,7 +8311,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX8" s="12">
-        <f>IF($B8="BIG_SIDE",$N8-$P8-$AY8,IF($B8="SMALL_SIDE",$O8-$Q8-$R8,0))</f>
+        <f>IF($B8="BIG_SIDE",$N8-$P8-$AY8,0)</f>
         <v/>
       </c>
       <c r="AY8" s="12">
@@ -8324,15 +8324,15 @@
       </c>
       <c r="BA8" s="12">
         <f>IF($AK8=TRUE,MAX(0,$AJ8-$BD8),IF($B8="BLOCKED",MAX(0,$BA7-$BD8),0))</f>
-        <v>0.8</v>
+        <v>0.8052</v>
       </c>
       <c r="BB8" s="12">
         <f>IF($AK8=TRUE,MAX(0,$AG8-$BE8),IF($B8="BLOCKED",MAX(0,$BB7-$BE8),0))</f>
-        <v>0.897</v>
+        <v>0.7254</v>
       </c>
       <c r="BC8" s="12">
         <f>$BA8+$BB8</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="BD8" s="13">
         <v>0</v>
@@ -8439,7 +8439,7 @@
         <v/>
       </c>
       <c r="X9" s="19">
-        <f>IF($B9="BIG_SIDE",IF($AX9&gt;0,$AX9-$AS9,0),IF($S9&gt;0,$S9*0.5,0))</f>
+        <f>IF($B9="BIG_SIDE",IF($AX$9&gt;0,$AX$9-$AS$9,0),IF($S$9&gt;0,$S$9*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y9" s="19">
@@ -8456,26 +8456,26 @@
       </c>
       <c r="AB9" s="12">
         <f>IF($B9="BLOCKED",$BC9,$D9+$G9+$J9)</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AC9" s="12">
         <f>IF($B9="BLOCKED",$BC9,IF($B9="BIG_SIDE",$W9,IF($AK9=TRUE,$BC9,$AG9)))</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AD9" s="12">
         <f>$AB9*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AE9" s="12">
         <f>$AC9*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AF9" s="12">
         <f>IF($B9="BLOCKED",IF($BB9&gt;0,$AF8,$C9),IF($B9="SMALL_SIDE",$E9,$C9))</f>
         <v/>
       </c>
       <c r="AG9" s="12">
-        <f>IF($B9="BLOCKED",IF($BB9&gt;0,$BB9,$BA9),IF($B9="SMALL_SIDE",$AM9,$W9))</f>
+        <f>IF($B9="BLOCKED",IF($BB8&gt;0,$BB8,$BA8),IF($B9="SMALL_SIDE",$AM9,$W9))</f>
         <v/>
       </c>
       <c r="AH9" s="13" t="inlineStr">
@@ -8520,7 +8520,7 @@
       </c>
       <c r="AR9" s="12" t="str">
         <f>IF($B9="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B9="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ9="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS9" s="20">
         <f>IF($B9="BIG_SIDE",$V9*$U9,0)</f>
@@ -8543,7 +8543,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX9" s="12">
-        <f>IF($B9="BIG_SIDE",$N9-$P9-$AY9,IF($B9="SMALL_SIDE",$O9-$Q9-$R9,0))</f>
+        <f>IF($B9="BIG_SIDE",$N9-$P9-$AY9,0)</f>
         <v/>
       </c>
       <c r="AY9" s="12">
@@ -8556,15 +8556,15 @@
       </c>
       <c r="BA9" s="12">
         <f>IF($AK9=TRUE,MAX(0,$AJ9-$BD9),IF($B9="BLOCKED",MAX(0,$BA8-$BD9),0))</f>
-        <v>0.8</v>
+        <v>0.8052</v>
       </c>
       <c r="BB9" s="12">
         <f>IF($AK9=TRUE,MAX(0,$AG9-$BE9),IF($B9="BLOCKED",MAX(0,$BB8-$BE9),0))</f>
-        <v>0.897</v>
+        <v>0.7254</v>
       </c>
       <c r="BC9" s="12">
         <f>$BA9+$BB9</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="BD9" s="13">
         <v>0</v>
@@ -8671,7 +8671,7 @@
         <v/>
       </c>
       <c r="X10" s="19">
-        <f>IF($B10="BIG_SIDE",IF($AX10&gt;0,$AX10-$AS10,0),IF($S10&gt;0,$S10*0.5,0))</f>
+        <f>IF($B10="BIG_SIDE",IF($AX$10&gt;0,$AX$10-$AS$10,0),IF($S$10&gt;0,$S$10*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y10" s="19">
@@ -8688,26 +8688,26 @@
       </c>
       <c r="AB10" s="12">
         <f>IF($B10="BLOCKED",$BC10,$D10+$G10+$J10)</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AC10" s="12">
         <f>IF($B10="BLOCKED",$BC10,IF($B10="BIG_SIDE",$W10,IF($AK10=TRUE,$BC10,$AG10)))</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AD10" s="12">
         <f>$AB10*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AE10" s="12">
         <f>$AC10*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AF10" s="12">
         <f>IF($B10="BLOCKED",IF($BB10&gt;0,$AF9,$C10),IF($B10="SMALL_SIDE",$E10,$C10))</f>
         <v/>
       </c>
       <c r="AG10" s="12">
-        <f>IF($B10="BLOCKED",IF($BB10&gt;0,$BB10,$BA10),IF($B10="SMALL_SIDE",$AM10,$W10))</f>
+        <f>IF($B10="BLOCKED",IF($BB9&gt;0,$BB9,$BA9),IF($B10="SMALL_SIDE",$AM10,$W10))</f>
         <v/>
       </c>
       <c r="AH10" s="13" t="inlineStr">
@@ -8752,7 +8752,7 @@
       </c>
       <c r="AR10" s="12" t="str">
         <f>IF($B10="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B10="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ10="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS10" s="20">
         <f>IF($B10="BIG_SIDE",$V10*$U10,0)</f>
@@ -8775,7 +8775,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX10" s="12">
-        <f>IF($B10="BIG_SIDE",$N10-$P10-$AY10,IF($B10="SMALL_SIDE",$O10-$Q10-$R10,0))</f>
+        <f>IF($B10="BIG_SIDE",$N10-$P10-$AY10,0)</f>
         <v/>
       </c>
       <c r="AY10" s="12">
@@ -8788,15 +8788,15 @@
       </c>
       <c r="BA10" s="12">
         <f>IF($AK10=TRUE,MAX(0,$AJ10-$BD10),IF($B10="BLOCKED",MAX(0,$BA9-$BD10),0))</f>
-        <v>0.8</v>
+        <v>0.8052</v>
       </c>
       <c r="BB10" s="12">
         <f>IF($AK10=TRUE,MAX(0,$AG10-$BE10),IF($B10="BLOCKED",MAX(0,$BB9-$BE10),0))</f>
-        <v>0.897</v>
+        <v>0.7254</v>
       </c>
       <c r="BC10" s="12">
         <f>$BA10+$BB10</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="BD10" s="13">
         <v>0</v>
@@ -8903,7 +8903,7 @@
         <v/>
       </c>
       <c r="X11" s="19">
-        <f>IF($B11="BIG_SIDE",IF($AX11&gt;0,$AX11-$AS11,0),IF($S11&gt;0,$S11*0.5,0))</f>
+        <f>IF($B11="BIG_SIDE",IF($AX$11&gt;0,$AX$11-$AS$11,0),IF($S$11&gt;0,$S$11*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="Y11" s="19">
@@ -8920,26 +8920,26 @@
       </c>
       <c r="AB11" s="12">
         <f>IF($B11="BLOCKED",$BC11,$D11+$G11+$J11)</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AC11" s="12">
         <f>IF($B11="BLOCKED",$BC11,IF($B11="BIG_SIDE",$W11,IF($AK11=TRUE,$BC11,$AG11)))</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="AD11" s="12">
         <f>$AB11*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AE11" s="12">
         <f>$AC11*Settings!$B$10</f>
-        <v>1697</v>
+        <v>1530.6</v>
       </c>
       <c r="AF11" s="12">
         <f>IF($B11="BLOCKED",IF($BB11&gt;0,$AF10,$C11),IF($B11="SMALL_SIDE",$E11,$C11))</f>
         <v/>
       </c>
       <c r="AG11" s="12">
-        <f>IF($B11="BLOCKED",IF($BB11&gt;0,$BB11,$BA11),IF($B11="SMALL_SIDE",$AM11,$W11))</f>
+        <f>IF($B11="BLOCKED",IF($BB10&gt;0,$BB10,$BA10),IF($B11="SMALL_SIDE",$AM11,$W11))</f>
         <v/>
       </c>
       <c r="AH11" s="13" t="inlineStr">
@@ -8984,7 +8984,7 @@
       </c>
       <c r="AR11" s="12" t="str">
         <f>IF($B11="BLOCKED","Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия",IF($B11="BIG_SIDE","BIG_SIDE: Big и Small закрыты 100%; баланс учитывает RealizedFarLoss",IF($AQ11="DUAL_TAIL","SMALL_SIDE: старый и новый хвост одновременно; новый уровень запрещён","SMALL_SIDE: Small закрыт 100%, Big закрыт 22%, остаток Big = новый хвост")))</f>
-        <v>Заблокировано: предыдущий уровень не разрешил новый полноценный уровень</v>
+        <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS11" s="20">
         <f>IF($B11="BIG_SIDE",$V11*$U11,0)</f>
@@ -9007,7 +9007,7 @@
         <v>DUAL_TAIL persistence: оба хвоста сохранены</v>
       </c>
       <c r="AX11" s="12">
-        <f>IF($B11="BIG_SIDE",$N11-$P11-$AY11,IF($B11="SMALL_SIDE",$O11-$Q11-$R11,0))</f>
+        <f>IF($B11="BIG_SIDE",$N11-$P11-$AY11,0)</f>
         <v/>
       </c>
       <c r="AY11" s="12">
@@ -9020,15 +9020,15 @@
       </c>
       <c r="BA11" s="12">
         <f>IF($AK11=TRUE,MAX(0,$AJ11-$BD11),IF($B11="BLOCKED",MAX(0,$BA10-$BD11),0))</f>
-        <v>0.8</v>
+        <v>0.8052</v>
       </c>
       <c r="BB11" s="12">
         <f>IF($AK11=TRUE,MAX(0,$AG11-$BE11),IF($B11="BLOCKED",MAX(0,$BB10-$BE11),0))</f>
-        <v>0.897</v>
+        <v>0.7254</v>
       </c>
       <c r="BC11" s="12">
         <f>$BA11+$BB11</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="BD11" s="13">
         <v>0</v>
@@ -9578,7 +9578,7 @@
       </c>
       <c r="C26">
         <f>SUM(Calculator!N2:O11,Trend_UP!N2:O11,Trend_DOWN!N2:O11)+SUMIF(Calculator!AI2:AI11,"&gt;0",Calculator!AI2:AI11)+SUMIF(Trend_UP!AI2:AI11,"&gt;0",Trend_UP!AI2:AI11)+SUMIF(Trend_DOWN!AI2:AI11,"&gt;0",Trend_DOWN!AI2:AI11)</f>
-        <v/>
+        <v>900</v>
       </c>
       <c r="D26">
         <f>C26</f>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="C27">
         <f>SUM(Calculator!P2:R11,Trend_UP!P2:R11,Trend_DOWN!P2:R11)+SUM(Calculator!AS2:AS11,Trend_UP!AS2:AS11,Trend_DOWN!AS2:AS11)-SUMIF(Calculator!AI2:AI11,"&lt;0",Calculator!AI2:AI11)-SUMIF(Trend_UP!AI2:AI11,"&lt;0",Trend_UP!AI2:AI11)-SUMIF(Trend_DOWN!AI2:AI11,"&lt;0",Trend_DOWN!AI2:AI11)</f>
-        <v/>
+        <v>300</v>
       </c>
       <c r="D27">
         <f>C27</f>
@@ -9738,7 +9738,7 @@
       </c>
       <c r="C34">
         <f>MAX(Calculator!BB2:BB11,Trend_UP!BB2:BB11,Trend_DOWN!BB2:BB11)</f>
-        <v>1.697</v>
+        <v>1.5306</v>
       </c>
       <c r="D34">
         <f>C34</f>
@@ -9776,7 +9776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -13102,6 +13102,384 @@
       <c r="H79" t="inlineStr">
         <is>
           <t>Excel recalculates formulas on open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>V7-01</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>No circular reference warning in Excel</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Workbook formulas</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>No direct self-reference and no known circular formula pattern</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>openpyxl direct self-reference scan + formula review</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Excel desktop manual warning cannot be opened in this headless environment; direct/cross-row formulas were cleaned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>V7-02</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>No direct self-reference in formulas</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>All formula cells</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>No cell coordinate appears in its own formula</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Python openpyxl scan</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Simple Excel-style direct self-reference smoke check passes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>V7-03</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Trend_DOWN BLOCKED old tail from DUAL_TAIL</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Trend_DOWN row after DUAL_TAIL</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>ActiveOldFarLot = previous ActiveOldFarLot</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>pytest data-only</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Trend_DOWN uses real previous DUAL_TAIL old tail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>V7-04</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Trend_DOWN BLOCKED new tail from DUAL_TAIL</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Trend_DOWN row after DUAL_TAIL</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>ActiveNewFarLot = previous ActiveNewFarLot</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>pytest data-only</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Trend_DOWN uses real previous DUAL_TAIL new tail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>V7-05</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Trend_DOWN dual total</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Trend_DOWN BLOCKED rows</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>DualTailTotalLot = ActiveOldFarLot + ActiveNewFarLot</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>pytest data-only</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Dual total equals two active tails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>V7-06</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Global Total Closed Profit populated</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Risk_Analysis</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Formula/value is not blank</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Risk_Analysis formula/data-only check</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Global profit aggregates Calculator + Trend_UP + Trend_DOWN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>V7-07</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Global Total Closed Loss populated</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Risk_Analysis</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Formula/value is not blank</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Risk_Analysis formula/data-only check</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Global loss aggregates Calculator + Trend_UP + Trend_DOWN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>V7-08</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Global DUAL/BLOCKED/STOP visible</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Risk_Analysis</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Counts and max exposure &gt; 0 when scenarios contain them</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>pytest data-only</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Global summary sees DUAL_TAIL, BLOCKED and STOP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>V7-09</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>BLOCKED key fields not blank</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Calculator/Trend_UP/Trend_DOWN</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Required key fields contain 0 or text</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>pytest data-only</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>BLOCKED rows are readable and complete.</t>
         </is>
       </c>
     </row>
@@ -21356,59 +21734,59 @@
         <v>2</v>
       </c>
       <c r="D2">
-        <f>Trend_UP!C2&amp;" "&amp;TEXT(Trend_UP!D2,"0.00")</f>
+        <f>Trend_UP!$C$2&amp;" "&amp;TEXT(Trend_UP!$D$2,"0.00")</f>
         <v/>
       </c>
       <c r="E2">
-        <f>Trend_UP!E2&amp;" "&amp;TEXT(Trend_UP!G2,"0.00")</f>
+        <f>Trend_UP!$E$2&amp;" "&amp;TEXT(Trend_UP!$G$2,"0.00")</f>
         <v/>
       </c>
       <c r="F2">
-        <f>Trend_UP!H2&amp;" "&amp;TEXT(Trend_UP!J2,"0.00")</f>
+        <f>Trend_UP!$H$2&amp;" "&amp;TEXT(Trend_UP!$J$2,"0.00")</f>
         <v/>
       </c>
       <c r="G2">
-        <f>Trend_UP!B2</f>
+        <f>Trend_UP!$B$2</f>
         <v/>
       </c>
       <c r="H2">
-        <f>Trend_UP!S2</f>
+        <f>Trend_UP!$S$2</f>
         <v/>
       </c>
       <c r="I2">
-        <f>Trend_UP!T2</f>
+        <f>Trend_UP!$T$2</f>
         <v/>
       </c>
       <c r="J2">
-        <f>Trend_UP!X2</f>
+        <f>Trend_UP!$X$2</f>
         <v/>
       </c>
       <c r="K2">
-        <f>Trend_UP!AZ2</f>
+        <f>Trend_UP!$AZ$2</f>
         <v/>
       </c>
       <c r="L2">
-        <f>Trend_UP!BA2</f>
+        <f>Trend_UP!$BA$2</f>
         <v/>
       </c>
       <c r="M2">
-        <f>Trend_UP!BB2</f>
+        <f>Trend_UP!$BB$2</f>
         <v/>
       </c>
       <c r="N2">
-        <f>Trend_UP!AB2</f>
+        <f>Trend_UP!$AB$2</f>
         <v/>
       </c>
       <c r="O2">
-        <f>Trend_UP!AD2</f>
+        <f>Trend_UP!$AD$2</f>
         <v/>
       </c>
       <c r="P2">
-        <f>Trend_UP!AQ2</f>
+        <f>Trend_UP!$AQ$2</f>
         <v/>
       </c>
       <c r="Q2">
-        <f>Trend_UP!AR2</f>
+        <f>Trend_UP!$AR$2</f>
         <v/>
       </c>
     </row>
@@ -21427,59 +21805,59 @@
         <v>5</v>
       </c>
       <c r="D3">
-        <f>Trend_UP!C5&amp;" "&amp;TEXT(Trend_UP!D5,"0.00")</f>
+        <f>Trend_UP!$C$5&amp;" "&amp;TEXT(Trend_UP!$D$5,"0.00")</f>
         <v/>
       </c>
       <c r="E3">
-        <f>Trend_UP!E5&amp;" "&amp;TEXT(Trend_UP!G5,"0.00")</f>
+        <f>Trend_UP!$E$5&amp;" "&amp;TEXT(Trend_UP!$G$5,"0.00")</f>
         <v/>
       </c>
       <c r="F3">
-        <f>Trend_UP!H5&amp;" "&amp;TEXT(Trend_UP!J5,"0.00")</f>
+        <f>Trend_UP!$H$5&amp;" "&amp;TEXT(Trend_UP!$J$5,"0.00")</f>
         <v/>
       </c>
       <c r="G3">
-        <f>Trend_UP!B5</f>
+        <f>Trend_UP!$B$5</f>
         <v/>
       </c>
       <c r="H3">
-        <f>Trend_UP!S5</f>
+        <f>Trend_UP!$S$5</f>
         <v/>
       </c>
       <c r="I3">
-        <f>Trend_UP!T5</f>
+        <f>Trend_UP!$T$5</f>
         <v/>
       </c>
       <c r="J3">
-        <f>Trend_UP!X5</f>
+        <f>Trend_UP!$X$5</f>
         <v/>
       </c>
       <c r="K3">
-        <f>Trend_UP!AZ5</f>
+        <f>Trend_UP!$AZ$5</f>
         <v/>
       </c>
       <c r="L3">
-        <f>Trend_UP!BA5</f>
+        <f>Trend_UP!$BA$5</f>
         <v/>
       </c>
       <c r="M3">
-        <f>Trend_UP!BB5</f>
+        <f>Trend_UP!$BB$5</f>
         <v/>
       </c>
       <c r="N3">
-        <f>Trend_UP!AB5</f>
+        <f>Trend_UP!$AB$5</f>
         <v/>
       </c>
       <c r="O3">
-        <f>Trend_UP!AD5</f>
+        <f>Trend_UP!$AD$5</f>
         <v/>
       </c>
       <c r="P3">
-        <f>Trend_UP!AQ5</f>
+        <f>Trend_UP!$AQ$5</f>
         <v/>
       </c>
       <c r="Q3">
-        <f>Trend_UP!AR5</f>
+        <f>Trend_UP!$AR$5</f>
         <v/>
       </c>
     </row>
@@ -21498,59 +21876,59 @@
         <v>4</v>
       </c>
       <c r="D4">
-        <f>Trend_DOWN!C4&amp;" "&amp;TEXT(Trend_DOWN!D4,"0.00")</f>
+        <f>Trend_DOWN!$C$4&amp;" "&amp;TEXT(Trend_DOWN!$D$4,"0.00")</f>
         <v/>
       </c>
       <c r="E4">
-        <f>TEXT(Trend_DOWN!G4,"0.00")</f>
+        <f>TEXT(Trend_DOWN!$G$4,"0.00")</f>
         <v/>
       </c>
       <c r="F4">
-        <f>TEXT(Trend_DOWN!J4,"0.00")</f>
+        <f>TEXT(Trend_DOWN!$J$4,"0.00")</f>
         <v/>
       </c>
       <c r="G4">
-        <f>Trend_DOWN!B4</f>
+        <f>Trend_DOWN!$B$4</f>
         <v/>
       </c>
       <c r="H4">
-        <f>Trend_DOWN!S4</f>
+        <f>Trend_DOWN!$S$4</f>
         <v/>
       </c>
       <c r="I4">
-        <f>Trend_DOWN!T4</f>
+        <f>Trend_DOWN!$T$4</f>
         <v/>
       </c>
       <c r="J4">
-        <f>Trend_DOWN!X4</f>
+        <f>Trend_DOWN!$X$4</f>
         <v/>
       </c>
       <c r="K4">
-        <f>Trend_DOWN!AZ4</f>
+        <f>Trend_DOWN!$AZ$4</f>
         <v/>
       </c>
       <c r="L4">
-        <f>Trend_DOWN!BA4</f>
+        <f>Trend_DOWN!$BA$4</f>
         <v/>
       </c>
       <c r="M4">
-        <f>Trend_DOWN!BB4</f>
+        <f>Trend_DOWN!$BB$4</f>
         <v/>
       </c>
       <c r="N4">
-        <f>Trend_DOWN!AB4</f>
+        <f>Trend_DOWN!$AB$4</f>
         <v/>
       </c>
       <c r="O4">
-        <f>Trend_DOWN!AD4</f>
+        <f>Trend_DOWN!$AD$4</f>
         <v/>
       </c>
       <c r="P4">
-        <f>Trend_DOWN!AQ4</f>
+        <f>Trend_DOWN!$AQ$4</f>
         <v/>
       </c>
       <c r="Q4">
-        <f>Trend_DOWN!AR4</f>
+        <f>Trend_DOWN!$AR$4</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix global dual-tail exposure and add settings geometry table
</commit_message>
<xml_diff>
--- a/work/MinusLock_SelfCompressing_BigSmall_v2/MinusLock_SelfCompressing_BigSmall_v2.xlsx
+++ b/work/MinusLock_SelfCompressing_BigSmall_v2/MinusLock_SelfCompressing_BigSmall_v2.xlsx
@@ -28,7 +28,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -54,7 +56,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -116,6 +118,26 @@
         <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -143,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -199,6 +221,27 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -598,13 +641,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -914,7 +958,264 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>Справочная геометрия лотов Big-N / Small-N / Close-N</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>FarStart-N</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t>Big-N</t>
+        </is>
+      </c>
+      <c r="D21" s="30" t="inlineStr">
+        <is>
+          <t>Small-N</t>
+        </is>
+      </c>
+      <c r="E21" s="31" t="inlineStr">
+        <is>
+          <t>Close-N</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="32">
+        <f>IF(1&lt;=Settings!$B$12,1,"")</f>
+        <v>1</v>
+      </c>
+      <c r="B22" s="33">
+        <f>IF($A22="","",Settings!$B$2)</f>
+        <v>1</v>
+      </c>
+      <c r="C22" s="33">
+        <f>IF($A22="","",ROUND(($B22*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>1.15</v>
+      </c>
+      <c r="D22" s="33">
+        <f>IF($A22="","",ROUND(($C22*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.44</v>
+      </c>
+      <c r="E22" s="33">
+        <f>IF($A22="","",ROUND(($B22*Settings!$B$5)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="32">
+        <f>IF(2&lt;=Settings!$B$12,2,"")</f>
+        <v>2</v>
+      </c>
+      <c r="B23" s="33">
+        <f>IF($A23="","",$B22*(1-Settings!$B$5))</f>
+        <v>0.8</v>
+      </c>
+      <c r="C23" s="33">
+        <f>IF($A23="","",ROUND(($B23*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.92</v>
+      </c>
+      <c r="D23" s="33">
+        <f>IF($A23="","",ROUND(($C23*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.35</v>
+      </c>
+      <c r="E23" s="33">
+        <f>IF($A23="","",ROUND(($B23*Settings!$B$5)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="32">
+        <f>IF(3&lt;=Settings!$B$12,3,"")</f>
+        <v>3</v>
+      </c>
+      <c r="B24" s="33">
+        <f>IF($A24="","",$B23*(1-Settings!$B$5))</f>
+        <v>0.64</v>
+      </c>
+      <c r="C24" s="33">
+        <f>IF($A24="","",ROUND(($B24*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.74</v>
+      </c>
+      <c r="D24" s="33">
+        <f>IF($A24="","",ROUND(($C24*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.28</v>
+      </c>
+      <c r="E24" s="33">
+        <f>IF($A24="","",ROUND(($B24*Settings!$B$5)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="32">
+        <f>IF(4&lt;=Settings!$B$12,4,"")</f>
+        <v>4</v>
+      </c>
+      <c r="B25" s="33">
+        <f>IF($A25="","",$B24*(1-Settings!$B$5))</f>
+        <v>0.512</v>
+      </c>
+      <c r="C25" s="33">
+        <f>IF($A25="","",ROUND(($B25*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.59</v>
+      </c>
+      <c r="D25" s="33">
+        <f>IF($A25="","",ROUND(($C25*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.22</v>
+      </c>
+      <c r="E25" s="33">
+        <f>IF($A25="","",ROUND(($B25*Settings!$B$5)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="32">
+        <f>IF(5&lt;=Settings!$B$12,5,"")</f>
+        <v>5</v>
+      </c>
+      <c r="B26" s="33">
+        <f>IF($A26="","",$B25*(1-Settings!$B$5))</f>
+        <v>0.4096</v>
+      </c>
+      <c r="C26" s="33">
+        <f>IF($A26="","",ROUND(($B26*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.47</v>
+      </c>
+      <c r="D26" s="33">
+        <f>IF($A26="","",ROUND(($C26*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.18</v>
+      </c>
+      <c r="E26" s="33">
+        <f>IF($A26="","",ROUND(($B26*Settings!$B$5)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="32">
+        <f>IF(6&lt;=Settings!$B$12,6,"")</f>
+        <v>6</v>
+      </c>
+      <c r="B27" s="33">
+        <f>IF($A27="","",$B26*(1-Settings!$B$5))</f>
+        <v>0.32768</v>
+      </c>
+      <c r="C27" s="33">
+        <f>IF($A27="","",ROUND(($B27*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.38</v>
+      </c>
+      <c r="D27" s="33">
+        <f>IF($A27="","",ROUND(($C27*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.14</v>
+      </c>
+      <c r="E27" s="33">
+        <f>IF($A27="","",ROUND(($B27*Settings!$B$5)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.07</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="32">
+        <f>IF(7&lt;=Settings!$B$12,7,"")</f>
+        <v>7</v>
+      </c>
+      <c r="B28" s="33">
+        <f>IF($A28="","",$B27*(1-Settings!$B$5))</f>
+        <v>0.262144</v>
+      </c>
+      <c r="C28" s="33">
+        <f>IF($A28="","",ROUND(($B28*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.3</v>
+      </c>
+      <c r="D28" s="33">
+        <f>IF($A28="","",ROUND(($C28*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.11</v>
+      </c>
+      <c r="E28" s="33">
+        <f>IF($A28="","",ROUND(($B28*Settings!$B$5)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="32">
+        <f>IF(8&lt;=Settings!$B$12,8,"")</f>
+        <v>8</v>
+      </c>
+      <c r="B29" s="33">
+        <f>IF($A29="","",$B28*(1-Settings!$B$5))</f>
+        <v>0.2097152</v>
+      </c>
+      <c r="C29" s="33">
+        <f>IF($A29="","",ROUND(($B29*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.24</v>
+      </c>
+      <c r="D29" s="33">
+        <f>IF($A29="","",ROUND(($C29*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.09</v>
+      </c>
+      <c r="E29" s="33">
+        <f>IF($A29="","",ROUND(($B29*Settings!$B$5)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="32">
+        <f>IF(9&lt;=Settings!$B$12,9,"")</f>
+        <v>9</v>
+      </c>
+      <c r="B30" s="33">
+        <f>IF($A30="","",$B29*(1-Settings!$B$5))</f>
+        <v>0.16777216</v>
+      </c>
+      <c r="C30" s="33">
+        <f>IF($A30="","",ROUND(($B30*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.19</v>
+      </c>
+      <c r="D30" s="33">
+        <f>IF($A30="","",ROUND(($C30*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.07</v>
+      </c>
+      <c r="E30" s="33">
+        <f>IF($A30="","",ROUND(($B30*Settings!$B$5)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="32">
+        <f>IF(10&lt;=Settings!$B$12,10,"")</f>
+        <v>10</v>
+      </c>
+      <c r="B31" s="33">
+        <f>IF($A31="","",$B30*(1-Settings!$B$5))</f>
+        <v>0.134217728</v>
+      </c>
+      <c r="C31" s="33">
+        <f>IF($A31="","",ROUND(($B31*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.15</v>
+      </c>
+      <c r="D31" s="33">
+        <f>IF($A31="","",ROUND(($C31*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.06</v>
+      </c>
+      <c r="E31" s="33">
+        <f>IF($A31="","",ROUND(($B31*Settings!$B$5)/Settings!$B$11,0)*Settings!$B$11)</f>
+        <v>0.03</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A20:E20"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9326,7 +9627,7 @@
       </c>
       <c r="C12">
         <f>COUNTIF(Calculator!AQ2:AQ11,"DUAL_TAIL")</f>
-        <v>1</v>
+        <v/>
       </c>
       <c r="D12">
         <f>C12</f>
@@ -9366,7 +9667,7 @@
       </c>
       <c r="C14">
         <f>COUNTIF(Calculator!AQ2:AQ11,"STOP")</f>
-        <v>7</v>
+        <v/>
       </c>
       <c r="D14">
         <f>C14</f>
@@ -9410,7 +9711,7 @@
       </c>
       <c r="D16">
         <f>C16</f>
-        <v/>
+        <v>0.9896</v>
       </c>
     </row>
     <row r="17">
@@ -9426,7 +9727,7 @@
       </c>
       <c r="C17">
         <f>LOOKUP(2,1/(Calculator!AZ2:AZ11&lt;&gt;""),Calculator!AZ2:AZ11)</f>
-        <v>0.5216</v>
+        <v/>
       </c>
       <c r="D17">
         <f>C17</f>
@@ -9446,7 +9747,7 @@
       </c>
       <c r="C18">
         <f>LOOKUP(2,1/(Calculator!BA2:BA11&lt;&gt;""),Calculator!BA2:BA11)</f>
-        <v>0.468</v>
+        <v/>
       </c>
       <c r="D18">
         <f>C18</f>
@@ -9466,7 +9767,7 @@
       </c>
       <c r="C19">
         <f>LOOKUP(2,1/(Calculator!BB2:BB11&lt;&gt;""),Calculator!BB2:BB11)</f>
-        <v>0.9896</v>
+        <v/>
       </c>
       <c r="D19">
         <f>C19</f>
@@ -9510,7 +9811,7 @@
       </c>
       <c r="D21">
         <f>C21</f>
-        <v/>
+        <v>7</v>
       </c>
     </row>
     <row r="22">
@@ -9582,7 +9883,7 @@
       </c>
       <c r="D26">
         <f>C26</f>
-        <v/>
+        <v>900</v>
       </c>
     </row>
     <row r="27">
@@ -9602,7 +9903,7 @@
       </c>
       <c r="D27">
         <f>C27</f>
-        <v/>
+        <v>300</v>
       </c>
     </row>
     <row r="28">
@@ -9618,7 +9919,7 @@
       </c>
       <c r="C28">
         <f>SUM(Calculator!AS2:AS11,Trend_UP!AS2:AS11,Trend_DOWN!AS2:AS11)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="D28">
         <f>C28</f>
@@ -9638,7 +9939,7 @@
       </c>
       <c r="C29">
         <f>MAX(Calculator!AD2:AD11,Trend_UP!AD2:AD11,Trend_DOWN!AD2:AD11)</f>
-        <v>2590</v>
+        <v/>
       </c>
       <c r="D29">
         <f>C29</f>
@@ -9658,7 +9959,7 @@
       </c>
       <c r="C30">
         <f>MAX(Calculator!AB2:AB11,Trend_UP!AB2:AB11,Trend_DOWN!AB2:AB11)</f>
-        <v>2.59</v>
+        <v/>
       </c>
       <c r="D30">
         <f>C30</f>
@@ -9682,7 +9983,7 @@
       </c>
       <c r="D31">
         <f>C31</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
@@ -9702,7 +10003,7 @@
       </c>
       <c r="D32">
         <f>C32</f>
-        <v/>
+        <v>14</v>
       </c>
     </row>
     <row r="33">
@@ -9722,7 +10023,7 @@
       </c>
       <c r="D33">
         <f>C33</f>
-        <v/>
+        <v>14</v>
       </c>
     </row>
     <row r="34">
@@ -9737,12 +10038,12 @@
         </is>
       </c>
       <c r="C34">
-        <f>MAX(Calculator!BB2:BB11,Trend_UP!BB2:BB11,Trend_DOWN!BB2:BB11)</f>
+        <f>MAX(Calculator!BC2:BC11,Trend_UP!BC2:BC11,Trend_DOWN!BC2:BC11)</f>
         <v>1.5306</v>
       </c>
       <c r="D34">
         <f>C34</f>
-        <v/>
+        <v>1.5306</v>
       </c>
     </row>
     <row r="35">
@@ -9758,7 +10059,7 @@
       </c>
       <c r="C35">
         <f>COUNTIF(Calculator!AQ2:AQ11,"DANGER")+COUNTIF(Trend_UP!AQ2:AQ11,"DANGER")+COUNTIF(Trend_DOWN!AQ2:AQ11,"DANGER")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="D35">
         <f>C35</f>
@@ -9776,7 +10077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -13480,6 +13781,342 @@
       <c r="H88" t="inlineStr">
         <is>
           <t>BLOCKED rows are readable and complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>V8-01</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Global Max DualTail Exposure uses DualTailTotalLot</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Risk_Analysis formula</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>MAX Calculator/Trend_UP/Trend_DOWN DualTailTotalLot ranges</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Formula inspection</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Uses BC DualTailTotalLot ranges, not ActiveNewFarLot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>V8-02</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Global Max DualTail Exposure expected value</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Current scenario data</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>1.5306</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>data_only Risk_Analysis cache</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Global max equals Trend_DOWN dual-tail total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>V8-03</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Settings geometry table exists</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Settings sheet</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>N / FarStart-N / Big-N / Small-N / Close-N</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Header inspection</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Geometry table is below parameter block.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>V8-04</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Big-N formula</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Settings geometry table</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Big-N = FarStart-N × BigRatio rounded by LotStep</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Formula inspection</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Formula references Settings!$B$3 and Settings!$B$11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>V8-05</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Small-N formula</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Settings geometry table</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Small-N = Big-N × SmallRatio rounded by LotStep</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Formula inspection</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Formula references Settings!$B$4 and Settings!$B$11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>V8-06</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Close-N formula</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Settings geometry table</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Close-N = FarStart-N × CloseFarShare rounded by LotStep</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Formula inspection</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Formula references Settings!$B$5 and Settings!$B$11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>V8-07</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Geometry uses Settings references</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Settings geometry table</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>No static ratios in formulas</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Formula inspection</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Uses StartLot, BigRatio, SmallRatio, CloseFarShare, LotStep, MaxLevels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>V8-08</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Close-N reference only</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Calculator close logic</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Calculator remains money-mode: CloseFarBudget / LossPerLotToClose</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Formula inspection</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Close-N is not used in Calculator formulas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Big-harvest LotStep rounding and final close logic
</commit_message>
<xml_diff>
--- a/work/MinusLock_SelfCompressing_BigSmall_v2/MinusLock_SelfCompressing_BigSmall_v2.xlsx
+++ b/work/MinusLock_SelfCompressing_BigSmall_v2/MinusLock_SelfCompressing_BigSmall_v2.xlsx
@@ -170,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -260,6 +260,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -659,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -673,9 +676,16 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -988,7 +998,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>Big Harvest Geometry — денежное закрытие Far через CloseFarBudget</t>
+          <t>Big Harvest Geometry — LotStep rounding and final-close validation</t>
         </is>
       </c>
     </row>
@@ -1050,17 +1060,52 @@
       </c>
       <c r="L21" s="31" t="inlineStr">
         <is>
-          <t>CloseFarLot</t>
-        </is>
-      </c>
-      <c r="M21" s="29" t="inlineStr">
-        <is>
-          <t>FarRemain</t>
-        </is>
-      </c>
-      <c r="N21" s="31" t="inlineStr">
+          <t>CloseFarLotRaw</t>
+        </is>
+      </c>
+      <c r="M21" s="31" t="inlineStr">
+        <is>
+          <t>CloseFarLotRounded</t>
+        </is>
+      </c>
+      <c r="N21" s="29" t="inlineStr">
+        <is>
+          <t>FarRemainAfterRounded</t>
+        </is>
+      </c>
+      <c r="O21" s="31" t="inlineStr">
         <is>
           <t>CloseFarPercent</t>
+        </is>
+      </c>
+      <c r="P21" s="36" t="inlineStr">
+        <is>
+          <t>CannotCloseBelowLotStep</t>
+        </is>
+      </c>
+      <c r="Q21" s="36" t="inlineStr">
+        <is>
+          <t>FarRemainLoss</t>
+        </is>
+      </c>
+      <c r="R21" s="37" t="inlineStr">
+        <is>
+          <t>TotalReserve</t>
+        </is>
+      </c>
+      <c r="S21" s="28" t="inlineStr">
+        <is>
+          <t>FinalCloseAllowed</t>
+        </is>
+      </c>
+      <c r="T21" s="36" t="inlineStr">
+        <is>
+          <t>FinalClosePL</t>
+        </is>
+      </c>
+      <c r="U21" s="31" t="inlineStr">
+        <is>
+          <t>LostToRounding</t>
         </is>
       </c>
     </row>
@@ -1110,16 +1155,44 @@
         <v>8.3</v>
       </c>
       <c r="L22" s="33">
-        <f>IF($A22="","",MIN($B22,IFERROR($J22/($D22*Settings!$B$9),0)))</f>
+        <f>IF($A22="","",IFERROR($J22/($D22*Settings!$B$9),0))</f>
         <v>0.3735</v>
       </c>
       <c r="M22" s="33">
-        <f>IF($A22="","",MAX(0,$B22-$L22))</f>
-        <v>0.6265</v>
+        <f>IF($A22="","",MIN($B22,FLOOR(MAX(0,$L22),Settings!$B$11)))</f>
+        <v>0.37</v>
       </c>
       <c r="N22" s="33">
-        <f>IF($A22="","",IFERROR($L22/$B22,0))</f>
-        <v>0.3735</v>
+        <f>IF($A22="","",MAX(0,$B22-$M22))</f>
+        <v>0.63</v>
+      </c>
+      <c r="O22" s="33">
+        <f>IF($A22="","",IFERROR($M22/$B22,0))</f>
+        <v>0.37</v>
+      </c>
+      <c r="P22" s="39" t="str">
+        <f>IF($A22="","",IF(AND($L22&gt;0,$L22&lt;Settings!$B$11),"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="Q22" s="33">
+        <f>IF($A22="","",$N22*$D22*Settings!$B$9)</f>
+        <v>126</v>
+      </c>
+      <c r="R22" s="33">
+        <f>IF($A22="","",SUM($K$22:$K22))</f>
+        <v>8.3</v>
+      </c>
+      <c r="S22" s="39" t="str">
+        <f>IF($A22="","",IF($R22&gt;=$Q22,"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="T22" s="33">
+        <f>IF($A22="","",$R22-$Q22)</f>
+        <v>-117.7</v>
+      </c>
+      <c r="U22" s="33">
+        <f>IF($A22="","",MAX(0,$L22-$M22))</f>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="23">
@@ -1128,8 +1201,8 @@
         <v>2</v>
       </c>
       <c r="B23" s="33">
-        <f>IF($A23="","",$M22)</f>
-        <v>0.6265</v>
+        <f>IF($A23="","",$N22)</f>
+        <v>0.63</v>
       </c>
       <c r="C23" s="32">
         <f>IF($A23="","",100)</f>
@@ -1141,19 +1214,19 @@
       </c>
       <c r="E23" s="33">
         <f>IF($A23="","",ROUND(($B23*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.81</v>
+        <v>0.82</v>
       </c>
       <c r="F23" s="33">
         <f>IF($A23="","",ROUND(($E23*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="G23" s="33">
         <f>IF($A23="","",$E23*$C23*Settings!$B$9)</f>
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H23" s="33">
         <f>IF($A23="","",$F23*$C23*Settings!$B$9)</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I23" s="33">
         <f>IF($A23="","",$G23-$H23)</f>
@@ -1168,16 +1241,44 @@
         <v>5.2</v>
       </c>
       <c r="L23" s="33">
-        <f>IF($A23="","",MIN($B23,IFERROR($J23/($D23*Settings!$B$9),0)))</f>
+        <f>IF($A23="","",IFERROR($J23/($D23*Settings!$B$9),0))</f>
         <v>0.234</v>
       </c>
       <c r="M23" s="33">
-        <f>IF($A23="","",MAX(0,$B23-$L23))</f>
-        <v>0.3925</v>
+        <f>IF($A23="","",MIN($B23,FLOOR(MAX(0,$L23),Settings!$B$11)))</f>
+        <v>0.23</v>
       </c>
       <c r="N23" s="33">
-        <f>IF($A23="","",IFERROR($L23/$B23,0))</f>
-        <v>0.373503591381</v>
+        <f>IF($A23="","",MAX(0,$B23-$M23))</f>
+        <v>0.4</v>
+      </c>
+      <c r="O23" s="33">
+        <f>IF($A23="","",IFERROR($M23/$B23,0))</f>
+        <v>0.365079365079</v>
+      </c>
+      <c r="P23" s="39" t="str">
+        <f>IF($A23="","",IF(AND($L23&gt;0,$L23&lt;Settings!$B$11),"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="Q23" s="33">
+        <f>IF($A23="","",$N23*$D23*Settings!$B$9)</f>
+        <v>80</v>
+      </c>
+      <c r="R23" s="33">
+        <f>IF($A23="","",SUM($K$22:$K23))</f>
+        <v>13.5</v>
+      </c>
+      <c r="S23" s="39" t="str">
+        <f>IF($A23="","",IF($R23&gt;=$Q23,"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="T23" s="33">
+        <f>IF($A23="","",$R23-$Q23)</f>
+        <v>-66.5</v>
+      </c>
+      <c r="U23" s="33">
+        <f>IF($A23="","",MAX(0,$L23-$M23))</f>
+        <v>0.004</v>
       </c>
     </row>
     <row r="24">
@@ -1186,8 +1287,8 @@
         <v>3</v>
       </c>
       <c r="B24" s="33">
-        <f>IF($A24="","",$M23)</f>
-        <v>0.3925</v>
+        <f>IF($A24="","",$N23)</f>
+        <v>0.4</v>
       </c>
       <c r="C24" s="32">
         <f>IF($A24="","",100)</f>
@@ -1199,19 +1300,19 @@
       </c>
       <c r="E24" s="33">
         <f>IF($A24="","",ROUND(($B24*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="F24" s="33">
         <f>IF($A24="","",ROUND(($E24*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="G24" s="33">
         <f>IF($A24="","",$E24*$C24*Settings!$B$9)</f>
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H24" s="33">
         <f>IF($A24="","",$F24*$C24*Settings!$B$9)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I24" s="33">
         <f>IF($A24="","",$G24-$H24)</f>
@@ -1226,16 +1327,44 @@
         <v>3.3</v>
       </c>
       <c r="L24" s="33">
-        <f>IF($A24="","",MIN($B24,IFERROR($J24/($D24*Settings!$B$9),0)))</f>
+        <f>IF($A24="","",IFERROR($J24/($D24*Settings!$B$9),0))</f>
         <v>0.1485</v>
       </c>
       <c r="M24" s="33">
-        <f>IF($A24="","",MAX(0,$B24-$L24))</f>
-        <v>0.244</v>
+        <f>IF($A24="","",MIN($B24,FLOOR(MAX(0,$L24),Settings!$B$11)))</f>
+        <v>0.14</v>
       </c>
       <c r="N24" s="33">
-        <f>IF($A24="","",IFERROR($L24/$B24,0))</f>
-        <v>0.378343949045</v>
+        <f>IF($A24="","",MAX(0,$B24-$M24))</f>
+        <v>0.26</v>
+      </c>
+      <c r="O24" s="33">
+        <f>IF($A24="","",IFERROR($M24/$B24,0))</f>
+        <v>0.35</v>
+      </c>
+      <c r="P24" s="39" t="str">
+        <f>IF($A24="","",IF(AND($L24&gt;0,$L24&lt;Settings!$B$11),"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="Q24" s="33">
+        <f>IF($A24="","",$N24*$D24*Settings!$B$9)</f>
+        <v>52</v>
+      </c>
+      <c r="R24" s="33">
+        <f>IF($A24="","",SUM($K$22:$K24))</f>
+        <v>16.8</v>
+      </c>
+      <c r="S24" s="39" t="str">
+        <f>IF($A24="","",IF($R24&gt;=$Q24,"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="T24" s="33">
+        <f>IF($A24="","",$R24-$Q24)</f>
+        <v>-35.2</v>
+      </c>
+      <c r="U24" s="33">
+        <f>IF($A24="","",MAX(0,$L24-$M24))</f>
+        <v>0.0085</v>
       </c>
     </row>
     <row r="25">
@@ -1244,8 +1373,8 @@
         <v>4</v>
       </c>
       <c r="B25" s="33">
-        <f>IF($A25="","",$M24)</f>
-        <v>0.244</v>
+        <f>IF($A25="","",$N24)</f>
+        <v>0.26</v>
       </c>
       <c r="C25" s="32">
         <f>IF($A25="","",100)</f>
@@ -1257,7 +1386,7 @@
       </c>
       <c r="E25" s="33">
         <f>IF($A25="","",ROUND(($B25*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="F25" s="33">
         <f>IF($A25="","",ROUND(($E25*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
@@ -1265,7 +1394,7 @@
       </c>
       <c r="G25" s="33">
         <f>IF($A25="","",$E25*$C25*Settings!$B$9)</f>
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H25" s="33">
         <f>IF($A25="","",$F25*$C25*Settings!$B$9)</f>
@@ -1273,27 +1402,55 @@
       </c>
       <c r="I25" s="33">
         <f>IF($A25="","",$G25-$H25)</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J25" s="33">
         <f>IF($A25="","",MAX(0,$I25*Settings!$B$5))</f>
-        <v>18</v>
+        <v>19.8</v>
       </c>
       <c r="K25" s="33">
         <f>IF($A25="","",MAX(0,$I25*Settings!$B$6))</f>
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="L25" s="33">
-        <f>IF($A25="","",MIN($B25,IFERROR($J25/($D25*Settings!$B$9),0)))</f>
+        <f>IF($A25="","",IFERROR($J25/($D25*Settings!$B$9),0))</f>
+        <v>0.099</v>
+      </c>
+      <c r="M25" s="33">
+        <f>IF($A25="","",MIN($B25,FLOOR(MAX(0,$L25),Settings!$B$11)))</f>
         <v>0.09</v>
       </c>
-      <c r="M25" s="33">
-        <f>IF($A25="","",MAX(0,$B25-$L25))</f>
-        <v>0.154</v>
-      </c>
       <c r="N25" s="33">
-        <f>IF($A25="","",IFERROR($L25/$B25,0))</f>
-        <v>0.368852459016</v>
+        <f>IF($A25="","",MAX(0,$B25-$M25))</f>
+        <v>0.17</v>
+      </c>
+      <c r="O25" s="33">
+        <f>IF($A25="","",IFERROR($M25/$B25,0))</f>
+        <v>0.346153846154</v>
+      </c>
+      <c r="P25" s="39" t="str">
+        <f>IF($A25="","",IF(AND($L25&gt;0,$L25&lt;Settings!$B$11),"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="Q25" s="33">
+        <f>IF($A25="","",$N25*$D25*Settings!$B$9)</f>
+        <v>34</v>
+      </c>
+      <c r="R25" s="33">
+        <f>IF($A25="","",SUM($K$22:$K25))</f>
+        <v>19</v>
+      </c>
+      <c r="S25" s="39" t="str">
+        <f>IF($A25="","",IF($R25&gt;=$Q25,"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="T25" s="33">
+        <f>IF($A25="","",$R25-$Q25)</f>
+        <v>-15</v>
+      </c>
+      <c r="U25" s="33">
+        <f>IF($A25="","",MAX(0,$L25-$M25))</f>
+        <v>0.009</v>
       </c>
     </row>
     <row r="26">
@@ -1302,8 +1459,8 @@
         <v>5</v>
       </c>
       <c r="B26" s="33">
-        <f>IF($A26="","",$M25)</f>
-        <v>0.154</v>
+        <f>IF($A26="","",$N25)</f>
+        <v>0.17</v>
       </c>
       <c r="C26" s="32">
         <f>IF($A26="","",100)</f>
@@ -1315,43 +1472,71 @@
       </c>
       <c r="E26" s="33">
         <f>IF($A26="","",ROUND(($B26*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="F26" s="33">
         <f>IF($A26="","",ROUND(($E26*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.07</v>
+        <v>0.08</v>
       </c>
       <c r="G26" s="33">
         <f>IF($A26="","",$E26*$C26*Settings!$B$9)</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H26" s="33">
         <f>IF($A26="","",$F26*$C26*Settings!$B$9)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I26" s="33">
         <f>IF($A26="","",$G26-$H26)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J26" s="33">
         <f>IF($A26="","",MAX(0,$I26*Settings!$B$5))</f>
-        <v>11.7</v>
+        <v>12.6</v>
       </c>
       <c r="K26" s="33">
         <f>IF($A26="","",MAX(0,$I26*Settings!$B$6))</f>
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="L26" s="33">
-        <f>IF($A26="","",MIN($B26,IFERROR($J26/($D26*Settings!$B$9),0)))</f>
-        <v>0.0585</v>
+        <f>IF($A26="","",IFERROR($J26/($D26*Settings!$B$9),0))</f>
+        <v>0.063</v>
       </c>
       <c r="M26" s="33">
-        <f>IF($A26="","",MAX(0,$B26-$L26))</f>
-        <v>0.0955</v>
+        <f>IF($A26="","",MIN($B26,FLOOR(MAX(0,$L26),Settings!$B$11)))</f>
+        <v>0.06</v>
       </c>
       <c r="N26" s="33">
-        <f>IF($A26="","",IFERROR($L26/$B26,0))</f>
-        <v>0.37987012987</v>
+        <f>IF($A26="","",MAX(0,$B26-$M26))</f>
+        <v>0.11</v>
+      </c>
+      <c r="O26" s="33">
+        <f>IF($A26="","",IFERROR($M26/$B26,0))</f>
+        <v>0.352941176471</v>
+      </c>
+      <c r="P26" s="39" t="str">
+        <f>IF($A26="","",IF(AND($L26&gt;0,$L26&lt;Settings!$B$11),"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="Q26" s="33">
+        <f>IF($A26="","",$N26*$D26*Settings!$B$9)</f>
+        <v>22</v>
+      </c>
+      <c r="R26" s="33">
+        <f>IF($A26="","",SUM($K$22:$K26))</f>
+        <v>20.4</v>
+      </c>
+      <c r="S26" s="39" t="str">
+        <f>IF($A26="","",IF($R26&gt;=$Q26,"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="T26" s="33">
+        <f>IF($A26="","",$R26-$Q26)</f>
+        <v>-1.6</v>
+      </c>
+      <c r="U26" s="33">
+        <f>IF($A26="","",MAX(0,$L26-$M26))</f>
+        <v>0.003</v>
       </c>
     </row>
     <row r="27">
@@ -1360,8 +1545,8 @@
         <v>6</v>
       </c>
       <c r="B27" s="33">
-        <f>IF($A27="","",$M26)</f>
-        <v>0.0955</v>
+        <f>IF($A27="","",$N26)</f>
+        <v>0.11</v>
       </c>
       <c r="C27" s="32">
         <f>IF($A27="","",100)</f>
@@ -1373,43 +1558,71 @@
       </c>
       <c r="E27" s="33">
         <f>IF($A27="","",ROUND(($B27*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="F27" s="33">
         <f>IF($A27="","",ROUND(($E27*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="G27" s="33">
         <f>IF($A27="","",$E27*$C27*Settings!$B$9)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H27" s="33">
         <f>IF($A27="","",$F27*$C27*Settings!$B$9)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I27" s="33">
         <f>IF($A27="","",$G27-$H27)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J27" s="33">
         <f>IF($A27="","",MAX(0,$I27*Settings!$B$5))</f>
-        <v>7.2</v>
+        <v>8.1</v>
       </c>
       <c r="K27" s="33">
         <f>IF($A27="","",MAX(0,$I27*Settings!$B$6))</f>
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="L27" s="33">
-        <f>IF($A27="","",MIN($B27,IFERROR($J27/($D27*Settings!$B$9),0)))</f>
-        <v>0.036</v>
+        <f>IF($A27="","",IFERROR($J27/($D27*Settings!$B$9),0))</f>
+        <v>0.0405</v>
       </c>
       <c r="M27" s="33">
-        <f>IF($A27="","",MAX(0,$B27-$L27))</f>
-        <v>0.0595</v>
+        <f>IF($A27="","",MIN($B27,FLOOR(MAX(0,$L27),Settings!$B$11)))</f>
+        <v>0.04</v>
       </c>
       <c r="N27" s="33">
-        <f>IF($A27="","",IFERROR($L27/$B27,0))</f>
-        <v>0.376963350785</v>
+        <f>IF($A27="","",MAX(0,$B27-$M27))</f>
+        <v>0.07</v>
+      </c>
+      <c r="O27" s="33">
+        <f>IF($A27="","",IFERROR($M27/$B27,0))</f>
+        <v>0.363636363636</v>
+      </c>
+      <c r="P27" s="39" t="str">
+        <f>IF($A27="","",IF(AND($L27&gt;0,$L27&lt;Settings!$B$11),"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="Q27" s="33">
+        <f>IF($A27="","",$N27*$D27*Settings!$B$9)</f>
+        <v>14</v>
+      </c>
+      <c r="R27" s="33">
+        <f>IF($A27="","",SUM($K$22:$K27))</f>
+        <v>21.3</v>
+      </c>
+      <c r="S27" s="39" t="str">
+        <f>IF($A27="","",IF($R27&gt;=$Q27,"YES","NO"))</f>
+        <v>YES</v>
+      </c>
+      <c r="T27" s="33">
+        <f>IF($A27="","",$R27-$Q27)</f>
+        <v>7.3</v>
+      </c>
+      <c r="U27" s="33">
+        <f>IF($A27="","",MAX(0,$L27-$M27))</f>
+        <v>0.0005</v>
       </c>
     </row>
     <row r="28">
@@ -1418,8 +1631,8 @@
         <v>7</v>
       </c>
       <c r="B28" s="33">
-        <f>IF($A28="","",$M27)</f>
-        <v>0.0595</v>
+        <f>IF($A28="","",$N27)</f>
+        <v>0.07</v>
       </c>
       <c r="C28" s="32">
         <f>IF($A28="","",100)</f>
@@ -1431,7 +1644,7 @@
       </c>
       <c r="E28" s="33">
         <f>IF($A28="","",ROUND(($B28*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="F28" s="33">
         <f>IF($A28="","",ROUND(($E28*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
@@ -1439,7 +1652,7 @@
       </c>
       <c r="G28" s="33">
         <f>IF($A28="","",$E28*$C28*Settings!$B$9)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H28" s="33">
         <f>IF($A28="","",$F28*$C28*Settings!$B$9)</f>
@@ -1447,27 +1660,55 @@
       </c>
       <c r="I28" s="33">
         <f>IF($A28="","",$G28-$H28)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J28" s="33">
         <f>IF($A28="","",MAX(0,$I28*Settings!$B$5))</f>
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
       <c r="K28" s="33">
         <f>IF($A28="","",MAX(0,$I28*Settings!$B$6))</f>
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="L28" s="33">
-        <f>IF($A28="","",MIN($B28,IFERROR($J28/($D28*Settings!$B$9),0)))</f>
-        <v>0.0225</v>
+        <f>IF($A28="","",IFERROR($J28/($D28*Settings!$B$9),0))</f>
+        <v>0.027</v>
       </c>
       <c r="M28" s="33">
-        <f>IF($A28="","",MAX(0,$B28-$L28))</f>
-        <v>0.037</v>
+        <f>IF($A28="","",MIN($B28,FLOOR(MAX(0,$L28),Settings!$B$11)))</f>
+        <v>0.02</v>
       </c>
       <c r="N28" s="33">
-        <f>IF($A28="","",IFERROR($L28/$B28,0))</f>
-        <v>0.378151260504</v>
+        <f>IF($A28="","",MAX(0,$B28-$M28))</f>
+        <v>0.05</v>
+      </c>
+      <c r="O28" s="33">
+        <f>IF($A28="","",IFERROR($M28/$B28,0))</f>
+        <v>0.285714285714</v>
+      </c>
+      <c r="P28" s="39" t="str">
+        <f>IF($A28="","",IF(AND($L28&gt;0,$L28&lt;Settings!$B$11),"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="Q28" s="33">
+        <f>IF($A28="","",$N28*$D28*Settings!$B$9)</f>
+        <v>10</v>
+      </c>
+      <c r="R28" s="33">
+        <f>IF($A28="","",SUM($K$22:$K28))</f>
+        <v>21.9</v>
+      </c>
+      <c r="S28" s="39" t="str">
+        <f>IF($A28="","",IF($R28&gt;=$Q28,"YES","NO"))</f>
+        <v>YES</v>
+      </c>
+      <c r="T28" s="33">
+        <f>IF($A28="","",$R28-$Q28)</f>
+        <v>11.9</v>
+      </c>
+      <c r="U28" s="33">
+        <f>IF($A28="","",MAX(0,$L28-$M28))</f>
+        <v>0.007</v>
       </c>
     </row>
     <row r="29">
@@ -1476,8 +1717,8 @@
         <v>8</v>
       </c>
       <c r="B29" s="33">
-        <f>IF($A29="","",$M28)</f>
-        <v>0.037</v>
+        <f>IF($A29="","",$N28)</f>
+        <v>0.05</v>
       </c>
       <c r="C29" s="32">
         <f>IF($A29="","",100)</f>
@@ -1489,7 +1730,7 @@
       </c>
       <c r="E29" s="33">
         <f>IF($A29="","",ROUND(($B29*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="F29" s="33">
         <f>IF($A29="","",ROUND(($E29*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
@@ -1497,7 +1738,7 @@
       </c>
       <c r="G29" s="33">
         <f>IF($A29="","",$E29*$C29*Settings!$B$9)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H29" s="33">
         <f>IF($A29="","",$F29*$C29*Settings!$B$9)</f>
@@ -1505,27 +1746,55 @@
       </c>
       <c r="I29" s="33">
         <f>IF($A29="","",$G29-$H29)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J29" s="33">
         <f>IF($A29="","",MAX(0,$I29*Settings!$B$5))</f>
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
       <c r="K29" s="33">
         <f>IF($A29="","",MAX(0,$I29*Settings!$B$6))</f>
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L29" s="33">
-        <f>IF($A29="","",MIN($B29,IFERROR($J29/($D29*Settings!$B$9),0)))</f>
-        <v>0.0135</v>
+        <f>IF($A29="","",IFERROR($J29/($D29*Settings!$B$9),0))</f>
+        <v>0.018</v>
       </c>
       <c r="M29" s="33">
-        <f>IF($A29="","",MAX(0,$B29-$L29))</f>
-        <v>0.0235</v>
+        <f>IF($A29="","",MIN($B29,FLOOR(MAX(0,$L29),Settings!$B$11)))</f>
+        <v>0.01</v>
       </c>
       <c r="N29" s="33">
-        <f>IF($A29="","",IFERROR($L29/$B29,0))</f>
-        <v>0.364864864865</v>
+        <f>IF($A29="","",MAX(0,$B29-$M29))</f>
+        <v>0.04</v>
+      </c>
+      <c r="O29" s="33">
+        <f>IF($A29="","",IFERROR($M29/$B29,0))</f>
+        <v>0.2</v>
+      </c>
+      <c r="P29" s="39" t="str">
+        <f>IF($A29="","",IF(AND($L29&gt;0,$L29&lt;Settings!$B$11),"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="Q29" s="33">
+        <f>IF($A29="","",$N29*$D29*Settings!$B$9)</f>
+        <v>8</v>
+      </c>
+      <c r="R29" s="33">
+        <f>IF($A29="","",SUM($K$22:$K29))</f>
+        <v>22.3</v>
+      </c>
+      <c r="S29" s="39" t="str">
+        <f>IF($A29="","",IF($R29&gt;=$Q29,"YES","NO"))</f>
+        <v>YES</v>
+      </c>
+      <c r="T29" s="33">
+        <f>IF($A29="","",$R29-$Q29)</f>
+        <v>14.3</v>
+      </c>
+      <c r="U29" s="33">
+        <f>IF($A29="","",MAX(0,$L29-$M29))</f>
+        <v>0.008</v>
       </c>
     </row>
     <row r="30">
@@ -1534,8 +1803,8 @@
         <v>9</v>
       </c>
       <c r="B30" s="33">
-        <f>IF($A30="","",$M29)</f>
-        <v>0.0235</v>
+        <f>IF($A30="","",$N29)</f>
+        <v>0.04</v>
       </c>
       <c r="C30" s="32">
         <f>IF($A30="","",100)</f>
@@ -1547,43 +1816,71 @@
       </c>
       <c r="E30" s="33">
         <f>IF($A30="","",ROUND(($B30*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="F30" s="33">
         <f>IF($A30="","",ROUND(($E30*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="G30" s="33">
         <f>IF($A30="","",$E30*$C30*Settings!$B$9)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H30" s="33">
         <f>IF($A30="","",$F30*$C30*Settings!$B$9)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I30" s="33">
         <f>IF($A30="","",$G30-$H30)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J30" s="33">
         <f>IF($A30="","",MAX(0,$I30*Settings!$B$5))</f>
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="K30" s="33">
         <f>IF($A30="","",MAX(0,$I30*Settings!$B$6))</f>
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L30" s="33">
-        <f>IF($A30="","",MIN($B30,IFERROR($J30/($D30*Settings!$B$9),0)))</f>
-        <v>0.009</v>
+        <f>IF($A30="","",IFERROR($J30/($D30*Settings!$B$9),0))</f>
+        <v>0.0135</v>
       </c>
       <c r="M30" s="33">
-        <f>IF($A30="","",MAX(0,$B30-$L30))</f>
-        <v>0.0145</v>
+        <f>IF($A30="","",MIN($B30,FLOOR(MAX(0,$L30),Settings!$B$11)))</f>
+        <v>0.01</v>
       </c>
       <c r="N30" s="33">
-        <f>IF($A30="","",IFERROR($L30/$B30,0))</f>
-        <v>0.382978723404</v>
+        <f>IF($A30="","",MAX(0,$B30-$M30))</f>
+        <v>0.03</v>
+      </c>
+      <c r="O30" s="33">
+        <f>IF($A30="","",IFERROR($M30/$B30,0))</f>
+        <v>0.25</v>
+      </c>
+      <c r="P30" s="39" t="str">
+        <f>IF($A30="","",IF(AND($L30&gt;0,$L30&lt;Settings!$B$11),"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="Q30" s="33">
+        <f>IF($A30="","",$N30*$D30*Settings!$B$9)</f>
+        <v>6</v>
+      </c>
+      <c r="R30" s="33">
+        <f>IF($A30="","",SUM($K$22:$K30))</f>
+        <v>22.6</v>
+      </c>
+      <c r="S30" s="39" t="str">
+        <f>IF($A30="","",IF($R30&gt;=$Q30,"YES","NO"))</f>
+        <v>YES</v>
+      </c>
+      <c r="T30" s="33">
+        <f>IF($A30="","",$R30-$Q30)</f>
+        <v>16.6</v>
+      </c>
+      <c r="U30" s="33">
+        <f>IF($A30="","",MAX(0,$L30-$M30))</f>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="31">
@@ -1592,8 +1889,8 @@
         <v>10</v>
       </c>
       <c r="B31" s="33">
-        <f>IF($A31="","",$M30)</f>
-        <v>0.0145</v>
+        <f>IF($A31="","",$N30)</f>
+        <v>0.03</v>
       </c>
       <c r="C31" s="32">
         <f>IF($A31="","",100)</f>
@@ -1605,7 +1902,7 @@
       </c>
       <c r="E31" s="33">
         <f>IF($A31="","",ROUND(($B31*Settings!$B$3)/Settings!$B$11,0)*Settings!$B$11)</f>
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="F31" s="33">
         <f>IF($A31="","",ROUND(($E31*Settings!$B$4)/Settings!$B$11,0)*Settings!$B$11)</f>
@@ -1613,7 +1910,7 @@
       </c>
       <c r="G31" s="33">
         <f>IF($A31="","",$E31*$C31*Settings!$B$9)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H31" s="33">
         <f>IF($A31="","",$F31*$C31*Settings!$B$9)</f>
@@ -1621,32 +1918,60 @@
       </c>
       <c r="I31" s="33">
         <f>IF($A31="","",$G31-$H31)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J31" s="33">
         <f>IF($A31="","",MAX(0,$I31*Settings!$B$5))</f>
-        <v>0.9</v>
+        <v>2.7</v>
       </c>
       <c r="K31" s="33">
         <f>IF($A31="","",MAX(0,$I31*Settings!$B$6))</f>
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="L31" s="33">
-        <f>IF($A31="","",MIN($B31,IFERROR($J31/($D31*Settings!$B$9),0)))</f>
-        <v>0.0045</v>
+        <f>IF($A31="","",IFERROR($J31/($D31*Settings!$B$9),0))</f>
+        <v>0.0135</v>
       </c>
       <c r="M31" s="33">
-        <f>IF($A31="","",MAX(0,$B31-$L31))</f>
+        <f>IF($A31="","",MIN($B31,FLOOR(MAX(0,$L31),Settings!$B$11)))</f>
         <v>0.01</v>
       </c>
       <c r="N31" s="33">
-        <f>IF($A31="","",IFERROR($L31/$B31,0))</f>
-        <v>0.310344827586</v>
+        <f>IF($A31="","",MAX(0,$B31-$M31))</f>
+        <v>0.02</v>
+      </c>
+      <c r="O31" s="33">
+        <f>IF($A31="","",IFERROR($M31/$B31,0))</f>
+        <v>0.333333333333</v>
+      </c>
+      <c r="P31" s="39" t="str">
+        <f>IF($A31="","",IF(AND($L31&gt;0,$L31&lt;Settings!$B$11),"YES","NO"))</f>
+        <v>NO</v>
+      </c>
+      <c r="Q31" s="33">
+        <f>IF($A31="","",$N31*$D31*Settings!$B$9)</f>
+        <v>4</v>
+      </c>
+      <c r="R31" s="33">
+        <f>IF($A31="","",SUM($K$22:$K31))</f>
+        <v>22.9</v>
+      </c>
+      <c r="S31" s="39" t="str">
+        <f>IF($A31="","",IF($R31&gt;=$Q31,"YES","NO"))</f>
+        <v>YES</v>
+      </c>
+      <c r="T31" s="33">
+        <f>IF($A31="","",$R31-$Q31)</f>
+        <v>18.9</v>
+      </c>
+      <c r="U31" s="33">
+        <f>IF($A31="","",MAX(0,$L31-$M31))</f>
+        <v>0.0035</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:N20"/>
+    <mergeCell ref="A20:U20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1658,7 +1983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BO11"/>
+  <dimension ref="A1:BU11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1728,6 +2053,12 @@
     <col width="17" customWidth="1" min="65" max="65"/>
     <col width="15" customWidth="1" min="66" max="66"/>
     <col width="14" customWidth="1" min="67" max="67"/>
+    <col width="16" customWidth="1" min="68" max="68"/>
+    <col width="20" customWidth="1" min="69" max="69"/>
+    <col width="23" customWidth="1" min="70" max="70"/>
+    <col width="25" customWidth="1" min="71" max="71"/>
+    <col width="19" customWidth="1" min="72" max="72"/>
+    <col width="16" customWidth="1" min="73" max="73"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2066,6 +2397,36 @@
           <t>FinalClosePL</t>
         </is>
       </c>
+      <c r="BP1" s="38" t="inlineStr">
+        <is>
+          <t>CloseFarLotRaw</t>
+        </is>
+      </c>
+      <c r="BQ1" s="38" t="inlineStr">
+        <is>
+          <t>CloseFarLotRounded</t>
+        </is>
+      </c>
+      <c r="BR1" s="38" t="inlineStr">
+        <is>
+          <t>FarRemainAfterRounded</t>
+        </is>
+      </c>
+      <c r="BS1" s="38" t="inlineStr">
+        <is>
+          <t>CannotCloseBelowLotStep</t>
+        </is>
+      </c>
+      <c r="BT1" s="38" t="inlineStr">
+        <is>
+          <t>FinalCloseAllowed</t>
+        </is>
+      </c>
+      <c r="BU1" s="38" t="inlineStr">
+        <is>
+          <t>LostToRounding</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="n">
@@ -2155,12 +2516,12 @@
         <v>200</v>
       </c>
       <c r="V2" s="12">
-        <f>IF($B2="BIG_SIDE",IFERROR(MIN($D2,MAX(0,$T2/$U2)),0),0)</f>
-        <v>0.3735</v>
+        <f>$BQ2</f>
+        <v>0.37</v>
       </c>
       <c r="W2" s="12">
-        <f>IF($B2="BIG_SIDE",MAX(0,$D2-$V2),$AJ2)</f>
-        <v>0.6265</v>
+        <f>IF($B2="BIG_SIDE",$BR2,$AJ2)</f>
+        <v>0.63</v>
       </c>
       <c r="X2" s="19">
         <f>IF($B2="BIG_SIDE",IF($AX$2&gt;0,$AX$2*Settings!$B$6,0),IF($S$2&gt;0,$S$2*Settings!$B$6,0))</f>
@@ -2175,7 +2536,7 @@
       </c>
       <c r="AA2" s="12">
         <f>IF($B2="BLOCKED",$Z2+$BF2,IF($B2="BIG_SIDE",$Z2+$S2-$AS2,IF($B2="SMALL_SIDE",$Z2+$S2+$AI2,$Z2+$S2)))</f>
-        <v>8.3</v>
+        <v>9</v>
       </c>
       <c r="AB2" s="12">
         <f>IF($B2="BLOCKED",$BC2,$D2+$G2+$J2)</f>
@@ -2246,11 +2607,11 @@
         <v/>
       </c>
       <c r="AS2" s="20">
-        <f>IF($B2="BIG_SIDE",$V2*$U2,0)</f>
-        <v>74.7</v>
+        <f>IF($B2="BIG_SIDE",$BQ2*$U2,0)</f>
+        <v>74</v>
       </c>
       <c r="AT2" s="12">
-        <f>IF($B2="BIG_SIDE",$G2+$J2+$V2,IF($B2="SMALL_SIDE",$J2+$AL2+$AV2,0))</f>
+        <f>IF($B2="BIG_SIDE",$G2+$J2+$BQ2,IF($B2="SMALL_SIDE",$J2+$AL2+$AV2,0))</f>
         <v/>
       </c>
       <c r="AU2" s="12">
@@ -2320,20 +2681,44 @@
         <v>1</v>
       </c>
       <c r="BL2">
-        <f>IF($D2&gt;0,IFERROR($V2/$D2,0),0)</f>
-        <v>0.3735</v>
+        <f>IF($D2&gt;0,IFERROR($BQ2/$D2,0),0)</f>
+        <v>0.37</v>
       </c>
       <c r="BM2" t="b">
-        <f>IF($BN2&lt;=0,FALSE,$Y2&gt;=$BN2)</f>
+        <f>$BT2</f>
         <v>0</v>
       </c>
       <c r="BN2">
-        <f>MAX(0,$W2*$BI2*Settings!$B$9)</f>
-        <v>125.3</v>
+        <f>MAX(0,$BR2*$BI2*Settings!$B$9)</f>
+        <v>126</v>
       </c>
       <c r="BO2">
         <f>$Y2-$BN2</f>
-        <v>-117</v>
+        <v>-117.7</v>
+      </c>
+      <c r="BP2">
+        <f>IF($B2="BIG_SIDE",IFERROR($T2/$U2,0),0)</f>
+        <v>0.3735</v>
+      </c>
+      <c r="BQ2">
+        <f>IF($B2="BIG_SIDE",MIN($D2,FLOOR(MAX(0,$BP2),Settings!$B$11)),0)</f>
+        <v>0.37</v>
+      </c>
+      <c r="BR2">
+        <f>IF($B2="BIG_SIDE",MAX(0,$D2-$BQ2),$AJ2)</f>
+        <v>0.63</v>
+      </c>
+      <c r="BS2" t="str">
+        <f>IF(AND($BP2&gt;0,$BP2&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT2" t="str">
+        <f>IF($Y2&gt;=$BN2,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU2">
+        <f>MAX(0,$BP2-$BQ2)</f>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="3">
@@ -2421,11 +2806,11 @@
         <v/>
       </c>
       <c r="V3" s="12">
-        <f>IF($B3="BIG_SIDE",IFERROR(MIN($D3,MAX(0,$T3/$U3)),0),0)</f>
+        <f>$BQ3</f>
         <v/>
       </c>
       <c r="W3" s="12">
-        <f>IF($B3="BIG_SIDE",MAX(0,$D3-$V3),$AJ3)</f>
+        <f>IF($B3="BIG_SIDE",$BR3,$AJ3)</f>
         <v/>
       </c>
       <c r="X3" s="19">
@@ -2513,11 +2898,11 @@
         <v/>
       </c>
       <c r="AS3" s="20">
-        <f>IF($B3="BIG_SIDE",$V3*$U3,0)</f>
+        <f>IF($B3="BIG_SIDE",$BQ3*$U3,0)</f>
         <v/>
       </c>
       <c r="AT3" s="12">
-        <f>IF($B3="BIG_SIDE",$G3+$J3+$V3,IF($B3="SMALL_SIDE",$J3+$AL3+$AV3,0))</f>
+        <f>IF($B3="BIG_SIDE",$G3+$J3+$BQ3,IF($B3="SMALL_SIDE",$J3+$AL3+$AV3,0))</f>
         <v/>
       </c>
       <c r="AU3" s="12">
@@ -2587,19 +2972,43 @@
         <v/>
       </c>
       <c r="BL3">
-        <f>IF($D3&gt;0,IFERROR($V3/$D3,0),0)</f>
+        <f>IF($D3&gt;0,IFERROR($BQ3/$D3,0),0)</f>
         <v/>
       </c>
       <c r="BM3">
-        <f>IF($BN3&lt;=0,FALSE,$Y3&gt;=$BN3)</f>
+        <f>$BT3</f>
         <v/>
       </c>
       <c r="BN3">
-        <f>MAX(0,$W3*$BI3*Settings!$B$9)</f>
+        <f>MAX(0,$BR3*$BI3*Settings!$B$9)</f>
         <v/>
       </c>
       <c r="BO3">
         <f>$Y3-$BN3</f>
+        <v/>
+      </c>
+      <c r="BP3">
+        <f>IF($B3="BIG_SIDE",IFERROR($T3/$U3,0),0)</f>
+        <v/>
+      </c>
+      <c r="BQ3">
+        <f>IF($B3="BIG_SIDE",MIN($D3,FLOOR(MAX(0,$BP3),Settings!$B$11)),0)</f>
+        <v/>
+      </c>
+      <c r="BR3">
+        <f>IF($B3="BIG_SIDE",MAX(0,$D3-$BQ3),$AJ3)</f>
+        <v/>
+      </c>
+      <c r="BS3">
+        <f>IF(AND($BP3&gt;0,$BP3&lt;Settings!$B$11),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BT3">
+        <f>IF($Y3&gt;=$BN3,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BU3">
+        <f>MAX(0,$BP3-$BQ3)</f>
         <v/>
       </c>
     </row>
@@ -2688,11 +3097,11 @@
         <v/>
       </c>
       <c r="V4" s="12">
-        <f>IF($B4="BIG_SIDE",IFERROR(MIN($D4,MAX(0,$T4/$U4)),0),0)</f>
+        <f>$BQ4</f>
         <v/>
       </c>
       <c r="W4" s="12">
-        <f>IF($B4="BIG_SIDE",MAX(0,$D4-$V4),$AJ4)</f>
+        <f>IF($B4="BIG_SIDE",$BR4,$AJ4)</f>
         <v/>
       </c>
       <c r="X4" s="19">
@@ -2780,11 +3189,11 @@
         <v/>
       </c>
       <c r="AS4" s="20">
-        <f>IF($B4="BIG_SIDE",$V4*$U4,0)</f>
+        <f>IF($B4="BIG_SIDE",$BQ4*$U4,0)</f>
         <v/>
       </c>
       <c r="AT4" s="12">
-        <f>IF($B4="BIG_SIDE",$G4+$J4+$V4,IF($B4="SMALL_SIDE",$J4+$AL4+$AV4,0))</f>
+        <f>IF($B4="BIG_SIDE",$G4+$J4+$BQ4,IF($B4="SMALL_SIDE",$J4+$AL4+$AV4,0))</f>
         <v/>
       </c>
       <c r="AU4" s="12">
@@ -2854,19 +3263,43 @@
         <v/>
       </c>
       <c r="BL4">
-        <f>IF($D4&gt;0,IFERROR($V4/$D4,0),0)</f>
+        <f>IF($D4&gt;0,IFERROR($BQ4/$D4,0),0)</f>
         <v/>
       </c>
       <c r="BM4">
-        <f>IF($BN4&lt;=0,FALSE,$Y4&gt;=$BN4)</f>
+        <f>$BT4</f>
         <v/>
       </c>
       <c r="BN4">
-        <f>MAX(0,$W4*$BI4*Settings!$B$9)</f>
+        <f>MAX(0,$BR4*$BI4*Settings!$B$9)</f>
         <v/>
       </c>
       <c r="BO4">
         <f>$Y4-$BN4</f>
+        <v/>
+      </c>
+      <c r="BP4">
+        <f>IF($B4="BIG_SIDE",IFERROR($T4/$U4,0),0)</f>
+        <v/>
+      </c>
+      <c r="BQ4">
+        <f>IF($B4="BIG_SIDE",MIN($D4,FLOOR(MAX(0,$BP4),Settings!$B$11)),0)</f>
+        <v/>
+      </c>
+      <c r="BR4">
+        <f>IF($B4="BIG_SIDE",MAX(0,$D4-$BQ4),$AJ4)</f>
+        <v/>
+      </c>
+      <c r="BS4">
+        <f>IF(AND($BP4&gt;0,$BP4&lt;Settings!$B$11),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BT4">
+        <f>IF($Y4&gt;=$BN4,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BU4">
+        <f>MAX(0,$BP4-$BQ4)</f>
         <v/>
       </c>
     </row>
@@ -2955,11 +3388,11 @@
         <v/>
       </c>
       <c r="V5" s="12">
-        <f>IF($B5="BIG_SIDE",IFERROR(MIN($D5,MAX(0,$T5/$U5)),0),0)</f>
+        <f>$BQ5</f>
         <v/>
       </c>
       <c r="W5" s="12">
-        <f>IF($B5="BIG_SIDE",MAX(0,$D5-$V5),$AJ5)</f>
+        <f>IF($B5="BIG_SIDE",$BR5,$AJ5)</f>
         <v/>
       </c>
       <c r="X5" s="19">
@@ -3047,11 +3480,11 @@
         <v/>
       </c>
       <c r="AS5" s="20">
-        <f>IF($B5="BIG_SIDE",$V5*$U5,0)</f>
+        <f>IF($B5="BIG_SIDE",$BQ5*$U5,0)</f>
         <v/>
       </c>
       <c r="AT5" s="12">
-        <f>IF($B5="BIG_SIDE",$G5+$J5+$V5,IF($B5="SMALL_SIDE",$J5+$AL5+$AV5,0))</f>
+        <f>IF($B5="BIG_SIDE",$G5+$J5+$BQ5,IF($B5="SMALL_SIDE",$J5+$AL5+$AV5,0))</f>
         <v/>
       </c>
       <c r="AU5" s="12">
@@ -3121,19 +3554,43 @@
         <v/>
       </c>
       <c r="BL5">
-        <f>IF($D5&gt;0,IFERROR($V5/$D5,0),0)</f>
+        <f>IF($D5&gt;0,IFERROR($BQ5/$D5,0),0)</f>
         <v/>
       </c>
       <c r="BM5">
-        <f>IF($BN5&lt;=0,FALSE,$Y5&gt;=$BN5)</f>
+        <f>$BT5</f>
         <v/>
       </c>
       <c r="BN5">
-        <f>MAX(0,$W5*$BI5*Settings!$B$9)</f>
+        <f>MAX(0,$BR5*$BI5*Settings!$B$9)</f>
         <v/>
       </c>
       <c r="BO5">
         <f>$Y5-$BN5</f>
+        <v/>
+      </c>
+      <c r="BP5">
+        <f>IF($B5="BIG_SIDE",IFERROR($T5/$U5,0),0)</f>
+        <v/>
+      </c>
+      <c r="BQ5">
+        <f>IF($B5="BIG_SIDE",MIN($D5,FLOOR(MAX(0,$BP5),Settings!$B$11)),0)</f>
+        <v/>
+      </c>
+      <c r="BR5">
+        <f>IF($B5="BIG_SIDE",MAX(0,$D5-$BQ5),$AJ5)</f>
+        <v/>
+      </c>
+      <c r="BS5">
+        <f>IF(AND($BP5&gt;0,$BP5&lt;Settings!$B$11),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BT5">
+        <f>IF($Y5&gt;=$BN5,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BU5">
+        <f>MAX(0,$BP5-$BQ5)</f>
         <v/>
       </c>
     </row>
@@ -3222,11 +3679,11 @@
         <v/>
       </c>
       <c r="V6" s="12">
-        <f>IF($B6="BIG_SIDE",IFERROR(MIN($D6,MAX(0,$T6/$U6)),0),0)</f>
+        <f>$BQ6</f>
         <v/>
       </c>
       <c r="W6" s="12">
-        <f>IF($B6="BIG_SIDE",MAX(0,$D6-$V6),$AJ6)</f>
+        <f>IF($B6="BIG_SIDE",$BR6,$AJ6)</f>
         <v/>
       </c>
       <c r="X6" s="19">
@@ -3314,11 +3771,11 @@
         <v/>
       </c>
       <c r="AS6" s="20">
-        <f>IF($B6="BIG_SIDE",$V6*$U6,0)</f>
+        <f>IF($B6="BIG_SIDE",$BQ6*$U6,0)</f>
         <v/>
       </c>
       <c r="AT6" s="12">
-        <f>IF($B6="BIG_SIDE",$G6+$J6+$V6,IF($B6="SMALL_SIDE",$J6+$AL6+$AV6,0))</f>
+        <f>IF($B6="BIG_SIDE",$G6+$J6+$BQ6,IF($B6="SMALL_SIDE",$J6+$AL6+$AV6,0))</f>
         <v/>
       </c>
       <c r="AU6" s="12">
@@ -3388,19 +3845,43 @@
         <v/>
       </c>
       <c r="BL6">
-        <f>IF($D6&gt;0,IFERROR($V6/$D6,0),0)</f>
+        <f>IF($D6&gt;0,IFERROR($BQ6/$D6,0),0)</f>
         <v/>
       </c>
       <c r="BM6">
-        <f>IF($BN6&lt;=0,FALSE,$Y6&gt;=$BN6)</f>
+        <f>$BT6</f>
         <v/>
       </c>
       <c r="BN6">
-        <f>MAX(0,$W6*$BI6*Settings!$B$9)</f>
+        <f>MAX(0,$BR6*$BI6*Settings!$B$9)</f>
         <v/>
       </c>
       <c r="BO6">
         <f>$Y6-$BN6</f>
+        <v/>
+      </c>
+      <c r="BP6">
+        <f>IF($B6="BIG_SIDE",IFERROR($T6/$U6,0),0)</f>
+        <v/>
+      </c>
+      <c r="BQ6">
+        <f>IF($B6="BIG_SIDE",MIN($D6,FLOOR(MAX(0,$BP6),Settings!$B$11)),0)</f>
+        <v/>
+      </c>
+      <c r="BR6">
+        <f>IF($B6="BIG_SIDE",MAX(0,$D6-$BQ6),$AJ6)</f>
+        <v/>
+      </c>
+      <c r="BS6">
+        <f>IF(AND($BP6&gt;0,$BP6&lt;Settings!$B$11),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BT6">
+        <f>IF($Y6&gt;=$BN6,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BU6">
+        <f>MAX(0,$BP6-$BQ6)</f>
         <v/>
       </c>
     </row>
@@ -3489,11 +3970,11 @@
         <v/>
       </c>
       <c r="V7" s="12">
-        <f>IF($B7="BIG_SIDE",IFERROR(MIN($D7,MAX(0,$T7/$U7)),0),0)</f>
+        <f>$BQ7</f>
         <v/>
       </c>
       <c r="W7" s="12">
-        <f>IF($B7="BIG_SIDE",MAX(0,$D7-$V7),$AJ7)</f>
+        <f>IF($B7="BIG_SIDE",$BR7,$AJ7)</f>
         <v/>
       </c>
       <c r="X7" s="19">
@@ -3581,11 +4062,11 @@
         <v/>
       </c>
       <c r="AS7" s="20">
-        <f>IF($B7="BIG_SIDE",$V7*$U7,0)</f>
+        <f>IF($B7="BIG_SIDE",$BQ7*$U7,0)</f>
         <v/>
       </c>
       <c r="AT7" s="12">
-        <f>IF($B7="BIG_SIDE",$G7+$J7+$V7,IF($B7="SMALL_SIDE",$J7+$AL7+$AV7,0))</f>
+        <f>IF($B7="BIG_SIDE",$G7+$J7+$BQ7,IF($B7="SMALL_SIDE",$J7+$AL7+$AV7,0))</f>
         <v/>
       </c>
       <c r="AU7" s="12">
@@ -3655,19 +4136,43 @@
         <v/>
       </c>
       <c r="BL7">
-        <f>IF($D7&gt;0,IFERROR($V7/$D7,0),0)</f>
+        <f>IF($D7&gt;0,IFERROR($BQ7/$D7,0),0)</f>
         <v/>
       </c>
       <c r="BM7">
-        <f>IF($BN7&lt;=0,FALSE,$Y7&gt;=$BN7)</f>
+        <f>$BT7</f>
         <v/>
       </c>
       <c r="BN7">
-        <f>MAX(0,$W7*$BI7*Settings!$B$9)</f>
+        <f>MAX(0,$BR7*$BI7*Settings!$B$9)</f>
         <v/>
       </c>
       <c r="BO7">
         <f>$Y7-$BN7</f>
+        <v/>
+      </c>
+      <c r="BP7">
+        <f>IF($B7="BIG_SIDE",IFERROR($T7/$U7,0),0)</f>
+        <v/>
+      </c>
+      <c r="BQ7">
+        <f>IF($B7="BIG_SIDE",MIN($D7,FLOOR(MAX(0,$BP7),Settings!$B$11)),0)</f>
+        <v/>
+      </c>
+      <c r="BR7">
+        <f>IF($B7="BIG_SIDE",MAX(0,$D7-$BQ7),$AJ7)</f>
+        <v/>
+      </c>
+      <c r="BS7">
+        <f>IF(AND($BP7&gt;0,$BP7&lt;Settings!$B$11),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BT7">
+        <f>IF($Y7&gt;=$BN7,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BU7">
+        <f>MAX(0,$BP7-$BQ7)</f>
         <v/>
       </c>
     </row>
@@ -3756,11 +4261,11 @@
         <v/>
       </c>
       <c r="V8" s="12">
-        <f>IF($B8="BIG_SIDE",IFERROR(MIN($D8,MAX(0,$T8/$U8)),0),0)</f>
+        <f>$BQ8</f>
         <v/>
       </c>
       <c r="W8" s="12">
-        <f>IF($B8="BIG_SIDE",MAX(0,$D8-$V8),$AJ8)</f>
+        <f>IF($B8="BIG_SIDE",$BR8,$AJ8)</f>
         <v/>
       </c>
       <c r="X8" s="19">
@@ -3848,11 +4353,11 @@
         <v/>
       </c>
       <c r="AS8" s="20">
-        <f>IF($B8="BIG_SIDE",$V8*$U8,0)</f>
+        <f>IF($B8="BIG_SIDE",$BQ8*$U8,0)</f>
         <v/>
       </c>
       <c r="AT8" s="12">
-        <f>IF($B8="BIG_SIDE",$G8+$J8+$V8,IF($B8="SMALL_SIDE",$J8+$AL8+$AV8,0))</f>
+        <f>IF($B8="BIG_SIDE",$G8+$J8+$BQ8,IF($B8="SMALL_SIDE",$J8+$AL8+$AV8,0))</f>
         <v/>
       </c>
       <c r="AU8" s="12">
@@ -3922,19 +4427,43 @@
         <v/>
       </c>
       <c r="BL8">
-        <f>IF($D8&gt;0,IFERROR($V8/$D8,0),0)</f>
+        <f>IF($D8&gt;0,IFERROR($BQ8/$D8,0),0)</f>
         <v/>
       </c>
       <c r="BM8">
-        <f>IF($BN8&lt;=0,FALSE,$Y8&gt;=$BN8)</f>
+        <f>$BT8</f>
         <v/>
       </c>
       <c r="BN8">
-        <f>MAX(0,$W8*$BI8*Settings!$B$9)</f>
+        <f>MAX(0,$BR8*$BI8*Settings!$B$9)</f>
         <v/>
       </c>
       <c r="BO8">
         <f>$Y8-$BN8</f>
+        <v/>
+      </c>
+      <c r="BP8">
+        <f>IF($B8="BIG_SIDE",IFERROR($T8/$U8,0),0)</f>
+        <v/>
+      </c>
+      <c r="BQ8">
+        <f>IF($B8="BIG_SIDE",MIN($D8,FLOOR(MAX(0,$BP8),Settings!$B$11)),0)</f>
+        <v/>
+      </c>
+      <c r="BR8">
+        <f>IF($B8="BIG_SIDE",MAX(0,$D8-$BQ8),$AJ8)</f>
+        <v/>
+      </c>
+      <c r="BS8">
+        <f>IF(AND($BP8&gt;0,$BP8&lt;Settings!$B$11),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BT8">
+        <f>IF($Y8&gt;=$BN8,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BU8">
+        <f>MAX(0,$BP8-$BQ8)</f>
         <v/>
       </c>
     </row>
@@ -4023,11 +4552,11 @@
         <v/>
       </c>
       <c r="V9" s="12">
-        <f>IF($B9="BIG_SIDE",IFERROR(MIN($D9,MAX(0,$T9/$U9)),0),0)</f>
+        <f>$BQ9</f>
         <v/>
       </c>
       <c r="W9" s="12">
-        <f>IF($B9="BIG_SIDE",MAX(0,$D9-$V9),$AJ9)</f>
+        <f>IF($B9="BIG_SIDE",$BR9,$AJ9)</f>
         <v/>
       </c>
       <c r="X9" s="19">
@@ -4115,11 +4644,11 @@
         <v/>
       </c>
       <c r="AS9" s="20">
-        <f>IF($B9="BIG_SIDE",$V9*$U9,0)</f>
+        <f>IF($B9="BIG_SIDE",$BQ9*$U9,0)</f>
         <v/>
       </c>
       <c r="AT9" s="12">
-        <f>IF($B9="BIG_SIDE",$G9+$J9+$V9,IF($B9="SMALL_SIDE",$J9+$AL9+$AV9,0))</f>
+        <f>IF($B9="BIG_SIDE",$G9+$J9+$BQ9,IF($B9="SMALL_SIDE",$J9+$AL9+$AV9,0))</f>
         <v/>
       </c>
       <c r="AU9" s="12">
@@ -4189,19 +4718,43 @@
         <v/>
       </c>
       <c r="BL9">
-        <f>IF($D9&gt;0,IFERROR($V9/$D9,0),0)</f>
+        <f>IF($D9&gt;0,IFERROR($BQ9/$D9,0),0)</f>
         <v/>
       </c>
       <c r="BM9">
-        <f>IF($BN9&lt;=0,FALSE,$Y9&gt;=$BN9)</f>
+        <f>$BT9</f>
         <v/>
       </c>
       <c r="BN9">
-        <f>MAX(0,$W9*$BI9*Settings!$B$9)</f>
+        <f>MAX(0,$BR9*$BI9*Settings!$B$9)</f>
         <v/>
       </c>
       <c r="BO9">
         <f>$Y9-$BN9</f>
+        <v/>
+      </c>
+      <c r="BP9">
+        <f>IF($B9="BIG_SIDE",IFERROR($T9/$U9,0),0)</f>
+        <v/>
+      </c>
+      <c r="BQ9">
+        <f>IF($B9="BIG_SIDE",MIN($D9,FLOOR(MAX(0,$BP9),Settings!$B$11)),0)</f>
+        <v/>
+      </c>
+      <c r="BR9">
+        <f>IF($B9="BIG_SIDE",MAX(0,$D9-$BQ9),$AJ9)</f>
+        <v/>
+      </c>
+      <c r="BS9">
+        <f>IF(AND($BP9&gt;0,$BP9&lt;Settings!$B$11),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BT9">
+        <f>IF($Y9&gt;=$BN9,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BU9">
+        <f>MAX(0,$BP9-$BQ9)</f>
         <v/>
       </c>
     </row>
@@ -4209,9 +4762,9 @@
       <c r="A10" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="13" t="str">
         <f>IF(AND($AQ9="MANUAL_READY",$BG9="YES"),"BIG_SIDE",IF(OR($AP9="NO",$AQ9="DUAL_TAIL",$AQ9="DANGER",$AQ9="STOP",$AQ9="MANUAL_READY",$AQ9="STOP_CLEARED"),"BLOCKED","BIG_SIDE"))</f>
-        <v/>
+        <v>BIG_SIDE</v>
       </c>
       <c r="C10" s="13">
         <f>IF($B10="BLOCKED",$AF9,IF(AND($AQ9="MANUAL_READY",$BG9="YES"),$AF9,IF($AP9="YES",$AF9,$C9)))</f>
@@ -4219,7 +4772,7 @@
       </c>
       <c r="D10" s="13">
         <f>IF($B10="BLOCKED",0,IF(AND($AQ9="MANUAL_READY",$BG9="YES"),MAX($BA9,$BB9),IF($AP9="YES",MAX(0,$AG9),$D9)))</f>
-        <v/>
+        <v>0.1</v>
       </c>
       <c r="E10" s="12">
         <f>IF($B10="BLOCKED","",IF($C10="SELL","BUY","SELL"))</f>
@@ -4290,11 +4843,11 @@
         <v/>
       </c>
       <c r="V10" s="12">
-        <f>IF($B10="BIG_SIDE",IFERROR(MIN($D10,MAX(0,$T10/$U10)),0),0)</f>
-        <v/>
+        <f>$BQ10</f>
+        <v>0</v>
       </c>
       <c r="W10" s="12">
-        <f>IF($B10="BIG_SIDE",MAX(0,$D10-$V10),$AJ10)</f>
+        <f>IF($B10="BIG_SIDE",$BR10,$AJ10)</f>
         <v/>
       </c>
       <c r="X10" s="19">
@@ -4382,11 +4935,11 @@
         <v/>
       </c>
       <c r="AS10" s="20">
-        <f>IF($B10="BIG_SIDE",$V10*$U10,0)</f>
+        <f>IF($B10="BIG_SIDE",$BQ10*$U10,0)</f>
         <v/>
       </c>
       <c r="AT10" s="12">
-        <f>IF($B10="BIG_SIDE",$G10+$J10+$V10,IF($B10="SMALL_SIDE",$J10+$AL10+$AV10,0))</f>
+        <f>IF($B10="BIG_SIDE",$G10+$J10+$BQ10,IF($B10="SMALL_SIDE",$J10+$AL10+$AV10,0))</f>
         <v/>
       </c>
       <c r="AU10" s="12">
@@ -4456,20 +5009,44 @@
         <v/>
       </c>
       <c r="BL10">
-        <f>IF($D10&gt;0,IFERROR($V10/$D10,0),0)</f>
+        <f>IF($D10&gt;0,IFERROR($BQ10/$D10,0),0)</f>
         <v/>
       </c>
       <c r="BM10">
-        <f>IF($BN10&lt;=0,FALSE,$Y10&gt;=$BN10)</f>
+        <f>$BT10</f>
         <v/>
       </c>
       <c r="BN10">
-        <f>MAX(0,$W10*$BI10*Settings!$B$9)</f>
-        <v/>
+        <f>MAX(0,$BR10*$BI10*Settings!$B$9)</f>
+        <v>20</v>
       </c>
       <c r="BO10">
         <f>$Y10-$BN10</f>
-        <v/>
+        <v>-20</v>
+      </c>
+      <c r="BP10">
+        <f>IF($B10="BIG_SIDE",IFERROR($T10/$U10,0),0)</f>
+        <v>0.009</v>
+      </c>
+      <c r="BQ10">
+        <f>IF($B10="BIG_SIDE",MIN($D10,FLOOR(MAX(0,$BP10),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR10">
+        <f>IF($B10="BIG_SIDE",MAX(0,$D10-$BQ10),$AJ10)</f>
+        <v>0.1</v>
+      </c>
+      <c r="BS10" t="str">
+        <f>IF(AND($BP10&gt;0,$BP10&lt;Settings!$B$11),"YES","NO")</f>
+        <v>YES</v>
+      </c>
+      <c r="BT10" t="str">
+        <f>IF($Y10&gt;=$BN10,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU10">
+        <f>MAX(0,$BP10-$BQ10)</f>
+        <v>0.009</v>
       </c>
     </row>
     <row r="11">
@@ -4557,11 +5134,11 @@
         <v/>
       </c>
       <c r="V11" s="12">
-        <f>IF($B11="BIG_SIDE",IFERROR(MIN($D11,MAX(0,$T11/$U11)),0),0)</f>
+        <f>$BQ11</f>
         <v/>
       </c>
       <c r="W11" s="12">
-        <f>IF($B11="BIG_SIDE",MAX(0,$D11-$V11),$AJ11)</f>
+        <f>IF($B11="BIG_SIDE",$BR11,$AJ11)</f>
         <v/>
       </c>
       <c r="X11" s="19">
@@ -4649,11 +5226,11 @@
         <v/>
       </c>
       <c r="AS11" s="20">
-        <f>IF($B11="BIG_SIDE",$V11*$U11,0)</f>
+        <f>IF($B11="BIG_SIDE",$BQ11*$U11,0)</f>
         <v/>
       </c>
       <c r="AT11" s="12">
-        <f>IF($B11="BIG_SIDE",$G11+$J11+$V11,IF($B11="SMALL_SIDE",$J11+$AL11+$AV11,0))</f>
+        <f>IF($B11="BIG_SIDE",$G11+$J11+$BQ11,IF($B11="SMALL_SIDE",$J11+$AL11+$AV11,0))</f>
         <v/>
       </c>
       <c r="AU11" s="12">
@@ -4723,19 +5300,43 @@
         <v/>
       </c>
       <c r="BL11">
-        <f>IF($D11&gt;0,IFERROR($V11/$D11,0),0)</f>
+        <f>IF($D11&gt;0,IFERROR($BQ11/$D11,0),0)</f>
         <v/>
       </c>
       <c r="BM11">
-        <f>IF($BN11&lt;=0,FALSE,$Y11&gt;=$BN11)</f>
+        <f>$BT11</f>
         <v/>
       </c>
       <c r="BN11">
-        <f>MAX(0,$W11*$BI11*Settings!$B$9)</f>
+        <f>MAX(0,$BR11*$BI11*Settings!$B$9)</f>
         <v/>
       </c>
       <c r="BO11">
         <f>$Y11-$BN11</f>
+        <v/>
+      </c>
+      <c r="BP11">
+        <f>IF($B11="BIG_SIDE",IFERROR($T11/$U11,0),0)</f>
+        <v/>
+      </c>
+      <c r="BQ11">
+        <f>IF($B11="BIG_SIDE",MIN($D11,FLOOR(MAX(0,$BP11),Settings!$B$11)),0)</f>
+        <v/>
+      </c>
+      <c r="BR11">
+        <f>IF($B11="BIG_SIDE",MAX(0,$D11-$BQ11),$AJ11)</f>
+        <v/>
+      </c>
+      <c r="BS11">
+        <f>IF(AND($BP11&gt;0,$BP11&lt;Settings!$B$11),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BT11">
+        <f>IF($Y11&gt;=$BN11,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BU11">
+        <f>MAX(0,$BP11-$BQ11)</f>
         <v/>
       </c>
     </row>
@@ -4776,7 +5377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BO11"/>
+  <dimension ref="A1:BU11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4846,6 +5447,12 @@
     <col width="17" customWidth="1" min="65" max="65"/>
     <col width="15" customWidth="1" min="66" max="66"/>
     <col width="14" customWidth="1" min="67" max="67"/>
+    <col width="16" customWidth="1" min="68" max="68"/>
+    <col width="20" customWidth="1" min="69" max="69"/>
+    <col width="23" customWidth="1" min="70" max="70"/>
+    <col width="25" customWidth="1" min="71" max="71"/>
+    <col width="19" customWidth="1" min="72" max="72"/>
+    <col width="16" customWidth="1" min="73" max="73"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5184,6 +5791,36 @@
           <t>FinalClosePL</t>
         </is>
       </c>
+      <c r="BP1" s="38" t="inlineStr">
+        <is>
+          <t>CloseFarLotRaw</t>
+        </is>
+      </c>
+      <c r="BQ1" s="38" t="inlineStr">
+        <is>
+          <t>CloseFarLotRounded</t>
+        </is>
+      </c>
+      <c r="BR1" s="38" t="inlineStr">
+        <is>
+          <t>FarRemainAfterRounded</t>
+        </is>
+      </c>
+      <c r="BS1" s="38" t="inlineStr">
+        <is>
+          <t>CannotCloseBelowLotStep</t>
+        </is>
+      </c>
+      <c r="BT1" s="38" t="inlineStr">
+        <is>
+          <t>FinalCloseAllowed</t>
+        </is>
+      </c>
+      <c r="BU1" s="38" t="inlineStr">
+        <is>
+          <t>LostToRounding</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="n">
@@ -5273,12 +5910,12 @@
         <v>200</v>
       </c>
       <c r="V2" s="12">
-        <f>IF($B2="BIG_SIDE",IFERROR(MIN($D2,MAX(0,$T2/$U2)),0),0)</f>
-        <v>0.3735</v>
+        <f>$BQ2</f>
+        <v>0.37</v>
       </c>
       <c r="W2" s="12">
-        <f>IF($B2="BIG_SIDE",MAX(0,$D2-$V2),$AJ2)</f>
-        <v>0.6265</v>
+        <f>IF($B2="BIG_SIDE",$BR2,$AJ2)</f>
+        <v>0.63</v>
       </c>
       <c r="X2" s="19">
         <f>IF($B2="BIG_SIDE",IF($AX$2&gt;0,$AX$2*Settings!$B$6,0),IF($S$2&gt;0,$S$2*Settings!$B$6,0))</f>
@@ -5293,7 +5930,7 @@
       </c>
       <c r="AA2" s="12">
         <f>IF($B2="BLOCKED",$Z2+$BF2,IF($B2="BIG_SIDE",$Z2+$S2-$AS2,IF($B2="SMALL_SIDE",$Z2+$S2+$AI2,$Z2+$S2)))</f>
-        <v>8.3</v>
+        <v>9</v>
       </c>
       <c r="AB2" s="12">
         <f>IF($B2="BLOCKED",$BC2,$D2+$G2+$J2)</f>
@@ -5364,11 +6001,11 @@
         <v/>
       </c>
       <c r="AS2" s="20">
-        <f>IF($B2="BIG_SIDE",$V2*$U2,0)</f>
-        <v>74.7</v>
+        <f>IF($B2="BIG_SIDE",$BQ2*$U2,0)</f>
+        <v>74</v>
       </c>
       <c r="AT2" s="12">
-        <f>IF($B2="BIG_SIDE",$G2+$J2+$V2,IF($B2="SMALL_SIDE",$J2+$AL2+$AV2,0))</f>
+        <f>IF($B2="BIG_SIDE",$G2+$J2+$BQ2,IF($B2="SMALL_SIDE",$J2+$AL2+$AV2,0))</f>
         <v/>
       </c>
       <c r="AU2" s="12">
@@ -5438,20 +6075,44 @@
         <v>1</v>
       </c>
       <c r="BL2">
-        <f>IF($D2&gt;0,IFERROR($V2/$D2,0),0)</f>
-        <v>0.3735</v>
+        <f>IF($D2&gt;0,IFERROR($BQ2/$D2,0),0)</f>
+        <v>0.37</v>
       </c>
       <c r="BM2" t="b">
-        <f>IF($BN2&lt;=0,FALSE,$Y2&gt;=$BN2)</f>
+        <f>$BT2</f>
         <v>0</v>
       </c>
       <c r="BN2">
-        <f>MAX(0,$W2*$BI2*Settings!$B$9)</f>
-        <v>125.3</v>
+        <f>MAX(0,$BR2*$BI2*Settings!$B$9)</f>
+        <v>126</v>
       </c>
       <c r="BO2">
         <f>$Y2-$BN2</f>
-        <v>-117</v>
+        <v>-117.7</v>
+      </c>
+      <c r="BP2">
+        <f>IF($B2="BIG_SIDE",IFERROR($T2/$U2,0),0)</f>
+        <v>0.3735</v>
+      </c>
+      <c r="BQ2">
+        <f>IF($B2="BIG_SIDE",MIN($D2,FLOOR(MAX(0,$BP2),Settings!$B$11)),0)</f>
+        <v>0.37</v>
+      </c>
+      <c r="BR2">
+        <f>IF($B2="BIG_SIDE",MAX(0,$D2-$BQ2),$AJ2)</f>
+        <v>0.63</v>
+      </c>
+      <c r="BS2" t="str">
+        <f>IF(AND($BP2&gt;0,$BP2&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT2" t="str">
+        <f>IF($Y2&gt;=$BN2,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU2">
+        <f>MAX(0,$BP2-$BQ2)</f>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="3">
@@ -5539,11 +6200,11 @@
         <v/>
       </c>
       <c r="V3" s="12">
-        <f>IF($B3="BIG_SIDE",IFERROR(MIN($D3,MAX(0,$T3/$U3)),0),0)</f>
+        <f>$BQ3</f>
         <v/>
       </c>
       <c r="W3" s="12">
-        <f>IF($B3="BIG_SIDE",MAX(0,$D3-$V3),$AJ3)</f>
+        <f>IF($B3="BIG_SIDE",$BR3,$AJ3)</f>
         <v/>
       </c>
       <c r="X3" s="19">
@@ -5631,11 +6292,11 @@
         <v/>
       </c>
       <c r="AS3" s="20">
-        <f>IF($B3="BIG_SIDE",$V3*$U3,0)</f>
+        <f>IF($B3="BIG_SIDE",$BQ3*$U3,0)</f>
         <v/>
       </c>
       <c r="AT3" s="12">
-        <f>IF($B3="BIG_SIDE",$G3+$J3+$V3,IF($B3="SMALL_SIDE",$J3+$AL3+$AV3,0))</f>
+        <f>IF($B3="BIG_SIDE",$G3+$J3+$BQ3,IF($B3="SMALL_SIDE",$J3+$AL3+$AV3,0))</f>
         <v/>
       </c>
       <c r="AU3" s="12">
@@ -5705,19 +6366,43 @@
         <v/>
       </c>
       <c r="BL3">
-        <f>IF($D3&gt;0,IFERROR($V3/$D3,0),0)</f>
+        <f>IF($D3&gt;0,IFERROR($BQ3/$D3,0),0)</f>
         <v/>
       </c>
       <c r="BM3">
-        <f>IF($BN3&lt;=0,FALSE,$Y3&gt;=$BN3)</f>
+        <f>$BT3</f>
         <v/>
       </c>
       <c r="BN3">
-        <f>MAX(0,$W3*$BI3*Settings!$B$9)</f>
+        <f>MAX(0,$BR3*$BI3*Settings!$B$9)</f>
         <v/>
       </c>
       <c r="BO3">
         <f>$Y3-$BN3</f>
+        <v/>
+      </c>
+      <c r="BP3">
+        <f>IF($B3="BIG_SIDE",IFERROR($T3/$U3,0),0)</f>
+        <v/>
+      </c>
+      <c r="BQ3">
+        <f>IF($B3="BIG_SIDE",MIN($D3,FLOOR(MAX(0,$BP3),Settings!$B$11)),0)</f>
+        <v/>
+      </c>
+      <c r="BR3">
+        <f>IF($B3="BIG_SIDE",MAX(0,$D3-$BQ3),$AJ3)</f>
+        <v/>
+      </c>
+      <c r="BS3">
+        <f>IF(AND($BP3&gt;0,$BP3&lt;Settings!$B$11),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BT3">
+        <f>IF($Y3&gt;=$BN3,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BU3">
+        <f>MAX(0,$BP3-$BQ3)</f>
         <v/>
       </c>
     </row>
@@ -5806,11 +6491,11 @@
         <v/>
       </c>
       <c r="V4" s="12">
-        <f>IF($B4="BIG_SIDE",IFERROR(MIN($D4,MAX(0,$T4/$U4)),0),0)</f>
+        <f>$BQ4</f>
         <v/>
       </c>
       <c r="W4" s="12">
-        <f>IF($B4="BIG_SIDE",MAX(0,$D4-$V4),$AJ4)</f>
+        <f>IF($B4="BIG_SIDE",$BR4,$AJ4)</f>
         <v/>
       </c>
       <c r="X4" s="19">
@@ -5898,11 +6583,11 @@
         <v/>
       </c>
       <c r="AS4" s="20">
-        <f>IF($B4="BIG_SIDE",$V4*$U4,0)</f>
+        <f>IF($B4="BIG_SIDE",$BQ4*$U4,0)</f>
         <v/>
       </c>
       <c r="AT4" s="12">
-        <f>IF($B4="BIG_SIDE",$G4+$J4+$V4,IF($B4="SMALL_SIDE",$J4+$AL4+$AV4,0))</f>
+        <f>IF($B4="BIG_SIDE",$G4+$J4+$BQ4,IF($B4="SMALL_SIDE",$J4+$AL4+$AV4,0))</f>
         <v/>
       </c>
       <c r="AU4" s="12">
@@ -5972,19 +6657,43 @@
         <v/>
       </c>
       <c r="BL4">
-        <f>IF($D4&gt;0,IFERROR($V4/$D4,0),0)</f>
+        <f>IF($D4&gt;0,IFERROR($BQ4/$D4,0),0)</f>
         <v/>
       </c>
       <c r="BM4">
-        <f>IF($BN4&lt;=0,FALSE,$Y4&gt;=$BN4)</f>
+        <f>$BT4</f>
         <v/>
       </c>
       <c r="BN4">
-        <f>MAX(0,$W4*$BI4*Settings!$B$9)</f>
+        <f>MAX(0,$BR4*$BI4*Settings!$B$9)</f>
         <v/>
       </c>
       <c r="BO4">
         <f>$Y4-$BN4</f>
+        <v/>
+      </c>
+      <c r="BP4">
+        <f>IF($B4="BIG_SIDE",IFERROR($T4/$U4,0),0)</f>
+        <v/>
+      </c>
+      <c r="BQ4">
+        <f>IF($B4="BIG_SIDE",MIN($D4,FLOOR(MAX(0,$BP4),Settings!$B$11)),0)</f>
+        <v/>
+      </c>
+      <c r="BR4">
+        <f>IF($B4="BIG_SIDE",MAX(0,$D4-$BQ4),$AJ4)</f>
+        <v/>
+      </c>
+      <c r="BS4">
+        <f>IF(AND($BP4&gt;0,$BP4&lt;Settings!$B$11),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BT4">
+        <f>IF($Y4&gt;=$BN4,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BU4">
+        <f>MAX(0,$BP4-$BQ4)</f>
         <v/>
       </c>
     </row>
@@ -6073,11 +6782,11 @@
         <v/>
       </c>
       <c r="V5" s="12">
-        <f>IF($B5="BIG_SIDE",IFERROR(MIN($D5,MAX(0,$T5/$U5)),0),0)</f>
+        <f>$BQ5</f>
         <v/>
       </c>
       <c r="W5" s="12">
-        <f>IF($B5="BIG_SIDE",MAX(0,$D5-$V5),$AJ5)</f>
+        <f>IF($B5="BIG_SIDE",$BR5,$AJ5)</f>
         <v/>
       </c>
       <c r="X5" s="19">
@@ -6165,11 +6874,11 @@
         <v>DUAL_TAIL: старый и новый хвост сохранены</v>
       </c>
       <c r="AS5" s="20">
-        <f>IF($B5="BIG_SIDE",$V5*$U5,0)</f>
+        <f>IF($B5="BIG_SIDE",$BQ5*$U5,0)</f>
         <v/>
       </c>
       <c r="AT5" s="12">
-        <f>IF($B5="BIG_SIDE",$G5+$J5+$V5,IF($B5="SMALL_SIDE",$J5+$AL5+$AV5,0))</f>
+        <f>IF($B5="BIG_SIDE",$G5+$J5+$BQ5,IF($B5="SMALL_SIDE",$J5+$AL5+$AV5,0))</f>
         <v/>
       </c>
       <c r="AU5" s="12">
@@ -6239,19 +6948,43 @@
         <v/>
       </c>
       <c r="BL5">
-        <f>IF($D5&gt;0,IFERROR($V5/$D5,0),0)</f>
+        <f>IF($D5&gt;0,IFERROR($BQ5/$D5,0),0)</f>
         <v/>
       </c>
       <c r="BM5">
-        <f>IF($BN5&lt;=0,FALSE,$Y5&gt;=$BN5)</f>
+        <f>$BT5</f>
         <v/>
       </c>
       <c r="BN5">
-        <f>MAX(0,$W5*$BI5*Settings!$B$9)</f>
+        <f>MAX(0,$BR5*$BI5*Settings!$B$9)</f>
         <v/>
       </c>
       <c r="BO5">
         <f>$Y5-$BN5</f>
+        <v/>
+      </c>
+      <c r="BP5">
+        <f>IF($B5="BIG_SIDE",IFERROR($T5/$U5,0),0)</f>
+        <v/>
+      </c>
+      <c r="BQ5">
+        <f>IF($B5="BIG_SIDE",MIN($D5,FLOOR(MAX(0,$BP5),Settings!$B$11)),0)</f>
+        <v/>
+      </c>
+      <c r="BR5">
+        <f>IF($B5="BIG_SIDE",MAX(0,$D5-$BQ5),$AJ5)</f>
+        <v/>
+      </c>
+      <c r="BS5">
+        <f>IF(AND($BP5&gt;0,$BP5&lt;Settings!$B$11),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BT5">
+        <f>IF($Y5&gt;=$BN5,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BU5">
+        <f>MAX(0,$BP5-$BQ5)</f>
         <v/>
       </c>
     </row>
@@ -6340,16 +7073,16 @@
         <v/>
       </c>
       <c r="V6" s="12">
-        <f>IF($B6="BIG_SIDE",IFERROR(MIN($D6,MAX(0,$T6/$U6)),0),0)</f>
+        <f>$BQ6</f>
         <v>0</v>
       </c>
       <c r="W6" s="12">
-        <f>IF($B6="BIG_SIDE",MAX(0,$D6-$V6),$AJ6)</f>
+        <f>IF($B6="BIG_SIDE",$BR6,$AJ6)</f>
         <v/>
       </c>
       <c r="X6" s="19">
         <f>IF($B6="BIG_SIDE",IF($AX$6&gt;0,$AX$6*Settings!$B$6,0),IF($S$6&gt;0,$S$6*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y6" s="19">
         <f>IF(ROW()=2,$X6,$Y5+$X6)</f>
@@ -6432,11 +7165,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS6" s="20">
-        <f>IF($B6="BIG_SIDE",$V6*$U6,0)</f>
+        <f>IF($B6="BIG_SIDE",$BQ6*$U6,0)</f>
         <v>0</v>
       </c>
       <c r="AT6" s="12">
-        <f>IF($B6="BIG_SIDE",$G6+$J6+$V6,IF($B6="SMALL_SIDE",$J6+$AL6+$AV6,0))</f>
+        <f>IF($B6="BIG_SIDE",$G6+$J6+$BQ6,IF($B6="SMALL_SIDE",$J6+$AL6+$AV6,0))</f>
         <v/>
       </c>
       <c r="AU6" s="12">
@@ -6506,21 +7239,45 @@
         <v/>
       </c>
       <c r="BL6">
-        <f>IF($D6&gt;0,IFERROR($V6/$D6,0),0)</f>
+        <f>IF($D6&gt;0,IFERROR($BQ6/$D6,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM6" t="b">
-        <f>IF($BN6&lt;=0,FALSE,$Y6&gt;=$BN6)</f>
+        <f>$BT6</f>
         <v>0</v>
       </c>
       <c r="BN6">
-        <f>MAX(0,$W6*$BI6*Settings!$B$9)</f>
+        <f>MAX(0,$BR6*$BI6*Settings!$B$9)</f>
         <v>197.92</v>
       </c>
       <c r="BO6">
         <f>$Y6-$BN6</f>
         <v>-197.92</v>
       </c>
+      <c r="BP6">
+        <f>IF($B6="BIG_SIDE",IFERROR($T6/$U6,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ6">
+        <f>IF($B6="BIG_SIDE",MIN($D6,FLOOR(MAX(0,$BP6),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR6">
+        <f>IF($B6="BIG_SIDE",MAX(0,$D6-$BQ6),$AJ6)</f>
+        <v>0.9896</v>
+      </c>
+      <c r="BS6" t="str">
+        <f>IF(AND($BP6&gt;0,$BP6&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT6" t="str">
+        <f>IF($Y6&gt;=$BN6,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU6">
+        <f>MAX(0,$BP6-$BQ6)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="n">
@@ -6607,16 +7364,16 @@
         <v/>
       </c>
       <c r="V7" s="12">
-        <f>IF($B7="BIG_SIDE",IFERROR(MIN($D7,MAX(0,$T7/$U7)),0),0)</f>
+        <f>$BQ7</f>
         <v>0</v>
       </c>
       <c r="W7" s="12">
-        <f>IF($B7="BIG_SIDE",MAX(0,$D7-$V7),$AJ7)</f>
+        <f>IF($B7="BIG_SIDE",$BR7,$AJ7)</f>
         <v/>
       </c>
       <c r="X7" s="19">
         <f>IF($B7="BIG_SIDE",IF($AX$7&gt;0,$AX$7*Settings!$B$6,0),IF($S$7&gt;0,$S$7*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y7" s="19">
         <f>IF(ROW()=2,$X7,$Y6+$X7)</f>
@@ -6699,11 +7456,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS7" s="20">
-        <f>IF($B7="BIG_SIDE",$V7*$U7,0)</f>
+        <f>IF($B7="BIG_SIDE",$BQ7*$U7,0)</f>
         <v>0</v>
       </c>
       <c r="AT7" s="12">
-        <f>IF($B7="BIG_SIDE",$G7+$J7+$V7,IF($B7="SMALL_SIDE",$J7+$AL7+$AV7,0))</f>
+        <f>IF($B7="BIG_SIDE",$G7+$J7+$BQ7,IF($B7="SMALL_SIDE",$J7+$AL7+$AV7,0))</f>
         <v/>
       </c>
       <c r="AU7" s="12">
@@ -6773,21 +7530,45 @@
         <v/>
       </c>
       <c r="BL7">
-        <f>IF($D7&gt;0,IFERROR($V7/$D7,0),0)</f>
+        <f>IF($D7&gt;0,IFERROR($BQ7/$D7,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM7" t="b">
-        <f>IF($BN7&lt;=0,FALSE,$Y7&gt;=$BN7)</f>
+        <f>$BT7</f>
         <v>0</v>
       </c>
       <c r="BN7">
-        <f>MAX(0,$W7*$BI7*Settings!$B$9)</f>
+        <f>MAX(0,$BR7*$BI7*Settings!$B$9)</f>
         <v>197.92</v>
       </c>
       <c r="BO7">
         <f>$Y7-$BN7</f>
         <v>-197.92</v>
       </c>
+      <c r="BP7">
+        <f>IF($B7="BIG_SIDE",IFERROR($T7/$U7,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ7">
+        <f>IF($B7="BIG_SIDE",MIN($D7,FLOOR(MAX(0,$BP7),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR7">
+        <f>IF($B7="BIG_SIDE",MAX(0,$D7-$BQ7),$AJ7)</f>
+        <v>0.9896</v>
+      </c>
+      <c r="BS7" t="str">
+        <f>IF(AND($BP7&gt;0,$BP7&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT7" t="str">
+        <f>IF($Y7&gt;=$BN7,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU7">
+        <f>MAX(0,$BP7-$BQ7)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="n">
@@ -6874,16 +7655,16 @@
         <v/>
       </c>
       <c r="V8" s="12">
-        <f>IF($B8="BIG_SIDE",IFERROR(MIN($D8,MAX(0,$T8/$U8)),0),0)</f>
+        <f>$BQ8</f>
         <v>0</v>
       </c>
       <c r="W8" s="12">
-        <f>IF($B8="BIG_SIDE",MAX(0,$D8-$V8),$AJ8)</f>
+        <f>IF($B8="BIG_SIDE",$BR8,$AJ8)</f>
         <v/>
       </c>
       <c r="X8" s="19">
         <f>IF($B8="BIG_SIDE",IF($AX$8&gt;0,$AX$8*Settings!$B$6,0),IF($S$8&gt;0,$S$8*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y8" s="19">
         <f>IF(ROW()=2,$X8,$Y7+$X8)</f>
@@ -6966,11 +7747,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS8" s="20">
-        <f>IF($B8="BIG_SIDE",$V8*$U8,0)</f>
+        <f>IF($B8="BIG_SIDE",$BQ8*$U8,0)</f>
         <v>0</v>
       </c>
       <c r="AT8" s="12">
-        <f>IF($B8="BIG_SIDE",$G8+$J8+$V8,IF($B8="SMALL_SIDE",$J8+$AL8+$AV8,0))</f>
+        <f>IF($B8="BIG_SIDE",$G8+$J8+$BQ8,IF($B8="SMALL_SIDE",$J8+$AL8+$AV8,0))</f>
         <v/>
       </c>
       <c r="AU8" s="12">
@@ -7040,21 +7821,45 @@
         <v/>
       </c>
       <c r="BL8">
-        <f>IF($D8&gt;0,IFERROR($V8/$D8,0),0)</f>
+        <f>IF($D8&gt;0,IFERROR($BQ8/$D8,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM8" t="b">
-        <f>IF($BN8&lt;=0,FALSE,$Y8&gt;=$BN8)</f>
+        <f>$BT8</f>
         <v>0</v>
       </c>
       <c r="BN8">
-        <f>MAX(0,$W8*$BI8*Settings!$B$9)</f>
+        <f>MAX(0,$BR8*$BI8*Settings!$B$9)</f>
         <v>197.92</v>
       </c>
       <c r="BO8">
         <f>$Y8-$BN8</f>
         <v>-197.92</v>
       </c>
+      <c r="BP8">
+        <f>IF($B8="BIG_SIDE",IFERROR($T8/$U8,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ8">
+        <f>IF($B8="BIG_SIDE",MIN($D8,FLOOR(MAX(0,$BP8),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR8">
+        <f>IF($B8="BIG_SIDE",MAX(0,$D8-$BQ8),$AJ8)</f>
+        <v>0.9896</v>
+      </c>
+      <c r="BS8" t="str">
+        <f>IF(AND($BP8&gt;0,$BP8&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT8" t="str">
+        <f>IF($Y8&gt;=$BN8,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU8">
+        <f>MAX(0,$BP8-$BQ8)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="n">
@@ -7141,16 +7946,16 @@
         <v/>
       </c>
       <c r="V9" s="12">
-        <f>IF($B9="BIG_SIDE",IFERROR(MIN($D9,MAX(0,$T9/$U9)),0),0)</f>
+        <f>$BQ9</f>
         <v>0</v>
       </c>
       <c r="W9" s="12">
-        <f>IF($B9="BIG_SIDE",MAX(0,$D9-$V9),$AJ9)</f>
+        <f>IF($B9="BIG_SIDE",$BR9,$AJ9)</f>
         <v/>
       </c>
       <c r="X9" s="19">
         <f>IF($B9="BIG_SIDE",IF($AX$9&gt;0,$AX$9*Settings!$B$6,0),IF($S$9&gt;0,$S$9*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y9" s="19">
         <f>IF(ROW()=2,$X9,$Y8+$X9)</f>
@@ -7233,11 +8038,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS9" s="20">
-        <f>IF($B9="BIG_SIDE",$V9*$U9,0)</f>
+        <f>IF($B9="BIG_SIDE",$BQ9*$U9,0)</f>
         <v>0</v>
       </c>
       <c r="AT9" s="12">
-        <f>IF($B9="BIG_SIDE",$G9+$J9+$V9,IF($B9="SMALL_SIDE",$J9+$AL9+$AV9,0))</f>
+        <f>IF($B9="BIG_SIDE",$G9+$J9+$BQ9,IF($B9="SMALL_SIDE",$J9+$AL9+$AV9,0))</f>
         <v/>
       </c>
       <c r="AU9" s="12">
@@ -7307,21 +8112,45 @@
         <v/>
       </c>
       <c r="BL9">
-        <f>IF($D9&gt;0,IFERROR($V9/$D9,0),0)</f>
+        <f>IF($D9&gt;0,IFERROR($BQ9/$D9,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM9" t="b">
-        <f>IF($BN9&lt;=0,FALSE,$Y9&gt;=$BN9)</f>
+        <f>$BT9</f>
         <v>0</v>
       </c>
       <c r="BN9">
-        <f>MAX(0,$W9*$BI9*Settings!$B$9)</f>
+        <f>MAX(0,$BR9*$BI9*Settings!$B$9)</f>
         <v>197.92</v>
       </c>
       <c r="BO9">
         <f>$Y9-$BN9</f>
         <v>-197.92</v>
       </c>
+      <c r="BP9">
+        <f>IF($B9="BIG_SIDE",IFERROR($T9/$U9,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ9">
+        <f>IF($B9="BIG_SIDE",MIN($D9,FLOOR(MAX(0,$BP9),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR9">
+        <f>IF($B9="BIG_SIDE",MAX(0,$D9-$BQ9),$AJ9)</f>
+        <v>0.9896</v>
+      </c>
+      <c r="BS9" t="str">
+        <f>IF(AND($BP9&gt;0,$BP9&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT9" t="str">
+        <f>IF($Y9&gt;=$BN9,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU9">
+        <f>MAX(0,$BP9-$BQ9)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="n">
@@ -7337,7 +8166,7 @@
       </c>
       <c r="D10" s="13">
         <f>IF($B10="BLOCKED",0,IF(AND($AQ9="MANUAL_READY",$BG9="YES"),MAX($BA9,$BB9),IF($AP9="YES",MAX(0,$AG9),$D9)))</f>
-        <v/>
+        <v>0.1</v>
       </c>
       <c r="E10" s="12">
         <f>IF($B10="BLOCKED","",IF($C10="SELL","BUY","SELL"))</f>
@@ -7408,16 +8237,16 @@
         <v/>
       </c>
       <c r="V10" s="12">
-        <f>IF($B10="BIG_SIDE",IFERROR(MIN($D10,MAX(0,$T10/$U10)),0),0)</f>
+        <f>$BQ10</f>
         <v>0</v>
       </c>
       <c r="W10" s="12">
-        <f>IF($B10="BIG_SIDE",MAX(0,$D10-$V10),$AJ10)</f>
+        <f>IF($B10="BIG_SIDE",$BR10,$AJ10)</f>
         <v/>
       </c>
       <c r="X10" s="19">
         <f>IF($B10="BIG_SIDE",IF($AX$10&gt;0,$AX$10*Settings!$B$6,0),IF($S$10&gt;0,$S$10*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y10" s="19">
         <f>IF(ROW()=2,$X10,$Y9+$X10)</f>
@@ -7500,11 +8329,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS10" s="20">
-        <f>IF($B10="BIG_SIDE",$V10*$U10,0)</f>
+        <f>IF($B10="BIG_SIDE",$BQ10*$U10,0)</f>
         <v>0</v>
       </c>
       <c r="AT10" s="12">
-        <f>IF($B10="BIG_SIDE",$G10+$J10+$V10,IF($B10="SMALL_SIDE",$J10+$AL10+$AV10,0))</f>
+        <f>IF($B10="BIG_SIDE",$G10+$J10+$BQ10,IF($B10="SMALL_SIDE",$J10+$AL10+$AV10,0))</f>
         <v/>
       </c>
       <c r="AU10" s="12">
@@ -7574,21 +8403,45 @@
         <v/>
       </c>
       <c r="BL10">
-        <f>IF($D10&gt;0,IFERROR($V10/$D10,0),0)</f>
+        <f>IF($D10&gt;0,IFERROR($BQ10/$D10,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM10" t="b">
-        <f>IF($BN10&lt;=0,FALSE,$Y10&gt;=$BN10)</f>
+        <f>$BT10</f>
         <v>0</v>
       </c>
       <c r="BN10">
-        <f>MAX(0,$W10*$BI10*Settings!$B$9)</f>
+        <f>MAX(0,$BR10*$BI10*Settings!$B$9)</f>
         <v>197.92</v>
       </c>
       <c r="BO10">
         <f>$Y10-$BN10</f>
         <v>-197.92</v>
       </c>
+      <c r="BP10">
+        <f>IF($B10="BIG_SIDE",IFERROR($T10/$U10,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ10">
+        <f>IF($B10="BIG_SIDE",MIN($D10,FLOOR(MAX(0,$BP10),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR10">
+        <f>IF($B10="BIG_SIDE",MAX(0,$D10-$BQ10),$AJ10)</f>
+        <v>0.9896</v>
+      </c>
+      <c r="BS10" t="str">
+        <f>IF(AND($BP10&gt;0,$BP10&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT10" t="str">
+        <f>IF($Y10&gt;=$BN10,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU10">
+        <f>MAX(0,$BP10-$BQ10)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="n">
@@ -7675,16 +8528,16 @@
         <v/>
       </c>
       <c r="V11" s="12">
-        <f>IF($B11="BIG_SIDE",IFERROR(MIN($D11,MAX(0,$T11/$U11)),0),0)</f>
+        <f>$BQ11</f>
         <v>0</v>
       </c>
       <c r="W11" s="12">
-        <f>IF($B11="BIG_SIDE",MAX(0,$D11-$V11),$AJ11)</f>
+        <f>IF($B11="BIG_SIDE",$BR11,$AJ11)</f>
         <v/>
       </c>
       <c r="X11" s="19">
         <f>IF($B11="BIG_SIDE",IF($AX$11&gt;0,$AX$11*Settings!$B$6,0),IF($S$11&gt;0,$S$11*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y11" s="19">
         <f>IF(ROW()=2,$X11,$Y10+$X11)</f>
@@ -7767,11 +8620,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS11" s="20">
-        <f>IF($B11="BIG_SIDE",$V11*$U11,0)</f>
+        <f>IF($B11="BIG_SIDE",$BQ11*$U11,0)</f>
         <v>0</v>
       </c>
       <c r="AT11" s="12">
-        <f>IF($B11="BIG_SIDE",$G11+$J11+$V11,IF($B11="SMALL_SIDE",$J11+$AL11+$AV11,0))</f>
+        <f>IF($B11="BIG_SIDE",$G11+$J11+$BQ11,IF($B11="SMALL_SIDE",$J11+$AL11+$AV11,0))</f>
         <v/>
       </c>
       <c r="AU11" s="12">
@@ -7841,20 +8694,44 @@
         <v/>
       </c>
       <c r="BL11">
-        <f>IF($D11&gt;0,IFERROR($V11/$D11,0),0)</f>
+        <f>IF($D11&gt;0,IFERROR($BQ11/$D11,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM11" t="b">
-        <f>IF($BN11&lt;=0,FALSE,$Y11&gt;=$BN11)</f>
+        <f>$BT11</f>
         <v>0</v>
       </c>
       <c r="BN11">
-        <f>MAX(0,$W11*$BI11*Settings!$B$9)</f>
+        <f>MAX(0,$BR11*$BI11*Settings!$B$9)</f>
         <v>197.92</v>
       </c>
       <c r="BO11">
         <f>$Y11-$BN11</f>
         <v>-197.92</v>
+      </c>
+      <c r="BP11">
+        <f>IF($B11="BIG_SIDE",IFERROR($T11/$U11,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ11">
+        <f>IF($B11="BIG_SIDE",MIN($D11,FLOOR(MAX(0,$BP11),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR11">
+        <f>IF($B11="BIG_SIDE",MAX(0,$D11-$BQ11),$AJ11)</f>
+        <v>0.9896</v>
+      </c>
+      <c r="BS11" t="str">
+        <f>IF(AND($BP11&gt;0,$BP11&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT11" t="str">
+        <f>IF($Y11&gt;=$BN11,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU11">
+        <f>MAX(0,$BP11-$BQ11)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -7894,7 +8771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BO11"/>
+  <dimension ref="A1:BU11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7964,6 +8841,12 @@
     <col width="17" customWidth="1" min="65" max="65"/>
     <col width="15" customWidth="1" min="66" max="66"/>
     <col width="14" customWidth="1" min="67" max="67"/>
+    <col width="16" customWidth="1" min="68" max="68"/>
+    <col width="20" customWidth="1" min="69" max="69"/>
+    <col width="23" customWidth="1" min="70" max="70"/>
+    <col width="25" customWidth="1" min="71" max="71"/>
+    <col width="19" customWidth="1" min="72" max="72"/>
+    <col width="16" customWidth="1" min="73" max="73"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8302,6 +9185,36 @@
           <t>FinalClosePL</t>
         </is>
       </c>
+      <c r="BP1" s="38" t="inlineStr">
+        <is>
+          <t>CloseFarLotRaw</t>
+        </is>
+      </c>
+      <c r="BQ1" s="38" t="inlineStr">
+        <is>
+          <t>CloseFarLotRounded</t>
+        </is>
+      </c>
+      <c r="BR1" s="38" t="inlineStr">
+        <is>
+          <t>FarRemainAfterRounded</t>
+        </is>
+      </c>
+      <c r="BS1" s="38" t="inlineStr">
+        <is>
+          <t>CannotCloseBelowLotStep</t>
+        </is>
+      </c>
+      <c r="BT1" s="38" t="inlineStr">
+        <is>
+          <t>FinalCloseAllowed</t>
+        </is>
+      </c>
+      <c r="BU1" s="38" t="inlineStr">
+        <is>
+          <t>LostToRounding</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="n">
@@ -8391,12 +9304,12 @@
         <v>200</v>
       </c>
       <c r="V2" s="12">
-        <f>IF($B2="BIG_SIDE",IFERROR(MIN($D2,MAX(0,$T2/$U2)),0),0)</f>
-        <v>0.3735</v>
+        <f>$BQ2</f>
+        <v>0.37</v>
       </c>
       <c r="W2" s="12">
-        <f>IF($B2="BIG_SIDE",MAX(0,$D2-$V2),$AJ2)</f>
-        <v>0.6265</v>
+        <f>IF($B2="BIG_SIDE",$BR2,$AJ2)</f>
+        <v>0.63</v>
       </c>
       <c r="X2" s="19">
         <f>IF($B2="BIG_SIDE",IF($AX$2&gt;0,$AX$2*Settings!$B$6,0),IF($S$2&gt;0,$S$2*Settings!$B$6,0))</f>
@@ -8411,7 +9324,7 @@
       </c>
       <c r="AA2" s="12">
         <f>IF($B2="BLOCKED",$Z2+$BF2,IF($B2="BIG_SIDE",$Z2+$S2-$AS2,IF($B2="SMALL_SIDE",$Z2+$S2+$AI2,$Z2+$S2)))</f>
-        <v>8.3</v>
+        <v>9</v>
       </c>
       <c r="AB2" s="12">
         <f>IF($B2="BLOCKED",$BC2,$D2+$G2+$J2)</f>
@@ -8482,11 +9395,11 @@
         <v/>
       </c>
       <c r="AS2" s="20">
-        <f>IF($B2="BIG_SIDE",$V2*$U2,0)</f>
-        <v>74.7</v>
+        <f>IF($B2="BIG_SIDE",$BQ2*$U2,0)</f>
+        <v>74</v>
       </c>
       <c r="AT2" s="12">
-        <f>IF($B2="BIG_SIDE",$G2+$J2+$V2,IF($B2="SMALL_SIDE",$J2+$AL2+$AV2,0))</f>
+        <f>IF($B2="BIG_SIDE",$G2+$J2+$BQ2,IF($B2="SMALL_SIDE",$J2+$AL2+$AV2,0))</f>
         <v/>
       </c>
       <c r="AU2" s="12">
@@ -8556,20 +9469,44 @@
         <v>1</v>
       </c>
       <c r="BL2">
-        <f>IF($D2&gt;0,IFERROR($V2/$D2,0),0)</f>
-        <v>0.3735</v>
+        <f>IF($D2&gt;0,IFERROR($BQ2/$D2,0),0)</f>
+        <v>0.37</v>
       </c>
       <c r="BM2" t="b">
-        <f>IF($BN2&lt;=0,FALSE,$Y2&gt;=$BN2)</f>
+        <f>$BT2</f>
         <v>0</v>
       </c>
       <c r="BN2">
-        <f>MAX(0,$W2*$BI2*Settings!$B$9)</f>
-        <v>125.3</v>
+        <f>MAX(0,$BR2*$BI2*Settings!$B$9)</f>
+        <v>126</v>
       </c>
       <c r="BO2">
         <f>$Y2-$BN2</f>
-        <v>-117</v>
+        <v>-117.7</v>
+      </c>
+      <c r="BP2">
+        <f>IF($B2="BIG_SIDE",IFERROR($T2/$U2,0),0)</f>
+        <v>0.3735</v>
+      </c>
+      <c r="BQ2">
+        <f>IF($B2="BIG_SIDE",MIN($D2,FLOOR(MAX(0,$BP2),Settings!$B$11)),0)</f>
+        <v>0.37</v>
+      </c>
+      <c r="BR2">
+        <f>IF($B2="BIG_SIDE",MAX(0,$D2-$BQ2),$AJ2)</f>
+        <v>0.63</v>
+      </c>
+      <c r="BS2" t="str">
+        <f>IF(AND($BP2&gt;0,$BP2&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT2" t="str">
+        <f>IF($Y2&gt;=$BN2,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU2">
+        <f>MAX(0,$BP2-$BQ2)</f>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="3">
@@ -8657,11 +9594,11 @@
         <v/>
       </c>
       <c r="V3" s="12">
-        <f>IF($B3="BIG_SIDE",IFERROR(MIN($D3,MAX(0,$T3/$U3)),0),0)</f>
+        <f>$BQ3</f>
         <v/>
       </c>
       <c r="W3" s="12">
-        <f>IF($B3="BIG_SIDE",MAX(0,$D3-$V3),$AJ3)</f>
+        <f>IF($B3="BIG_SIDE",$BR3,$AJ3)</f>
         <v/>
       </c>
       <c r="X3" s="19">
@@ -8749,11 +9686,11 @@
         <v>DUAL_TAIL: старый и новый хвост сохранены</v>
       </c>
       <c r="AS3" s="20">
-        <f>IF($B3="BIG_SIDE",$V3*$U3,0)</f>
+        <f>IF($B3="BIG_SIDE",$BQ3*$U3,0)</f>
         <v/>
       </c>
       <c r="AT3" s="12">
-        <f>IF($B3="BIG_SIDE",$G3+$J3+$V3,IF($B3="SMALL_SIDE",$J3+$AL3+$AV3,0))</f>
+        <f>IF($B3="BIG_SIDE",$G3+$J3+$BQ3,IF($B3="SMALL_SIDE",$J3+$AL3+$AV3,0))</f>
         <v/>
       </c>
       <c r="AU3" s="12">
@@ -8823,19 +9760,43 @@
         <v/>
       </c>
       <c r="BL3">
-        <f>IF($D3&gt;0,IFERROR($V3/$D3,0),0)</f>
+        <f>IF($D3&gt;0,IFERROR($BQ3/$D3,0),0)</f>
         <v/>
       </c>
       <c r="BM3">
-        <f>IF($BN3&lt;=0,FALSE,$Y3&gt;=$BN3)</f>
+        <f>$BT3</f>
         <v/>
       </c>
       <c r="BN3">
-        <f>MAX(0,$W3*$BI3*Settings!$B$9)</f>
+        <f>MAX(0,$BR3*$BI3*Settings!$B$9)</f>
         <v/>
       </c>
       <c r="BO3">
         <f>$Y3-$BN3</f>
+        <v/>
+      </c>
+      <c r="BP3">
+        <f>IF($B3="BIG_SIDE",IFERROR($T3/$U3,0),0)</f>
+        <v/>
+      </c>
+      <c r="BQ3">
+        <f>IF($B3="BIG_SIDE",MIN($D3,FLOOR(MAX(0,$BP3),Settings!$B$11)),0)</f>
+        <v/>
+      </c>
+      <c r="BR3">
+        <f>IF($B3="BIG_SIDE",MAX(0,$D3-$BQ3),$AJ3)</f>
+        <v/>
+      </c>
+      <c r="BS3">
+        <f>IF(AND($BP3&gt;0,$BP3&lt;Settings!$B$11),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BT3">
+        <f>IF($Y3&gt;=$BN3,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="BU3">
+        <f>MAX(0,$BP3-$BQ3)</f>
         <v/>
       </c>
     </row>
@@ -8924,16 +9885,16 @@
         <v/>
       </c>
       <c r="V4" s="12">
-        <f>IF($B4="BIG_SIDE",IFERROR(MIN($D4,MAX(0,$T4/$U4)),0),0)</f>
+        <f>$BQ4</f>
         <v>0</v>
       </c>
       <c r="W4" s="12">
-        <f>IF($B4="BIG_SIDE",MAX(0,$D4-$V4),$AJ4)</f>
+        <f>IF($B4="BIG_SIDE",$BR4,$AJ4)</f>
         <v/>
       </c>
       <c r="X4" s="19">
         <f>IF($B4="BIG_SIDE",IF($AX$4&gt;0,$AX$4*Settings!$B$6,0),IF($S$4&gt;0,$S$4*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y4" s="19">
         <f>IF(ROW()=2,$X4,$Y3+$X4)</f>
@@ -9016,11 +9977,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS4" s="20">
-        <f>IF($B4="BIG_SIDE",$V4*$U4,0)</f>
+        <f>IF($B4="BIG_SIDE",$BQ4*$U4,0)</f>
         <v>0</v>
       </c>
       <c r="AT4" s="12">
-        <f>IF($B4="BIG_SIDE",$G4+$J4+$V4,IF($B4="SMALL_SIDE",$J4+$AL4+$AV4,0))</f>
+        <f>IF($B4="BIG_SIDE",$G4+$J4+$BQ4,IF($B4="SMALL_SIDE",$J4+$AL4+$AV4,0))</f>
         <v/>
       </c>
       <c r="AU4" s="12">
@@ -9090,21 +10051,45 @@
         <v/>
       </c>
       <c r="BL4">
-        <f>IF($D4&gt;0,IFERROR($V4/$D4,0),0)</f>
+        <f>IF($D4&gt;0,IFERROR($BQ4/$D4,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM4" t="b">
-        <f>IF($BN4&lt;=0,FALSE,$Y4&gt;=$BN4)</f>
+        <f>$BT4</f>
         <v>0</v>
       </c>
       <c r="BN4">
-        <f>MAX(0,$W4*$BI4*Settings!$B$9)</f>
+        <f>MAX(0,$BR4*$BI4*Settings!$B$9)</f>
         <v>306.12</v>
       </c>
       <c r="BO4">
         <f>$Y4-$BN4</f>
         <v>-306.12</v>
       </c>
+      <c r="BP4">
+        <f>IF($B4="BIG_SIDE",IFERROR($T4/$U4,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ4">
+        <f>IF($B4="BIG_SIDE",MIN($D4,FLOOR(MAX(0,$BP4),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR4">
+        <f>IF($B4="BIG_SIDE",MAX(0,$D4-$BQ4),$AJ4)</f>
+        <v>1.5306</v>
+      </c>
+      <c r="BS4" t="str">
+        <f>IF(AND($BP4&gt;0,$BP4&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT4" t="str">
+        <f>IF($Y4&gt;=$BN4,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU4">
+        <f>MAX(0,$BP4-$BQ4)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="n">
@@ -9191,16 +10176,16 @@
         <v/>
       </c>
       <c r="V5" s="12">
-        <f>IF($B5="BIG_SIDE",IFERROR(MIN($D5,MAX(0,$T5/$U5)),0),0)</f>
+        <f>$BQ5</f>
         <v>0</v>
       </c>
       <c r="W5" s="12">
-        <f>IF($B5="BIG_SIDE",MAX(0,$D5-$V5),$AJ5)</f>
+        <f>IF($B5="BIG_SIDE",$BR5,$AJ5)</f>
         <v/>
       </c>
       <c r="X5" s="19">
         <f>IF($B5="BIG_SIDE",IF($AX$5&gt;0,$AX$5*Settings!$B$6,0),IF($S$5&gt;0,$S$5*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y5" s="19">
         <f>IF(ROW()=2,$X5,$Y4+$X5)</f>
@@ -9283,11 +10268,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS5" s="20">
-        <f>IF($B5="BIG_SIDE",$V5*$U5,0)</f>
+        <f>IF($B5="BIG_SIDE",$BQ5*$U5,0)</f>
         <v>0</v>
       </c>
       <c r="AT5" s="12">
-        <f>IF($B5="BIG_SIDE",$G5+$J5+$V5,IF($B5="SMALL_SIDE",$J5+$AL5+$AV5,0))</f>
+        <f>IF($B5="BIG_SIDE",$G5+$J5+$BQ5,IF($B5="SMALL_SIDE",$J5+$AL5+$AV5,0))</f>
         <v/>
       </c>
       <c r="AU5" s="12">
@@ -9357,21 +10342,45 @@
         <v/>
       </c>
       <c r="BL5">
-        <f>IF($D5&gt;0,IFERROR($V5/$D5,0),0)</f>
+        <f>IF($D5&gt;0,IFERROR($BQ5/$D5,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM5" t="b">
-        <f>IF($BN5&lt;=0,FALSE,$Y5&gt;=$BN5)</f>
+        <f>$BT5</f>
         <v>0</v>
       </c>
       <c r="BN5">
-        <f>MAX(0,$W5*$BI5*Settings!$B$9)</f>
+        <f>MAX(0,$BR5*$BI5*Settings!$B$9)</f>
         <v>306.12</v>
       </c>
       <c r="BO5">
         <f>$Y5-$BN5</f>
         <v>-306.12</v>
       </c>
+      <c r="BP5">
+        <f>IF($B5="BIG_SIDE",IFERROR($T5/$U5,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ5">
+        <f>IF($B5="BIG_SIDE",MIN($D5,FLOOR(MAX(0,$BP5),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR5">
+        <f>IF($B5="BIG_SIDE",MAX(0,$D5-$BQ5),$AJ5)</f>
+        <v>1.5306</v>
+      </c>
+      <c r="BS5" t="str">
+        <f>IF(AND($BP5&gt;0,$BP5&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT5" t="str">
+        <f>IF($Y5&gt;=$BN5,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU5">
+        <f>MAX(0,$BP5-$BQ5)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="n">
@@ -9458,16 +10467,16 @@
         <v/>
       </c>
       <c r="V6" s="12">
-        <f>IF($B6="BIG_SIDE",IFERROR(MIN($D6,MAX(0,$T6/$U6)),0),0)</f>
+        <f>$BQ6</f>
         <v>0</v>
       </c>
       <c r="W6" s="12">
-        <f>IF($B6="BIG_SIDE",MAX(0,$D6-$V6),$AJ6)</f>
+        <f>IF($B6="BIG_SIDE",$BR6,$AJ6)</f>
         <v/>
       </c>
       <c r="X6" s="19">
         <f>IF($B6="BIG_SIDE",IF($AX$6&gt;0,$AX$6*Settings!$B$6,0),IF($S$6&gt;0,$S$6*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y6" s="19">
         <f>IF(ROW()=2,$X6,$Y5+$X6)</f>
@@ -9550,11 +10559,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS6" s="20">
-        <f>IF($B6="BIG_SIDE",$V6*$U6,0)</f>
+        <f>IF($B6="BIG_SIDE",$BQ6*$U6,0)</f>
         <v>0</v>
       </c>
       <c r="AT6" s="12">
-        <f>IF($B6="BIG_SIDE",$G6+$J6+$V6,IF($B6="SMALL_SIDE",$J6+$AL6+$AV6,0))</f>
+        <f>IF($B6="BIG_SIDE",$G6+$J6+$BQ6,IF($B6="SMALL_SIDE",$J6+$AL6+$AV6,0))</f>
         <v/>
       </c>
       <c r="AU6" s="12">
@@ -9624,21 +10633,45 @@
         <v/>
       </c>
       <c r="BL6">
-        <f>IF($D6&gt;0,IFERROR($V6/$D6,0),0)</f>
+        <f>IF($D6&gt;0,IFERROR($BQ6/$D6,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM6" t="b">
-        <f>IF($BN6&lt;=0,FALSE,$Y6&gt;=$BN6)</f>
+        <f>$BT6</f>
         <v>0</v>
       </c>
       <c r="BN6">
-        <f>MAX(0,$W6*$BI6*Settings!$B$9)</f>
+        <f>MAX(0,$BR6*$BI6*Settings!$B$9)</f>
         <v>306.12</v>
       </c>
       <c r="BO6">
         <f>$Y6-$BN6</f>
         <v>-306.12</v>
       </c>
+      <c r="BP6">
+        <f>IF($B6="BIG_SIDE",IFERROR($T6/$U6,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ6">
+        <f>IF($B6="BIG_SIDE",MIN($D6,FLOOR(MAX(0,$BP6),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR6">
+        <f>IF($B6="BIG_SIDE",MAX(0,$D6-$BQ6),$AJ6)</f>
+        <v>1.5306</v>
+      </c>
+      <c r="BS6" t="str">
+        <f>IF(AND($BP6&gt;0,$BP6&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT6" t="str">
+        <f>IF($Y6&gt;=$BN6,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU6">
+        <f>MAX(0,$BP6-$BQ6)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="n">
@@ -9725,16 +10758,16 @@
         <v/>
       </c>
       <c r="V7" s="12">
-        <f>IF($B7="BIG_SIDE",IFERROR(MIN($D7,MAX(0,$T7/$U7)),0),0)</f>
+        <f>$BQ7</f>
         <v>0</v>
       </c>
       <c r="W7" s="12">
-        <f>IF($B7="BIG_SIDE",MAX(0,$D7-$V7),$AJ7)</f>
+        <f>IF($B7="BIG_SIDE",$BR7,$AJ7)</f>
         <v/>
       </c>
       <c r="X7" s="19">
         <f>IF($B7="BIG_SIDE",IF($AX$7&gt;0,$AX$7*Settings!$B$6,0),IF($S$7&gt;0,$S$7*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y7" s="19">
         <f>IF(ROW()=2,$X7,$Y6+$X7)</f>
@@ -9817,11 +10850,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS7" s="20">
-        <f>IF($B7="BIG_SIDE",$V7*$U7,0)</f>
+        <f>IF($B7="BIG_SIDE",$BQ7*$U7,0)</f>
         <v>0</v>
       </c>
       <c r="AT7" s="12">
-        <f>IF($B7="BIG_SIDE",$G7+$J7+$V7,IF($B7="SMALL_SIDE",$J7+$AL7+$AV7,0))</f>
+        <f>IF($B7="BIG_SIDE",$G7+$J7+$BQ7,IF($B7="SMALL_SIDE",$J7+$AL7+$AV7,0))</f>
         <v/>
       </c>
       <c r="AU7" s="12">
@@ -9891,21 +10924,45 @@
         <v/>
       </c>
       <c r="BL7">
-        <f>IF($D7&gt;0,IFERROR($V7/$D7,0),0)</f>
+        <f>IF($D7&gt;0,IFERROR($BQ7/$D7,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM7" t="b">
-        <f>IF($BN7&lt;=0,FALSE,$Y7&gt;=$BN7)</f>
+        <f>$BT7</f>
         <v>0</v>
       </c>
       <c r="BN7">
-        <f>MAX(0,$W7*$BI7*Settings!$B$9)</f>
+        <f>MAX(0,$BR7*$BI7*Settings!$B$9)</f>
         <v>306.12</v>
       </c>
       <c r="BO7">
         <f>$Y7-$BN7</f>
         <v>-306.12</v>
       </c>
+      <c r="BP7">
+        <f>IF($B7="BIG_SIDE",IFERROR($T7/$U7,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ7">
+        <f>IF($B7="BIG_SIDE",MIN($D7,FLOOR(MAX(0,$BP7),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR7">
+        <f>IF($B7="BIG_SIDE",MAX(0,$D7-$BQ7),$AJ7)</f>
+        <v>1.5306</v>
+      </c>
+      <c r="BS7" t="str">
+        <f>IF(AND($BP7&gt;0,$BP7&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT7" t="str">
+        <f>IF($Y7&gt;=$BN7,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU7">
+        <f>MAX(0,$BP7-$BQ7)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="n">
@@ -9992,16 +11049,16 @@
         <v/>
       </c>
       <c r="V8" s="12">
-        <f>IF($B8="BIG_SIDE",IFERROR(MIN($D8,MAX(0,$T8/$U8)),0),0)</f>
+        <f>$BQ8</f>
         <v>0</v>
       </c>
       <c r="W8" s="12">
-        <f>IF($B8="BIG_SIDE",MAX(0,$D8-$V8),$AJ8)</f>
+        <f>IF($B8="BIG_SIDE",$BR8,$AJ8)</f>
         <v/>
       </c>
       <c r="X8" s="19">
         <f>IF($B8="BIG_SIDE",IF($AX$8&gt;0,$AX$8*Settings!$B$6,0),IF($S$8&gt;0,$S$8*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y8" s="19">
         <f>IF(ROW()=2,$X8,$Y7+$X8)</f>
@@ -10084,11 +11141,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS8" s="20">
-        <f>IF($B8="BIG_SIDE",$V8*$U8,0)</f>
+        <f>IF($B8="BIG_SIDE",$BQ8*$U8,0)</f>
         <v>0</v>
       </c>
       <c r="AT8" s="12">
-        <f>IF($B8="BIG_SIDE",$G8+$J8+$V8,IF($B8="SMALL_SIDE",$J8+$AL8+$AV8,0))</f>
+        <f>IF($B8="BIG_SIDE",$G8+$J8+$BQ8,IF($B8="SMALL_SIDE",$J8+$AL8+$AV8,0))</f>
         <v/>
       </c>
       <c r="AU8" s="12">
@@ -10158,21 +11215,45 @@
         <v/>
       </c>
       <c r="BL8">
-        <f>IF($D8&gt;0,IFERROR($V8/$D8,0),0)</f>
+        <f>IF($D8&gt;0,IFERROR($BQ8/$D8,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM8" t="b">
-        <f>IF($BN8&lt;=0,FALSE,$Y8&gt;=$BN8)</f>
+        <f>$BT8</f>
         <v>0</v>
       </c>
       <c r="BN8">
-        <f>MAX(0,$W8*$BI8*Settings!$B$9)</f>
+        <f>MAX(0,$BR8*$BI8*Settings!$B$9)</f>
         <v>306.12</v>
       </c>
       <c r="BO8">
         <f>$Y8-$BN8</f>
         <v>-306.12</v>
       </c>
+      <c r="BP8">
+        <f>IF($B8="BIG_SIDE",IFERROR($T8/$U8,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ8">
+        <f>IF($B8="BIG_SIDE",MIN($D8,FLOOR(MAX(0,$BP8),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR8">
+        <f>IF($B8="BIG_SIDE",MAX(0,$D8-$BQ8),$AJ8)</f>
+        <v>1.5306</v>
+      </c>
+      <c r="BS8" t="str">
+        <f>IF(AND($BP8&gt;0,$BP8&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT8" t="str">
+        <f>IF($Y8&gt;=$BN8,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU8">
+        <f>MAX(0,$BP8-$BQ8)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="n">
@@ -10259,16 +11340,16 @@
         <v/>
       </c>
       <c r="V9" s="12">
-        <f>IF($B9="BIG_SIDE",IFERROR(MIN($D9,MAX(0,$T9/$U9)),0),0)</f>
+        <f>$BQ9</f>
         <v>0</v>
       </c>
       <c r="W9" s="12">
-        <f>IF($B9="BIG_SIDE",MAX(0,$D9-$V9),$AJ9)</f>
+        <f>IF($B9="BIG_SIDE",$BR9,$AJ9)</f>
         <v/>
       </c>
       <c r="X9" s="19">
         <f>IF($B9="BIG_SIDE",IF($AX$9&gt;0,$AX$9*Settings!$B$6,0),IF($S$9&gt;0,$S$9*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y9" s="19">
         <f>IF(ROW()=2,$X9,$Y8+$X9)</f>
@@ -10351,11 +11432,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS9" s="20">
-        <f>IF($B9="BIG_SIDE",$V9*$U9,0)</f>
+        <f>IF($B9="BIG_SIDE",$BQ9*$U9,0)</f>
         <v>0</v>
       </c>
       <c r="AT9" s="12">
-        <f>IF($B9="BIG_SIDE",$G9+$J9+$V9,IF($B9="SMALL_SIDE",$J9+$AL9+$AV9,0))</f>
+        <f>IF($B9="BIG_SIDE",$G9+$J9+$BQ9,IF($B9="SMALL_SIDE",$J9+$AL9+$AV9,0))</f>
         <v/>
       </c>
       <c r="AU9" s="12">
@@ -10425,21 +11506,45 @@
         <v/>
       </c>
       <c r="BL9">
-        <f>IF($D9&gt;0,IFERROR($V9/$D9,0),0)</f>
+        <f>IF($D9&gt;0,IFERROR($BQ9/$D9,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM9" t="b">
-        <f>IF($BN9&lt;=0,FALSE,$Y9&gt;=$BN9)</f>
+        <f>$BT9</f>
         <v>0</v>
       </c>
       <c r="BN9">
-        <f>MAX(0,$W9*$BI9*Settings!$B$9)</f>
+        <f>MAX(0,$BR9*$BI9*Settings!$B$9)</f>
         <v>306.12</v>
       </c>
       <c r="BO9">
         <f>$Y9-$BN9</f>
         <v>-306.12</v>
       </c>
+      <c r="BP9">
+        <f>IF($B9="BIG_SIDE",IFERROR($T9/$U9,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ9">
+        <f>IF($B9="BIG_SIDE",MIN($D9,FLOOR(MAX(0,$BP9),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR9">
+        <f>IF($B9="BIG_SIDE",MAX(0,$D9-$BQ9),$AJ9)</f>
+        <v>1.5306</v>
+      </c>
+      <c r="BS9" t="str">
+        <f>IF(AND($BP9&gt;0,$BP9&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT9" t="str">
+        <f>IF($Y9&gt;=$BN9,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU9">
+        <f>MAX(0,$BP9-$BQ9)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="n">
@@ -10455,7 +11560,7 @@
       </c>
       <c r="D10" s="13">
         <f>IF($B10="BLOCKED",0,IF(AND($AQ9="MANUAL_READY",$BG9="YES"),MAX($BA9,$BB9),IF($AP9="YES",MAX(0,$AG9),$D9)))</f>
-        <v/>
+        <v>0.1</v>
       </c>
       <c r="E10" s="12">
         <f>IF($B10="BLOCKED","",IF($C10="SELL","BUY","SELL"))</f>
@@ -10526,16 +11631,16 @@
         <v/>
       </c>
       <c r="V10" s="12">
-        <f>IF($B10="BIG_SIDE",IFERROR(MIN($D10,MAX(0,$T10/$U10)),0),0)</f>
+        <f>$BQ10</f>
         <v>0</v>
       </c>
       <c r="W10" s="12">
-        <f>IF($B10="BIG_SIDE",MAX(0,$D10-$V10),$AJ10)</f>
+        <f>IF($B10="BIG_SIDE",$BR10,$AJ10)</f>
         <v/>
       </c>
       <c r="X10" s="19">
         <f>IF($B10="BIG_SIDE",IF($AX$10&gt;0,$AX$10*Settings!$B$6,0),IF($S$10&gt;0,$S$10*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y10" s="19">
         <f>IF(ROW()=2,$X10,$Y9+$X10)</f>
@@ -10618,11 +11723,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS10" s="20">
-        <f>IF($B10="BIG_SIDE",$V10*$U10,0)</f>
+        <f>IF($B10="BIG_SIDE",$BQ10*$U10,0)</f>
         <v>0</v>
       </c>
       <c r="AT10" s="12">
-        <f>IF($B10="BIG_SIDE",$G10+$J10+$V10,IF($B10="SMALL_SIDE",$J10+$AL10+$AV10,0))</f>
+        <f>IF($B10="BIG_SIDE",$G10+$J10+$BQ10,IF($B10="SMALL_SIDE",$J10+$AL10+$AV10,0))</f>
         <v/>
       </c>
       <c r="AU10" s="12">
@@ -10692,21 +11797,45 @@
         <v/>
       </c>
       <c r="BL10">
-        <f>IF($D10&gt;0,IFERROR($V10/$D10,0),0)</f>
+        <f>IF($D10&gt;0,IFERROR($BQ10/$D10,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM10" t="b">
-        <f>IF($BN10&lt;=0,FALSE,$Y10&gt;=$BN10)</f>
+        <f>$BT10</f>
         <v>0</v>
       </c>
       <c r="BN10">
-        <f>MAX(0,$W10*$BI10*Settings!$B$9)</f>
+        <f>MAX(0,$BR10*$BI10*Settings!$B$9)</f>
         <v>306.12</v>
       </c>
       <c r="BO10">
         <f>$Y10-$BN10</f>
         <v>-306.12</v>
       </c>
+      <c r="BP10">
+        <f>IF($B10="BIG_SIDE",IFERROR($T10/$U10,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ10">
+        <f>IF($B10="BIG_SIDE",MIN($D10,FLOOR(MAX(0,$BP10),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR10">
+        <f>IF($B10="BIG_SIDE",MAX(0,$D10-$BQ10),$AJ10)</f>
+        <v>1.5306</v>
+      </c>
+      <c r="BS10" t="str">
+        <f>IF(AND($BP10&gt;0,$BP10&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT10" t="str">
+        <f>IF($Y10&gt;=$BN10,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU10">
+        <f>MAX(0,$BP10-$BQ10)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="n">
@@ -10793,16 +11922,16 @@
         <v/>
       </c>
       <c r="V11" s="12">
-        <f>IF($B11="BIG_SIDE",IFERROR(MIN($D11,MAX(0,$T11/$U11)),0),0)</f>
+        <f>$BQ11</f>
         <v>0</v>
       </c>
       <c r="W11" s="12">
-        <f>IF($B11="BIG_SIDE",MAX(0,$D11-$V11),$AJ11)</f>
+        <f>IF($B11="BIG_SIDE",$BR11,$AJ11)</f>
         <v/>
       </c>
       <c r="X11" s="19">
         <f>IF($B11="BIG_SIDE",IF($AX$11&gt;0,$AX$11*Settings!$B$6,0),IF($S$11&gt;0,$S$11*Settings!$B$6,0))</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y11" s="19">
         <f>IF(ROW()=2,$X11,$Y10+$X11)</f>
@@ -10885,11 +12014,11 @@
         <v>Заблокировано: DUAL_TAIL сохраняет оба хвоста до ручного закрытия</v>
       </c>
       <c r="AS11" s="20">
-        <f>IF($B11="BIG_SIDE",$V11*$U11,0)</f>
+        <f>IF($B11="BIG_SIDE",$BQ11*$U11,0)</f>
         <v>0</v>
       </c>
       <c r="AT11" s="12">
-        <f>IF($B11="BIG_SIDE",$G11+$J11+$V11,IF($B11="SMALL_SIDE",$J11+$AL11+$AV11,0))</f>
+        <f>IF($B11="BIG_SIDE",$G11+$J11+$BQ11,IF($B11="SMALL_SIDE",$J11+$AL11+$AV11,0))</f>
         <v/>
       </c>
       <c r="AU11" s="12">
@@ -10959,20 +12088,44 @@
         <v/>
       </c>
       <c r="BL11">
-        <f>IF($D11&gt;0,IFERROR($V11/$D11,0),0)</f>
+        <f>IF($D11&gt;0,IFERROR($BQ11/$D11,0),0)</f>
         <v>0</v>
       </c>
       <c r="BM11" t="b">
-        <f>IF($BN11&lt;=0,FALSE,$Y11&gt;=$BN11)</f>
+        <f>$BT11</f>
         <v>0</v>
       </c>
       <c r="BN11">
-        <f>MAX(0,$W11*$BI11*Settings!$B$9)</f>
+        <f>MAX(0,$BR11*$BI11*Settings!$B$9)</f>
         <v>306.12</v>
       </c>
       <c r="BO11">
         <f>$Y11-$BN11</f>
         <v>-306.12</v>
+      </c>
+      <c r="BP11">
+        <f>IF($B11="BIG_SIDE",IFERROR($T11/$U11,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ11">
+        <f>IF($B11="BIG_SIDE",MIN($D11,FLOOR(MAX(0,$BP11),Settings!$B$11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR11">
+        <f>IF($B11="BIG_SIDE",MAX(0,$D11-$BQ11),$AJ11)</f>
+        <v>1.5306</v>
+      </c>
+      <c r="BS11" t="str">
+        <f>IF(AND($BP11&gt;0,$BP11&lt;Settings!$B$11),"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BT11" t="str">
+        <f>IF($Y11&gt;=$BN11,"YES","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="BU11">
+        <f>MAX(0,$BP11-$BQ11)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -11012,7 +12165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -11748,11 +12901,11 @@
       </c>
       <c r="C38">
         <f>SUM(Calculator!AS2:AS11,Trend_UP!AS2:AS11,Trend_DOWN!AS2:AS11)</f>
-        <v>74.7</v>
+        <v>74</v>
       </c>
       <c r="D38">
         <f>C38</f>
-        <v>74.7</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39">
@@ -11788,11 +12941,11 @@
       </c>
       <c r="C40">
         <f>LOOKUP(2,1/(Calculator!W2:W11&lt;&gt;""),Calculator!W2:W11)</f>
-        <v>0.6265</v>
+        <v>0.63</v>
       </c>
       <c r="D40">
         <f>C40</f>
-        <v>0.6265</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="41">
@@ -11808,11 +12961,11 @@
       </c>
       <c r="C41">
         <f>LOOKUP(2,1/(Calculator!BN2:BN11&lt;&gt;""),Calculator!BN2:BN11)</f>
-        <v>125.3</v>
+        <v>126</v>
       </c>
       <c r="D41">
         <f>C41</f>
-        <v>125.3</v>
+        <v>126</v>
       </c>
     </row>
     <row r="42">
@@ -11848,11 +13001,131 @@
       </c>
       <c r="C43">
         <f>LOOKUP(2,1/(Calculator!BO2:BO11&lt;&gt;""),Calculator!BO2:BO11)</f>
-        <v>-117</v>
+        <v>-117.7</v>
       </c>
       <c r="D43">
         <f>C43</f>
-        <v>-117</v>
+        <v>-117.7</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Total CloseFarLotRaw</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>LotStep Rounding Risk Checks</t>
+        </is>
+      </c>
+      <c r="C44">
+        <f>SUM(Calculator!BP2:BP11,Trend_UP!BP2:BP11,Trend_DOWN!BP2:BP11)</f>
+        <v>0.3735</v>
+      </c>
+      <c r="D44">
+        <f>C44</f>
+        <v>0.3735</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Total CloseFarLotRounded</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>LotStep Rounding Risk Checks</t>
+        </is>
+      </c>
+      <c r="C45">
+        <f>SUM(Calculator!BQ2:BQ11,Trend_UP!BQ2:BQ11,Trend_DOWN!BQ2:BQ11)</f>
+        <v>0.37</v>
+      </c>
+      <c r="D45">
+        <f>C45</f>
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Total LostToRounding</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>LotStep Rounding Risk Checks</t>
+        </is>
+      </c>
+      <c r="C46">
+        <f>SUM(Calculator!BU2:BU11,Trend_UP!BU2:BU11,Trend_DOWN!BU2:BU11)</f>
+        <v>0.0035</v>
+      </c>
+      <c r="D46">
+        <f>C46</f>
+        <v>0.0035</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Final FarRemainAfterRounded</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>LotStep Rounding Risk Checks</t>
+        </is>
+      </c>
+      <c r="C47">
+        <f>LOOKUP(2,1/(Calculator!BR2:BR11&lt;&gt;""),Calculator!BR2:BR11)</f>
+        <v>0.63</v>
+      </c>
+      <c r="D47">
+        <f>C47</f>
+        <v>0.63</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>CannotCloseBelowLotStep Count</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>LotStep Rounding Risk Checks</t>
+        </is>
+      </c>
+      <c r="C48">
+        <f>COUNTIF(Calculator!BS2:BS11,"YES")+COUNTIF(Trend_UP!BS2:BS11,"YES")+COUNTIF(Trend_DOWN!BS2:BS11,"YES")</f>
+        <v>1</v>
+      </c>
+      <c r="D48">
+        <f>C48</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>FinalCloseAllowed Count</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>LotStep Rounding Risk Checks</t>
+        </is>
+      </c>
+      <c r="C49">
+        <f>COUNTIF(Calculator!BT2:BT11,"YES")+COUNTIF(Trend_UP!BT2:BT11,"YES")+COUNTIF(Trend_DOWN!BT2:BT11,"YES")</f>
+        <v>0</v>
+      </c>
+      <c r="D49">
+        <f>C49</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>